<commit_message>
vault backup: 2026-09-27 19:11:33
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shaah\Documents\Obsidian Vault\FYP\Matrices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{968AD984-5C3B-40A3-820D-DD7A88531EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BA16D0A-8F77-42CC-B70D-F1D6754C160D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Literature Survey" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1755" uniqueCount="1489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1938" uniqueCount="1638">
   <si>
     <t>Term</t>
   </si>
@@ -3978,7 +3978,7 @@
     <t>Verified - fetched the endpoint or page myself</t>
   </si>
   <si>
-    <t>Technical/valuation agent; trader agent; simulated exchange (volume profile).</t>
+    <t>A_T technical and A_L liquidity (price, volume, turnover), plus the friction-aware evaluation layer, which is gated on exactly the same data.</t>
   </si>
   <si>
     <t>The only source with real per-ticker CSE coverage. Free, no auth, and the announcement endpoints are also how I discover the annual report PDFs.</t>
@@ -3993,6 +3993,54 @@
     <t>There is effectively no alternative. Yahoo and Investing.com are index-only, EODHD's CSE exchange code is contaminated, and TradingView has no free export. Build a local archive from day one and probe chartData depth in week one, because if the history is too short the whole RL design has to change.</t>
   </si>
   <si>
+    <t>D02</t>
+  </si>
+  <si>
+    <t>cse.lk Python package</t>
+  </si>
+  <si>
+    <t>PyPI (community)</t>
+  </si>
+  <si>
+    <t>https://pypi.org/project/cse.lk/</t>
+  </si>
+  <si>
+    <t>CSE, wraps D01.</t>
+  </si>
+  <si>
+    <t>Ingestion tooling.</t>
+  </si>
+  <si>
+    <t>Same as D01.</t>
+  </si>
+  <si>
+    <t>Wraps 13+ CSE endpoints.</t>
+  </si>
+  <si>
+    <t>pip install. Python 3.8+.</t>
+  </si>
+  <si>
+    <t>MIT. One of the clean licences - see the Read Me for the full list.</t>
+  </si>
+  <si>
+    <t>Inherits every limitation of D01, including no OHLCV and unknown history depth.</t>
+  </si>
+  <si>
+    <t>Ingestion layer for A_T and A_L.</t>
+  </si>
+  <si>
+    <t>Fastest route to a working prototype, and MIT-licensed so it's safe to build on. Marked Production/Stable.</t>
+  </si>
+  <si>
+    <t>Thin wrapper - it doesn't solve any of D01's underlying problems.</t>
+  </si>
+  <si>
+    <t>USE - ingestion wrapper</t>
+  </si>
+  <si>
+    <t>No reason to hand-roll the HTTP layer when a stable MIT-licensed wrapper exists. Just don't mistake it for a different data source.</t>
+  </si>
+  <si>
     <t>D03</t>
   </si>
   <si>
@@ -4035,7 +4083,7 @@
     <t>Snapshot only on the free tier - no historical series.</t>
   </si>
   <si>
-    <t>Universe construction for every agent.</t>
+    <t>Universe construction for all four agents.</t>
   </si>
   <si>
     <t>The best free confirmation of the complete CSE ticker universe I found. 296 names with market caps is exactly what I need to define the investable set.</t>
@@ -4089,7 +4137,7 @@
     <t>No programmatic access without paying, so it can't be part of an automated pipeline.</t>
   </si>
   <si>
-    <t>Manual cross-check for the technical agent.</t>
+    <t>Manual cross-check for A_T. Confirmed ten years of depth at index level.</t>
   </si>
   <si>
     <t>Best third-party per-stock CSE coverage I confirmed, and useful for eyeballing whether D01's numbers look right.</t>
@@ -4140,7 +4188,7 @@
     <t>Index only, and the useful access is paywalled.</t>
   </si>
   <si>
-    <t>Risk/volatility agent (long ASPI history for regime analysis).</t>
+    <t>A_V volatility and risk - long index history for the persistence estimates and regime splitting.</t>
   </si>
   <si>
     <t>1993-2026 daily index history would comfortably support the walk-forward scheme and regime decomposition, which is exactly what D01's unknown depth might not.</t>
@@ -4191,7 +4239,7 @@
     <t>Index-only coverage is the killer. One Sri Lankan equity listed.</t>
   </si>
   <si>
-    <t>Risk/volatility agent, as a cross-check on index series.</t>
+    <t>A_V, as a cross-check on the index series.</t>
   </si>
   <si>
     <t>Gives proper OHLCV at index level, which D01 does not.</t>
@@ -4251,7 +4299,7 @@
     <t>No XBRL, so nothing is machine-structured. Report layout varies considerably company to company. Older filings more likely to be scanned rather than text-native, which is exactly the OCR failure mode P07 warns breaks element-based chunking.</t>
   </si>
   <si>
-    <t>Fundamental analyst agent (RAG).</t>
+    <t>A_F fundamental. After the September 2026 scope decision this is the framework's only text modality, so it carries the heterogeneity claim in the main gap.</t>
   </si>
   <si>
     <t>The best-provisioned component of the whole project. Text-native full-statement PDFs for every listed company on an open CDN - I verified one end to end (Office Equipment PLC FY2025, full audited statements).</t>
@@ -4263,7 +4311,7 @@
     <t>USE - primary RAG corpus</t>
   </si>
   <si>
-    <t>This is what G4 is built on. Text-native PDFs mean element-based chunking (P07) has something real to work with, and the variance in layout across companies is precisely what makes testing whether SEC-derived methods transfer an actual research question rather than a formality.</t>
+    <t>This is what A_F is built on, and after the scope cut it is the framework's only text channel rather than a demoted system feature. Text-native PDFs mean element-based chunking has something real to work with. The architectural novelty is closed by the 2025 CSE Neo4j Graph-RAG work (Shamila, Silva and Talagala, ERU 2025, DOI 10.31705/ERU.2025.35), now verified, so what remains for A_F is numeric statement extraction, point-in-time correctness and the orchestration that consumes the signal. Every document needs a publication-date field and a retrieval filter keyed to the simulation clock, because their graph is a static snapshot with no as-of field and that is a lookahead hazard in a backtest rather than an inconvenience.</t>
   </si>
   <si>
     <t>D08</t>
@@ -4308,7 +4356,7 @@
     <t>Exchange-level only - no company fundamentals.</t>
   </si>
   <si>
-    <t>Background / market microstructure context for G1.</t>
+    <t>None directly. Background for the Sub-gap 1 execution model, market structure and turnover context.</t>
   </si>
   <si>
     <t>Useful for understanding CSE turnover patterns and market structure when I'm designing the simulated exchange.</t>
@@ -4362,7 +4410,7 @@
     <t>Note the domain: cbsl.lk, not cbsl.gov.lk - the .gov.lk/eresearch path 404s. Everything about access format is unconfirmed.</t>
   </si>
   <si>
-    <t>Risk/volatility agent.</t>
+    <t>A_V, and the macro context for regime labelling.</t>
   </si>
   <si>
     <t>If it offers structured downloads it's a much better route than parsing the PDF-only publications (D15).</t>
@@ -4374,7 +4422,7 @@
     <t>EVALUATE FIRST - this decides the macro ingestion design</t>
   </si>
   <si>
-    <t>Worth an hour before committing to a PDF-extraction pipeline, because if this portal exports CSV the whole macro problem gets much easier. The user-guide PDF referenced on the landing page is the place to start.</t>
+    <t>Worth an hour before committing to a PDF-extraction pipeline, because if this portal exports CSV the macro problem gets much easier. Evaluate it ahead of D10 and D11, which are PDF-first. The CSE macro papers confirm the acquisition method is manual in practice, mostly Excel downloads with inflation data transcribed out of PDFs, and name the Department of Census and Statistics as the NCPI source alongside CBSL.</t>
   </si>
   <si>
     <t>D10</t>
@@ -4413,7 +4461,7 @@
     <t>Download formats not stated on the index pages. The treasury-endpoint disallow is a real constraint, not a formality.</t>
   </si>
   <si>
-    <t>Risk/volatility agent; risk-free rate for Sharpe and excess-return calculations.</t>
+    <t>A_V, plus the risk-free rate for Sharpe and excess-return calculations in the evaluation layer.</t>
   </si>
   <si>
     <t>Confirmed categories cover everything I need: CCPI and NCPI inflation, policy rates, exchange rates, SLIBOR, government securities (T-bill and T-bond yields), commercial bank lending and deposit rates, open market operations. P11 uses 91-day T-bill auction rates as the risk-free rate, and those live here.</t>
@@ -4461,30 +4509,51 @@
     <t>PDF only - no Excel or CSV offered. This is a real ingestion cost, not a minor inconvenience.</t>
   </si>
   <si>
+    <t>A_V.</t>
+  </si>
+  <si>
     <t>Comprehensive and current, with a long archive.</t>
   </si>
   <si>
     <t>PDF-first means the risk agent needs a table-extraction pipeline before it can use any of it. Ironically I'd be doing the same structural PDF parsing here that G4 does for company filings.</t>
   </si>
   <si>
-    <t>USE - but check D13 and D10 first</t>
+    <t>USE - but evaluate D09 first</t>
   </si>
   <si>
     <t>If D13 or Lanka Data can supply the same series as structured data, take that route. If not, at least the table-extraction work overlaps with the fundamental agent's pipeline so it's not entirely duplicated effort.</t>
   </si>
   <si>
-    <t>News / social</t>
+    <t>D12</t>
+  </si>
+  <si>
+    <t>D13</t>
+  </si>
+  <si>
+    <t>D14</t>
+  </si>
+  <si>
+    <t>D15</t>
   </si>
   <si>
     <t>Unlabelled.</t>
   </si>
   <si>
+    <t>D16</t>
+  </si>
+  <si>
+    <t>D17</t>
+  </si>
+  <si>
     <t>D18</t>
   </si>
   <si>
     <t>CSE announcements feed</t>
   </si>
   <si>
+    <t>Disclosures</t>
+  </si>
+  <si>
     <t>Via the D01 POST API - 8 announcement categories</t>
   </si>
   <si>
@@ -4512,7 +4581,7 @@
     <t>Historical depth unconfirmed, same as everything else on the CSE API.</t>
   </si>
   <si>
-    <t>News analyst agent; fundamental agent (this is how report PDFs get discovered).</t>
+    <t>A_F. This is how the report PDFs in D07 are discovered, which is the whole reason it survives the scope cut.</t>
   </si>
   <si>
     <t>Primary-source corporate disclosure, which is higher-signal and less ambiguous than news coverage of the same events. Also the discovery mechanism for D11.</t>
@@ -4524,7 +4593,10 @@
     <t>USE - primary disclosure feed</t>
   </si>
   <si>
-    <t>Doubles as the news source and the RAG discovery layer, which makes it the highest-leverage endpoint on the whole CSE API.</t>
+    <t>The only survivor of the news and social block, and it survives for a structural reason rather than a sentimental one: it is a primary disclosure feed, not commentary, and it is how the report PDFs in D07 are discovered. It also carries the timestamp that makes point-in-time retrieval possible - a document is only visible to A_F after the announcement datetime, which is what keeps the backtest free of lookahead. Treat it as metadata and routing for A_F, not as a text signal in its own right.</t>
+  </si>
+  <si>
+    <t>D19</t>
   </si>
   <si>
     <t>D20</t>
@@ -4572,7 +4644,7 @@
     <t>Verified - cloned the repo and parsed the full CSV myself</t>
   </si>
   <si>
-    <t>Technical/valuation agent - backfill for the price archive. Market-cap and issued-quantity series also feed the portfolio-weighting layer.</t>
+    <t>A_T and A_L. The confirmed per-counter archive and currently the single most important row in this sheet.</t>
   </si>
   <si>
     <t>Seventeen months of already-collected daily CSE cross-section, free, and it directly attacks the biggest unknown in this matrix - D01's retention depth - without waiting. Per-day market cap and issued quantity are not available from any other source I checked. The Actions workflow is a working template for my own archiver.</t>
@@ -4629,7 +4701,7 @@
     <t>Verified - cloned and read the source; the extraction has not been re-run end to end since 30 January 2026</t>
   </si>
   <si>
-    <t>Technical/valuation agent - the OHLCV feed D01 cannot provide.</t>
+    <t>A_T. The OHLCV feed D01 cannot provide.</t>
   </si>
   <si>
     <t>The only route in the matrix to true per-ticker OHLCV with an open price and multi-year depth for CSE. It is my own code, so it does not depend on a third party maintaining anything, and alt_scraper.py needs no TradingView account at all.</t>
@@ -4642,6 +4714,381 @@
   </si>
   <si>
     <t>It answers the OHLCV gap nothing else here answers, which is exactly what makes it dangerous - easy to build on, hard to justify. Use it offline to validate D01 and D38 against an independent source, and either obtain written permission or a paid TradingView data plan, or keep it out of the published pipeline. D04 is this same finding without the code attached.</t>
+  </si>
+  <si>
+    <t>CSE Price Index / ASPI ten-year daily series</t>
+  </si>
+  <si>
+    <t>Colombo Stock Exchange official database</t>
+  </si>
+  <si>
+    <t>Via CSE directly; published route evidenced by the 2026 ARIMA study in the Literature Survey sheet</t>
+  </si>
+  <si>
+    <t>CSE, index level only.</t>
+  </si>
+  <si>
+    <t>1 July 2014 to 30 June 2024 is the published, verified span. 2,362 usable observations after differencing and lag adjustment.</t>
+  </si>
+  <si>
+    <t>~2,400 daily observations.</t>
+  </si>
+  <si>
+    <t>Index close. No per-counter fields.</t>
+  </si>
+  <si>
+    <t>Obtained by the source study from the official CSE database and cross-checked against Bloomberg historical series. Acquisition described as manual.</t>
+  </si>
+  <si>
+    <t>Not stated in the source study. CSE data-reuse terms remain unconfirmed and should be resolved in the same written request as everything else.</t>
+  </si>
+  <si>
+    <t>Index level only, so it cannot feed A_T, A_L or the friction model. Spans the Easter attacks, the COVID low of 4,247.95, the January 2022 peak of 13,462.39 and the 2022 crisis, so it contains real trading halts and extended closure periods that a continuous series silently stitches over.</t>
+  </si>
+  <si>
+    <t>Verified in the published record - a 2026 study reports this exact span from the official database.</t>
+  </si>
+  <si>
+    <t>A_V above all. Also the baselines and the regime-split reporting in the evaluation layer.</t>
+  </si>
+  <si>
+    <t>THE INDEX TRACK IS SECURE. Roughly 2,400 daily observations is in the same range as the 2,922 the CSE FIGARCH study used, so Sub-gap 2's persistence estimator can be fitted even if per-counter depth never improves. Three distinct regime episodes for labelling.</t>
+  </si>
+  <si>
+    <t>Index only. Per-regime it splits to roughly 1,500 / 500 / 600 observations, so the COVID window is thin for a fractional differencing estimate even though it is an order of magnitude past the four-month failure case in the literature.</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>USE - the confirmed index track</t>
+  </si>
+  <si>
+    <t>This is the row that de-risks Sub-gap 2. The persistence work does not wait on the per-counter data request. Ask for it by name rather than asking for 'ten years of data', because an index series would satisfy that phrasing and leave A_T, A_L and the friction model no better off.</t>
+  </si>
+  <si>
+    <t>Listing and delisting register with effective dates</t>
+  </si>
+  <si>
+    <t>Reference data</t>
+  </si>
+  <si>
+    <t>Not located. Part of the CSE R&amp;D request.</t>
+  </si>
+  <si>
+    <t>CSE, all counters including those no longer listed.</t>
+  </si>
+  <si>
+    <t>Tradability mask. Reference table.</t>
+  </si>
+  <si>
+    <t>As far back as the archive goes.</t>
+  </si>
+  <si>
+    <t>Event-level.</t>
+  </si>
+  <si>
+    <t>Unknown.</t>
+  </si>
+  <si>
+    <t>None directly - this is the mask applied to the price data.</t>
+  </si>
+  <si>
+    <t>Listing date, delisting date, and reason where available.</t>
+  </si>
+  <si>
+    <t>Not available through any route identified so far. The cse.lk API almost certainly serves only currently-listed counters.</t>
+  </si>
+  <si>
+    <t>Unconfirmed.</t>
+  </si>
+  <si>
+    <t>Unobtained. Without it every backtest on this market is survivorship-biased by an unmeasured amount, and the bias flatters returns.</t>
+  </si>
+  <si>
+    <t>REQUIRED, NOT OBTAINED.</t>
+  </si>
+  <si>
+    <t>All four agents, via the universe definition, plus the evaluation layer.</t>
+  </si>
+  <si>
+    <t>A counter should leave the investable universe on the day it delisted, not retrospectively for the whole sample. This is the tradability-mask correction that the diversified-portfolio framework in the Literature Survey sheet builds explicitly from membership history, and whose absence is flagged there as a possible thirty-year survivorship filter in a comparable study.</t>
+  </si>
+  <si>
+    <t>May be unobtainable. The counters that delisted through the 2022 default and currency collapse are disproportionately the ones that failed, and they are also disproportionately thin - which is exactly the part of the book Sub-gap 1 is about, so excluding them removes the phenomenon under study.</t>
+  </si>
+  <si>
+    <t>REQUIRED - ask for it explicitly; if refused, state the bias and its direction</t>
+  </si>
+  <si>
+    <t>If it cannot be obtained, the honest move is to write that the universe is survivorship-biased because delisted counters were not retrievable, which flatters reported returns by an unmeasured amount. That is a limitation an examiner accepts; an unmentioned one is not. Even the delisting DATES alone, without price history, would let the size of the missing universe be quantified.</t>
+  </si>
+  <si>
+    <t>Counter liquidity screen and tier table</t>
+  </si>
+  <si>
+    <t>Derived dataset</t>
+  </si>
+  <si>
+    <t>Own computation over D20</t>
+  </si>
+  <si>
+    <t>Derived from the D20 archive</t>
+  </si>
+  <si>
+    <t>CSE, all counters present in the archive.</t>
+  </si>
+  <si>
+    <t>Derived reference table sizing every downstream component.</t>
+  </si>
+  <si>
+    <t>The D20 span, 2025-04-10 to 2026-09-18.</t>
+  </si>
+  <si>
+    <t>Per counter.</t>
+  </si>
+  <si>
+    <t>374 trading days across roughly 300 counters in the source archive.</t>
+  </si>
+  <si>
+    <t>Per counter: trading-day frequency (share of days with volume greater than zero), median daily turnover in LKR, Amihud mean of absolute return over turnover, and zero-return frequency reported separately from non-trading.</t>
+  </si>
+  <si>
+    <t>Liquidity tier per counter.</t>
+  </si>
+  <si>
+    <t>One pass over data already held. No external dependency, no permission required.</t>
+  </si>
+  <si>
+    <t>n/a - derived.</t>
+  </si>
+  <si>
+    <t>A genuine flat print and a stale carry-forward both read as a zero return in a close-only series and are completely different events, so the screen must test volume rather than price change. One year is also one liquidity regime, so a screen fixed on it is not valid for a longer backtest and must be re-run inside each training fold.</t>
+  </si>
+  <si>
+    <t>Not yet computed.</t>
+  </si>
+  <si>
+    <t>Sizes A_T, calibrates A_L, and sets the friction model's scale. Also the first empirical fit of the L_t conditioning variable.</t>
+  </si>
+  <si>
+    <t>The cheapest high-value computation available and it needs nothing that is not already held. It answers the question the cross-sectional reframe actually turns on, which is how many counters clear a liquidity screen rather than how many years of history exist. It is also a publishable CSE liquidity statistic in its own right.</t>
+  </si>
+  <si>
+    <t>Do not reduce it to a single threshold. Screening for liquid counters removes the thin-book conditions Sub-gap 1 is about, so report results BY TIER and let the cutoff become a result rather than a choice. That also aligns with the CSE finding that small caps are more exposed to illiquidity shocks than large, at -0.071 against -0.060.</t>
+  </si>
+  <si>
+    <t>COMPUTE NEXT - no dependency on the data request</t>
+  </si>
+  <si>
+    <t>At a 30-day lookback the D20 archive gives roughly 345 usable windows per counter, so with ~300 counters the sequence count is around 100,000, materially better than the earlier ~240-day working assumption. The tier table converts that headline into a per-tier figure, which is what actually sizes the model.</t>
+  </si>
+  <si>
+    <t>University of Moratuwa CSE Graph-RAG corpus and code</t>
+  </si>
+  <si>
+    <t>Shamila, Silva and Talagala, Dept of Computer Science and Engineering, University of Moratuwa</t>
+  </si>
+  <si>
+    <t>DOI 10.31705/ERU.2025.35, with a public GitHub repository linked from the paper</t>
+  </si>
+  <si>
+    <t>CSE annual reports. Company count and date range not reported.</t>
+  </si>
+  <si>
+    <t>Prior art for A_F, plus a data-access lead.</t>
+  </si>
+  <si>
+    <t>Not reported in the paper.</t>
+  </si>
+  <si>
+    <t>Document level.</t>
+  </si>
+  <si>
+    <t>Over 6,000 unique entities reported, against roughly 280 listed companies.</t>
+  </si>
+  <si>
+    <t>English. CSE annual report PDFs.</t>
+  </si>
+  <si>
+    <t>A Neo4j knowledge graph of corporate structure, governance and ownership. Tabular financial data is explicitly out of scope in their work.</t>
+  </si>
+  <si>
+    <t>Public repository. The authors are at the same university and are reachable.</t>
+  </si>
+  <si>
+    <t>The paper gives NO information on how the CSE documents were obtained, how many companies, or what date range - which is the single most useful thing it could have reported for my purposes.</t>
+  </si>
+  <si>
+    <t>Verified. Two-page extended abstract, ERU Symposium 2025.</t>
+  </si>
+  <si>
+    <t>A_F, as prior art and as adoptable tooling.</t>
+  </si>
+  <si>
+    <t>Closes the architectural novelty of structure-aware retrieval over CSE annual reports, which is settled and not recoverable. More useful to me now as a data-access lead: same department, same university, reachable, with working extraction code.</t>
+  </si>
+  <si>
+    <t>A two-page abstract, so the pipeline constants are adoptable as defaults but not as validated settings. Their graph is a static snapshot with no as-of field.</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>USE as prior art and as tooling; CONTACT the authors</t>
+  </si>
+  <si>
+    <t>The best warm route to the CSE data-access question. A local research group that already extracted CSE annual reports at scale knows how they got them, and that is worth an email before the formal R&amp;D request rather than after.</t>
+  </si>
+  <si>
+    <t>FinQA</t>
+  </si>
+  <si>
+    <t>Benchmark</t>
+  </si>
+  <si>
+    <t>Chen et al., EMNLP 2021</t>
+  </si>
+  <si>
+    <t>https://github.com/czyssrs/FinQA</t>
+  </si>
+  <si>
+    <t>US filings, English.</t>
+  </si>
+  <si>
+    <t>Development artefact for A_F. Tables plus text.</t>
+  </si>
+  <si>
+    <t>n/a.</t>
+  </si>
+  <si>
+    <t>Question level.</t>
+  </si>
+  <si>
+    <t>Built over FinTabNet.</t>
+  </si>
+  <si>
+    <t>Question, answer, and an executable reasoning program.</t>
+  </si>
+  <si>
+    <t>Public GitHub.</t>
+  </si>
+  <si>
+    <t>CDLA-Permissive via FinTabNet. The cleanest licence of the A_F development set.</t>
+  </si>
+  <si>
+    <t>US filings with page-local, pre-located context and no as-of notion, so it does not transfer to CSE documents as data.</t>
+  </si>
+  <si>
+    <t>Verified.</t>
+  </si>
+  <si>
+    <t>A_F, development and the C_F,t confidence signal.</t>
+  </si>
+  <si>
+    <t>Pull the DSL and the program executor directly rather than reimplement. Supplies the retrieve-then-program architecture and, importantly, a structural confidence signal for A_F: whether the program parses under the grammar, whether every argument traces to a retrieved number, and program step count as a calibrated difficulty proxy at 67.61 / 59.08 / 22.78 per cent for one, two and three-plus steps.</t>
+  </si>
+  <si>
+    <t>Not usable as a CSE evaluation set. Its 61.24 / 91.16 difficulty prior is explicitly non-portable and should be cited as an order of magnitude, never as a target.</t>
+  </si>
+  <si>
+    <t>USE - A_F development only</t>
+  </si>
+  <si>
+    <t>The planning band agreed across three independent papers is below 50% on computed quantities over CSE filings, nearer 40% than 60% on first build. A_F is expected to be unusable more often than not, and the orchestrator has to be designed for a channel that is frequently unusable rather than occasionally imperfect.</t>
+  </si>
+  <si>
+    <t>ConvFinQA and TAT-QA</t>
+  </si>
+  <si>
+    <t>Chen et al., EMNLP 2022; Zhu et al., ACL-IJCNLP 2021</t>
+  </si>
+  <si>
+    <t>https://github.com/czyssrs/ConvFinQA and https://nextplusplus.github.io/TAT-QA</t>
+  </si>
+  <si>
+    <t>Development artefacts and taxonomy for A_F.</t>
+  </si>
+  <si>
+    <t>ConvFinQA: 3,037 / 421 / 434 conversations. TAT-QA: hybrid table-and-text questions.</t>
+  </si>
+  <si>
+    <t>ConvFinQA adds multi-turn context; TAT-QA adds a scale taxonomy of None / Thousand / Million / Billion / Percent and an answer-type by answer-source split.</t>
+  </si>
+  <si>
+    <t>Public.</t>
+  </si>
+  <si>
+    <t>ConvFinQA inherits FinTabNet. TAT-QA is public for NON-COMMERCIAL USE ONLY - the one explicit restriction in the A_F set.</t>
+  </si>
+  <si>
+    <t>Same non-transferability as D26.</t>
+  </si>
+  <si>
+    <t>A_F, probe-set design and taxonomy.</t>
+  </si>
+  <si>
+    <t>ConvFinQA pairs with FinQA as one probe corpus with and without conversational context, which is the cheapest available ablation on whether a reference-resolution layer does anything. TAT-QA's scale taxonomy and two-round validation pattern lift directly into the CSE probe-set design and are affordable at ten to twenty questions.</t>
+  </si>
+  <si>
+    <t>Neither is a CSE evaluation set. TAT-QA's operator accuracy runs from 100.0 down to 0.0 across classes, so a single posterior is not comparable across classes without per-operator reliability estimated on my own probe set.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>USE - taxonomy and probe design</t>
+  </si>
+  <si>
+    <t>The convergent conclusion across the benchmark papers is the same: build a hand-checked probe set of ten to twenty questions over a handful of CSE annual reports, stratified by reasoning type and answer source, scored on the four-state taxonomy of correct, incorrect, failure-to-answer and no parseable answer.</t>
+  </si>
+  <si>
+    <t>Level-III message data and multi-level depth for CSE</t>
+  </si>
+  <si>
+    <t>Microstructure</t>
+  </si>
+  <si>
+    <t>Not located. cse.lk/api/chartData almost certainly does not expose it.</t>
+  </si>
+  <si>
+    <t>CSE, per counter.</t>
+  </si>
+  <si>
+    <t>Order-book microstructure.</t>
+  </si>
+  <si>
+    <t>Tick or message level.</t>
+  </si>
+  <si>
+    <t>Order arrival, market order and cancellation intensities by queue size, or at minimum multi-level depth snapshots.</t>
+  </si>
+  <si>
+    <t>Not available through any identified route. Whether the CSE exposes anything below top-of-book is unknown.</t>
+  </si>
+  <si>
+    <t>Assessed as almost certainly out of reach. The queue-reactive execution simulator in the literature needs order-level message data; the deep LOB model needs ten levels per side tick-by-tick plus roughly 7,192 GPU hours in its own evidentiary standard.</t>
+  </si>
+  <si>
+    <t>Not obtained; judged unlikely.</t>
+  </si>
+  <si>
+    <t>A_L and the friction-aware evaluation layer, which are gated on exactly the same data and should therefore be one workstream and one request.</t>
+  </si>
+  <si>
+    <t>There is a decisive and nearly free fallback that runs FIRST: the tick-size classification needs only the best bid, the best ask and the exchange's tick schedule. If liquid CSE counters come out small-tick, the microstructural route is ruled out at almost no cost and the friction work becomes daily-bar-based by necessity rather than by preference.</t>
+  </si>
+  <si>
+    <t>If none of it is observable, A_L falls back to turnover, traded value, zero-return frequency and Amihud-style measures from daily bars, and the friction model falls back to a parametric temporary and permanent impact model calibrated against observed turnover and daily price moves. Weaker, but honest.</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>EVALUATE via the top-of-book tick test first</t>
+  </si>
+  <si>
+    <t>Fold the level-III feature list and the queue-intensity calibration data into the SAME written request rather than two, because whatever cannot be observed also cannot be simulated, and the depth of the request determines how strong both A_L and the evaluation layer can be.</t>
   </si>
 </sst>
 </file>
@@ -4693,9 +5140,7 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4803,9 +5248,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -4875,15 +5319,14 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -9451,10 +9894,10 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9648,16 +10091,11 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.21875" customWidth="1"/>
-    <col min="6" max="6" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="5" width="30.21875" customWidth="1"/>
+    <col min="6" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -9795,7 +10233,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:W14"/>
+  <dimension ref="A1:W22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" bestFit="1" customWidth="1"/>
@@ -9955,291 +10393,291 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="396" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:23" ht="224.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>1272</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>1273</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>1253</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>1274</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="5" t="s">
         <v>1275</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="5" t="s">
         <v>1276</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="5" t="s">
         <v>1277</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="5" t="s">
         <v>1278</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="5" t="s">
+        <v>1278</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>1279</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="5" t="s">
+        <v>1278</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>1280</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="O3" s="5" t="s">
         <v>1281</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="P3" s="5" t="s">
         <v>1282</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="Q3" s="5" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>1283</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>1284</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>1285</v>
+      </c>
+      <c r="U3" s="9">
+        <v>4</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>1286</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="396" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>1290</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>1291</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>1292</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>1294</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>1295</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>1296</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>1298</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="N3" s="3" t="s">
-        <v>1283</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>1284</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>1285</v>
-      </c>
-      <c r="Q3" s="3" t="s">
+      <c r="N4" s="3" t="s">
+        <v>1299</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>1300</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>1301</v>
+      </c>
+      <c r="Q4" s="3" t="s">
         <v>1266</v>
       </c>
-      <c r="R3" s="3" t="s">
-        <v>1286</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>1287</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>1288</v>
-      </c>
-      <c r="U3" s="8">
+      <c r="R4" s="3" t="s">
+        <v>1302</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>1303</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>1304</v>
+      </c>
+      <c r="U4" s="8">
         <v>4</v>
       </c>
-      <c r="V3" s="7" t="s">
-        <v>1289</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>1290</v>
+      <c r="V4" s="7" t="s">
+        <v>1305</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>1306</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="277.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>1292</v>
-      </c>
-      <c r="C4" s="5" t="s">
+    <row r="5" spans="1:23" ht="277.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>1253</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>1293</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>1294</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="D5" s="5" t="s">
+        <v>1309</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>1310</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>1311</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>1312</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>1313</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>1314</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>1315</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>1316</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>1317</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>1318</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>1319</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>1320</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>1321</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>1322</v>
+      </c>
+      <c r="U5" s="9">
+        <v>2</v>
+      </c>
+      <c r="V5" s="6" t="s">
+        <v>1323</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>1324</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>1328</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>1330</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>1331</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>1295</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>1296</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>1297</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>1298</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>1299</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>1300</v>
-      </c>
-      <c r="L4" s="5" t="s">
+      <c r="J6" s="3" t="s">
+        <v>1332</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>1333</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="N4" s="5" t="s">
-        <v>1301</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>1302</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>1303</v>
-      </c>
-      <c r="Q4" s="5" t="s">
+      <c r="N6" s="3" t="s">
+        <v>1334</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>1335</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>1336</v>
+      </c>
+      <c r="Q6" s="3" t="s">
         <v>1266</v>
       </c>
-      <c r="R4" s="5" t="s">
-        <v>1304</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>1305</v>
-      </c>
-      <c r="T4" s="5" t="s">
-        <v>1306</v>
-      </c>
-      <c r="U4" s="9">
-        <v>2</v>
-      </c>
-      <c r="V4" s="6" t="s">
-        <v>1307</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>1308</v>
+      <c r="R6" s="3" t="s">
+        <v>1337</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>1338</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>1339</v>
+      </c>
+      <c r="U6" s="8">
+        <v>3</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>1340</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>1341</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>1310</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>1253</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>1311</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>1312</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>1313</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>1314</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>1315</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>1279</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>1316</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>1317</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>1318</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>1319</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>1320</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>1266</v>
-      </c>
-      <c r="R5" s="3" t="s">
-        <v>1321</v>
-      </c>
-      <c r="S5" s="3" t="s">
-        <v>1322</v>
-      </c>
-      <c r="T5" s="3" t="s">
-        <v>1323</v>
-      </c>
-      <c r="U5" s="8">
-        <v>3</v>
-      </c>
-      <c r="V5" s="6" t="s">
-        <v>1324</v>
-      </c>
-      <c r="W5" s="3" t="s">
-        <v>1325</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" ht="237.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>1326</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>1327</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>1253</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>1328</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>1329</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>1330</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>1331</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>1332</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>1279</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>1333</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>1334</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>1335</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>1336</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>1337</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>1266</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>1338</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>1339</v>
-      </c>
-      <c r="T6" s="5" t="s">
-        <v>1340</v>
-      </c>
-      <c r="U6" s="9">
-        <v>2</v>
-      </c>
-      <c r="V6" s="6" t="s">
-        <v>1307</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>1341</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="330" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" ht="237.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>1342</v>
       </c>
@@ -10247,572 +10685,1136 @@
         <v>1343</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>1344</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>1345</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>1346</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>1347</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="5" t="s">
         <v>1348</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="5" t="s">
+        <v>1295</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>1349</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="K7" s="5" t="s">
         <v>1350</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="L7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="N7" s="5" t="s">
         <v>1351</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="O7" s="5" t="s">
         <v>1352</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="P7" s="5" t="s">
         <v>1353</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>1354</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>1355</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>1356</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>1357</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>1266</v>
       </c>
       <c r="R7" s="5" t="s">
+        <v>1354</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>1355</v>
+      </c>
+      <c r="T7" s="5" t="s">
+        <v>1356</v>
+      </c>
+      <c r="U7" s="9">
+        <v>2</v>
+      </c>
+      <c r="V7" s="6" t="s">
+        <v>1323</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="330" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>1358</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>1359</v>
       </c>
-      <c r="T7" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>1360</v>
       </c>
-      <c r="U7" s="9">
+      <c r="D8" s="5" t="s">
+        <v>1361</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>1362</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>1363</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>1364</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>1365</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>1366</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>1367</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>1368</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>1369</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>1370</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>1371</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>1372</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>1373</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>1374</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>1375</v>
+      </c>
+      <c r="T8" s="5" t="s">
+        <v>1376</v>
+      </c>
+      <c r="U8" s="9">
         <v>5</v>
       </c>
-      <c r="V7" s="7" t="s">
-        <v>1361</v>
-      </c>
-      <c r="W7" s="5" t="s">
-        <v>1362</v>
+      <c r="V8" s="7" t="s">
+        <v>1377</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>1378</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="171.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>1363</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>1364</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>1344</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>1365</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>1366</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>1367</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>1368</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>1369</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>1370</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>1371</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>1372</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>1373</v>
-      </c>
-      <c r="M8" s="3" t="s">
+    <row r="9" spans="1:23" ht="171.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>1381</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>1382</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>1383</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>1384</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>1385</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>1386</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>1387</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>1388</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>1389</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="N8" s="3" t="s">
-        <v>1374</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>1375</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>1376</v>
-      </c>
-      <c r="Q8" s="3" t="s">
+      <c r="N9" s="3" t="s">
+        <v>1390</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>1391</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>1392</v>
+      </c>
+      <c r="Q9" s="3" t="s">
         <v>1266</v>
       </c>
-      <c r="R8" s="3" t="s">
-        <v>1377</v>
-      </c>
-      <c r="S8" s="3" t="s">
-        <v>1378</v>
-      </c>
-      <c r="T8" s="3" t="s">
-        <v>1379</v>
-      </c>
-      <c r="U8" s="8">
+      <c r="R9" s="3" t="s">
+        <v>1393</v>
+      </c>
+      <c r="S9" s="3" t="s">
+        <v>1394</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>1395</v>
+      </c>
+      <c r="U9" s="8">
         <v>3</v>
       </c>
-      <c r="V8" s="7" t="s">
-        <v>1380</v>
-      </c>
-      <c r="W8" s="3" t="s">
+      <c r="V9" s="7" t="s">
+        <v>1396</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>1397</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>1399</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>1402</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>1403</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>1404</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>1405</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>1406</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>1407</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>1408</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>1389</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>1409</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>1407</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>1410</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>1411</v>
+      </c>
+      <c r="S10" s="5" t="s">
+        <v>1412</v>
+      </c>
+      <c r="T10" s="5" t="s">
+        <v>1413</v>
+      </c>
+      <c r="U10" s="9">
+        <v>3</v>
+      </c>
+      <c r="V10" s="6" t="s">
+        <v>1414</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>1415</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" ht="369.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>1416</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>1417</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>1419</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>1420</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>1421</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>1422</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>1423</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>1424</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>1425</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>1426</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>1427</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R11" s="3" t="s">
+        <v>1428</v>
+      </c>
+      <c r="S11" s="3" t="s">
+        <v>1429</v>
+      </c>
+      <c r="T11" s="3" t="s">
+        <v>1430</v>
+      </c>
+      <c r="U11" s="8">
+        <v>4</v>
+      </c>
+      <c r="V11" s="7" t="s">
+        <v>1431</v>
+      </c>
+      <c r="W11" s="3" t="s">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" ht="290.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>1435</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>1436</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>1437</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>1438</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>1439</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>1440</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>1389</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>1441</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>1442</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>1443</v>
+      </c>
+      <c r="Q12" s="5" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R12" s="5" t="s">
+        <v>1444</v>
+      </c>
+      <c r="S12" s="5" t="s">
+        <v>1445</v>
+      </c>
+      <c r="T12" s="5" t="s">
+        <v>1446</v>
+      </c>
+      <c r="U12" s="9">
+        <v>3</v>
+      </c>
+      <c r="V12" s="7" t="s">
+        <v>1447</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>1449</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>1458</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>1381</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>1382</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>1383</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>1384</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>1385</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>1386</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>1387</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>1388</v>
-      </c>
-      <c r="H9" s="5" t="s">
+      <c r="E13" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>1460</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>1461</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>1462</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>1463</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>1464</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L13" s="3" t="s">
         <v>1389</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>1390</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>1391</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>1392</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>1373</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="N9" s="5" t="s">
-        <v>1393</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>1391</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>1394</v>
-      </c>
-      <c r="Q9" s="5" t="s">
+      <c r="M13" s="3" t="s">
+        <v>1453</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>1465</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>1466</v>
+      </c>
+      <c r="P13" s="3" t="s">
+        <v>1467</v>
+      </c>
+      <c r="Q13" s="3" t="s">
         <v>1266</v>
       </c>
-      <c r="R9" s="5" t="s">
-        <v>1395</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>1396</v>
-      </c>
-      <c r="T9" s="5" t="s">
-        <v>1397</v>
-      </c>
-      <c r="U9" s="9">
-        <v>3</v>
-      </c>
-      <c r="V9" s="6" t="s">
-        <v>1398</v>
-      </c>
-      <c r="W9" s="5" t="s">
-        <v>1399</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="369.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>1400</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>1401</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>1384</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>1385</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>1402</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>1403</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>1404</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>1405</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>1406</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>1407</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>1408</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>1409</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>1410</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>1411</v>
-      </c>
-      <c r="Q10" s="3" t="s">
-        <v>1266</v>
-      </c>
-      <c r="R10" s="3" t="s">
-        <v>1412</v>
-      </c>
-      <c r="S10" s="3" t="s">
-        <v>1413</v>
-      </c>
-      <c r="T10" s="3" t="s">
-        <v>1414</v>
-      </c>
-      <c r="U10" s="8">
-        <v>4</v>
-      </c>
-      <c r="V10" s="7" t="s">
-        <v>1415</v>
-      </c>
-      <c r="W10" s="3" t="s">
-        <v>1416</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" ht="290.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>1417</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>1418</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>1384</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>1385</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>1419</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>1420</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>1421</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>1422</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>1423</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>1424</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>1373</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>1425</v>
-      </c>
-      <c r="O11" s="5" t="s">
-        <v>1426</v>
-      </c>
-      <c r="P11" s="5" t="s">
-        <v>1427</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>1266</v>
-      </c>
-      <c r="R11" s="5" t="s">
-        <v>1395</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>1428</v>
-      </c>
-      <c r="T11" s="5" t="s">
-        <v>1429</v>
-      </c>
-      <c r="U11" s="9">
-        <v>3</v>
-      </c>
-      <c r="V11" s="7" t="s">
-        <v>1430</v>
-      </c>
-      <c r="W11" s="5" t="s">
-        <v>1431</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>1434</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>1435</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>1432</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>1365</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>1436</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>1437</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>1438</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>1439</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>1440</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>1441</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>1373</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>1433</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>1442</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>1443</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>1444</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>1266</v>
-      </c>
-      <c r="R12" s="3" t="s">
-        <v>1445</v>
-      </c>
-      <c r="S12" s="3" t="s">
-        <v>1446</v>
-      </c>
-      <c r="T12" s="3" t="s">
-        <v>1447</v>
-      </c>
-      <c r="U12" s="8">
+      <c r="R13" s="3" t="s">
+        <v>1468</v>
+      </c>
+      <c r="S13" s="3" t="s">
+        <v>1469</v>
+      </c>
+      <c r="T13" s="3" t="s">
+        <v>1470</v>
+      </c>
+      <c r="U13" s="8">
         <v>5</v>
       </c>
-      <c r="V12" s="7" t="s">
-        <v>1448</v>
-      </c>
-      <c r="W12" s="3" t="s">
-        <v>1449</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" ht="409.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>1450</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>1451</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>1253</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>1452</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>1453</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>1454</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>1455</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>1456</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>1457</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>1458</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>1459</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>1460</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>1461</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>1462</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>1463</v>
-      </c>
-      <c r="Q13" s="3" t="s">
-        <v>1464</v>
-      </c>
-      <c r="R13" s="3" t="s">
-        <v>1465</v>
-      </c>
-      <c r="S13" s="3" t="s">
-        <v>1466</v>
-      </c>
-      <c r="T13" s="3" t="s">
-        <v>1467</v>
-      </c>
-      <c r="U13" s="8">
-        <v>4</v>
-      </c>
       <c r="V13" s="7" t="s">
-        <v>1468</v>
+        <v>1471</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>1469</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="409.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>1470</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>1471</v>
-      </c>
-      <c r="C14" s="5" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>1475</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>1253</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>1472</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="D14" s="3" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>1478</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>1479</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>1480</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>1481</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>1482</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>1483</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>1484</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>1485</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>1486</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>1487</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>1488</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>1489</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>1490</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>1491</v>
+      </c>
+      <c r="U14" s="8">
+        <v>4</v>
+      </c>
+      <c r="V14" s="7" t="s">
+        <v>1492</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="409.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>1496</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>1497</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>1498</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>1499</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>1500</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>1501</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>1502</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>1503</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>1504</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>1505</v>
+      </c>
+      <c r="P15" s="5" t="s">
+        <v>1506</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>1507</v>
+      </c>
+      <c r="R15" s="5" t="s">
+        <v>1508</v>
+      </c>
+      <c r="S15" s="5" t="s">
+        <v>1509</v>
+      </c>
+      <c r="T15" s="5" t="s">
+        <v>1510</v>
+      </c>
+      <c r="U15" s="9">
+        <v>2</v>
+      </c>
+      <c r="V15" s="6" t="s">
+        <v>1511</v>
+      </c>
+      <c r="W15" s="5" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>1514</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>1515</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>1516</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>1330</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>1517</v>
+      </c>
+      <c r="I16" s="20" t="s">
+        <v>1295</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>1518</v>
+      </c>
+      <c r="K16" s="20" t="s">
+        <v>1519</v>
+      </c>
+      <c r="L16" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="M16" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="N16" s="20" t="s">
+        <v>1520</v>
+      </c>
+      <c r="O16" s="20" t="s">
+        <v>1521</v>
+      </c>
+      <c r="P16" s="20" t="s">
+        <v>1522</v>
+      </c>
+      <c r="Q16" s="20" t="s">
+        <v>1523</v>
+      </c>
+      <c r="R16" s="20" t="s">
+        <v>1524</v>
+      </c>
+      <c r="S16" s="20" t="s">
+        <v>1525</v>
+      </c>
+      <c r="T16" s="20" t="s">
+        <v>1526</v>
+      </c>
+      <c r="U16" s="20" t="s">
+        <v>1527</v>
+      </c>
+      <c r="V16" s="20" t="s">
+        <v>1528</v>
+      </c>
+      <c r="W16" s="20" t="s">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>1531</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>1381</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>1532</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>1533</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>1534</v>
+      </c>
+      <c r="H17" s="23" t="s">
+        <v>1535</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>1536</v>
+      </c>
+      <c r="J17" s="23" t="s">
+        <v>1537</v>
+      </c>
+      <c r="K17" s="23" t="s">
+        <v>1538</v>
+      </c>
+      <c r="L17" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="M17" s="23" t="s">
+        <v>1539</v>
+      </c>
+      <c r="N17" s="23" t="s">
+        <v>1540</v>
+      </c>
+      <c r="O17" s="23" t="s">
+        <v>1541</v>
+      </c>
+      <c r="P17" s="23" t="s">
+        <v>1542</v>
+      </c>
+      <c r="Q17" s="23" t="s">
+        <v>1543</v>
+      </c>
+      <c r="R17" s="23" t="s">
+        <v>1544</v>
+      </c>
+      <c r="S17" s="23" t="s">
+        <v>1545</v>
+      </c>
+      <c r="T17" s="23" t="s">
+        <v>1546</v>
+      </c>
+      <c r="U17" s="23" t="s">
+        <v>1527</v>
+      </c>
+      <c r="V17" s="23" t="s">
+        <v>1547</v>
+      </c>
+      <c r="W17" s="23" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>1455</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>1550</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>1551</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>1552</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>1553</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>1554</v>
+      </c>
+      <c r="H18" s="20" t="s">
+        <v>1555</v>
+      </c>
+      <c r="I18" s="20" t="s">
+        <v>1556</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>1557</v>
+      </c>
+      <c r="K18" s="20" t="s">
+        <v>1558</v>
+      </c>
+      <c r="L18" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="M18" s="20" t="s">
+        <v>1559</v>
+      </c>
+      <c r="N18" s="20" t="s">
+        <v>1560</v>
+      </c>
+      <c r="O18" s="20" t="s">
+        <v>1561</v>
+      </c>
+      <c r="P18" s="20" t="s">
+        <v>1562</v>
+      </c>
+      <c r="Q18" s="20" t="s">
+        <v>1563</v>
+      </c>
+      <c r="R18" s="20" t="s">
+        <v>1564</v>
+      </c>
+      <c r="S18" s="20" t="s">
+        <v>1565</v>
+      </c>
+      <c r="T18" s="20" t="s">
+        <v>1566</v>
+      </c>
+      <c r="U18" s="20" t="s">
+        <v>1527</v>
+      </c>
+      <c r="V18" s="20" t="s">
+        <v>1567</v>
+      </c>
+      <c r="W18" s="20" t="s">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>1570</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>1571</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>1572</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>1573</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>1574</v>
+      </c>
+      <c r="I19" s="20" t="s">
+        <v>1575</v>
+      </c>
+      <c r="J19" s="20" t="s">
+        <v>1576</v>
+      </c>
+      <c r="K19" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="L19" s="20" t="s">
+        <v>1577</v>
+      </c>
+      <c r="M19" s="20" t="s">
+        <v>1578</v>
+      </c>
+      <c r="N19" s="20" t="s">
+        <v>1579</v>
+      </c>
+      <c r="O19" s="20" t="s">
+        <v>1407</v>
+      </c>
+      <c r="P19" s="20" t="s">
+        <v>1580</v>
+      </c>
+      <c r="Q19" s="20" t="s">
+        <v>1581</v>
+      </c>
+      <c r="R19" s="20" t="s">
+        <v>1582</v>
+      </c>
+      <c r="S19" s="20" t="s">
+        <v>1583</v>
+      </c>
+      <c r="T19" s="20" t="s">
+        <v>1584</v>
+      </c>
+      <c r="U19" s="20" t="s">
+        <v>1585</v>
+      </c>
+      <c r="V19" s="20" t="s">
+        <v>1586</v>
+      </c>
+      <c r="W19" s="20" t="s">
+        <v>1587</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
         <v>1473</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="B20" s="20" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>1589</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>1590</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>1591</v>
+      </c>
+      <c r="F20" s="20" t="s">
+        <v>1592</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>1593</v>
+      </c>
+      <c r="H20" s="20" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I20" s="20" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J20" s="20" t="s">
+        <v>1596</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="L20" s="20" t="s">
+        <v>1389</v>
+      </c>
+      <c r="M20" s="20" t="s">
+        <v>1597</v>
+      </c>
+      <c r="N20" s="20" t="s">
+        <v>1598</v>
+      </c>
+      <c r="O20" s="20" t="s">
+        <v>1599</v>
+      </c>
+      <c r="P20" s="20" t="s">
+        <v>1600</v>
+      </c>
+      <c r="Q20" s="20" t="s">
+        <v>1601</v>
+      </c>
+      <c r="R20" s="20" t="s">
+        <v>1602</v>
+      </c>
+      <c r="S20" s="20" t="s">
+        <v>1603</v>
+      </c>
+      <c r="T20" s="20" t="s">
+        <v>1604</v>
+      </c>
+      <c r="U20" s="20" t="s">
+        <v>1585</v>
+      </c>
+      <c r="V20" s="20" t="s">
+        <v>1605</v>
+      </c>
+      <c r="W20" s="20" t="s">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
         <v>1474</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>1475</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>1476</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>1477</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>1478</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>1479</v>
-      </c>
-      <c r="L14" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="M14" s="5" t="s">
+      <c r="B21" s="20" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>1589</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>1608</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>1609</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>1592</v>
+      </c>
+      <c r="G21" s="20" t="s">
+        <v>1610</v>
+      </c>
+      <c r="H21" s="20" t="s">
+        <v>1594</v>
+      </c>
+      <c r="I21" s="20" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J21" s="20" t="s">
+        <v>1611</v>
+      </c>
+      <c r="K21" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="N14" s="5" t="s">
-        <v>1480</v>
-      </c>
-      <c r="O14" s="5" t="s">
-        <v>1481</v>
-      </c>
-      <c r="P14" s="5" t="s">
-        <v>1482</v>
-      </c>
-      <c r="Q14" s="5" t="s">
-        <v>1483</v>
-      </c>
-      <c r="R14" s="5" t="s">
-        <v>1484</v>
-      </c>
-      <c r="S14" s="5" t="s">
-        <v>1485</v>
-      </c>
-      <c r="T14" s="5" t="s">
-        <v>1486</v>
-      </c>
-      <c r="U14" s="9">
-        <v>2</v>
-      </c>
-      <c r="V14" s="6" t="s">
-        <v>1487</v>
-      </c>
-      <c r="W14" s="5" t="s">
-        <v>1488</v>
+      <c r="L21" s="20" t="s">
+        <v>1389</v>
+      </c>
+      <c r="M21" s="20" t="s">
+        <v>1612</v>
+      </c>
+      <c r="N21" s="20" t="s">
+        <v>1613</v>
+      </c>
+      <c r="O21" s="20" t="s">
+        <v>1614</v>
+      </c>
+      <c r="P21" s="20" t="s">
+        <v>1615</v>
+      </c>
+      <c r="Q21" s="20" t="s">
+        <v>1601</v>
+      </c>
+      <c r="R21" s="20" t="s">
+        <v>1616</v>
+      </c>
+      <c r="S21" s="20" t="s">
+        <v>1617</v>
+      </c>
+      <c r="T21" s="20" t="s">
+        <v>1618</v>
+      </c>
+      <c r="U21" s="20" t="s">
+        <v>1619</v>
+      </c>
+      <c r="V21" s="20" t="s">
+        <v>1620</v>
+      </c>
+      <c r="W21" s="20" t="s">
+        <v>1621</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="24" t="s">
+        <v>1494</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>1622</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>1623</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>1381</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>1624</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>1625</v>
+      </c>
+      <c r="G22" s="20" t="s">
+        <v>1626</v>
+      </c>
+      <c r="H22" s="20" t="s">
+        <v>1537</v>
+      </c>
+      <c r="I22" s="20" t="s">
+        <v>1627</v>
+      </c>
+      <c r="J22" s="20" t="s">
+        <v>1537</v>
+      </c>
+      <c r="K22" s="20" t="s">
+        <v>1628</v>
+      </c>
+      <c r="L22" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="M22" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="N22" s="20" t="s">
+        <v>1629</v>
+      </c>
+      <c r="O22" s="20" t="s">
+        <v>1541</v>
+      </c>
+      <c r="P22" s="20" t="s">
+        <v>1630</v>
+      </c>
+      <c r="Q22" s="20" t="s">
+        <v>1631</v>
+      </c>
+      <c r="R22" s="20" t="s">
+        <v>1632</v>
+      </c>
+      <c r="S22" s="20" t="s">
+        <v>1633</v>
+      </c>
+      <c r="T22" s="20" t="s">
+        <v>1634</v>
+      </c>
+      <c r="U22" s="20" t="s">
+        <v>1635</v>
+      </c>
+      <c r="V22" s="20" t="s">
+        <v>1636</v>
+      </c>
+      <c r="W22" s="20" t="s">
+        <v>1637</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{6E677F0D-D3A5-43AC-A643-930ACE350978}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{3EF0E9F0-9BAB-4C94-8CFD-061F065A29BA}"/>
-    <hyperlink ref="E9" r:id="rId3" xr:uid="{84A8C5B7-CA38-4EF3-819B-787F208F51A1}"/>
-  </hyperlinks>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-08 10:52:04
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -80,7 +80,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -152,6 +152,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -209,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -299,6 +304,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -698,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X54"/>
+  <dimension ref="A1:X61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1765,7 +1779,7 @@
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>RAG pipelines have a lot of knobs and nobody had isolated which ones actually matter in finance. Runs 1,620 experiments - 6 LLMs x 15 retrieval conditions x 9 prompts x 2 datasets x 2 quality aspects.</t>
+          <t>RAG pipelines have a lot of knobs and which ones actually matter in finance had not been isolated. Runs 1,620 experiments - 6 LLMs x 15 retrieval conditions x 9 prompts x 2 datasets x 2 quality aspects.</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
@@ -2380,7 +2394,7 @@
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Prior Sri Lankan volatility studies contradict each other on whether there's a leverage effect, and nobody had run the full symmetric versus asymmetric GARCH lineup against a consistent mean equation on CSE data. Also targets 2018-2022 specifically, a window that swallows the Easter Sunday attacks, COVID-19 and the 2022 economic crisis.</t>
+          <t>Prior Sri Lankan volatility studies contradict each other on whether there's a leverage effect, and the full symmetric versus asymmetric GARCH lineup had not been run against a consistent mean equation on CSE data. Also targets 2018-2022 specifically, a window that swallows the Easter Sunday attacks, COVID-19 and the 2022 economic crisis.</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
@@ -2471,125 +2485,198 @@
       </c>
     </row>
     <row r="15" ht="409.6" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>P14</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Aldasoro, I., Hordahl, P., Schrimpf, A. &amp; Zhu, S. (BIS)</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Aldasoro, I., Hördahl, P., Schrimpf, A. and Zhu, S. (2025). Predicting financial market stress with machine learning. Bank for International Settlements, BIS Working Paper 1250, February 2025. Affiliations as recorded in my note: all four authors out of the BIS Monetary and Economic Department, with Schrimpf also at CEPR. No DOI recorded in the note frontmatter (doi field empty). Citekey: aldasoroPredictingFinancialMarket2025.</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>BIS Working Papers No. 1250, 17 March 2025. Also CEPR Discussion Paper DP20439</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>https://www.bis.org/publ/work1250.pdf</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>Market stress / tail-risk forecasting</t>
-        </is>
-      </c>
-      <c r="G15" s="18" t="inlineStr">
-        <is>
-          <t>Forecasts financial market stress as a full conditional distribution rather than a point estimate, using newly constructed market condition indicators.</t>
-        </is>
-      </c>
-      <c r="H15" s="18" t="inlineStr">
-        <is>
-          <t>US Treasury, FX and money markets.</t>
-        </is>
-      </c>
-      <c r="I15" s="18" t="inlineStr">
-        <is>
-          <t>Newly constructed market condition indicators (MCIs) for the three markets above.</t>
-        </is>
-      </c>
-      <c r="J15" s="18" t="inlineStr">
-        <is>
-          <t>Funding liquidity, global financial cycle and macro stress inputs aggregated into the MCIs.</t>
-        </is>
-      </c>
-      <c r="K15" s="18" t="inlineStr">
-        <is>
-          <t>Tree-based machine learning - random forests with quantile regression to map the full conditional distribution of future stress, with SHAP values to identify which factors are contributing.</t>
-        </is>
-      </c>
-      <c r="L15" s="18" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="M15" s="18" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N15" s="18" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="O15" s="18" t="inlineStr">
-        <is>
-          <t>This is the whole paper - forecasting the probability of extreme stress episodes rather than modelling conditional variance directly.</t>
-        </is>
-      </c>
-      <c r="P15" s="18" t="inlineStr">
-        <is>
-          <t>Funding liquidity is one of the MCI inputs, so liquidity enters as a stress driver rather than an execution cost.</t>
-        </is>
-      </c>
-      <c r="Q15" s="18" t="inlineStr">
-        <is>
-          <t>SHAP values identify which risk factors are driving a given stress forecast, which is the part that matters for a guardrail you have to justify.</t>
-        </is>
-      </c>
-      <c r="R15" s="18" t="inlineStr">
-        <is>
-          <t>Quantile loss, against autoregressive time-series benchmarks.</t>
-        </is>
-      </c>
-      <c r="S15" s="18" t="inlineStr">
-        <is>
-          <t>Random forests achieve up to 27% lower quantile loss than the autoregressive benchmarks, with the largest gains at 3-12 month horizons.</t>
-        </is>
-      </c>
-      <c r="T15" s="18" t="inlineStr">
-        <is>
-          <t>Heavy dependence on structural macro data. US markets only. Likely to struggle across abrupt regime switches unless paired with something real-time.</t>
-        </is>
-      </c>
-      <c r="U15" s="18" t="inlineStr">
-        <is>
-          <t>NOT YET REVIEWED - fields here come from the source paper, not my own read. I couldn't find it on Semantic Scholar so I left it; the PDF is at bis.org/publ/work1250.pdf. Worth coming back to for the risk agent though: forecasting the whole conditional distribution of stress rather than a point estimate, plus SHAP attribution for which factor is driving it, is the right shape for a risk guardrail that has to explain itself.</t>
-        </is>
-      </c>
-      <c r="V15" s="18" t="inlineStr">
-        <is>
-          <t>US Treasury, FX and money markets. CSE has nothing like the MCI inputs available, so the method transfers but the features don't - I'd have to construct a Sri Lankan equivalent from what CBSL actually publishes.</t>
-        </is>
-      </c>
-      <c r="W15" s="18" t="inlineStr">
-        <is>
-          <t>[[Predicting Financial Market Stress with Machine Learning]] - NOT YET REVIEWED</t>
-        </is>
-      </c>
-      <c r="X15" s="18" t="inlineStr">
-        <is>
-          <t>SPEAKS TO: A_V.
-STILL NOT REVIEWED. Fields are from the source paper, not my own read.</t>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>Bank for International Settlements, Working Paper 1250, February 2025. Central bank working paper, not a peer-reviewed venue.</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>https://www.bis.org/publications/working-paper-1250-predicting-financial-market-stress-machine-learning (accessed 21 September 2026). Zotero: zotero://select/library/items/PYNXNGJT</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>Stream field is empty in the note frontmatter, as is market. In my own framing this is state measurement and state forecasting, not an architecture paper: "This is not a competitor architecture, there are no agents here and nothing resembling an orchestrator, and the horizon is monthly over three to twelve months rather than daily. It earns a full note because it is the closest thing in my set to a worked specification of the thing my weighting function conditions on."</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>Two contributions stacked on each other. First, build daily market condition indicators (MCIs) for three US markets, Treasury, FX and money markets, out of microstructure inputs rather than the equity-volatility inputs that dominate conventional stress indices, aggregating each market's inputs through a rolling-window PCA so the index at any date uses only past information. Second, forecast the full conditional distribution of those indicators three to twelve months ahead with quantile regression, benchmarking a random forest against a quantile AR and a 44-predictor multivariate quantile regression, then open the forest up with Shapley values. The MCI series are released with the paper.
+Gaps as the authors frame them, as I recorded:
+- Aggregate stress and financial conditions indices conflate broad sentiment with structural vulnerability. FSIs and FCIs give a snapshot of market health but mix broad sentiment shifts, equity volatility via the VIX above all, with liquidity shortages and arbitrage breakdowns; the supporting observation is that the OFR's FSI and Goldman's US FCI both correlate very highly with the VIX despite the VIX being one input among many. "The consequence they care about is that a stress signal you cannot attribute to a market is a stress signal you cannot act on with a targeted intervention."
+- The missing object is a market-specific indicator built from market-specific frictions. Three indices for three segments rather than one for the system, each built from dislocations diagnostic of that segment: bid-ask spreads, on/off-the-run spreads and repo-OIS for illiquidity; covered interest parity deviations and triangular no-arbitrage violations for impaired arbitrage. The claim is that these capture balance-sheet constraints on intermediaries in a way a volatility index cannot.
+- Distribution rather than mean, "and it is the one that transfers." Policymakers care about the upper percentile stress scenarios that could trigger contagion, not the conditional mean, and linear regression on conditional means flattens precisely those extremes. Quantile regression gives the whole distribution, which lets them ask what drives the worst 10% of money market outcomes rather than the average one.
+- Two properties of the forecasting problem are argued to suit tree-based models specifically: the quantile loss is non-smooth, and many of the 44 predictors are uninformative on average while mattering in specific quantiles, both conditions under which [[Empirical Asset Pricing via Machine Learning]] and the tabular-data result they lean on say trees do well. Trees also stay interpretable through TreeSHAP in a way a network does not.
+Premise I flagged once rather than relitigating: "the first principal component of a dozen standardised friction measures is a meaningful scalar state of a market. The paper asserts this, validates it informally against known episodes, and never tests it against an alternative aggregation."</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>US Treasury market, US money market, and FX centred on the dollar. Market-level, not asset-level. Monthly forecasting frequency over daily index construction. My bounding note: "Everything is market-level, monthly and US, which bounds how far any of it transfers. The inputs exist because these are the deepest markets in the world, cross-currency bases, repo-OIS, on-the-run premia, failed deliveries, dealer coupon holdings. The construction method is portable, this particular input set is not, and the paper makes no claim about frontier or thinly traded markets."</t>
+        </is>
+      </c>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>Daily series from Bloomberg, Tradeweb, Datascope and the Fed for the index inputs, EPFR and ICI for fund flows, over 01/01/2003 to 31/05/2024, then aggregated to monthly for the forecasting exercise.
+Setup grid as recorded:
+- Markets: US Treasury, US money market, FX centred on the dollar
+- Period: Jan 2003 to May 2024, 239 monthly observations
+- MCI inputs: FX 4 series, Treasury 8 series, money market 4 series
+- Aggregation: rolling-window PCA, first principal component
+- Initial PCA window: 3 years, expanded by one month at each step
+- Predictors: 44, in two families, overextension and risk perception, versus funding liquidity and market-making capacity
+- Estimation-test window: 84 months, rolled forward
+- Horizons: h = 1 to 12 months
+- Test windows: 153 at h = 1, 142 at h = 12
+- Quantiles: median, 75th, 90th, 95th
+- Metric: average out-of-sample quantile loss</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="inlineStr">
+        <is>
+          <t>Microstructure and macro-financial time series only. No text, no images.
+MCI construction: for each market, the input series are signed so higher means worse conditions, z-scored to mean zero and unit variance, then reduced to their first principal component, which is re-normalised to zero mean and unit standard deviation. Positive values mean tighter-than-average conditions. All three are right-skewed as expected of a stress measure: MCI(TR) runs -1.80 to 6.34, MCI(MM) -1.53 to 5.02, MCI(FX) -1.77 to 4.15, each against a standard deviation of roughly 0.95.
+Index input families: illiquidity (bid-ask spreads, on/off-the-run spreads, repo-OIS) and impaired arbitrage (covered interest parity deviations, triangular no-arbitrage violations).
+The 44 predictors split into: Fed and government balance-sheet variables (Treasury purchases in level and six-month moving average, the Treasury General Account, failed deliveries, dealer coupon holdings); fund flows (EPFR cross-border flows, ICI intra-family flows into money market, high-yield and equity funds); macro-financial state (excess bond premium, broad dollar index, the Rey global financial cycle index, Citi surprise indices, futures margin, bill issuance, curve slopes); and risk proxies (MOVE, VIX, SKEW, three-month implied vol on EUR, GBP and JPY).</t>
+        </is>
+      </c>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>Rolling-window PCA for index construction, then quantile regression forecasting of the index's conditional distribution at h = 1 to 12 months, then TreeSHAP attribution.
+Common objective, the check-function quantile loss, "which is the piece I would need to reimplement and the reason the comparison across models is apples to apples":
+(1/N) * sum_{t=1}^{T} rho_tau( y_t - beta * x_t^T ),  where rho_tau(u) = tau*u if u &gt; 0, and (tau - 1)*u if u &lt;= 0
+where tau is the quantile being fitted and the asymmetry of rho_tau is what makes the fitted line a quantile rather than a mean, under-prediction and over-prediction being penalised at different rates.
+Benchmark 1, the one the rest of the paper actually competes against: a quantile AR(1) on the market's own lagged MCI, extended so that each market sees all three.
+Benchmark 2 adds the 44 predictors on top:
+y^tau_{i,t} ~ beta_1 * y_{tr,t-1} + beta_2 * y_{mm,t-1} + beta_3 * y_{fx,t-1} + sum_{k=1}^{K} gamma_k * x_{k,t-1} + epsilon_t,  for i in {tr, mm, fx}
+ML model: a quantile regression forest in the Meinshausen sense, a random forest read as an estimate of the full conditional distribution rather than the conditional mean. No hyperparameters are reported anywhere, no tuning procedure is described, and the XGBoost comparison that would show the choice of tree ensemble does not drive the result is explicitly "unreported".
+Attribution: TreeSHAP, with the Shapley value in the usual cooperative-game form:
+phi_i = sum over S subset of N\{i} of [ |S|! * (|N| - |S| - 1)! / |N|! ] * [ f(S union {i}) - f(S) ]
+where N is the full feature set and S a subset not containing feature i; f(S) is the model's prediction using only the features in S; and the combinatorial weight averages i's marginal contribution over every possible ordering of the features. "The reason this is affordable at all is that the exact computation is exponential in |N| and the Lundberg tree solution reduces it to a polynomial traversal of the tree structure, which is why the attribution layer here costs almost nothing while the same thing on a network would not."
+Output: the full conditional distribution (median, 75th, 90th, 95th quantiles) of each market's MCI at horizons of one to twelve months, plus Shapley attributions over the 44 predictors.</t>
+        </is>
+      </c>
+      <c r="L15" s="28" t="inlineStr">
+        <is>
+          <t>None. "There are no agents here and nothing resembling an orchestrator." The paper is a state-measurement and state-forecasting exercise, and it enters my matrix as a specification for the objects my orchestrator conditions on rather than as a competitor architecture.</t>
+        </is>
+      </c>
+      <c r="M15" s="28" t="inlineStr">
+        <is>
+          <t>No text sentiment and no NLP. "Sentiment" appears only as the name of a numeric predictor in the Shapley rankings (Sentiment and Sentiment (6ma) rank second, third and fourth for Treasury and fourth for FX by mean absolute Shapley value); the note does not record how that series is constructed. The paper's framing argument is in fact the opposite of a sentiment approach: it objects that conventional FSIs and FCIs "mix broad sentiment shifts, equity volatility via the VIX above all, with liquidity shortages and arbitrage breakdowns," and builds friction-based indices instead. Nothing here is a sentiment component, so the scope decision does not bite on this row.</t>
+        </is>
+      </c>
+      <c r="N15" s="28" t="inlineStr">
+        <is>
+          <t>Not recorded in the note. There is no retrieval, no document corpus and no fundamental-data channel. The relevant cross-reference is to my explainability plan rather than to A_F: "The explainability component is attribution over risk features, RAG citation tracing, interpretable FIGARCH and GJR-GARCH parameters, and the orchestrator's weight vector, and this paper is a central-bank-grade instance of the first of those on a tree model."</t>
+        </is>
+      </c>
+      <c r="O15" s="28" t="inlineStr">
+        <is>
+          <t>Central to the paper, but as a state to be measured and forecast rather than as a model of returns. Volatility enters three ways. As an object of criticism: the whole motivation is that conventional stress indices are dominated by equity volatility (the VIX), and that the OFR FSI and Goldman US FCI both correlate very highly with the VIX. As inputs: the risk-proxy family of predictors is MOVE, VIX, SKEW and three-month implied volatility on EUR, GBP and JPY. And as the target's tail: the forecasting exercise targets the median, 75th, 90th and 95th quantiles of each MCI rather than its mean, on the argument that policymakers care about the upper percentile stress scenarios that could trigger contagion, not the conditional mean, and that linear regression on conditional means flattens precisely those extremes.
+Evidence bearing on persistence: attribution is dominated by the indicator's own lag in all three markets. For the money market, current MCI(MM) is the top feature by a wide margin; for FX, MCI(FX) ranks second; for Treasury, MCI(TR) is first. The authors read this as stress being self-reinforcing within a market and transmitting across markets that are distinct but intertwined through market-making and collateral. My caveat: "That reading is consistent with the attribution but is not separately tested, there is no spillover identification here and no decomposition of own-lag persistence into anything finer."
+My own reading of what that does and does not give me on P_t: "The same result read the other way is independent large-sample support for P_t having something to measure, since the current MCI is the top feature for its own three-month tail in all three markets, but it does not distinguish hyperbolic from exponential decay and estimates nothing like d, so [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] stays the only local evidence on the shape."</t>
+        </is>
+      </c>
+      <c r="P15" s="28" t="inlineStr">
+        <is>
+          <t>This is the paper's core material. The indices are built from illiquidity and arbitrage-breakdown inputs specifically: bid-ask spreads, on/off-the-run spreads and repo-OIS for illiquidity; covered interest parity deviations and triangular no-arbitrage violations for impaired arbitrage. The claim is that these capture balance-sheet constraints on intermediaries in a way a volatility index cannot. Funding-liquidity and market-making-capacity variables form one of the two predictor families, and the paper's headline attribution finding is that funding liquidity, investor overextension and the global financial cycle carry most of the attribution.
+Market-specific split of what predicts the tails: "Money market tails are predicted by funding and official-sector supply, lower Fed purchases and lower bill issuance and lower TGA balances predicting tighter conditions ahead, together with the global financial cycle. FX tails are predicted overwhelmingly by risk perception, implied volatility on EUR and GBP and intra-family equity flows, with funding and market-making variables present but lower."
+What is absent on the friction side: any execution cost, trading decision or economic objective. "There is no economic evaluation of any kind, on a paper whose stated purpose is real-time vulnerability monitoring. Quantile loss is the only metric."</t>
+        </is>
+      </c>
+      <c r="Q15" s="28" t="inlineStr">
+        <is>
+          <t>TreeSHAP over the 44 predictors, presented as the second contribution ("opening black boxes"). Shapley value defined in the cooperative-game form given above, with the Lundberg tree solution reducing an exponential computation to a polynomial traversal, which is why the attribution layer costs almost nothing on a forest.
+Two problems I recorded. First, the explainability contribution sits on a model whose own specification is undocumented: "No forest hyperparameters, no tuning protocol, no seed or ensemble treatment, no report of whether the forest is refit at every rolling window or periodically, and the XGBoost robustness check appears only as an assertion that performance is comparable at higher computational cost. Combined with the unstated interval construction noted above, the random forest is effectively a black box in a paper whose second contribution is opening black boxes." Second, Shapley results are presented for the Treasury market where the forecasting model does not beat the benchmark. The authors do caveat it, saying Treasury results should be interpreted with caution since out-of-sample performance is not significantly better than the AR, "and they are right to, but the plot is still there at the same size as the other two and will be cited. The general issue is sharper than this one instance: SHAP explains what the model does, not what the market does, so attributions from a model with no demonstrated out-of-sample edge are describing a fitted artefact."</t>
+        </is>
+      </c>
+      <c r="R15" s="28" t="inlineStr">
+        <is>
+          <t>Metric: average out-of-sample quantile loss under the check function, the same objective for every model, "which is the reason the comparison across models is apples to apples."
+Protocol: 84-month estimation-test window rolled forward over 239 monthly observations, horizons h = 1 to 12, 153 test windows at h = 1 and 142 at h = 12, quantiles median, 75th, 90th and 95th. Both in-sample and out-of-sample results are reported for the linear specifications.
+Baselines: a quantile AR(1) on the market's own lagged MCI extended so each market sees all three (the benchmark the paper actually competes against), and an unpenalised 44-predictor multivariate quantile regression on top of it.
+Look-ahead discipline: the rolling PCA is adopted specifically because the full-sample version used in the authors' earlier policy article computes the components from the entire dataset and therefore introduces future information into every historical value of the index. "They run both and plot them together, which is the cheapest possible honesty about look-ahead bias and something almost nothing else in my set does." The two series are close in the crises and visibly apart elsewhere, the Treasury panel in particular, where the rolling estimate carries a spike in early 2020 more than twice the height of the full-sample one.
+Caveat I recorded as a warning: "The test windows overlap heavily and the paper does not say how the confidence intervals handle it. With 153 rolling 84-month windows over a 239-month sample and forecast horizons out to twelve months, successive forecast errors share almost all of their training data and, at h = 12, eleven months of their target window. The 90% intervals in Figure 4 are the only uncertainty quantification in the paper and the correction used to produce them is not stated, so I read the significance claims as indicative rather than as clean tests."
+Also recorded as a structural caveat on the estimation window: "That is 84 monthly observations against 44 predictors in the multivariate specification and against a random forest in the ML specification, which is a very small training set by any ML standard and is the fact that makes the parsimony result below more than a curiosity."
+No economic evaluation: no decision rule, no threshold, no cost of a false alarm against a missed episode, no comparison against a policymaker's existing FSI on the same test windows.</t>
+        </is>
+      </c>
+      <c r="S15" s="28" t="inlineStr">
+        <is>
+          <t>- Headline: the random forest achieves up to 27% lower quantile loss than the AR benchmark at the 90th quantile of FX stress three months out; the 44-predictor linear model wins in-sample everywhere and loses out-of-sample everywhere; funding liquidity, investor overextension and the global financial cycle carry most of the attribution.
+- The MCIs carry market-specific stress that the VIX does not, and the 2015-16 window is the cleanest demonstration. The FX MCI rose significantly through the Swiss franc de-peg, Brexit and the US money market fund reform without a commensurate VIX spike, "which is the single episode that justifies the whole construction, because an index tightly linked to the VIX by design cannot produce that divergence." The Treasury MCI moves into positive territory after the 2013 taper tantrum and during the idiosyncratic flash events of 2014 and 2021, and all three spike in the GFC and the pandemic to differing degrees, the money market one remaining largely subdued outside those two. My caveat: "I would read the known-episode matching as construct validation rather than as a result, since the inputs were chosen partly because they are known to move in those episodes."
+- Out of sample the 44-predictor model loses to a one-lag AR everywhere, and the reversal against in-sample is total. In-sample the multivariate model has lower quantile loss than the AR unambiguously, every market, every quantile, every horizon from one to twelve months. Out of sample the ordering flips just as completely, across horizons, markets and quantiles, and at the twelve-month horizon for the Treasury MCI the multivariate model's quantile loss exceeds the AR's by 18%. "The out-of-sample panels are also visibly unstable, the full-model loss sawtoothing between adjacent horizons while the AR line rises smoothly, which is what estimation noise rather than mis-specification looks like."
+- The random forest's gains are real in two markets out of three and the third is a null the authors state plainly. RF has significantly lower quantile loss than the AR in money and FX markets across horizons and quantiles, reaching 27% lower loss at the 90th quantile of FX stress at the three-month horizon, with money market performance comparable at h = 1 and significantly better from h = 2 onward, and FX improving monotonically out to h = 11. For the Treasury market RF does not significantly outperform, slightly underperforming on median predictions and improving only in the upper tail at three to five month horizons, with intervals that cross zero throughout. "The gain is therefore conditional on the market, and the market where it fails is the one with the deepest book and the most intermediary structure in its inputs."
+- Attribution is dominated by the indicator's own lag in all three markets, with the other markets' indicators ranking high. For the money market, current MCI(MM) is the top feature by a wide margin and MCI(FX) ranks eleventh; for FX, MCI(FX) ranks second and MCI(TR) third; for Treasury, MCI(TR) is first. The authors read this as self-reinforcing illiquidity plus spillover; I record that the reading is consistent with the attribution but not separately tested.
+- Top five predictors by mean absolute Shapley value:
+  Money market: 1 MCI (MM), 2 Fed Treasury purchases (6ma), 3 three-month bill issuance, 4 Global financial cycle index, 5 Treasury General Account.
+  FX: 1 IV EUR 3m, 2 MCI (FX), 3 MCI (TR), 4 Sentiment (6ma), 5 IV GBP 3m.
+  Treasury: 1 MCI (TR), 2 Sentiment (6ma), 3 Sentiment, 4 Swap 3m2y, 5 CP issuance.
+  "The authors' summary, that investor overextension in seemingly calm and low-volatility periods often sows the seeds for subsequent market stress, is the right shape of claim for a Shapley plot, directional and conditional rather than causal."
+- MCI ranges: MCI(TR) -1.80 to 6.34, MCI(MM) -1.53 to 5.02, MCI(FX) -1.77 to 4.15, each against a standard deviation of roughly 0.95.
+- The MCI series are released with the paper.</t>
+        </is>
+      </c>
+      <c r="T15" s="28" t="inlineStr">
+        <is>
+          <t>- The headline comparison is partly regularised against unregularised, not machine learning against linear. "The multivariate benchmark is an unpenalised quantile regression fitting 44 coefficients on 84 observations, which is nearly saturated and would be expected to overfit catastrophically whatever the data-generating process looks like. A penalised quantile regression, lasso or elastic net, is the benchmark that would separate 'trees capture non-linearities' from 'the linear model had no shrinkage', and it is absent. The result that survives cleanly is the narrower and still useful one, that the forest beats a one-lag AR in two markets, and I read the in-sample versus out-of-sample reversal as evidence about the benchmark's specification rather than about linearity."
+- No economic evaluation of any kind, on a paper whose stated purpose is real-time vulnerability monitoring. Quantile loss is the only metric. No decision rule, no threshold, no cost of a false alarm against a missed episode, no comparison against a policymaker's existing FSI on the same test windows, no statement of how much of the 27% loss improvement is concentrated in the two crisis episodes that dominate the sample. "With roughly 240 monthly observations containing two large stress events, a model that gets those two periods slightly better will post a materially lower average quantile loss while being no more useful in the other 220 months, and nothing in the paper rules that out."
+- The look-ahead discipline covers aggregation but not variable selection, and the input set is not stable over the sample. "The PCA is rolling, which is the right call and done well, but which variables enter each market's index was decided once with the full 2003 to 2024 sample in view, including knowledge of which spreads blew out in which crisis. The inputs also change composition mid-sample, Treasury quoted spreads being measured one way before 2008 and another after, time-to-quote being Tradeweb-dependent, and LIBOR-based money market inputs spanning the period in which LIBOR was discontinued. None of this is addressed and it means the index is not quite the same object at both ends of the sample."
+- The modelling details that would let anyone reproduce the ML result are missing: no forest hyperparameters, no tuning protocol, no seed or ensemble treatment, no report of whether the forest is refit at every rolling window or periodically, and the XGBoost robustness check appears only as an assertion that performance is comparable at higher computational cost.
+- Shapley results are presented for the Treasury market where the forecasting model does not beat the benchmark. Caveated by the authors, but shown at the same size as the other two. "SHAP explains what the model does, not what the market does, so attributions from a model with no demonstrated out-of-sample edge are describing a fitted artefact."
+- Everything is market-level, monthly and US. "The construction method is portable, this particular input set is not, and the paper makes no claim about frontier or thinly traded markets."
+- Test-window overlap and unstated interval construction (recorded as a warning): significance claims read as indicative rather than as clean tests.
+- Unvalidated premise: the first principal component of a dozen standardised friction measures as a meaningful scalar state of a market is asserted, validated informally against known episodes, and never tested against an alternative aggregation.</t>
+        </is>
+      </c>
+      <c r="U15" s="28" t="inlineStr">
+        <is>
+          <t>- The rolling-window PCA as the construction recipe for L_t, built from what the CSE actually prints. "The method is the transferable part: sign every input so higher means worse, z-score, take the first principal component over an expanding window starting from a three-year block, re-normalise. The CSE analogues of their input families are Amihud illiquidity, turnover ratio, zero-return frequency, quoted spread where the book is visible, and Parkinson or Garman-Klass range volatility, which is the estimator already pinned for V_t since five-minute realised volatility is unavailable here. That converts the liquidity state from a single Amihud number into a composite with the same construction discipline as a published central bank indicator, and it costs nothing I am not already computing for the cost model."
+- Their look-ahead test as a standing check. "Running the full-sample PCA alongside the rolling one and plotting both is a half-day of work that produces direct evidence of how much look-ahead bias a naive construction would have injected. The same check generalises to every fitted transform in my pipeline, which is the same question I ended up asking of decomposition boundaries in [[Extending machine learning prediction capabilities by explainable AI in financial time series prediction]], and it belongs in the methodology chapter rather than in a footnote."
+- The parsimony result as a pre-registered constraint on my conditioning set. "Eighty-four observations and 44 predictors produced a model that beat its benchmark in-sample everywhere and lost out-of-sample everywhere, at monthly frequency on the deepest markets in the world. My orchestrator conditions on four state variables plus a per-agent confidence term, which is far smaller, but the training sample is roughly 374 trading days per counter and the temptation to widen the state vector as reviews suggest additions is exactly the pressure that produced their Figure 3. The concrete commitment is that any proposed addition to f(L_t, V_t, P_t, C_{i,t}) has to beat the existing set out-of-sample on the ablation protocol, not in-sample, and the static learned-weight baseline stays in as the shrinkage-equivalent control."
+- The idea of conditioning on a forecast tail of the state rather than its current level, with the horizon named. "An orchestrator that down-weights A_T when liquidity is already bad is reacting, one that down-weights it when the upper tail of the liquidity state is forecast to widen is anticipating. The horizon mismatch is the hard part, their three to twelve months is a policy horizon and mine is days to a few weeks, so the honest version is to test a short-horizon quantile forecast of L_t on CSE data and report whether it beats the contemporaneous value as a conditioning input, as a named experiment rather than an assumed improvement."
+- The Treasury null as a scoping test for whether state-forecasting machinery is worth building at all. "The check that comes before the agent build is whether the CSE liquidity state is AR-dominated: if a quantile AR(1) on L_t is as good as anything richer, the orchestrator conditions on the lag and the state-forecasting machinery is dead weight."
+- SHAP over risk and liquidity features as the published precedent for my re-scoped attribution plan, plus the discipline that goes with it: "attribution is only reported for components whose out-of-sample performance clears the benchmark, so no SHAP plot for an agent that has not beaten its own baseline."
+- The check-function quantile loss itself, as the objective I would reimplement if I forecast a state tail.
+- The demand for economic evaluation, which this paper does not supply: "A better quantile loss on a state variable is not a better decision, and with two dominant crises in the sample it is not even clearly a better forecast in normal conditions. My equivalent trap is an orchestrator whose weights move impressively in the two or three most volatile CSE months and are inert the rest of the time, so the evaluation has to report weight variation and return against the equal-weight and static-learned baselines over quiet sub-periods separately, not only pooled, and with friction charged either way."</t>
+        </is>
+      </c>
+      <c r="V15" s="28" t="inlineStr">
+        <is>
+          <t>No agents, no orchestrator, no decision layer. The state is measured and forecast and then nothing is done with it: there is no decision rule, no threshold, no cost of a false alarm against a missed episode, and no economic evaluation on a paper whose stated purpose is real-time vulnerability monitoring. The horizon is three to twelve months at monthly frequency, a policy horizon, not the days-to-weeks horizon an orchestrator needs. Everything is market-level and US, built on inputs that exist because these are the deepest markets in the world, so the construction method is portable but the input set is not, and the paper makes no claim about frontier or thinly traded markets. On persistence specifically: own-lag dominance in the Shapley rankings is evidence that the state is persistent, but the paper does not decompose that persistence into anything finer, does not distinguish hyperbolic from exponential decay and estimates nothing like a memory parameter d, so the operationalisation of P_t is untouched. There is no treatment of how liquidity state conditions the reliability of any downstream signal, only of what predicts the liquidity state itself. And the minimum-estimation-window question I have open is left half-answered: their 84-month window is a demonstration of what too few observations against too many predictors does, not a derivation of a minimum.</t>
+        </is>
+      </c>
+      <c r="W15" s="28" t="inlineStr">
+        <is>
+          <t>[[Predicting Financial Market Stress with Machine Learning]]</t>
+        </is>
+      </c>
+      <c r="X15" s="28" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: The measurement half of the main gap, directly and in detail. "My orchestrator is supposed to vary agent influence as a function of measured exogenous market state, and the measurement half of that sentence has so far been a promise, L_t and V_t named and not constructed. This paper constructs exactly that object from illiquidity, volatility and arbitrage-breakdown inputs, enforces the look-ahead discipline that makes it usable in a forecasting exercise, forecasts its upper tail rather than its level, and attributes the forecast with SHAP, which is the same attribution layer the re-scoped explainability plan commits to. It speaks directly to A_L and A_V and to the orchestrator's state vector, and the parsimony result in the middle of it is the most useful thing I have read against my own conditioning set."
+EFFECT ON MAIN GAP: Does not close it, and sharpens the constraints on how I close it. It supplies no orchestration, no agents and no decision layer, so w(i,t) = f(L_t, V_t, P_t, C_{i,t}) stands untouched as a gap. What it changes is the discipline around f. The parsimony result is the binding one: 84 monthly observations against 44 predictors produced a model that beat its benchmark in-sample everywhere, across every market, quantile and horizon, and lost out-of-sample everywhere, with the Treasury twelve-month quantile loss exceeding the AR's by 18% and the out-of-sample loss curve sawtoothing between adjacent horizons in the way estimation noise rather than mis-specification looks. That happened at monthly frequency on the deepest markets in the world; my sample is roughly 374 trading days per counter. The commitment that follows is that any proposed addition to f has to beat the existing four-plus-confidence set out-of-sample on the ablation protocol, never in-sample, and that the static learned-weight baseline stays in as the shrinkage-equivalent control. It also reframes what the state input should be: conditioning on a forecast upper tail of the state rather than its current level is anticipating rather than reacting, and the honest version given the horizon mismatch is to test a short-horizon quantile forecast of L_t on CSE data and report whether it beats the contemporaneous value as a conditioning input, as a named experiment rather than an assumed improvement. The Treasury null gives me a cheap scoping test to run before the agent build: if a quantile AR(1) on L_t is as good as anything richer, the orchestrator conditions on the lag and the state-forecasting machinery is dead weight.
+EFFECT ON SUB-GAP 1: Substantial, on the measurement side only. This is the published, central-bank-grade recipe for turning a set of friction measures into a single scalar liquidity state: sign every input so higher means worse, z-score to mean zero and unit variance, take the first principal component over an expanding window starting from a three-year block, re-normalise to zero mean and unit standard deviation so positive means tighter than average. The CSE analogues of their input families are Amihud illiquidity, turnover ratio, zero-return frequency, quoted spread where the book is visible, and Parkinson or Garman-Klass range volatility (the estimator already pinned for V_t, since five-minute realised volatility is unavailable here), and the whole set is already being computed for the cost model, so the composite costs me nothing extra. That converts L_t from a single Amihud number into a composite with the same construction discipline as a published central bank indicator. What it does not supply is the other half of sub-gap 1: there is no execution cost anywhere, no trading objective, no friction charged, and nothing at all about liquidity conditioning the reliability of price-derived agents. The paper predicts the liquidity state; it never uses it. The cross-market spillover finding, that each market's MCI helps predict the others', has a cross-counter analogue worth testing: sector-level or market-wide liquidity state predicting an individual counter's, the structure the graph approach in [[Forecasting realized volatility with spillover effects, Perspectives from graph neural networks]] formalises. Under the scope rules that goes in as a candidate, a market-wide L_t alongside the counter-level one, to be tested on the ablation protocol rather than adopted.
+EFFECT ON SUB-GAP 2: Partial and asymmetric. On the supporting side, this is independent large-sample evidence that persistence has something to measure: the current MCI is the top feature for its own three-month tail in all three markets (first for money market by a wide margin, first for Treasury, second for FX), with the other markets' indicators also ranking high, and the authors read that as stress being self-reinforcing within a market. On the limiting side, the paper stops exactly where my sub-gap starts: own-lag dominance in a Shapley ranking is not a persistence model. There is no decomposition of own-lag persistence into anything finer, no distinction between hyperbolic and exponential decay, and nothing resembling an estimate of d, so [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] stays the only local evidence on the shape. The attribution is also not separately tested as a spillover claim; there is no spillover identification in the paper. On my open item about the minimum estimation window for persistence plus a turbulence indicator: this gives me a cautionary data point rather than an answer. Their 84-month estimation window is the thing that broke the 44-predictor specification, and the paper neither derives a minimum nor reports a sensitivity sweep over window length, so the minimum-window question is still mine to answer empirically. The turbulence-indicator side is better served: the MCI construction is a worked turbulence indicator, right-skewed as a stress measure should be (MCI(TR) -1.80 to 6.34, MCI(MM) -1.53 to 5.02, MCI(FX) -1.77 to 4.15 against a standard deviation of roughly 0.95), validated informally against the GFC, the pandemic, the 2013 taper tantrum, the 2014 and 2021 flash events, and the 2015-16 Swiss franc de-peg, Brexit and money market fund reform window, that last episode being the one where the FX MCI rose without a commensurate VIX spike. I would read that episode matching as construct validation rather than as a result, since the inputs were chosen partly because they are known to move in those episodes. And the regime-identification claim is weaker than it looks in one respect I should carry: with roughly 240 monthly observations containing two large stress events, a model that gets those two periods slightly better posts a materially lower average quantile loss while being no more useful in the other 220 months, and nothing in the paper rules that out.
+CSE DATA EVIDENCE: None directly, and the paper is explicit about its own bounds. Everything is market-level, monthly and US, and the inputs exist because these are the deepest markets in the world: cross-currency bases, repo-OIS, on-the-run premia, failed deliveries, dealer coupon holdings. The construction method is portable, this particular input set is not, and the paper makes no claim about frontier or thinly traded markets. The transfer I record is the recipe plus a CSE-specific substitution list (Amihud illiquidity, turnover ratio, zero-return frequency, quoted spread where the book is visible, Parkinson or Garman-Klass range volatility), not the inputs. The one quantitative CSE fact this interacts with is my own sample size, roughly 374 trading days per counter, which is what makes the parsimony result a live constraint rather than a curiosity.
+PROPOSED REVISION STATED IN THE NOTE: Build L_t as a rolling-window-PCA composite over CSE friction measures rather than as a single Amihud number, using the sign/z-score/first-PC/re-normalise recipe with an expanding window from a three-year block. Add the full-sample-versus-rolling PCA comparison as a standing look-ahead check in the methodology chapter, and generalise it to every fitted transform in the pipeline. Pre-register the parsimony response: any addition to f(L_t, V_t, P_t, C_{i,t}) must beat the existing set out-of-sample on the ablation protocol, with the static learned-weight baseline retained as the shrinkage-equivalent control. Run the AR-dominance test on the CSE liquidity state before building any state-forecasting machinery, and if a quantile AR(1) on L_t is as good as anything richer, condition on the lag. Test a short-horizon quantile forecast of L_t against its contemporaneous value as a conditioning input, as a named experiment. Add a market-wide L_t alongside the counter-level one as an ablation candidate, not an adopted feature. Adopt the rule that no SHAP plot is reported for an agent that has not beaten its own baseline out-of-sample. Report weight variation and return against the equal-weight and static-learned baselines over quiet sub-periods separately rather than only pooled, with friction charged either way, so the system is not credited for moving only in the two or three most volatile CSE months.
+STATUS: Reviewed in full from my own read, October 2026. This replaces the earlier provisional entry whose fields came from the source paper.</t>
         </is>
       </c>
     </row>
@@ -3947,122 +4034,122 @@
       </c>
     </row>
     <row r="27" ht="409.6" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>P26</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="28" t="inlineStr">
         <is>
           <t>Xia, You, Wang, Liu, Qi, Wu and Zhang, Shenzhen University with one author at the Shenzhen Audencia Financial Technology Institute, 2026. Fifty-nine pages, roughly the last fifteen appendices and references.</t>
         </is>
       </c>
-      <c r="C27" s="20" t="inlineStr">
+      <c r="C27" s="28" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>Not recorded in the note</t>
-        </is>
-      </c>
-      <c r="E27" s="20" t="inlineStr">
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>arXiv preprint (survey). Recovered from the Research Papers Grid entry 51 and the note header.</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
         <is>
           <t>staged note only; no DOI/URL recorded in the note.</t>
         </is>
       </c>
-      <c r="F27" s="20" t="inlineStr">
+      <c r="F27" s="28" t="inlineStr">
         <is>
           <t>Survey / systematic review and reproducibility audit of LLM-based trading agents. Note stresses "It presents itself as a survey of LLM-based trading agents, but the taxonomy is not what it is selling."</t>
         </is>
       </c>
-      <c r="G27" s="20" t="inlineStr">
+      <c r="G27" s="28" t="inlineStr">
         <is>
           <t>Prior reviews "organise the field by task coverage or by model-level benchmark performance and treat execution as an afterthought," producing three misclassifications — execution read as a byproduct of reasoning rather than a first-class architectural component, mechanism conflated with function (a multi-agent alpha-miner and a multi-agent trading system land in the same bucket), and adaptation treated as an implementation detail. Answer: the Architecture-Capability-Adaptation (A-C-A) lens, "offered explicitly as a working analytical lens rather than a validated taxonomy," plus an evidence ledger, a reproducibility audit and a reporting checklist, "which they name as the actual contributions."</t>
         </is>
       </c>
-      <c r="H27" s="20" t="inlineStr">
+      <c r="H27" s="28" t="inlineStr">
         <is>
           <t>Not a market study. Audited corpus is overwhelmingly US/crypto instruments; the note flags the named evaluation arenas (AI-Trader, Agent Market Arena, LiveTradeBench, ContestTrade, PredictionMarketBench) as "all of which are US or crypto instruments."  Agentic trading systems generally — alpha discovery, portfolio management, risk management, execution.</t>
         </is>
       </c>
-      <c r="I27" s="20" t="inlineStr">
+      <c r="I27" s="28" t="inlineStr">
         <is>
           <t>Literature corpus, not market data. Search 2022-01-01 through 2026-03-09 over ACM DL, IEEE Xplore, arXiv, SSRN, Google Scholar with backward/forward citation chaining. Funnel: 92 candidate records, 15 final exclusions, 77 included, partitioned 19 primary / 58 background. Reliability audits: S1 screening-boundary audit over 182 raw screening records (retained only as a screening-stage quality check, explicitly refused as evidence for extraction-level fields); S3 extraction-level audit over 15 fixed-seed primary studies, seed 20260426, 100.0% agreement after adjudication. Missing reporting coded conservatively as NR/Unknown. Corpus frame: "18/19 primary studies were published between 2024 and 2026, and 17/19 are currently coded as non-peer-reviewed against 2/19 peer-reviewed."</t>
         </is>
       </c>
-      <c r="J27" s="20" t="inlineStr">
+      <c r="J27" s="28" t="inlineStr">
         <is>
           <t>N/A (paper-level extraction fields: data &amp; universe, split protocol, action semantics, execution &amp; costs, leakage, artifacts, multi-agent reporting).</t>
         </is>
       </c>
-      <c r="K27" s="20" t="inlineStr">
+      <c r="K27" s="28" t="inlineStr">
         <is>
           <t>Four-step screening (keyword search, dedup, title/abstract screening against the finance/trading domain, full-text screening assigning primary vs background). Two criteria decide the primary subset and "the whole paper hangs off them": *Action Output* (system emits tradable actions — orders, position changes, portfolio allocations) and *Closed-Loop Evaluation* (actions evaluated in backtest, simulation or live trading rather than only through predictive metrics).  Not a system. Three reimplementable rules the note singles out, "each is a rule rather than a model": 1. Reasoning module as a typed contract — f(O_t, M_episodic, P_portfolio) → (A_cand, α, V_check), where O_t is a timestamped state observation at decision time t, M_episodic retrievable episodic memory, P_portfolio read-only portfolio state (positions, risk limits), A_cand a set of candidate actions, α ∈ [0,1] a confidence score, V_check a validity check such as holds &lt; max_leverage. Purpose: "risk constraints are enforced during or immediately after reasoning rather than at the final execution layer, so a hallucinated action never reaches the order interface." 2. Outcome Embargo against the "Oracle Fallacy" (retrieving a past episode whose stored text already contains a post-hoc narrative of how it turned out). Valid episode is (S_t, A_t, O_{t+k}, τ); retrieval constraint: retrieve(S_t, A_t, O_{t+k}) permitted only if t_now ≥ t+k. Paired with a recency decay term e^{−λ(t_now − t_k)} on the relevance score "so that retrieval does not keep surfacing high-similarity episodes from a regime that has ended." 3. Exposure cap: w_i(t) = min(w_i^max, risk_budget / risk_per_unit_i). Note: "deliberately simple, and it is in the paper because risk triggers, latency budgets and audit logs are inconsistently reported across the corpus, so the argument is about the disclosure convention rather than the formula." Action module formalised as f(D_t) → (A_order, A_algo) with typed order fields and explicit failure modes for rejection, partial fill and timeout fed back into memory; feasible actions conditioned on O_{t−δ} to respect processing latency.</t>
         </is>
       </c>
-      <c r="L27" s="20" t="inlineStr">
+      <c r="L27" s="28" t="inlineStr">
         <is>
           <t>- Number/heterogeneity: not a system; audits others. Only 9/19 primary studies address coordination mechanisms at all; multi-agent chapter section-level primary count is 12, "with the larger citation list made up of benchmarks and background agent-based modelling work that does not enter the primary total." - Combination: three coordination patterns compared — role-based, hierarchical, market-ecology. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." - Anything varying influence by market state? No — not in the survey's own design and not reported as present in the audited corpus. The survey's contribution here is negative evidence plus a protocol demand: "cross-play evaluation swapping individual agents to test interoperability against team overfitting, explicit communication constraints, crowding and impact metrics, and role or communication ablations to attribute gains to coordination rather than to compute. On their reading, complex decomposition currently obscures the source of gains rather than demonstrating them." - Confidence per agent: yes as an interface — α ∈ [0,1] emitted per decision inside the reasoning contract alongside V_check. Note: "it tells me the confidence score belongs in the agent's typed output rather than being inferred by the orchestrator after the fact." No comparability mechanism.</t>
         </is>
       </c>
-      <c r="M27" s="20" t="inlineStr">
+      <c r="M27" s="28" t="inlineStr">
         <is>
           <t>Not separately audited; text/news appears under MR-1 timestamp availability ("especially text and news").</t>
         </is>
       </c>
-      <c r="N27" s="20" t="inlineStr">
+      <c r="N27" s="28" t="inlineStr">
         <is>
           <t>Memory and RAG mapped to "the knowledge base" in the expert-system reading. Follow-up flagged: "the FinSage provenance-versioned knowledge-base design, which is the one semantic-memory entry in their comparison that reports both a versioned timestamp rule and a drift check."</t>
         </is>
       </c>
-      <c r="O27" s="20" t="inlineStr">
+      <c r="O27" s="28" t="inlineStr">
         <is>
           <t>Risk and compliance mapped to "rule constraints"; risk enforced inside the reasoning contract via V_check and the exposure cap above. Note records that "risk triggers, latency budgets and audit logs are inconsistently reported across the corpus." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): No cost model of the survey's own. Its audit finding is the cost datum: "1/19 (5.3%) specifies a transaction-cost model," and "the one I would quote first is the cost figure, because a literature in which one paper in nineteen models transaction costs cannot adjudicate any claim about net profitability." Microstructure signals (imbalance, spread, queue position) framed as "hard feasibility constraints filtering the action space rather than optimisation inputs." MR-4 demands execution timing and price assumption, rebalancing frequency, fees, spread, slippage, impact model, execution metrics plus sensitivity to cost assumptions.</t>
         </is>
       </c>
-      <c r="P27" s="20" t="inlineStr">
+      <c r="P27" s="28" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="Q27" s="20" t="inlineStr">
+      <c r="Q27" s="28" t="inlineStr">
         <is>
           <t>Accountability layer = logs plus human oversight; MR-6 demands "immutable logs linking order IDs to traces, rollback criteria for adaptive systems." Author-coined "Log-to-Narrative Verification" (flagged by the note as author synthesis, not surveyed evidence).</t>
         </is>
       </c>
-      <c r="R27" s="20" t="inlineStr">
+      <c r="R27" s="28" t="inlineStr">
         <is>
           <t>No performance synthesis at all. Reproducibility tiers R0–R3; evaluation-type counts 11 backtest, 3 live, 2 simulation, 3 benchmark. Seven minimum reporting items MR-1 to MR-7 (data &amp; universe; time-consistent splitting; action semantics; execution &amp; costs; leakage audit; artifacts &amp; logs; multi-agent evaluation), graded mandatory/recommended/optional by study type. KEY RESULTS (numbers): Within the 19 primary studies — "2/19 (10.5%) report an extractable time-consistent split protocol, 1/19 (5.3%) specifies a transaction-cost model, 1/19 documents universe or survivorship handling, 11/19 (57.9%) report execution timing or semantics, and 4/19 expose artifacts beyond narrative description." On split protocol, "17/19 are coded Unknown, 2 are coded other, and zero report walk-forward or rolling evaluation." Reproducibility: "Fifteen of nineteen primary studies sit at R0, no runnable artifacts at all, one at R1, three at R2, and none reaches R3, so R2 or above is 15.8%." "That zero in the R3 row is, on this sample, the single most citable number in the paper." Coordination: "Nine of the nineteen primary studies address coordination mechanisms at all," section-level primary count for the multi-agent chapter is 12. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." Adaptation: "The section-level primary count for supervised fine-tuning is N=0 and for meta-learning it is N=0, learning paradigms overall rest on 3 primary studies, one in-context learning and two reinforcement learning, and self-evolution carries 4 primary studies with every row of its comparison table tagged as background." The only performance figure anywhere: "the 53.17% cumulative return on SSE50 reported by Automate Strategy Finding, is quoted with Split: NR, Execution: NR, Cost: NR, Universe: SSE50, Tier: BG attached precisely to demonstrate that the number is illustrative rather than protocol-comparable." LIMITATIONS (quoting the note): "The lens and the checklist are both author-curated and neither is externally validated.… The standard the field is measured against was set by the people doing the measuring, and while the paper says so plainly in three places, a different set of authors could have made MR-7 mandatory for multi-agent systems and produced a different set of failing grades." "A denominator of 19 makes every percentage brittle, and the section-level zeros are the most brittle of all. One paper moves the headline figures by 5.3 points, so 10.5% for split protocols and 5.3% for cost models should be read as two papers and one paper, which is how I will quote them." "The audit measures papers and the narrative occasionally slips into measuring systems… for a corpus that is 89% preprints, much of what is missing is appendix material that a journal round would have forced out." "Several named frameworks are the authors' own inventions presented in the same register as surveyed evidence" — Cascaded Controller, Alpha-to-Trade Contract, Hierarchy of Truth, Log-to-Narrative Verification, Oracle Fallacy; "HiveMind (Xia et al. 2026) also appears as background in the coordination chapter without the self-citation being flagged." "It deliberately contains no performance synthesis, so it cannot tell me what works… it means the paper is a citation for why comparisons are unsafe and never a citation for a comparison."</t>
         </is>
       </c>
-      <c r="S27" s="20" t="inlineStr">
+      <c r="S27" s="28" t="inlineStr">
         <is>
           <t>Not recorded in the note.</t>
         </is>
       </c>
-      <c r="T27" s="20" t="inlineStr">
+      <c r="T27" s="28" t="inlineStr">
         <is>
           <t>Not recorded in the note.</t>
         </is>
       </c>
-      <c r="U27" s="20" t="inlineStr">
+      <c r="U27" s="28" t="inlineStr">
         <is>
           <t>"The reporting checklist becomes the spine of my evaluation chapter, with the CSE specifics filled in under each item" — universe construction and survivorship under MR-1 matter because "delistings, long trading suspensions and illiquid counters make the definition of the tradable universe a design decision that changes results"; MR-2 commits to "walk-forward with a stated embargo, which also settles how the orchestrator's own tuning is separated from final evaluation." "The execution-friction work is now positioned by the field's own counts rather than by my assertion. One paper in nineteen specifying a transaction-cost model, and zero coordination patterns reporting execution semantics, is a much stronger warrant for state-dependent friction in a thin book than the individual-paper evidence I have been leaning on, such as MacroHFT's flat 0.02% over roughly twenty round trips." "The reasoning I/O contract gives the heterogeneous-confidence problem a shape without solving it." "The outcome embargo and the recency decay are two memory rules I can implement, test and report in a paragraph"; memory settings are an "evaluation knob" — "retrieval window, similarity function and truncation all change decisions under the same base model, so ablations have to report memory settings or they are not ablations." "Role and communication ablations are the published form of the diagnostic I already pre-registered… Reporting it under MR-7 alongside a cross-play check, swapping one agent for a weaker or differently-specified version, converts a defensive self-check into a positive methodological contribution, and it is the answer to the objection that a heterogeneous ensemble is just more compute." "Fifteen of nineteen at R0 has a direct planning consequence and a direct opportunity… with 0/19 reaching R3 on this sample, a CSE system released with pinned environment, data access instructions, seeds and an end-to-end evaluation pipeline would be at a tier no audited paper in this corpus occupies." Time-scale taxonomy (reactive / reflective / strategic) justifies the reasoning budget: "LLM-mediated deliberation operates at second-scale latency at best and cannot support genuine high-frequency decisions… A daily or intraday CSE rebalance sits comfortably in the reflective band." Search budget: "iterative refinement against validation metrics mines the validation set unless the final result is reported on a sealed test set never exposed to the refinement loop"; also a stated "reflection budget," "because retrying until a profitable trade appears is testing into success."</t>
         </is>
       </c>
-      <c r="V27" s="20" t="inlineStr">
+      <c r="V27" s="28" t="inlineStr">
         <is>
           <t>No performance synthesis, no architecture recommendation, no evidence any design works — by construction. On the main gap specifically, it supplies α as a typed per-decision output but "does not supply is comparability, because an LLM analyst's self-reported α, an econometric estimator's interval width and an RL policy's value spread are on three different scales and the paper never addresses cross-agent calibration." Cross-play evaluation "I have not seen operationalised anywhere and may need to define myself."</t>
         </is>
       </c>
-      <c r="W27" s="20" t="inlineStr">
+      <c r="W27" s="28" t="inlineStr">
         <is>
           <t>[[Agentic Trading, When LLM Agents Meet Financial Markets]]</t>
         </is>
       </c>
-      <c r="X27" s="20" t="inlineStr">
+      <c r="X27" s="28" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (MR-7, cross-play, role/communication ablations, the α contract) and friction-aware evaluation layer (MR-1 to MR-6, the 1/19 cost figure, the microstructure-as-feasibility-constraint framing). Secondarily A_F via the episodic-memory/embargo rules.
 EFFECT ON MAIN GAP: Leaves it open and materially strengthens it. It supplies counted, denominator-attached evidence that coordination is under-evidenced (9/19), that no audited coordination pattern reports execution semantics, and that adaptation claims rest on 3 primary studies. Nothing in it does state-conditioned agent weighting. It does narrow the *shape* of one sub-problem: confidence is now specified as a typed per-agent output, so the residual is calibration, not representation.
@@ -4451,128 +4538,128 @@
       </c>
     </row>
     <row r="31" ht="409.6" customHeight="1">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="31" t="inlineStr">
         <is>
           <t>P30</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="28" t="inlineStr">
         <is>
           <t>Kou, Yu, Luo, Peng, Li, Liu, Dai, Chen, Han and Guo. HKUST, HKUST Guangzhou and Peking University.</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
-        <is>
-          <t>Not recorded in the note</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>Not recorded in the note</t>
-        </is>
-      </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="C31" s="28" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D31" s="28" t="inlineStr">
+        <is>
+          <t>arXiv preprint, arXiv:2409.06289v4 dated 3 November 2025. Recovered from the note header; the Research Papers Grid entry 43 left the year blank.</t>
+        </is>
+      </c>
+      <c r="E31" s="28" t="inlineStr">
         <is>
           <t>arXiv:2409.06289v4, 3 November 2025, seventeen pages plus seven-page appendix; code at github.com/kouzhizhuo/Automate-Strategy-Finding-with-LLM-in-Quant-investment.</t>
         </is>
       </c>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="F31" s="28" t="inlineStr">
         <is>
           <t>LLM-driven alpha factor mining plus multi-agent factor evaluation and weight optimisation.</t>
         </is>
       </c>
-      <c r="G31" s="20" t="inlineStr">
+      <c r="G31" s="28" t="inlineStr">
         <is>
           <t>Brittleness of deep learning in quant finance, decomposed into three challenges — "traditional alpha mining methods are rigid and do not adapt to dynamic markets, machine learning approaches struggle to integrate diverse data, and strategies do not adapt to market variability." Three-stage pipeline: LLMs generate executable alpha factor candidates from the alpha-mining literature; a multi-agent evaluation filters them on market status and predictive quality while maintaining category balance; a weight optimisation stage combines the survivors. Most important framing in the note: "I came to this from the BlackRock survey, which describes it as employing an adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions. That is not what the paper does, and the difference is the most useful thing I got out of reading it. The adaptivity here is at selection, not at weighting."</t>
         </is>
       </c>
-      <c r="H31" s="20" t="inlineStr">
+      <c r="H31" s="28" t="inlineStr">
         <is>
           <t>SSE50 (main), CSI300 and SP500 (cross-market).  Equity factor investing / daily long-only stock selection.</t>
         </is>
       </c>
-      <c r="I31" s="20" t="inlineStr">
+      <c r="I31" s="28" t="inlineStr">
         <is>
           <t>Six primary features (open, high, low, close, volume, VWAP) plus quarterly and annual reports of index constituents, January 2019 to June 2024. Main backtest SSE50: train Jan 2021 – Jun 2022, validation Jul – Dec 2022, test Jan 2023 – Jan 2024. Cross-market Table 5 uses rolling annual partitions with six-month test windows, H1 2021, H1 2022, H1 2023 for CSI300 and SP500. Ablation uses SSE50 data 2010–2022.</t>
         </is>
       </c>
-      <c r="J31" s="20" t="inlineStr">
+      <c r="J31" s="28" t="inlineStr">
         <is>
           <t>OHLCV + VWAP + financial reports. Seed alpha library from eleven documents given to GPT-4o including Kakushadze's *101 Formulaic Alphas* and Lopez de Prado's *Causal Factor Investing*. Every object is a formulaic alpha, "a short arithmetic expression over OHLCV and fundamentals such as CLOSE - DELAY(SMA(CLOSE, 14), 7)." Counts do not hold up: "the appendix taxonomy is introduced as eight categories and then lists nine, and the actual experimental prompt in A.7 describes 37 factors in eight groups. Liquidity is a category in the taxonomy, is absent from the eight groups the experiment's prompt actually names, and is absent from the five categories evaluated in Table 2, yet two liquidity expressions appear in the twelve selected alphas of Table 3."</t>
         </is>
       </c>
-      <c r="K31" s="20" t="inlineStr">
+      <c r="K31" s="28" t="inlineStr">
         <is>
           <t>Phase 2 — two agents each score every candidate alpha α_ij in category j against market condition M^(t): θ_ij = E[IC(α_ij | M^(t))] from the Confidence Score Agent, and ρ_ij = f_risk(α_ij, M^(t)) from the Risk Preference Agent. Mixed linearly with the best-scoring alpha in each category kept, subject to a confidence threshold: α*_j = argmax_{α_ij} [w_c · θ_ij + w_r · ρ_ij]. Phase 3 — a three-layer MLP, input width equal to the number of selected alphas, ten ReLU hidden nodes, one output, mapping historical daily alpha values to future yields, with a held-out validation set; its learned parameters become the combination weights. Composite signal: α^(t)_i = Σ_j w_j · α^(t)_ij. "Read the subscripts. The alpha values carry t, the weights do not, here or in Algorithm 2 line 30 or in the paper's equation 8. The abstract's 'dynamic weight optimization that adapts to market conditions' and the survey's 'real time' gating both describe w_j as though it were w_j^(t), and nothing in the method produces that. The weights change when the model is retrained on a new window, which is retraining, not gating."  Three-stage pipeline → composite alpha → portfolio. A.8: "daily reconstruction, rank all securities by composite alpha, take the top k = 13, limit churn to n = 5 names per day, equal weight across holdings. That is roughly 38% daily turnover, which the paper states and then never prices."</t>
         </is>
       </c>
-      <c r="L31" s="20" t="inlineStr">
+      <c r="L31" s="28" t="inlineStr">
         <is>
           <t>- Two agents in Phase 2 plus an MLP in Phase 3. Homogeneous in evidence type: "the paper is not proposing a new way to combine heterogeneous *analysts*. Every object in the system is a formulaic alpha… The two agents both evaluate those same expressions. This is one evidence type scored two ways, not four evidence types that have to be reconciled." Confidence Score Agent sees candidate alphas plus the market condition M^(t) and outputs an expected conditional IC; Risk Preference Agent sees the same and outputs a risk-character score. - Combination: two stages. Agent scores are mixed by a fixed linear rule α*_j = argmax [w_c θ_ij + w_r ρ_ij] with w_c = 0.6, w_r = 0.4; the surviving factors are combined by a static MLP whose weights carry no time index. - Does anything vary influence by market state? Selection yes, weighting no — and this is the single most important correction in the note. Which factors enter is conditioned on M^(t), because M^(t) is passed to both evaluating agents. How much each selected factor counts is "a weight vector produced once by a small MLP trained on a fixed historical window, and it carries no time index anywhere in the paper's equations or in its algorithm listing." Quoting the note's headline: "The adaptivity here is at selection, not at weighting." And: "So this is not a competitor to my orchestrator. It is the strongest published instantiation I have of Baseline 2, the static learned weight, which the supervisor identified as the baseline that actually matters, and it is the reference design I should implement that arm against." - Confidence per agent: yes, and it is the most directly reusable confidence construct in the set — θ_ij = E[IC(α_ij | M^(t))], an expected conditional information coefficient, paired with a separate risk score, mixed linearly. Comparability is trivial here because both scores are over the same object type. The note's port: "each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target."</t>
         </is>
       </c>
-      <c r="M31" s="20" t="inlineStr">
+      <c r="M31" s="28" t="inlineStr">
         <is>
           <t>None used. "Multimodality is claimed in the abstract, drawn in Figure 1 and tabulated in the appendix, and never used. Table 11 lists audio data, financial morning news radio and market discussion radio, and video data, CCTV Securities Information Channel, as framework inputs. No experiment in the paper uses audio or video… The multimodal architecture is a taxonomy presented as a capability."</t>
         </is>
       </c>
-      <c r="N31" s="20" t="inlineStr">
+      <c r="N31" s="28" t="inlineStr">
         <is>
           <t>Quarterly and annual reports enter as factor inputs; no retrieval system.</t>
         </is>
       </c>
-      <c r="O31" s="20" t="inlineStr">
+      <c r="O31" s="28" t="inlineStr">
         <is>
           <t>The Risk Preference Agent scores "how the alpha behaves under different risk scenarios," conditional on market state. No explicit volatility model. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): None stated. "Table 4 reports final return, Sharpe, volatility, Sortino and Calmar with no cost column, and A.8 says only that the turnover level 'demonstrates favorable characteristics in our transaction cost modeling' without giving a rate anywhere in the paper." Liquidity as a factor category is defined and then dropped from the evaluated groups; two volume-based expressions nonetheless survive into the final twelve.</t>
         </is>
       </c>
-      <c r="P31" s="20" t="inlineStr">
+      <c r="P31" s="28" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="Q31" s="20" t="inlineStr">
+      <c r="Q31" s="28" t="inlineStr">
         <is>
           <t>Factors are human-readable arithmetic expressions; the weights come from an MLP, so the combination is not interpretable. IC sign confusion undermines readability: "Table 3's weighted combination scores −0.0587 against individual alphas in the ±0.02 range, and the text calls this 'quite high', reading the magnitude and ignoring the sign."</t>
         </is>
       </c>
-      <c r="R31" s="20" t="inlineStr">
+      <c r="R31" s="28" t="inlineStr">
         <is>
           <t>SSE50 backtest against LLM baselines FinCon (22.47%) and SEP (17.89%), benchmark −13.22%. Ablations removing each of the two agents. Regime breakdown (bull/bear/sideways). Cross-market Table 5/6. Sensitivity sweeps over the confidence-to-risk mixing weight and hyperparameters.</t>
         </is>
       </c>
-      <c r="S31" s="20" t="inlineStr">
+      <c r="S31" s="28" t="inlineStr">
         <is>
           <t>"Removing the Confidence Score Agent drops out-of-sample IC from 0.047 to 0.032, a 31.9% fall, and removing the Risk Preference Agent drops it to 0.039." Full model 0.059 in-sample / 0.047 out-of-sample / Sharpe 1.94; without Confidence 0.054 / 0.032 / 1.51; without Risk 0.056 / 0.039 / 1.34. Regime: "the full model holds out-of-sample IC at 0.051 bull, 0.042 bear and 0.045 sideways, while without the confidence agent the bear-market figure collapses to 0.021, half the full model's. On this sample, conditioning *which* factors are used on the market state is doing real work, and it is doing most of it when conditions are bad." Headline "53.17% is gross, on 38% daily turnover, against a benchmark of −13.22%." Sensitivity sweep of the confidence/risk mix: overall Sharpe 8.10, −2.68, 11.39, −5.10, −8.04, 9.00, −4.35 across the seven settings, with the chosen 0.6/0.4 at 11.39 "sitting directly between two negative results." Regularisation 0.0005 / 0.001 / 0.002 gives −1.88 / 13.33 / −6.91. Drawdown: "maximum drawdown is deeper than the benchmark's in four, −19.40 against −10.86 and −17.03 against −8.44 on CSI300, −7.89 against −4.23 and −11.52 against −7.75 on SP500, and shallower only in the H1 2022 downturn in both markets." LIMITATIONS (quoting the note): "The comparison that would isolate the weighting stage is not run. Both ablations remove an *agent* from the selection phase. Neither removes the MLP, so there is no arm anywhere in the paper showing what an equal-weighted combination of the same twelve selected alphas would have returned, and therefore no evidence that learning the weights contributes anything over the selection that precedes it… This is the limitation that most directly shapes my own design, because the missing arm is exactly the comparison my three-way weighting study is built to make." "Look-ahead exposure is structural and unaddressed. GPT-4o, whose training data extends well past the 2023 test period, is asked in the A.7 prompt to 'select the factors that will perform best in the last quarter of the SSE 50' for the test window… The paper offers no contamination check… That does not mean the result is contaminated, it means the paper provides nothing that would let me rule it out, and the effect would look exactly like the reported outperformance." "The Sharpe ratio is reported on at least three mutually incompatible scales and the convention is never stated… No equity strategy has a Sharpe of 13, so at least two of these tables are measuring something other than what the label says… only the within-table comparisons are readable and no number here can be carried into a sentence of mine." "The sensitivity studies show instability rather than sensitivity… a surface that alternates sign under a one-step parameter change is not a surface with an optimum on it, and the reported configuration is better described as the best of a noisy sweep than as a tuned choice." "The two metrics in that ablation disagree about which agent matters, and the paper reports only one of the answers." "Internal inconsistencies are frequent enough to affect how much weight any single figure can bear."</t>
         </is>
       </c>
-      <c r="T31" s="20" t="inlineStr">
+      <c r="T31" s="28" t="inlineStr">
         <is>
           <t>Not recorded in the note.</t>
         </is>
       </c>
-      <c r="U31" s="20" t="inlineStr">
-        <is>
-          <t>"This is my static-learned-weight baseline, and I should build that arm to this design rather than to a strawman. Baseline 2 is the one the supervisor singled out, because beating equal weighting proves little if a fixed learned weight gets there too, and until now I had no reference implementation of it… The comparison this paper never runs, equal weight against learned static weight over an identical input set, is the first half of my experimental design, and I can now say plainly in the write-up that the nearest prior work does not report it." "Adaptivity at selection and adaptivity at weighting are separable, and I should evaluate both. This system conditions which factors are in the set on the market state and then weights them statically. Mine conditions the weights and keeps the agent set fixed… so the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically, and I would rather find that out in my own ablation than have it raised in a viva." "Keep the orchestrator low-capacity. A ten-node MLP over roughly twelve inputs, trained on a fifty-stock universe with eighteen months of daily data, produces a Sharpe surface that flips sign when L2 regularisation moves from 0.001 to 0.002… That argues for a weighting function with a handful of interpretable parameters, a gated linear form or a shallow regression on the four state variables, rather than a network, and it argues for reporting the stability sweep rather than only the tuned configuration." "The two-agent scoring scheme is a usable template for the agent-confidence term, with one caution attached. Expected conditional information coefficient as a confidence score and a separate risk-character score, mixed linearly, is implementable for my four agents as each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target. The caution is that the mixing ratio between the two components is exactly the parameter this paper's sensitivity table shows to be unstable, so if I adopt a two-component confidence I fix that ratio on the validation split and report the sweep, rather than selecting it on the test window as this paper appears to." "The liquidity factor definitions transfer to the CSE even though the experiment's factor set excludes them. Amihud illiquidity as ABS(RETURN) / VOLUME, turnover as VOLUME / SHARES_OUTSTANDING, the high-low spread proxy (HIGH - LOW) / CLOSE and VOLUME / MARKET_CAP are all computable from the OHLCV and shares-outstanding data I expect to have, with no quote feed required, and the high-low proxy is the one that survives if I never get bid-ask data." "Gross returns on 38% daily turnover make the friction layer a contribution rather than housekeeping… The turnover constraint itself, cap the number of names replaced per session rather than the fraction of capital traded, is a clean mechanism worth borrowing." "They name the stationarity assumption behind state-conditional weighting and do not test it, which is precisely my persistence ablation. Their own limitations section states that the multi-agent evaluation presupposes persistent historical relationships between market conditions and alpha performance, an assumption that may prove tenuous during regime shifts. That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment nobody in this line of work has run. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." "Prompt hygiene needs to be a stated part of my method… the evaluation window must not be named in any prompt, the agent instructions must not ask which factors performed best in a period that overlaps the test set, and I should report a contamination check of some kind."</t>
-        </is>
-      </c>
-      <c r="V31" s="20" t="inlineStr">
+      <c r="U31" s="28" t="inlineStr">
+        <is>
+          <t>"This is my static-learned-weight baseline, and I should build that arm to this design rather than to a strawman. Baseline 2 is the one the supervisor singled out, because beating equal weighting proves little if a fixed learned weight gets there too, and until now I had no reference implementation of it… The comparison this paper never runs, equal weight against learned static weight over an identical input set, is the first half of my experimental design, and I can now say plainly in the write-up that the nearest prior work does not report it." "Adaptivity at selection and adaptivity at weighting are separable, and I should evaluate both. This system conditions which factors are in the set on the market state and then weights them statically. Mine conditions the weights and keeps the agent set fixed… so the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically, and I would rather find that out in my own ablation than have it raised in a viva." "Keep the orchestrator low-capacity. A ten-node MLP over roughly twelve inputs, trained on a fifty-stock universe with eighteen months of daily data, produces a Sharpe surface that flips sign when L2 regularisation moves from 0.001 to 0.002… That argues for a weighting function with a handful of interpretable parameters, a gated linear form or a shallow regression on the four state variables, rather than a network, and it argues for reporting the stability sweep rather than only the tuned configuration." "The two-agent scoring scheme is a usable template for the agent-confidence term, with one caution attached. Expected conditional information coefficient as a confidence score and a separate risk-character score, mixed linearly, is implementable for my four agents as each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target. The caution is that the mixing ratio between the two components is exactly the parameter this paper's sensitivity table shows to be unstable, so if I adopt a two-component confidence I fix that ratio on the validation split and report the sweep, rather than selecting it on the test window as this paper appears to." "The liquidity factor definitions transfer to the CSE even though the experiment's factor set excludes them. Amihud illiquidity as ABS(RETURN) / VOLUME, turnover as VOLUME / SHARES_OUTSTANDING, the high-low spread proxy (HIGH - LOW) / CLOSE and VOLUME / MARKET_CAP are all computable from the OHLCV and shares-outstanding data I expect to have, with no quote feed required, and the high-low proxy is the one that survives if I never get bid-ask data." "Gross returns on 38% daily turnover make the friction layer a contribution rather than housekeeping… The turnover constraint itself, cap the number of names replaced per session rather than the fraction of capital traded, is a clean mechanism worth borrowing." "They name the stationarity assumption behind state-conditional weighting and do not test it, which is precisely my persistence ablation. Their own limitations section states that the multi-agent evaluation presupposes persistent historical relationships between market conditions and alpha performance, an assumption that may prove tenuous during regime shifts. That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." "Prompt hygiene needs to be a stated part of my method… the evaluation window must not be named in any prompt, the agent instructions must not ask which factors performed best in a period that overlaps the test set, and I should report a contamination check of some kind."</t>
+        </is>
+      </c>
+      <c r="V31" s="28" t="inlineStr">
         <is>
           <t>No time index on the weights; the weighting stage is never ablated; costs unpriced; look-ahead unaddressed; liquidity category defined and excluded.</t>
         </is>
       </c>
-      <c r="W31" s="20" t="inlineStr">
+      <c r="W31" s="28" t="inlineStr">
         <is>
           <t>[[Automate Strategy Finding with LLM in Quant investment]]</t>
         </is>
       </c>
-      <c r="X31" s="20" t="inlineStr">
+      <c r="X31" s="28" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (as Baseline 2, the static learned weight), A_T (formulaic alphas), A_L (liquidity factor definitions), friction-aware evaluation layer (38% turnover unpriced).
 EFFECT ON MAIN GAP: Leaves it open — and the note's rereading of this paper is what keeps it open. The BlackRock survey had nominated it as the nearest prior art with a "dynamic weighting mechanism"/"adaptive gating mechanism that tunes the influence of each signal in real time." On the paper's own equations that description is unsupported. Net effect: the one candidate the field itself pointed at as occupying the gap turns out to be a static-learned-weight baseline. It does, however, narrow the gap in one direction — it demonstrates that state-conditional *selection* carries real signal, mostly in bear regimes (bear IC 0.042 full vs 0.021 without the confidence agent), which obliges the student to add a state-conditional-inclusion / static-weight configuration to their own ablation to prove the weighting function is what is doing the work.
 CONFIDENCE SCORING: Yes — the cleanest formal template in the set, though not a cross-*heterogeneity* solution. Expected conditional IC as confidence plus a separate risk-character score, linearly mixed. Caution attached: the mixing ratio is exactly the unstable parameter in their sensitivity table, so fix it on validation and report the sweep.
 FIXED-INFLUENCE FAILURE EVIDENCE: Indirect. The weighting stage is never ablated, so no failure is observable by construction; the note treats that absence as the missing arm rather than as evidence. The nearest documented degradation is the drawdown result — the strategy is deeper in drawdown than the benchmark in four of six cross-market windows while the abstract claims general downside protection, with nothing in the system detecting it.
-PROPOSED REVISION STATED IN THE NOTE: To the experimental design rather than the pool, but it directly touches the conditioning set. Verbatim: "the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically." And on P_t, verbatim: "That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment nobody in this line of work has run. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." Also: "Keep the orchestrator low-capacity… a gated linear form or a shallow regression on the four state variables, rather than a network."</t>
+PROPOSED REVISION STATED IN THE NOTE: To the experimental design rather than the pool, but it directly touches the conditioning set. Verbatim: "the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically." And on P_t, verbatim: "That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." Also: "Keep the orchestrator low-capacity… a gated linear form or a shallow regression on the four state variables, rather than a network."</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4892,7 @@
       </c>
       <c r="U33" s="20" t="inlineStr">
         <is>
-          <t>"This is the third documented case of a fixed-influence component degrading a multi-agent system, and the first that puts a number on it. FinAgent has auxiliary strategies returning 16% on ETHUSD against a 29% passive benchmark, AlphaAgents drops its sentiment agent outright for insufficient coverage, and here a news agent costs 10.36 points of total return while the architecture has no way to notice. The three together are the evidentiary base for the main gap, and this one is the strongest because the degradation is measured under a controlled ablation rather than inferred. The obvious counterfactual, a system that could down-weight the news agent on days when it diverges, is exactly what I am proposing and exactly what nobody here builds." "Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem." "That gives me a pre-registered test rather than an assumption… If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses. Either outcome is publishable and the cost is one scoring pass." "Another paper where execution friction never binds, which keeps the thin-market case open… The CSE charges materially more, the book is thin enough that impact is a separate cost on top of the spread, and every one of these systems was designed and tuned in a regime where cost is a rounding error." "Sentiment is out of scope for my project as of this note, so the news half of the ablation is the part that still speaks to my design… of the two text agents tested here the news agent is the nearer analogue, dated factual material summarised for a decision rather than community tone. That is the agent that cost 10.36 points of total return. The lesson is not that filings will hurt… it is that a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to, and that the demonstration costs one on-off ablation. Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one." "The horizon reversal is a prior against an all-LLM design, and it argues for my heterogeneity claim from the other direction.… An orchestrator that can shift weight toward a recurrent or econometric component at long horizons and toward the reasoning agents at short ones is a concrete, testable instantiation of the main gap, and this paper supplies the horizon evidence for free." "The evaluation harness is the part I should copy wholesale, including the trade-count calibration." "An honest null on the orchestration weights is a better outcome than a 1.7-point win I cannot defend."</t>
+          <t>"This is the third documented case of a fixed-influence component degrading a multi-agent system, and the first that puts a number on it. FinAgent has auxiliary strategies returning 16% on ETHUSD against a 29% passive benchmark, AlphaAgents drops its sentiment agent outright for insufficient coverage, and here a news agent costs 10.36 points of total return while the architecture has no way to notice. The three together are the evidentiary base for the main gap, and this one is the strongest because the degradation is measured under a controlled ablation rather than inferred. The obvious counterfactual, a system that could down-weight the news agent on days when it diverges, is exactly what I am proposing and exactly what this paper does not build." "Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem." "That gives me a pre-registered test rather than an assumption… If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses. Either outcome is publishable and the cost is one scoring pass." "Another paper where execution friction never binds, which keeps the thin-market case open… The CSE charges materially more, the book is thin enough that impact is a separate cost on top of the spread, and every one of these systems was designed and tuned in a regime where cost is a rounding error." "Sentiment is out of scope for my project as of this note, so the news half of the ablation is the part that still speaks to my design… of the two text agents tested here the news agent is the nearer analogue, dated factual material summarised for a decision rather than community tone. That is the agent that cost 10.36 points of total return. The lesson is not that filings will hurt… it is that a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to, and that the demonstration costs one on-off ablation. Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one." "The horizon reversal is a prior against an all-LLM design, and it argues for my heterogeneity claim from the other direction.… An orchestrator that can shift weight toward a recurrent or econometric component at long horizons and toward the reasoning agents at short ones is a concrete, testable instantiation of the main gap, and this paper supplies the horizon evidence for free." "The evaluation harness is the part I should copy wholesale, including the trade-count calibration." "An honest null on the orchestration weights is a better outcome than a 1.7-point win I cannot defend."</t>
         </is>
       </c>
       <c r="V33" s="20" t="inlineStr">
@@ -6210,122 +6297,122 @@
       </c>
     </row>
     <row r="45" ht="409.6" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="A45" s="31" t="inlineStr">
         <is>
           <t>P44</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B45" s="28" t="inlineStr">
         <is>
           <t>European Journal of Operational Research 270(2), 654–669. Fischer and Krauss, Department of Statistics and Econometrics, Erlangen-Nürnberg.</t>
         </is>
       </c>
-      <c r="C45" s="20" t="inlineStr">
-        <is>
-          <t>Not recorded in the note</t>
-        </is>
-      </c>
-      <c r="D45" s="20" t="inlineStr">
-        <is>
-          <t>European Journal of Operational Research 270(2), 654–669.</t>
-        </is>
-      </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="C45" s="28" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D45" s="28" t="inlineStr">
+        <is>
+          <t>European Journal of Operational Research 270(2), 654-669. Recovered from the Research Papers Grid entry 53 and the note header.</t>
+        </is>
+      </c>
+      <c r="E45" s="28" t="inlineStr">
         <is>
           <t>none recorded. "No code release."</t>
         </is>
       </c>
-      <c r="F45" s="20" t="inlineStr">
+      <c r="F45" s="28" t="inlineStr">
         <is>
           <t>statistical arbitrage via cross-sectional directional prediction.</t>
         </is>
       </c>
-      <c r="G45" s="20" t="inlineStr">
+      <c r="G45" s="28" t="inlineStr">
         <is>
           <t>"LSTM networks applied to directional prediction on the full S&amp;P 500 constituent universe from December 1992 to October 2015, framed as statistical arbitrage rather than as forecasting, where the model takes a single feature, the standardised one-day return, over a 240-day sequence and outputs the probability that a stock beats the cross-sectional median return tomorrow." The note's positioning: "this learns a ranking signal and hands it to a fixed mechanical trading rule, which is exactly the shape of A_T feeding an orchestrator, so I am reading it as a specification for that one agent rather than as a competitor architecture."</t>
         </is>
       </c>
-      <c r="H45" s="20" t="inlineStr">
+      <c r="H45" s="28" t="inlineStr">
         <is>
           <t>US equities, S&amp;P 500 constituents, survivor-bias free.  deep learning for cross-sectional equity ranking.</t>
         </is>
       </c>
-      <c r="I45" s="20" t="inlineStr">
+      <c r="I45" s="28" t="inlineStr">
         <is>
           <t>constituent lists from Thomson Reuters December 1989 to September 2015 consolidated into a binary membership matrix; daily total return indices January 1990 to October 2015, cum-dividend, adjusted for corporate actions and splits. Study period = 750 training days plus 250 trading days, rolled forward by 250 days; 23 non-overlapping trading periods; out-of-sample December 1992 to October 2015, 5750 trading days.</t>
         </is>
       </c>
-      <c r="J45" s="20" t="inlineStr">
+      <c r="J45" s="28" t="inlineStr">
         <is>
           <t>a single feature, the standardised one-day return, sequence length 240. Standardisation R̃^{m,s}_t = (R^{m,s}_t − μ^m_train)/σ^m_train, moments from the training portion only — "footnoted as key in order to avoid look-ahead biases."</t>
         </is>
       </c>
-      <c r="K45" s="20" t="inlineStr">
+      <c r="K45" s="28" t="inlineStr">
         <is>
           <t>LSTM, h = 25 hidden units, dropout 0.1 on the recurrent layer, RMSprop, cross-entropy, early stopping on a 20% validation split with patience 10 against a ceiling of 1000 epochs. Benchmarks: random forest (1000 trees, max depth 20, m = √p), deep net (31/10/5/2, maxout, dropout 0.5), logistic regression (L2 cross-validated over 100 values from 0.0001 to 10,000), all fed 31 engineered cumulative returns over m ∈ {1,…,20} ∪ {40, 60, …, 240}.  binary cross-sectional target Y^s_{t+1} = 1 if R^{1,s}_{t+1} ≥ median over the cross-section, else 0. Output is a probability, used ordinally to rank; trade long top k, short flop k, k ∈ {10, 50, 100, 150, 200}, equal weight, one-day hold. Parameter count 4hi + 4h + 4h² = 4(h(i + h + 1)); at h=25, i=1 that is 2700 plus 52 for the dense output, "so 2752 trainable parameters against roughly 255,000 training sequences, which the paper reports as approximately 93 training examples per parameter".</t>
         </is>
       </c>
-      <c r="L45" s="20" t="inlineStr">
+      <c r="L45" s="28" t="inlineStr">
         <is>
           <t>none — and that absence is the note's central exhibit for the main gap.</t>
         </is>
       </c>
-      <c r="M45" s="20" t="inlineStr">
+      <c r="M45" s="28" t="inlineStr">
         <is>
           <t>none.</t>
         </is>
       </c>
-      <c r="N45" s="20" t="inlineStr">
+      <c r="N45" s="28" t="inlineStr">
         <is>
           <t>none.</t>
         </is>
       </c>
-      <c r="O45" s="20" t="inlineStr">
+      <c r="O45" s="28" t="inlineStr">
         <is>
           <t>no volatility model. Volatility appears only descriptively, as a property of what the network selects: selected stocks "sit at higher 240-day rolling volatility of 0.0303 against 0.0213, higher kurtosis of 5.81 against 4.80, and a market beta of 1.19 against 1.05, with the effect strengthening as k shrinks." Risk control is structural rather than modelled — it comes from the long-short construction, which yields "a market beta of −0.0023 that is not significantly different from zero." No conditional variance, no persistence, no exposure scaling, no risk budget.</t>
         </is>
       </c>
-      <c r="P45" s="20" t="inlineStr">
+      <c r="P45" s="28" t="inlineStr">
         <is>
           <t>cost is "5 basis points per half-turn", flat, "with no size or depth term, on a universe chosen for being the 500 largest US stocks. No spread, no depth, no impact and no partial fill anywhere." The note: "This is the same execution-friction blind spot I have written into every trading paper in the vault so far, with the difference that this one at least measures the VWAP haircut, so the friction is observed even though it is never modelled." The execution ladder is the measurement: daily close → daily VWAP → weekly close → weekly VWAP → weekly with a day's wait. Microstructure contamination is acknowledged by the authors: "buying recent losers means buying stocks more likely to be quoted at the ask and selling recent winners more likely to be quoted at the bid, so part of the measured return is bid-ask bounce."</t>
         </is>
       </c>
-      <c r="Q45" s="20" t="inlineStr">
+      <c r="Q45" s="28" t="inlineStr">
         <is>
           <t>a two-step template — characterise the selected set with descriptive statistics and factor loadings, then build the simplest transparent rule reproducing the dominant pattern and report what fraction of the return it captures. "Fifty percent from a five-day reversal rule says more about what the model learned than any saliency map and costs nothing beyond statistics I am computing anyway."</t>
         </is>
       </c>
-      <c r="R45" s="20" t="inlineStr">
+      <c r="R45" s="28" t="inlineStr">
         <is>
           <t>random forest, deep net, logistic regression on identical data; Diebold-Mariano with Bonferroni correction; Pesaran-Timmermann; Newey-West t-statistics; Fama-French-style factor regression.</t>
         </is>
       </c>
-      <c r="S45" s="20" t="inlineStr">
+      <c r="S45" s="28" t="inlineStr">
         <is>
           <t>"Before costs, 0.46 percent per day against 0.43, 0.32 and 0.26 for the random forest, the deep net and the logistic regression, at standard deviations of 2.09 against 2.15, 2.62 and 2.69, giving annualised Sharpe ratios of 5.83, 5.00, 2.43 and 1.70 and accuracies of 54.3, 53.8, 53.7 and 52.2 percent. After 5 basis points per half-turn those returns become 0.26, 0.23, 0.12 and 0.06, so costs remove 43 percent of the LSTM's gross return." The formal test is marginal: "the Diebold-Mariano p-value for the null that the LSTM's forecasts are inferior to the random forest's coming in at 0.0143 against a Bonferroni-adjusted threshold of 1.67 percent". Ranking-depth reversal: "Daily returns fall monotonically from 0.46 percent at k=10 to 0.10 percent at k=200 and the Sharpe ratio from 5.83 to 3.30, but the random forest decays more slowly and takes the Sharpe lead at k=150 with 3.82 against 3.68, holding it at k=200 with 3.58 against 3.30." Era instability: "From 1993 to 2000 the LSTM is superior in almost all years, cumulative payouts on a 1 USD average daily investment reaching roughly 11 USD against the random forest's 8. From 2001 to 2009 the two run together until the crisis, where the random forest posts close to 0.9 percent per day in 2008 against the LSTM's 0.15 and finishes the era at 5.6 USD against 4. From 2010 to 2015 the LSTM oscillates around zero while the random forest goes strictly negative to roughly −1.2 USD." Selection profile: "Top k=10 stocks enter the trade on a five-day cumulative return of −4.05 percent against the flop stocks' +4.54 and a cross-sectional mean of +0.26". Factor regression: "an intercept of 0.42 percent per day at an R² of 0.0330 with significant loadings on short-term reversal at 0.3792 and momentum at −0.1241, against the random forest's 0.34 percent at an R² of 0.1338". Transparent rule: "yields 0.23 percent per day before costs, roughly 50 percent of the LSTM's, and loses its edge entirely after costs." Execution ladder: "the daily close-execution baseline returns 0.20 percent per day after costs at 53.76 percent annualised. Executing on volume-weighted average prices instead drops it to 0.16 percent and 42.87 percent, a weekly close variant to 0.11 percent, a weekly VWAP variant to 0.09 percent, and a weekly variant with a full day of waiting between signal and execution to 0.09 percent at 20.52 percent annualised... the ladder from 53.76 to 20.52 percent annualised is the size of the gap between a close-price backtest and something closer to implementable, on the most liquid equity market in the world." LIMITATIONS (quoting the note): "The cost model is a flat 5 basis points per half-turn with no size or depth term." "The signal's core is short-term reversal, which is partly a microstructure artefact, and the tests bound the problem without resolving it... survival on a universe with penny spreads bounds nothing about a market where the spread is a meaningful fraction of the daily move." "Everything is one run and the crucial comparison is marginal... the defensible statement is that the two methods are close and the ordering depends on the slice, not that the LSTM is the better model." "Nothing conditions on market state, and Figure 5 is the bill for that... the paper observes its own signal decaying to zero after 2010 and its benchmark going strictly negative with no channel through which either observation could change behaviour... it is simultaneously a description of a system that cannot respond to its own deterioration." "The probability output is used ordinally and never checked for calibration... no reliability diagram, no Brier score... Since I want to use exactly this kind of score as an agent confidence input, the absence is worth naming as an open question." "The cross-sectional median target assumes a dense, simultaneously priced cross-section... It degrades quietly rather than loudly when it does."</t>
         </is>
       </c>
-      <c r="T45" s="20" t="inlineStr">
+      <c r="T45" s="28" t="inlineStr">
         <is>
           <t>Not recorded in the note.</t>
         </is>
       </c>
-      <c r="U45" s="20" t="inlineStr">
+      <c r="U45" s="28" t="inlineStr">
         <is>
           <t>the cross-sectional relative target, taken early; cross-sectional pooling as the answer to the data-depth blocker; Figure 5 as the flagship evidence for the main gap; the execution ladder as the friction-aware protocol; the black-box attribution template; the recognition that the missing short leg relocates risk control onto A_V.</t>
         </is>
       </c>
-      <c r="V45" s="20" t="inlineStr">
+      <c r="V45" s="28" t="inlineStr">
         <is>
           <t>no state conditioning, no calibration, no depth-aware cost model, no seeds, and a target that assumes a dense cross-section.</t>
         </is>
       </c>
-      <c r="W45" s="20" t="inlineStr">
+      <c r="W45" s="28" t="inlineStr">
         <is>
           <t>[[Deep Learning with Long Short-Term Memory Networks for Financial Market Predictions]]</t>
         </is>
       </c>
-      <c r="X45" s="20" t="inlineStr">
+      <c r="X45" s="28" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T (this is the specification for the technical agent), orchestrator (Figure 5 is the main gap's empirical exhibit; C_{A_T,t} design), A_L and A_V (the selection-bias argument for why they are agents rather than post-processing), evaluation layer (the execution ladder).
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap — this is the strongest published evidence in the set. "Figure 5 is the best single piece of published evidence I have for the main gap, and I should cite it as such. Two heterogeneous predictors trained on identical data, one winning 1993 to 2000, the other winning decisively through 2008, the first winning again 2010 to 2015 by virtue of losing less, with no mechanism anywhere in the design to shift weight between them. A static equal blend would have been beaten by one of its own members in each of the three eras, and a state-conditional blend is exactly what my orchestrator is. This is stronger than the FinAgent and AlphaAgents cases I have been leaning on, because those are failures of a component that should have been switched off, whereas here both components are genuinely useful and the useful one changes." It also dictates evaluation shape: "report the three-way weighting comparison per era or per volatility regime, not only in aggregate, since an aggregate hides exactly this pattern." Sub-gap 1 — strong bearing. The k-depth reversal locates the edge "concentrated in the extreme tails of its own ranking, which is precisely where a thin market cannot absorb the trade". The execution ladder quantifies what realism costs on the most liquid market in the world (53.76 → 20.52 percent annualised), and the note adapts it: the one-day-waiting variant becomes "the cheap test for whether an apparent reversal signal is bid-ask bounce... a validity check rather than a robustness afterthought", with the VWAP leg conditional on intraday CSE data that has not been confirmed to exist. And the selection bias makes liquidity a constraint on the agent rather than a downstream cost: "the liquidity channel is not only a cost model downstream of the decision, it is a constraint on the technical agent's selection, one measurement serving both."
@@ -6455,7 +6542,7 @@
         <is>
           <t>SPEAKS TO: orchestrator above all (abstention, and the common confidence scale for C_{i,t}), evaluation layer (coverage/accuracy pairing; the expectation band for honest CSE directional accuracy), A_L (the abstention-as-liquidity-screen check), A_T (the expectation band and the leak warning).
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap — this is the single most directly useful paper in the set for the orchestration argument's second half. "My orchestration argument has always had two parts, that an agent's reliability varies with conditions and that the agents do not know it, and the second part is the one with no published mechanism behind it. AlphaAgents deleted its sentiment agent by hand and FinAgent's auxiliary strategies degraded quietly on ETHUSD, both because nothing in either design could decline to speak. This paper declines to speak, measures what declining costs, and publishes the frontier." It also supplies a concrete route to the comparable-confidence problem in C_{i,t}: "the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not." And it names precisely what must not be copied: "What I cannot borrow is the combiner itself, since a forest over two static features has no channel for liquidity state or volatility persistence and therefore reproduces exactly the fixed-influence design the main gap objects to, the same structural limitation as the near-binary mixture in [[MacroHFT...]]. The compression is the reusable part, the conditioning is mine to add." Sub-gap 1 — real bearing via the abstention-as-liquidity-screen problem: "On the CSE, an abstention threshold is partly a liquidity screen and I need to say which... the counters clearing a confidence bar are very likely the ones printing densely... So the check is to regress trusted-day frequency per counter on Amihud illiquidity and turnover before claiming the threshold is measuring confidence, which is the same measurement already being computed for the cost model, serving a third purpose." Plus the exposure policy on abstained days: "The abstained days also need an explicit exposure policy, hold the previous position or go flat, since those are different strategies and on the CSE the flat option carries a round-trip cost each time."
-EFFECT ON SUB-GAP 2: LEAVES IT OPEN. There is no volatility quantity anywhere in this paper, so nothing is operationalised in the persistence direction. Its relevance is oblique but real in one respect: it is the only paper in the set where a *confidence* quantity is operationalised into a decision (trade or abstain), which is the structural template Sub-gap 2 needs for its own quantity — a measured scalar that gates action rather than describing it. The note's own framing of the missing economic check is also the Sub-gap-2-adjacent worry in reverse: abstention may be selecting low-volatility days, and nobody checked, so the interaction between the confidence filter and the volatility state is unexamined in exactly the way Sub-gap 2 says volatility states go unexamined.
+EFFECT ON SUB-GAP 2: LEAVES IT OPEN. There is no volatility quantity anywhere in this paper, so nothing is operationalised in the persistence direction. Its relevance is oblique but real in one respect: it is the only paper in the set where a *confidence* quantity is operationalised into a decision (trade or abstain), which is the structural template Sub-gap 2 needs for its own quantity — a measured scalar that gates action rather than describing it. The note's own framing of the missing economic check is also the Sub-gap-2-adjacent worry in reverse: abstention may be selecting low-volatility days, and the authors do not check it, so the interaction between the confidence filter and the volatility state is unexamined in exactly the way Sub-gap 2 says volatility states go unexamined.
 CSE DATA EVIDENCE: not a CSE paper. Two CSE-relevant implications: the coverage curve doubles as a measurement of how often a channel is live ("the coverage curve for the sentiment agent on CSE counters is directly the measurement of how often that channel is actually live"), and a calibrated expectation band is set — "my expectation band for a technical agent on CSE daily direction is somewhere near 0.54 to 0.58 on honest out-of-sample data, and a result above about 0.65 is a prompt to hunt for a leak rather than a success."
 PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On C_{i,t}, verbatim: "Realised conditional accuracy is the common scale for heterogeneous agent confidence, and this paper is the argument for it. The open question in my matrix is how an LLM analyst, an econometric estimator and an RL policy produce comparable confidence numbers, and the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not. It also inherits the calibration problem named above rather than solving it, so the curve has to be re-estimated as conditions move rather than fitted once." Implicitly this adds an abstention channel to the weighting function — w(i,t) should be able to go to zero for an agent on a given day — though the note never writes that as a change to f(·) itself.</t>
         </is>
@@ -7336,125 +7423,1400 @@
       </c>
     </row>
     <row r="54" ht="409.6" customHeight="1">
-      <c r="A54" s="17" t="inlineStr">
+      <c r="A54" s="32" t="inlineStr">
         <is>
           <t>P53</t>
         </is>
       </c>
-      <c r="B54" s="18" t="inlineStr">
-        <is>
-          <t>Not yet reviewed.</t>
-        </is>
-      </c>
-      <c r="C54" s="18" t="inlineStr">
-        <is>
-          <t>See citation</t>
-        </is>
-      </c>
-      <c r="D54" s="18" t="inlineStr">
-        <is>
-          <t>See Citation column</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
+      <c r="B54" s="33" t="inlineStr">
+        <is>
+          <t>Smart Trading Rule: A Modular Machine Learning Framework for Portfolio Optimization with Transaction Costs. Journal of Financial Data Science 8(2), 2026. Bibliographic details recovered from the Research Papers Grid entry 42; the paper itself is paywalled and has not been obtained.</t>
+        </is>
+      </c>
+      <c r="C54" s="33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D54" s="33" t="inlineStr">
+        <is>
+          <t>Journal of Financial Data Science 8(2)</t>
+        </is>
+      </c>
+      <c r="E54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="F54" s="18" t="inlineStr">
+      <c r="F54" s="33" t="inlineStr">
         <is>
           <t>Portfolio optimisation with transaction costs</t>
         </is>
       </c>
-      <c r="G54" s="18" t="inlineStr">
+      <c r="G54" s="33" t="inlineStr">
         <is>
           <t>NOT YET REVIEWED - the vault note is an empty file.</t>
         </is>
       </c>
-      <c r="H54" s="18" t="inlineStr">
+      <c r="H54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
+      <c r="I54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="J54" s="18" t="inlineStr">
+      <c r="J54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="K54" s="18" t="inlineStr">
+      <c r="K54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="L54" s="18" t="inlineStr">
+      <c r="L54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="M54" s="18" t="inlineStr">
+      <c r="M54" s="33" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="N54" s="18" t="inlineStr">
+      <c r="N54" s="33" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="O54" s="18" t="inlineStr">
+      <c r="O54" s="33" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="P54" s="18" t="inlineStr">
+      <c r="P54" s="33" t="inlineStr">
         <is>
           <t>Likely relevant to Sub-gap 1 given the title, but nothing is recorded.</t>
         </is>
       </c>
-      <c r="Q54" s="18" t="inlineStr">
+      <c r="Q54" s="33" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="R54" s="18" t="inlineStr">
+      <c r="R54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="S54" s="18" t="inlineStr">
+      <c r="S54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="T54" s="18" t="inlineStr">
+      <c r="T54" s="33" t="inlineStr">
         <is>
           <t>Not recorded.</t>
         </is>
       </c>
-      <c r="U54" s="18" t="inlineStr">
+      <c r="U54" s="33" t="inlineStr">
         <is>
           <t>NOT YET REVIEWED. The note file is empty. On the title alone this is likely to bear on Sub-gap 1, the modular framework for portfolio optimisation with transaction costs, so it should be read before Sub-gap 1 is defended.</t>
         </is>
       </c>
-      <c r="V54" s="18" t="inlineStr">
+      <c r="V54" s="33" t="inlineStr">
         <is>
           <t>Unknown until read.</t>
         </is>
       </c>
-      <c r="W54" s="18" t="inlineStr">
+      <c r="W54" s="33" t="inlineStr">
         <is>
           <t>[[Smart Trading Rule, A Modular Machine Learning Framework for Portfolio Optimization with Transaction Costs]] - EMPTY FILE</t>
         </is>
       </c>
-      <c r="X54" s="18" t="inlineStr">
+      <c r="X54" s="33" t="inlineStr">
         <is>
           <t>SPEAKS TO: probably A_T and the friction-aware evaluation layer, on the title alone.
-NOT YET REVIEWED.</t>
+NOT YET REVIEWED, AND BLOCKED ON ACCESS RATHER THAN ON EFFORT. The paper is paywalled. Routes to try, in order: institutional access, interlibrary loan, or emailing the authors for a copy.
+WHY IT MATTERS: on its title it is a modular framework for portfolio optimisation WITH TRANSACTION COSTS, which is exactly Sub-gap 1's territory, and it may narrow that sub-gap further. Sub-gap 1 should not be presented as final until this has been read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="409.6" customHeight="1">
+      <c r="A55" s="29" t="inlineStr">
+        <is>
+          <t>P54</t>
+        </is>
+      </c>
+      <c r="B55" s="30" t="inlineStr">
+        <is>
+          <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid–ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
+        </is>
+      </c>
+      <c r="C55" s="30" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>Journal of Financial Economics (JFE), volume 161, article 103916.</t>
+        </is>
+      </c>
+      <c r="E55" s="30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jfineco.2024.103916 — accessed 4 October 2026. Code and data: github.com/eguidotti/bidask.</t>
+        </is>
+      </c>
+      <c r="F55" s="30" t="inlineStr">
+        <is>
+          <t>Low-frequency microstructure econometrics — estimation of the effective bid–ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin–Schultz (2012) / Abdi–Ranaldo (2017) lineage.</t>
+        </is>
+      </c>
+      <c r="G55" s="30" t="inlineStr">
+        <is>
+          <t>Produce an estimator of the effective bid–ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
+The object being estimated is the effective spread, not the quoted spread. The quoted spread is the posted distance between best bid and best ask; the effective spread is the realised distance between the transaction price and the unobserved fundamental price, S = 2D(P − P̃)/P̃, with D = +1 for buyer-initiated and −1 for seller-initiated trades. They differ because dealers often execute inside the quotes, and "one of this paper's headline empirical results is that the end-of-day quoted spread overstates the effective spread by up to 100%." For a cost model the effective spread is the right object and the harder one, since P̃ is never observed.
+The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid–ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed — Roll additionally required equally likely buys and sells; Corwin–Schultz and Abdi–Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
+        </is>
+      </c>
+      <c r="H55" s="30" t="inlineStr">
+        <is>
+          <t>US equities (NYSE / AMEX / NASDAQ) as the main empirical setting, plus a cryptocurrency application on Binance. No emerging or frontier market anywhere in the paper. The note records: "Emerging and thin markets" are represented only by the crypto section, which "is the closest thing here to an illiquid non-US market" and "has no benchmark whatsoever".</t>
+        </is>
+      </c>
+      <c r="I55" s="30" t="inlineStr">
+        <is>
+          <t>Two evaluations (a simulation and a CRSP–TAQ empirical study) plus three applications.
+Simulation: Corwin and Schultz (2012) design as reused by Abdi and Ranaldo (2017). 10,000 months, each 21 trading days, each day 390 minutes. Fundamental price P̃_m = P̃_{m−1}e^{σz}, P̃_0 = 1, z standard Gaussian. Daily sd 3%, per-minute sd 3%/√390. Trade prices are P̃_m times one minus (plus) half the spread, 50% chance of a bid (ask). Trade probability varied so expected trades per day runs from 1 to 390. On no-trade days the previous day's close is forward-filled into all four prices. Spreads tested: 0.50%, 1.00%, 2.00% through 8.00%.
+Empirical: CRSP US Stock Database, 1926–2021, NYSE / AMEX / NASDAQ, share codes 10 and 11. Benchmark is the Holden and Jacobsen (2014) effective spread from TAQ, May 1993 – December 2021. Merged sample 1,637,621 stock-months, CUSIP and ticker matching recovering 99% of CRSP stocks. Intraday sample 711,161 stock-months with both minute and daily estimates, October 2003 – December 2021. Crypto: Binance, 2163 pairs, 53,865 pair-months, July 2017 – December 2021, at daily / hourly / minute frequency.
+Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high–low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
+        </is>
+      </c>
+      <c r="J55" s="30" t="inlineStr">
+        <is>
+          <t>Daily (or intraday) open, high, low and close prices and nothing else. No quote feed, no trade-by-trade data, no vendor dependency. The derived quantities are: o_t, h_t, l_t, c_t as log-prices; η_t = (h_t + l_t)/2 the mid log-price; and the indicator τ_t that flags whether the high, the low and the previous close all coincide. The note flags the τ_t indicator as itself a usable feature — "the fraction of days on which the open or close coincides with the high or low, which falls out of the EDGE computation at no extra cost".</t>
+        </is>
+      </c>
+      <c r="K55" s="30" t="inlineStr">
+        <is>
+          <t>"There is no architecture, this is an estimator, and the whole mechanism rests on one indicator variable."
+τ_t = 0 if h_t = l_t = c_{t−1}, and 1 otherwise.
+τ_t = 0 flags the case where high, low and previous close all coincide, meaning either that every trade in the period executed at the previous closing price — "which becomes increasingly likely as trades per period fall" — or that there was no trading at all and the four prices were filled forward. Setting τ_t = 0 on those periods prevents the estimator from treating a forward-filled price as evidence about the spread, and conditioning every expectation on τ_t = 1 is what makes the derivation go through without assuming continuous observation.
+The spread estimator measured at the open:
+S_o² = −8·E[(η̄_t − ō_t)(o_t − c_{t−1})] / ( P[o_t ≠ h_t, τ_t = 1] + P[o_t ≠ l_t, τ_t = 1] )
+where bars denote de-meaned returns, r̄_t = r_t − τ_t·E[r_t]/E[τ_t], "which is the de-meaning that survives the conditioning on τ_t". The denominator is the entire discreteness correction and is the only thing separating this from the classical form: if prices are observed continuously the open and close can never coincide with the high or low, both probabilities equal one, the denominator collapses to two, and the expression reverts to the familiar −4E[·] shape.
+The note's reading: "The correction is therefore not a robustness patch bolted onto an existing estimator, it is a term that is identically one under the old assumption and shrinks the denominator, inflating the spread estimate, exactly in proportion to how often the price failed to move within the period."
+The same construction over other price combinations gives four Discrete Generalized Estimators — OHL, CHL, OHLC and CHLO — the first pair measuring the spread at the open and the second at the close. Their CHL estimator reduces exactly to the Abdi and Ranaldo (2017) estimator when continuous observation is imposed and returns are zero-mean, "so the prior work is recovered as a special case rather than contradicted."
+Efficiency half: the four estimators behave in opposite ways — when the spread is small relative to volatility the estimators using the mid-price have lower variance, and when the spread is large and observed returns are driven by bid–ask bounces, pairing mid-to-open with open-to-mid returns cancels a variance term that pairing with the closing price does not. Combining OHL with CHLO and OHLC with CHLO gives two moment conditions, and GMM with a diagonal weighting matrix reduces to a variance-weighted average:
+S²_EDGE = w₁·E[x_{1,t}] + w₂·E[x_{2,t}]
+x_{1,t} = (π_o/2)(η̄_t − ō_t)(o_t − η_{t−1}) + (π_c/2)(η̄_{t−1} − c̄_{t−1})(c_{t−1} − η_{t−1})
+x_{2,t} = (π_o/2)(η̄_t − ō_t)(o_t − c_{t−1}) + (π_c/2)(ō_t − c̄_{t−1})(c_{t−1} − η_{t−1})
+with π_o = −8/(P[o_t ≠ h_t, τ_t=1] + P[o_t ≠ l_t, τ_t=1]) and π_c its counterpart at the previous close, and weights w₁ = Var[x_{2,t}]/(Var[x_{1,t}] + Var[x_{2,t}]), w₂ = 1 − w₁.
+In estimation the sample counterparts replace the expectations, variances and probabilities, "so there is nothing to fit and nothing to tune, which is the practical appeal." Negative squared estimates are handled with Ŝ = √max{0, Ŝ²} applied once to the final estimate rather than within rolling windows, following Jahan-Parvar and Zikes's finding that the within-window version produces an upward bias that never declines.
+Output: an effective spread in basis points per asset per period, from OHLC alone.</t>
+        </is>
+      </c>
+      <c r="L55" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — this is a closed-form econometric estimator with no agents, no decision and no orchestration. The note states it plainly: "This is tooling, not a competitor architecture, there is no agent in it and no trading decision, but it goes at the part of my design that is currently weakest."</t>
+        </is>
+      </c>
+      <c r="M55" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — the paper uses only OHLC prices and contains no textual or sentiment component. (Sentiment is out of scope for this project in any case, per the supervisor decision.)</t>
+        </is>
+      </c>
+      <c r="N55" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no disclosures, filings, retrieval or text of any kind. The only inputs are the four daily prices.</t>
+        </is>
+      </c>
+      <c r="O55" s="30" t="inlineStr">
+        <is>
+          <t>No volatility model is estimated, but volatility enters the paper twice as a nuisance that drives the estimator's error. First, through the truncation channel: because Ŝ² can come out negative in small samples, standard practice is to reset negatives to zero, and Jahan-Parvar and Zikes (2023) show this introduces a strong upward bias that does not decline with sample size, "with volatility as its primary driver". Second, through the spread-to-volatility ratio: the degradation of correlation with the TAQ benchmark over time is attributed by the authors to spreads shrinking relative to volatility, consistent with the spread-quintile table where correlation runs 17.84% in the narrowest quintile against 71.38% in the widest.
+The note also flags a tension with the volatility side of the project's own literature: Assumption 1 rules out serially correlated fundamental returns, "which sits uneasily beside the long-memory results on the ASPI and SL20 in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], though that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it."
+Estimation variance is roughly proportional to σ₁⁴/N for N observations at per-period volatility σ₁, so the standard error scales with σ₁²/√N — which is the formula behind the frequency result below.</t>
+        </is>
+      </c>
+      <c r="P55" s="30" t="inlineStr">
+        <is>
+          <t>This is the whole paper. EDGE measures the effective spread — the realised cost of a marginal trade — directly, in basis points, from OHLC. The discreteness correction is explicitly a function of how thinly the asset trades: the probability that the open or close coincides with the high or low is "a direct consequence of too few trades per period", running from about 25% for large-cap US stocks to 75% for small-caps over 1926–2021, peaking in the 1930s and 1940s, collapsing after 2000 with electronification to roughly 2–5% for large-caps while small-caps still sit near 15% at the end of the sample. The authors' own reading is that "the correction is less significant for recent samples and becomes essential for small stocks and for older periods, and crucially that it also depends on sampling frequency, since going from daily to intraday prices reduces the trades observed per interval and pushes the probability back up."
+What the paper does NOT handle: order size. "There is no order size anywhere in the model, so what EDGE measures is the cost of a marginal trade." The effective spread is computed from the transaction prices that happened, at whatever sizes they happened in, and the estimator has no mechanism for saying what a larger order would have paid.</t>
+        </is>
+      </c>
+      <c r="Q55" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable in the ML sense — there is no black box. The estimator is closed-form, every term is interpretable, and the discreteness correction has a direct structural reading (the denominator is one under continuous observation and shrinks in proportion to how often the price failed to move). Reproducibility is strong: implementations in several languages, the computed spread data, and a Harvard Dataverse replication package.</t>
+        </is>
+      </c>
+      <c r="R55" s="30" t="inlineStr">
+        <is>
+          <t>Baselines: ROLL (Roll 1984), CS (Corwin and Schultz 2012), AR (Abdi and Ranaldo 2017), plus the paper's own intermediate estimators OHLC and CHL. Benchmark truth is the Holden and Jacobsen (2014) TAQ-based effective spread, May 1993 – December 2021.
+Evaluation axes: (i) simulation bias as a function of expected trades per day from 390 down to 1; (ii) simulation mean and standard deviation across true spreads 0.50%–8.00%; (iii) empirical Pearson and Spearman correlation, MAPE, RMSE and fraction of non-positive estimates on 1,637,621 merged stock-months, cut by market venue, sub-period, size quintile and decile, spread quintile and trading-frequency quintile; (iv) daily versus minute sampling on 711,161 stock-months; (v) the Binance crypto application across daily / hourly / minute, which has no benchmark.
+The note records a caveat on the empirical comparison: "The comparison is descriptive throughout, no standard errors on the differences and no formal test, which at this sample size is defensible but means the quintile tables are read by eye."</t>
+        </is>
+      </c>
+      <c r="S55" s="30" t="inlineStr">
+        <is>
+          <t>1. Infrequent trading breaks the alternatives and not EDGE. At 390 trades per day all estimators are unbiased and recover the 1% simulated spread. By 100 trades per day CS estimates 0.75%; by around twenty trades per day it has fallen to 0.1%; and below roughly thirteen trades per day CS returns exactly zero. AR degrades more gracefully but is still biased down to about 0.30% at one trade per day and 0.62% at roughly two. EDGE tracks 1.00% across the entire range, including simulations where only a single trade per period is expected on average. The note: "This is the single most transferable result in the paper for my purposes and I report it as the paper's evidence rather than as a general claim, since the simulation's price process is a geometric Brownian motion and its no-trade handling is forward-filling rather than genuine absence."
+2. Variance. Under infrequent trading, mean estimate with sd in parentheses against the true spread:
+True S | EDGE | OHLC | CHL | AR | CS | ROLL
+0.50% | 0.71 (0.75) | 0.77 (0.87) | 0.91 (0.97) | 0.65 (0.73) | 0.02 (0.07) | 1.44 (1.42)
+1.00% | 0.95 (0.83) | 0.99 (0.97) | 1.10 (1.04) | 0.81 (0.80) | 0.04 (0.10) | 1.56 (1.47)
+3.00% | 2.89 (0.83) | 2.76 (1.23) | 2.86 (1.19) | 2.26 (0.92) | 0.35 (0.36) | 2.89 (1.82)
+8.00% | 8.19 (0.96) | 8.10 (1.59) | 8.20 (1.26) | 6.59 (0.94) | 2.66 (0.96) | 7.71 (2.65)
+EDGE is within 0.21 of the true value at every spread size while AR is 1.41 low at 8.00% and CS is 5.34 low, and EDGE's standard deviation is the smallest or tied at every row. CS's small standard deviations are "the collapse to zero rather than precision". The uniformity comes from the building blocks swapping roles, OHLC and CHLO carrying lower variance for small spreads and OHL and CHL for large, with EDGE shifting weight between them rather than being tuned to a favoured region.
+3. Empirical dominance, widest where trading is thinnest. Against the TAQ benchmark EDGE achieves Pearson 78.86%, Spearman 66.68%, MAPE 16.21, RMSE 1.23, non-positive estimates 25.63% — against AR at 68.13 / 53.55 / 19.90 / 1.41 / 31.87 and CS at 45.55 / 33.77 / 35.90 / 2.61 / 29.18. EDGE is highest in every market venue, sub-period, size quintile, spread quintile and trading-frequency quintile. On the trading-frequency cut, EDGE scores 74.77% in the least-traded quintile falling to 55.48% in the most-traded, while ROLL runs the other way at 65.10% down to 22.29% and AR falls from 67.81% to 39.36%. The size-decile plot has the same shape, EDGE flat near 70% across all ten deciles while the others spread out below it. "The lead is therefore not an average that washes out in the hard cases, it is largest in the hard cases, which is the property a frontier-market application needs."
+4. Sampling frequency beats sampling length by three orders of magnitude. Standard error scales as σ₁²/√N. Going from a monthly sample of daily prices (N = 21) to a yearly one (N = 252) reduces the standard error by √(252/21) = 3.5 times; going instead to a monthly sample of minute prices (N = 21 × 390) reduces it by 390^{3/2} = 7702 times, which the authors note would take 1,245,699,037 daily prices to match, roughly five million years of trading. Empirically, on 711,161 stock-months, moving from daily to minute prices: negative estimates fall from 34.15% to 0.02%, Pearson rises from 56.17% to 88.79%, Spearman from 43.47% to 97.31%, MAPE from 23.68 to 5.17. The crypto application makes the point from the other side: AR and CS differ roughly tenfold between daily and minute sampling (0.18% against 0.02%, and 1.85% against 1.45% respectively) while EDGE stays within 0.68% to 0.70% at every frequency, "so the frequency-insensitivity is a property of the estimator rather than of the US sample."
+5. The discreteness term is itself a market-structure measurement: the coincidence probability ranges from ~25% (US large-cap) to 75% (small-cap) over 1926–2021, peaking in the 1930s–40s, collapsing after 2000 to 2–5% for large-caps with small-caps still near 15%.</t>
+        </is>
+      </c>
+      <c r="T55" s="30" t="inlineStr">
+        <is>
+          <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% — "a bias roughly seven times the quantity being measured" — and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
+2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid–ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information — Chen et al. (2017) being their example — is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
+3. No order size anywhere in the model. For a deep market the marginal-trade cost is close enough; "for a book where a single order can be a meaningful fraction of daily volume it is the intercept of a cost function and not the function." The scope is honest and never overclaimed, but EDGE answers only the first of the four open items in my cost work and leaves the nonlinear impact form, the participation-rate sweep and the thin-book depth calibration untouched.
+4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden–Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility — "plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation." The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
+5. The estimator needs at least three usable observations per stock-month and the paper never reports performance conditional on a small count. Periods with τ_t = 0 are excluded, and EDGE is missing in 1.24% of CRSP stock-months on that basis. "The thinnest cut they report is the bottom trading-frequency quintile of US-listed stocks, which still trades most days. For a counter with five trading days in a month the estimator is defined and will return a number computed from a handful of covariance terms, deep inside the small-sample regime where their own truncation bias is worst, and nothing in the paper tells me how that number behaves. That is the gap between what the paper validates and what I would be doing with it."
+6. The simulation's "infrequent trading" is not frontier-market infrequent. Panel B sets the daily trade probability to 1%, which on a 390-minute day means roughly four expected trades per day, and the bias plot extends down to one trade per day. "That is thin by US standards and it is the right stress test for the method, but a CSE counter in the bottom half of a liquidity screen can go whole days without a trade, and the paper's design forward-fills those days rather than modelling a counter that trades on five days in a month. The estimator handles the forward-fill correctly through its indicator; what is untested is the regime where the number of usable observations per stock-month falls into single digits."
+7. A premise doing quiet work throughout: that the effective spread is the whole of the transaction cost, since nothing in the model has an order size in it. The paper never claims otherwise and the title is honest about scope.</t>
+        </is>
+      </c>
+      <c r="U55" s="30" t="inlineStr">
+        <is>
+          <t>- EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC — the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
+- The infrequent-trading bias result as external evidence that thin-book calibration is a real problem, not a rhetorical one: below roughly thirteen trades per day CS returns exactly zero and AR is biased down by about a third at a few trades per day, "which means any cost model built on those estimators would charge approximately nothing for trading the least liquid counters on the CSE. That is backwards in the most expensive possible direction." Worth citing directly in the proposal when defending the thin-book calibration item.
+- Two new candidate inputs to the liquidity state L_t. (a) The measured spread itself, which unlike Amihud (price impact per unit volume), turnover (activity) and zero-return frequency (staleness) "is denominated in the same units as the objective". (b) The τ_t indicator — the fraction of days on which the open or close coincides with the high or low — which "falls out of the EDGE computation at no extra cost" and is a candidate staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both go into the ablation protocol "as additions to test rather than adopt".
+- A forced window decision. Given 25.63% non-positive daily-price estimates on CRSP and 41% negative for large-caps, and a monthly estimate from the per-counter archive being roughly 21 observations — "squarely in that regime" — the decision is a quarterly window on the per-counter track, accepting a cost term that cannot move within a quarter, and monthly on the index track where ten years of daily data supports it, "with the fraction of non-positive estimates reported alongside every spread series in both cases. Reporting that fraction is not optional here, it is the only visible signal that the truncation is distorting the number."
+- A reversal of my data priority. A month of minute prices gives a standard error 7702 times smaller than a month of daily prices, where a year of daily prices gives only 3.5 times. "So if any intraday CSE feed exists at any granularity, even hourly or five-minute, it is worth far more to the cost model than extending the daily archive backwards." This is a question to put to the supervisor before spending time on data depth, and it connects to the volatility estimator decision too, "since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE."
+- A positioning rule. EDGE is a 2024 JFE paper with public implementations, open spread data and a replication package, "so there is no contribution in running it on a new market and no reason to imply one." The defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered, and that the contribution is what an orchestrator does with a cost term that varies by counter and date rather than the estimator that produces it. "One sentence, offered before anyone asks."</t>
+        </is>
+      </c>
+      <c r="V55" s="30" t="inlineStr">
+        <is>
+          <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
+Second, the small-count regime is untested: the estimator is defined with three usable observations but the paper never characterises its behaviour there, and that is exactly the regime a CSE counter with five trading days in a month occupies.
+Third, the paper measures a spread; it never puts that spread inside a decision objective. "It sits alongside [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] as the measurement layer those papers assume and never supply." The claim that cost belongs inside the objective rather than deducted afterwards is still mine to make — and now has two separately validated pieces behind the cost term.
+Fourth, no validation against a quote-based benchmark in an emerging or frontier market: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."</t>
+        </is>
+      </c>
+      <c r="W55" s="30" t="inlineStr">
+        <is>
+          <t>[[Efficient estimation of bid–ask spreads from open, high, low, and close prices]]</t>
+        </is>
+      </c>
+      <c r="X55" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: A_L above all — this is the measurement instrument the liquidity agent currently lacks — plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
+EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency — "all proxies for illiquidity rather than measurements of what a trade pays" — and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade — "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren–Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
+The second half of Sub-gap 1 — that liquidity simultaneously conditions the reliability of price-derived agents — gets independent support from the paper's own mechanism rather than from my framing. The τ_t = 0 condition is literally the case where the price carries no information about the spread within the period, and the coincidence probability that drives the correction is "a direct consequence of too few trades per period". That is a measured, published statement that price-derived quantities degrade in a specific, quantifiable way as trading thins — which is precisely the premise under which L_t should down-weight A_T.
+EFFECT ON MAIN GAP: Indirect but real. The main gap is market-state-aware dynamic orchestration with w(i,t) = f(L_t, V_t, P_t, C_{i,t}), and the weakest-specified argument of that function is L_t. This paper contributes two candidate components to it that measure something the existing three proxies do not. The spread gives L_t a component denominated in the same units as the objective. The τ_t indicator gives a staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both enter the ablation protocol as additions to test rather than adopt, "which turns the question from whether liquidity matters into whether a measured spread and a measured staleness rate carry anything beyond the three proxies already there." That reframing is itself useful: it converts a soft claim about liquidity-awareness into a falsifiable ablation.
+EFFECT ON SUB-GAP 2: Minimal and only by friction. The paper estimates no volatility model and says nothing about persistence. The one contact point is Assumption 1, which rules out serially correlated fundamental returns and "sits uneasily beside the long-memory results on the ASPI and SL20" in the CSE volatility-memory work — but the note is careful that "that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it." So this does not move Sub-gap 2. There is one indirect operational link: the frequency result argues that any intraday CSE feed is worth far more to the cost model than more daily history, "and it connects to the volatility estimator decision too, since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE." The two data questions are the same question.
+CSE DATA EVIDENCE: The note's CSE-side commitments are: the CSE publishes daily OHLC for every listed counter, which is what makes EDGE applicable with no quote feed; the per-counter archive is roughly 374 trading days, giving ~21 observations per monthly estimate — "squarely in that regime" where 25.63% of CRSP daily-price estimates come out non-positive and 41% of large-cap stock-months come out negative before truncation; and a CSE counter in the bottom half of a liquidity screen "can go whole days without a trade", below anything the paper's simulation stresses (its thinnest panel is ~4 expected trades per day, with the bias plot extending to one trade per day, and no-trade days forward-filled rather than genuinely absent). The resulting design decisions are a quarterly window on the per-counter track, monthly on the index track where ten years of daily data supports it, and the fraction of non-positive estimates reported alongside every spread series in both cases.
+PROPOSED REVISION STATED IN THE NOTE: Re-scope the cost sub-gap as "EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part" — narrower and more defensible than the earlier wording, using this paper as support rather than letting it look like competition. Claim EDGE as an adopted measurement with the implementation cited and keep all novelty language off it; the one defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered. Add the measured spread and the τ_t staleness rate to the liquidity-state ablation as candidates to test rather than adopt. Fix the aggregation window before running anything (quarterly per-counter, monthly index-track) and report the non-positive fraction every time. Put the intraday-feed question to the supervisor before investing in deeper daily history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="409.6" customHeight="1">
+      <c r="A56" s="29" t="inlineStr">
+        <is>
+          <t>P55</t>
+        </is>
+      </c>
+      <c r="B56" s="30" t="inlineStr">
+        <is>
+          <t>Wang, X., Hyndman, R.J., Li, F. and Kang, Y. (2023). Forecast combinations: An over 50-year review. International Journal of Forecasting, 39(4), 1518–1547. DOI: 10.1016/j.ijforecast.2022.11.005. arXiv version 2205.04216v2 dated 26 September 2022. Affiliations: Xiaoqian Wang and Yanfei Kang at Beihang, Rob J Hyndman at Monash, Feng Li at the Central University of Finance and Economics — "about as authoritative an author list as this particular topic has". Citekey: wangForecastCombinations50year2023.</t>
+        </is>
+      </c>
+      <c r="C56" s="30" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D56" s="30" t="inlineStr">
+        <is>
+          <t>International Journal of Forecasting, 39(4), 1518–1547.</t>
+        </is>
+      </c>
+      <c r="E56" s="30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ijforecast.2022.11.005 (arXiv 2205.04216v2).</t>
+        </is>
+      </c>
+      <c r="F56" s="30" t="inlineStr">
+        <is>
+          <t>Forecast combination / forecast pooling — a narrative review of over fifty years of work on combining multiple forecasts of the same quantity, from Bates and Granger (1969) (and behind that Galton's 1906 ox-weight competition, where the average of 787 estimates came close to the animal's actual weight) through to the feature-based cross-learning methods that placed in M4. Organising split: point forecast combinations (section 2), probabilistic forecast combinations (section 3), eight open problems in closing, with a running commentary on which R and Python packages implement what.
+This is the most direct body of prior art on the orchestration half of my design. As the note puts it: "My orchestrator computes w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) over four heterogeneous agent outputs, and that object is a time-varying, feature-conditioned linear combination, which is a named construct in this literature with five decades of results attached to it, a good number of them inconvenient." It belongs next to the RL-in-quant-finance survey as the other half of the prior art: "that one establishes that coordination protocols among heterogeneous agents are underexplored in RL, this one establishes what fifty years of statistics already knows about combining their outputs once they exist."</t>
+        </is>
+      </c>
+      <c r="G56" s="30" t="inlineStr">
+        <is>
+          <t>Update the field's standing reviews — Clemen (1989) and Timmermann (2006) — and, structurally, set point and probabilistic combination side by side for the first time in a single survey. Three gaps motivate it:
+1. Both standing reviews predate the entire cross-learning and meta-learning strand, the M4 and M5 competitions, most of the probabilistic combination work, and the open-source tooling that now carries these methods into practice. The authors' Web of Science count puts combination papers at "13.80% of all published forecasting papers in 2021", up from roughly 1% in 1969, "so the case for an update is quantitative rather than rhetorical."
+2. Point and probabilistic combination had developed in parallel without being contrasted. In probabilistic combination, diversity among individuals becomes "more complex and less understood", and calibration and sharpness enter as considerations with no analogue in the point case. "Setting the two side by side is the structural contribution, and it is what produces the review's most useful result for me, because several intuitions do not survive the crossing."
+3. Model averaging and forecast combination get used interchangeably and shouldn't be. Model averaging is a general term for handling model uncertainty, chiefly in parameter estimation, with frequentist and Bayesian strands; forecast combination is narrower, operating on forecasts whose origin is irrelevant, carrying assumptions intended to keep the combination unbiased or optimal. "That is the right frame for my case, because my agents are not models of the same process with different parameters, they are methodologically different producers, and only the second framing accommodates that."
+The central empirical claim restated across fifty years of evidence: "the equally weighted average is extremely hard to beat", and the literature has a name for its own embarrassment about this — the forecast combination puzzle.
+SCOPE BOUND (the note flags this as bounding everything else): the authors take the individual forecasts "as given", do not discuss how they are generated, and restrict attention to forecasts derived from separate and non-interfering models for a single target series. Two adjacent literatures are named and excluded: manipulating one series into many and combining the results (Petropoulos and Spiliotis' "wisdom of the data", covering theta, bagging and temporal aggregation), and forecast reconciliation for hierarchical series following Hyndman et al. (2011). The target is always a realised value of one series and the loss is almost always quadratic. "There are no portfolios, no transaction costs, no execution, and no decisions. So this is prior art on the weighting mechanism and on the evidence about weighting, not on anything downstream of it, and the non-interfering assumption in particular is one my design may violate."</t>
+        </is>
+      </c>
+      <c r="H56" s="30" t="inlineStr">
+        <is>
+          <t>General forecasting, not finance-specific. Named application areas are retail, energy, economics, epidemiology and meteorology; the financial examples are macroeconomic series such as inflation and GDP growth. Competition datasets are M3, M4 (100,000 series), M5 and FRED. "Emerging and thin markets are absent from the entire paper."</t>
+        </is>
+      </c>
+      <c r="I56" s="30" t="inlineStr">
+        <is>
+          <t>No dataset of its own — the authors run no experiment. The evidence base is other people's results on M-competition data (M3, M4 at 100,000 series, M5), FRED, and individual case studies. Coverage spans 1969 to roughly 2022, with the Web of Science publication-share chart (Figure 1) the only quantitative artefact the authors produce. "There is no protocol, no screening count, and no stated inclusion criterion anywhere in the paper."</t>
+        </is>
+      </c>
+      <c r="J56" s="30" t="inlineStr">
+        <is>
+          <t>Univariate time series forecasts (point and probabilistic) as the inputs to be combined. The feature strand is the one that matters: FFORMA (Montero-Manso et al., 2020) extracts 42 statistical features of the series with the tsfeatures package and maps them to weights via an XGBoost meta-model. Collopy and Armstrong (1992) is the ancestor — a hand-built rule base of 99 rules over 18 time series features and four statistical models — and "the line from there to XGBoost over 42 features is the clearest trajectory in the paper." The feature pool has itself become a research object: Lemke and Gabrys (2010) add six features measuring diversity of the method pool rather than properties of the series, and Kang et al. (2021) build a combination model from a diversity matrix alone.</t>
+        </is>
+      </c>
+      <c r="K56" s="30" t="inlineStr">
+        <is>
+          <t>Not an architecture — a taxonomy of weighting schemes. The framing holding section 2 together is a one-dimensional aggregator over an N-vector of h-step-ahead forecasts:
+ỹ_{T+h|T} = C(ŷ_{T+h|T}; w_{T+h|T}), linear case ỹ_{T+h|T} = w'_{T+h|T} ŷ_{T+h|T}
+The ladder of weighting schemes, from no estimation to estimation over a whole dataset of series:
+Family | What determines the weights | Data needed | Section
+Simple combination | Nothing estimated. Mean, median, mode, trimmed and winsorized means | None | 2.1
+Optimal weights | Covariance matrix of the h-step forecast errors | Error history per method, all pairs | 2.2
+Regression weights | OLS of realisations on past individual forecasts, three restriction regimes | Aligned history of forecasts and outcomes | 2.2
+Performance-based | Inverse historical error, rolling window or exponentially discounted | Error history per method, no pairs | 2.2
+Rank-based | Position in the performance ordering, not error magnitude | Error history per method | 2.2
+Criteria-based | AIC, AICc or BIC differences across the model pool | In-sample fit of each model | 2.2
+Bayesian | Posterior model probabilities, or shrinkage toward a prior mean | Priors plus likelihood per model | 2.2, 3.4
+Nonlinear | A neural network or an explicit pairwise interaction term | As regression, plus far more | 2.3
+Combining by learning | A meta-model over features of the series and of the method pool | A dataset of many series | 2.4
+OPTIMAL WEIGHTS (Bates and Granger 1969 for pairs, Newbold and Granger 1974 in general) minimise the variance of the combined forecast error:
+w^opt_{T+h|T} = Σ⁻¹_{T+h|T} 1 / (1' Σ⁻¹_{T+h|T} 1)
+with Σ the N×N covariance matrix of h-step forecast errors. If the individuals are unbiased and their error variances stable, the combination is unbiased and its error variance is no greater than the minimum across individuals — "the diversification result the whole field rests on. The catch is in the last sentence of that passage: in practice Σ is unknown and has to be estimated, and that single sentence generates most of the rest of the literature."
+REGRESSION WEIGHTS (Granger and Ramanathan 1984): three regimes — weights summing to one with no intercept, which reproduces Bates–Granger exactly; unconstrained with no intercept; and unconstrained with an intercept, which they argued is superior regardless of whether constituents are biased because the intercept absorbs the bias. De Menezes et al. (2000) push back that the unrestricted version needs stationarity and runs into serial correlation and multicollinearity. Aksu and Gunter (1992) found empirically that constraining weights to be nonnegative is at least as robust as the simple average while beating the other regression variants — "which is the practical reading I'd take."
+PERFORMANCE-BASED, discounted variant (the one with a time dimension, and the one the note would implement first because it needs no pairwise estimation):
+w^{bg4}_{T+h|T,i} = ( Σ_{t=1}^{T} γ^t e²_{t|t−h,i} )⁻¹ / Σ_{j=1}^{N} ( Σ_{t=1}^{T} γ^t e²_{t|t−h,j} )⁻¹ , γ ≥ 1
+where e_{t|t−h,i} is the h-step error of method i made at t−h and realised at t, and γ controls how fast older errors are forgotten, with γ = 1 recovering the plain inverse-MSE weight over the full history. The rolling-window variant replaces the discount with a sum over the most recent ν observations. Both are adapted to non-stationary relationships between methods, and both, as Timmermann (2006) is quoted saying, "increase the variance of the parameter estimates and work quite poorly if the data generating process really is covariance stationary." Stock and Watson (1998) generalise by making weights inversely proportional to the kth power of MSE, so k=0 is equal weights and larger k concentrates on the best performer — "a single interpretable dial between the two extremes."
+TIME-VARYING WEIGHTS: Diebold and Pauly (1987) use rolling weighted least squares and time-varying parameters that are either deterministic polynomial functions of time or stochastic; Deutsch et al. (1994) let weights switch abruptly or transition smoothly using switching and smooth transition regression; Terui and van Dijk (2002) model the coefficients as a random walk in state space estimated by the Kalman filter, with Raftery et al. (2010) adding forgetting factors to make the recursive update cheap.
+The note's key structural observation: "So the literature already contains weights that change over time, and it contains weights that change as a regression function of covariates, and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state. The closest thing is the smooth transition specification of Deutsch et al., where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step."
+COMBINING BY LEARNING: stacking series-by-series needs n meta-models for n series, "computationally expensive and wastes the training data". Cross-learning trains one meta-model across many series. M4 is the evidence: "the top three methods all used information across the whole dataset rather than a single series." FFORMA is the exemplar — 42 tsfeatures features, XGBoost meta-model mapping features to weights over nine traditional models fitted per series, second place in M4.
+PROBABILISTIC COMBINATION: the linear opinion pool is a finite mixture F̃(y_{T+h}|I_T) = Σ w_{T+h|T,i} F_i(y_{T+h}|I_T) with nonnegative weights summing to one. Its first two moments:
+μ̃ = Σ w_i μ_i   and   σ̃² = Σ w_i σ_i² + Σ w_i (μ_i − μ̃)²
+The mean of the pooled distribution is exactly the linear point combination, so nothing changes there. The variance carries a second term in the disagreement between component means, so pooled variance exceeds the weighted average of component variances whenever the components disagree about location.
+Quantile combination (Vincentization, after Vincent 1912): Q̃_{T+h|T}(τ) = Σ w_{T+h|T,i} Q_{T+h|T,i}(τ) for 0 &lt; τ ≤ 1. The geometric statement, which the note calls "the clearest sentence in section 3": "quantile combination averages the individuals' cdfs horizontally while linear pooling averages them vertically." If components are in the same location-scale family the quantile average stays in it, so averaging normals gives a normal and is always unimodal, where linear pooling can be multimodal. Both share the same mean. Quantile averaging is sharper because it does not absorb disagreement in location as extra spread — Lichtendahl et al. (2013) and Busetti (2017) both come down on its side, the former arguing the average probability forecast is generally under-confident while the average quantile forecast is always sharper.</t>
+        </is>
+      </c>
+      <c r="L56" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable as implemented — "a paper with no architecture in it, no trading decision anywhere, and nothing resembling an agent". But this is the closest named prior art to my orchestrator: combination weights over heterogeneous producers are exactly the orchestration object, and the survey supplies the ladder from equal weights to feature-conditioned meta-learned weights.
+CRITICAL CONSTRAINT: the non-interfering assumption. "The components here are separate models that do not see each other's outputs. Every LLM multi-agent trading system in my reading violates that: [[TradingAgents, Multi-Agents LLM Financial Trading Framework]] has agents debating, [[HedgeAgents, A Balanced-aware Multi-agent Financial Trading System]] runs conferences, and even the ones that do not communicate share the same underlying price history and the same disclosures. So the clean statistical properties derived here, the unbiasedness of the combination and the variance bound, hold under an assumption my pool does not satisfy. My four agents read overlapping data by construction, and the paper's own observation that component forecasts trained on overlapping information sets produce highly correlated errors is the mechanism by which that bites."
+Subset selection is named as prior art for an abstention channel: the paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme, citing Li et al. (2022).</t>
+        </is>
+      </c>
+      <c r="M56" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no textual or sentiment component anywhere; the inputs are numerical forecasts of a single target series. (Sentiment is out of scope for this project regardless, per the supervisor decision of 20 September 2026, status Final.)</t>
+        </is>
+      </c>
+      <c r="N56" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no documents, filings, retrieval or text. The only relevance is structural: the abstention channel exists because my fundamental agent will have no disclosure to work from "more than half the time", and the paper supplies the vocabulary (time-varying subset selection) for that.</t>
+        </is>
+      </c>
+      <c r="O56" s="30" t="inlineStr">
+        <is>
+          <t>No volatility modelling. One result touches the high-volatility regime: Zischke et al. (2022) report that when forecasting during high-volatility periods, weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample — which the note reads as "a result about choosing what to score rather than about how elaborate the pooling function is". This is the single exception in section 3 where sophistication earned its keep, and it is region-specific.
+Second-order relevance: the probabilistic variance decomposition means a deliberately heterogeneous pool produces an under-confident interval, which bears on any risk interval the orchestrator might emit.</t>
+        </is>
+      </c>
+      <c r="P56" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages."</t>
+        </is>
+      </c>
+      <c r="Q56" s="30" t="inlineStr">
+        <is>
+          <t>Interpreting combination weights is one of the paper's eight stated future directions — in the authors' words, "discussing if, how, and when it is helpful to interpret combination weights", prompted by the observation that some schemes drive poor forecasts to zero asymptotically while individually bad forecasts can still be useful. The paper also flags in future directions that "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts", which the note treats as a direct warning about significance testing on a weighted output.</t>
+        </is>
+      </c>
+      <c r="R56" s="30" t="inlineStr">
+        <is>
+          <t>The paper runs no evaluation of its own. "The authors run no experiment of their own and aggregate no results from the papers they cover, so there is no table anywhere comparing two weighting schemes on shared data. Every performance claim in the paper is a report of a single study's finding, which means I can cite this for the existence and the lineage of a method but never for its relative performance."
+The de facto benchmark throughout is the equally weighted average, and the evidence base is M-competition results plus individual case studies.</t>
+        </is>
+      </c>
+      <c r="S56" s="30" t="inlineStr">
+        <is>
+          <t>1. THE FORECAST COMBINATION PUZZLE — the field's central empirical result, fifty years old and still open. Stock and Watson (2004) named it: theoretically sophisticated weighting schemes should dominate the simple average, and empirically the simple average dominates them. Evidence runs from Makridakis et al. (1982) in the original M-competition through to M4, where "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) is the most recent restatement across M3, M4, M5 and FRED, finding that the winning combination method differs by data source while simple averaging shows, on average, more gain than complex methods. The explanations all centre on estimation error: Timmermann (2006) attributes it to parameter estimation error that simple schemes avoid entirely; Smith and Wallis (2009) to finite-sample estimation effects; Claeskens et al. (2016) prove that treating the weights as random rather than fixed can introduce bias into combinations of unbiased components and inflate the combination's variance past the fixed-weight case; Blanc and Setzer (2020) frame it as a bias-variance tradeoff where equal weights underfit and estimated weights carry estimation variance; Elliott (2011) bounds the available gain from optimal over equal weights and finds it is usually too small to pay for the estimation.
+2. CORRELATIONS AMONG FORECAST ERRORS SHOULD BE IGNORED RATHER THAN ESTIMATED — an empirical finding, not a convenience. Bates and Granger argued correlations are poorly estimated in practice and should be left out; Newbold and Granger (1974) and Winkler and Makridakis (1983) tested that over more series, methods and horizons and concluded that "combinations ignoring correlations are more successful than those attempting to account for them". The mechanism is visible in the optimal-weight formula: the full covariance matrix needs N(N+1)/2 parameters from the same short error history that a diagonal treatment needs N from, and with highly correlated forecast errors the sample estimator of Σ is unstable. Chan et al. (1999) add that OLS combination performs very poorly when N is large, which pushes the literature toward principal components regression and clustering.
+3. ACCURACY AND DIVERSITY BOTH CONSTRAIN WHAT COMBINING CAN DELIVER, AND A SUBSET USUALLY BEATS BOTH THE FULL POOL AND THE SINGLE BEST. Mannes et al. (2014) establish that the mean level of expertise in the pool sets a floor on combination performance, so including poor forecasts degrades the result; Lichtendahl and Winkler (2020) add that the variance of accuracy across series matters as much as the mean and the two have to be traded off when choosing the pool. On the other side, diversity produces the error cancellation in the first place, with Atiya (2020) deriving it through the bias-variance decomposition of MSE, and diversity usually measured as low correlation among forecast errors. The slogan the paper quotes is "many could be better than all": there are decreasing returns to adding forecasts, and subset selection — by discarding the worst performers, by Kourentzes et al.'s (2019) boxplot-outlier heuristic, by Lichtendahl and Winkler's two screens (removing models worse than Naïve2, excluding pairs with highly correlated errors), or by Diebold and Shin's (2019) two-step LASSO that zeroes some weights then shrinks the survivors toward equality — beats both using everything and selecting one.
+4. FEATURE-BASED CROSS-LEARNING IS WHERE THE FIELD'S MOMENTUM IS. The meta-model learns a mapping from features of a series to weights over a fixed method pool, trained across many series rather than within one, sidestepping the short-history problem that makes per-series weight estimation noisy. FFORMA placed second in M4 with 42 features and an XGBoost meta-learner; Montero-Manso et al.'s interval variant placed second for the uncertainty track over 100,000 series by predicting the interval radius as a linear combination of individual radii minimising the MSIS; the top three M4 methods all drew on cross-dataset information.
+5. DIVERSITY REVERSES SIGN WHEN THE OUTPUT IS A DISTRIBUTION. From the linear pool's variance decomposition: "seeking diverse forecasts, which is the standard advice for point combination, harms the probabilistic forecast by destroying sharpness and making the mixture under-confident", and Ranjan and Gneiting (2010) show the pool of individually calibrated forecasts is generally not calibrated. Hora (2004) gives the countervailing case that pooling helps calibration when components are overconfident; Jose et al. (2014) narrow it, that overconfident components with low diversity stay overconfident. The response is the trimmed opinion pool — exterior trimming removes components with extreme means to cut variance and address under-confidence, interior trimming removes the moderate ones to raise variance and address overconfidence.
+6. NONLINEAR POOLING DOES NOT PAY FOR ITS COMPLEXITY. Baran and Lerch (2018) compared state-of-the-art combination methods in case studies and found "no substantial difference in forecast performance between the simple linear pool and the theoretically superior but cumbersome nonlinear pooling approaches". The note: "That is the probabilistic restatement of the puzzle, which makes it two independent appearances of the same pattern in one paper." The one exception is Zischke et al. (2022) on high-volatility periods, which is about what to score rather than how elaborate the pooling function is.
+7. NONLINEAR COMBINATION OF POINT FORECASTS IS A THIN LITERATURE AND THE AUTHORS SAY SO PLAINLY. Two forms: a neural network over the individual forecasts (Donaldson and Kamstra, 1996), with purely linear and purely nonlinear specifications as special cases; and an additive pairwise term Σ_{i&lt;j} π_{ij} v_{ij} where v_{ij} is a nonlinear function of forecasts i and j. Reported results generally dominate simple averaging, OLS weights and performance-based weights, but the authors' own assessment of that evidence is that it rests on "fewer than ten time series, possibly hand-picked", alongside neglect of error correlations, unstable parameter estimation and multicollinearity from overlapping information sets.</t>
+        </is>
+      </c>
+      <c r="T56" s="30" t="inlineStr">
+        <is>
+          <t>1. Narrative review with no protocol, no screening counts and no meta-analysis, "so it establishes what exists and not what works." The Web of Science query is given in full but only for the Figure 1 publication-share chart, not for the review's own selection. Nothing states how papers were found, how many were screened, or what put one in or out. The authors run no experiment and aggregate no results, so there is no table anywhere comparing two weighting schemes on shared data. "I can cite this for the existence and the lineage of a method but never for its relative performance. This is the same structural weakness I recorded against [[The Evolution of Reinforcement Learning in Quantitative Finance, A Survey]], and the two surveys share it for the same reason, that coverage and adjudication are different jobs."
+2. The puzzle is reported rather than resolved, and where the paper gestures at a contradiction there is not actually one. Claeskens et al. (2016) derive that random combination weights can introduce bias and inflate the variance of the combined forecast relative to fixed weights; Zischke et al. (2022) are quoted as finding the opposite, that weight estimation imparts no bias or variability at all, and the authors record the opposition in a single clause and move on. The note's own reading: the opposition is a compression rather than a real disagreement — "Claeskens is a finite-sample result about the MSE of the combined point forecast under unbiased components, Zischke is a first-order asymptotic result about the sampling variability of the out-of-sample expected score", so the two answer different questions about different objects and neither refutes the other. "The genuine limitation is that the review leaves the question my contribution turns on, whether estimated weights can be expected to beat fixed ones, standing open, while the work that takes it considerably further was already in circulation when the review went to press."
+3. The non-interfering assumption excludes the systems I am actually positioned against (see AGENTS &amp; ORCHESTRATION above). The clean statistical properties — unbiasedness of the combination, the variance bound — hold under an assumption my pool does not satisfy.
+4. The target is always a realised value of one series under a symmetric loss, "so none of the optimality results transfer to a decision." The combined forecast is scored against y_{T+h} under MSE or a proper scoring rule; there is no portfolio, position, transaction cost, slippage or execution anywhere in forty pages. Elliott and Timmermann (2004) and Patton and Timmermann (2007) are cited as the asymmetric-loss extension, finding that optimal weights depend strongly on the degree of asymmetry in the loss and the skewness of the error distribution, "which is as far as this literature goes toward my setting. My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality."
+5. Cross-learning, the strand closest to what I'm building, is demonstrated at a scale I cannot reach. Results come from M4 at 100,000 series, M3, M5 and FRED, and the stated first limitation of the approach is the requirement for a large and diverse time series dataset to produce meaningful training. The workarounds offered are simulating series from assumed data generating processes or generating them with controllable characteristics using gratis, "both of which hand the researcher the features they then learn from. My per-counter archive is roughly 300 counters over 374 trading days, three orders of magnitude short of M4, and no result in this paper speaks to what a feature-to-weight meta-model does at that scale."
+6. Emerging and thin markets are absent from the entire paper. Applications named are retail, energy, economics, epidemiology and meteorology; the financial examples are macroeconomic series such as inflation and GDP growth. "Nothing addresses a market where the components themselves are estimated on short, illiquid, intermittently traded series, which is the condition under which every estimation-error argument in the puzzle section becomes more severe rather than less. The direction of that bias is at least clear, which is the useful part: everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
+7. (Recorded in the note as a WARNING against the paper, from work that postdates it.) The puzzle may be substantially a testing artefact. Frazier, Covey, Martin and Poskitt, "Solving the Forecast Combination Puzzle", Monash EBS working paper 18/2023 and arXiv:2308.05263, subsumes both positions above, characterising Claeskens as "more general than but ultimately commensurate with Smith and Wallis (2009)", i.e. one context-specific explanation among several rather than the general one. Their argument is that the puzzle is a consequence of the two-step estimation methodology itself: because estimated weights impart no first-order sampling variability into the usual predictive-accuracy statistic, that statistic converges to a non-standard generalised chi-squared rather than a normal, and their Theorem 1 states that when two weight vectors lie within O(T^{−1/4−ε}) of each other "the test has no power to distinguish them at all". An underpowered test defaults to the naive approach, which is the puzzle. Their remedy is one-step joint estimation of the constituent parameters and the combination weights against the final loss, which their Theorem 2 shows restores power. The note is explicit that this "needs a note of its own, and its publication status needs checking before it is cited as anything other than a working paper."</t>
+        </is>
+      </c>
+      <c r="U56" s="30" t="inlineStr">
+        <is>
+          <t>- A lineage and a precise statement of what is new, which the note judges "a stronger framing than novelty". My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) is a time-varying feature-conditioned linear combination, and the paper contains both halves separately: time-varying weights through the Kalman-filter and smooth-transition line, feature-conditioned weights through FFORMA. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That reads as a generalisation along an identified axis rather than new machinery. It also tells me what the honest comparison is: FFORMA's structure — a gradient-boosted meta-model mapping features to a weight simplex — is available to me as an implementation choice, "and if I use something simpler I should say why rather than let it look like I did not know."
+- The hardest possible equal-weight baseline, plus a falsification condition to pre-register.
+- A five-decade justification for having no pairwise interaction term in the weighting function. "With four agents that is ten parameters against four, from 374 days, so the argument has real force here. This is worth stating explicitly in the write-up, because a reviewer will ask why there is no interaction term, and the answer is that the literature tried that first and moved away from it."
+- Two cheap intermediate baselines: the Stock and Watson inverse-kth-power family (a one-parameter dial from k=0 equal weights to winner-take-all, "a sweep over k maps the whole continuum... for almost no implementation cost"), and the discounted inverse-MSE scheme, "which adds a time dimension without adding state" — the one the note names as "the baseline that actually threatens my contribution". So the planned three-way comparison (equal weights vs static learned weights vs state-conditioned weights) becomes four-way with a discounted performance-weighting arm.
+- An oracle-weight arm, weights fitted on the test window itself rather than on training, "because the gap between oracle and estimated performance is the estimation cost measured in my own data and in my own units: no gain under oracle weights means the conditioning hypothesis is simply wrong, a gain under oracle but not under estimated weights means it is an estimation problem I can put a number on, and it costs one further pass of the same pipeline."
+- Vocabulary for the abstention channel: time-varying subset selection via a pre-set threshold on a time-varying weighting scheme (Li et al., 2022). Plus Geweke and Amisano's observation that individually poor forecasts may still help in combination and one does not want to zero-weight them — "an argument for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero, which is a concrete design decision I had not settled."
+- An operational definition of diversity (low correlation among forecast errors, with Lemke and Gabrys' six diversity features and Thomson et al.'s coherence measure as alternatives), making my heterogeneity claim testable on my own pool.
+- Quantile averaging as the escape route if the orchestrator ever emits an interval, pairing with adaptive conformal inference.
+- A warning on inference: "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts."</t>
+        </is>
+      </c>
+      <c r="V56" s="30" t="inlineStr">
+        <is>
+          <t>The review contains weights that change over time and weights that change as a regression function of covariates, "and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state." The two nearest things are Deutsch et al.'s smooth transition specification, where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step. That is the axis along which my weighting function generalises existing work.
+Second, the review leaves standing open the question my contribution turns on — whether estimated weights can be expected to beat fixed ones — and its own two guidelines on the matter cut in opposite directions, with the paper clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature.
+Third, nothing in the paper speaks to a feature-to-weight meta-model at my data scale, nor to any market where the components themselves are estimated on short, illiquid, intermittently traded series.
+Fourth, the paper names interpretation of combination weights as an open research question; my orchestrator produces a weight per agent per step as a readable function of named market-state inputs, which is a direct response to that question rather than a byproduct.
+Fifth, subset selection has, in the paper's own assessment, "received scant attention, is mainly trimming on expertise alone", and "most existing algorithms are ad hoc and lack statistical rationale" — so a principled selection rule driven by a structural property of the output is defensible ground.</t>
+        </is>
+      </c>
+      <c r="W56" s="30" t="inlineStr">
+        <is>
+          <t>[[Forecast combinations, An over 50-year review]]</t>
+        </is>
+      </c>
+      <c r="X56" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: The orchestrator above everything else — this is the prior art for the weighting function itself, and the note is blunt that it is being written up precisely because "it is the most direct body of prior art on the half of my design I have covered least". Also the abstention channel (named here as time-varying subset selection), the confidence term C_{i,t} (via quantile averaging and calibrated intervals), the agent pool design (diversity as a measurable quantity rather than an asserted one), the explainability claim, and — most consequentially — the entire evaluation design.
+EFFECT ON MAIN GAP: THIS IS THE PAPER THAT BOTH LEGITIMISES AND THREATENS THE MAIN GAP, AND BOTH HALVES HAVE TO BE CARRIED THROUGH HONESTLY.
+The legitimising half. My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) stops being an invention and becomes a named construct with a lineage: a time-varying, feature-conditioned linear combination. The review contains time-varying weights (Diebold and Pauly, Deutsch et al., Terui and van Dijk's Kalman-filter random walk, Raftery et al.'s forgetting factors) and it contains feature-conditioned weights (FFORMA). What it does not contain, anywhere, is weights that are a function of measured exogenous market state. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That is a generalisation along an identified axis, which is a stronger and more defensible framing than novelty — and it is the framing the orchestration note already used. It also obliges me to be honest about implementation: FFORMA's gradient-boosted-meta-model-to-weight-simplex structure is available to me, and if I use something simpler I should say why.
+The threatening half, and it is serious. The forecast combination puzzle says that fifty years of evidence finds the equally weighted average extremely hard to beat, and that sophisticated weighting schemes lose because of estimation error. In M4, "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) across M3, M4, M5 and FRED find simple averaging shows, on average, more gain than complex methods. Elliott (2011) bounds the available gain from optimal over equal weights and finds it usually too small to pay for the estimation. Claeskens et al. (2016) prove random weights can introduce bias into combinations of unbiased components and inflate variance past the fixed-weight case. And the probabilistic side produces the same pattern independently: Baran and Lerch (2018) found no substantial difference between the simple linear pool and the theoretically superior nonlinear alternatives. "That is the probabilistic restatement of the puzzle, which makes it two independent appearances of the same pattern in one paper."
+Worse for me specifically: everything the paper says about estimation error swamping the gains from optimal weights "gets worse in my setting, not better", because my components are themselves estimated on short, illiquid, intermittently traded series. And the two practical guidelines the paper derives cut in opposite directions for me — "guideline one says that with limited historical data the simple average or weights ignoring covariances are recommended, which my 374 trading days per counter argues for, while guideline two says structural change impacts sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state."
+The honest consequence the note draws: the equal-weight baseline becomes the field's hardest benchmark, and "if my state-conditioned weighting fails to beat equal weights on the CSE, that is the expected outcome under the field's prior and not a surprise". The response is not to defend the gap but to pre-register — write down before the run what margin and what test would count as beating equal weights. And the note extracts a genuine contribution even from failure: "Which effect dominates on this data is the question, and the paper is clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature, so an answer in a thin frontier market is a contribution even if the answer is that equal weights win."
+How my setting differs — three ways the note identifies. (i) My weights condition on exogenous measured market state, not on properties of the series computed once; this is the axis the literature has not covered. (ii) My loss is not quadratic forecast MSE against a realised value — "My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality." The asymmetric-loss line (Elliott and Timmermann 2004, Patton and Timmermann 2007) is as close as this literature gets, and it finds optimal weights depend strongly on loss asymmetry and error skewness. (iii) My pool violates the review's non-interfering assumption: the four agents read overlapping data by construction, so the unbiasedness and variance-bound results do not hold for me, and the paper's own observation that overlapping information sets produce highly correlated errors is the mechanism by which that bites.
+A second threat, from the WARNING box rather than the paper itself. Frazier, Covey, Martin and Poskitt (Monash EBS WP 18/2023, arXiv:2308.05263) argue the puzzle is substantially an artefact of two-step estimation: estimated weights impart no first-order sampling variability into the usual predictive-accuracy statistic, so it converges to a generalised chi-squared rather than a normal, and their Theorem 1 says that when two weight vectors lie within O(T^{−1/4−ε}) of each other "the test has no power to distinguish them at all". Two consequences land directly on my design. "The O(T^{−1/4}) rate is not small at my sample sizes, roughly 0.23 at 374 trading days against roughly 0.14 on the ten-year index track, and with four agents sitting at 0.25 each under equal weights, a short sample puts almost any non-degenerate weighting scheme inside the dead zone. The constant is unknown so neither figure is a threshold, but the direction is unambiguous and it argues for running the weighting comparison on the index series rather than the per-counter panel." And their remedy, one-step joint estimation, is "mostly unavailable to me, since a retrieval agent is not jointly optimisable with a volatility model, so the partial version is to fit the parametric agents against the combined objective rather than against their own local losses." Caveat carried: this is a working paper and its publication status needs checking before it is cited as anything else.
+Design decisions this forces on the main gap: (a) no pairwise interaction term in the weighting function, backed by Bates and Granger, Newbold and Granger, and Winkler and Makridakis — ten covariance parameters against four diagonal ones, from 374 days; (b) a four-way rather than three-way comparison, adding a discounted inverse-MSE arm, because "if weights that merely react to recent agent performance do as well as weights conditioned on measured market state, then the state conditioning is not earning its place and I need to know that early"; (c) an oracle-weight arm to separate "the conditioning hypothesis is wrong" from "the estimation is too noisy"; (d) a Stock–Watson k-sweep to map the whole continuum from equal weights to winner-take-all cheaply; (e) pre-registration that separates two failure modes which look identical in the output — "the weighting genuinely not helping, which is the field's prior from the puzzle, against the weighting helping and the two-step test being unable to see it, because the first says abandon the conditioning and the second says change how it is estimated or tested."
+EFFECT ON THE ABSTENTION CHANNEL: Upgraded from a bespoke mechanism to named prior art. The paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme (Li et al., 2022). "That is structurally what the abstention channel does when the fundamental agent has no disclosure to work from, which is expected more than half the time, so I should present it in that vocabulary rather than as a bespoke mechanism." Two consequences: the paper's own assessment is that subset selection "has received scant attention, is mainly trimming on expertise alone, and that most existing algorithms are ad hoc and lack statistical rationale", so a principled selection rule driven by a structural property of the output is defensible ground; and Geweke and Amisano's observation that individually poor forecasts may still help in combination argues for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero — "a concrete design decision I had not settled."
+EFFECT ON THE CONFIDENCE TERM C_{i,t}: A route to making C_{i,t} a measured structural property rather than a self-report. If the orchestrator ever emits an interval rather than a point allocation, the linear pool's variance decomposition says component disagreement adds directly to pooled variance, "so a deliberately heterogeneous pool produces an under-confident interval, and that is the one place where my central design choice actively works against me." Quantile averaging avoids it — it averages cdfs horizontally, preserves the family for location-scale components, and is sharper for the same mean. "This connects to [[Adaptive Conformal Inference Under Distribution Shift]] more tightly than I expected, since adaptive conformal inference is a per-agent calibration wrapper and quantile averaging is the aggregation step, and the pair would give me a calibrated interval from a heterogeneous pool without the under-confidence that linear pooling would introduce. That is a route to the confidence term being a measured interval width rather than a self-report, which is what the scope revision asked for."
+EFFECT ON THE HETEROGENEITY CLAIM: The paper makes it testable and therefore falsifiable. "I describe the four agents as methodologically heterogeneous and that heterogeneity is load-bearing in the gap statement, but the paper's operational definition of diversity is low correlation among forecast errors... So the claim is testable on my own pool and I should run it: if the technical agent and the volatility agent produce errors that correlate at 0.8 on CSE data, the pool is substantially less diverse than the architecture diagram implies and the error-cancellation argument weakens accordingly. This is close to free, it uses data I will already have from the individual agent runs, and it is the kind of result that is much better found by me than by an examiner." Also relevant: Mannes et al. (2014) show the mean level of expertise in the pool sets a floor, so including a poor agent degrades the result — which bears on whether all four agents should always be in the pool.
+EFFECT ON EXPLAINABILITY: Upgraded from a feature to a positioned contribution. Interpreting combination weights is one of the paper's eight future directions — "discussing if, how, and when it is helpful to interpret combination weights". "My orchestrator produces a weight per agent per step as a readable function of named market-state inputs, so the trace of which agent was trusted when, and on what measured conditions, is a direct response to that question rather than a byproduct." Caveat carried from the layered-explainability reading: "a weight being readable is not the same as it being correct, so the claim is that the system exposes the quantity this literature identifies as unexamined, not that exposing it is sufficient."
+EFFECT ON SUB-GAP 1: Negative in the sense that it offers nothing — "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages" — but that absence is itself the boundary line. Everything in this paper is a weighting mechanism scored against a realised value under quadratic loss; none of its optimality results transfer to an after-cost decision objective. So the claim that execution cost belongs inside the decision objective is untouched by fifty years of combination theory, which is a clean separation to state.
+EFFECT ON SUB-GAP 2: Essentially none directly. The only contact point is Zischke et al. (2022), who find that in high-volatility periods weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample — "a result about choosing what to score rather than about how elaborate the pooling function is". That is about volatility level, not persistence, and the review contains nothing on persistence or on decay schedules. The structural-change guideline ("structural change impacts sophisticated schemes more than the simple average and changing weights are a legitimate response to it") is the nearest thing to support for conditioning on a regime, but it is a general statement with no persistence mechanism behind it.
+CSE DATA EVIDENCE: The note states my per-counter archive as roughly 300 counters over 374 trading days, "three orders of magnitude short of M4", with "no result in this paper" speaking to a feature-to-weight meta-model at that scale. The ten-year index track is the alternative. Those two sample sizes drive the O(T^{−1/4}) calculation — roughly 0.23 at 374 trading days against roughly 0.14 on the index track, against four agents at 0.25 each under equal weights — which argues for running the weighting comparison on the index series rather than the per-counter panel. The same 374 days drive the parameter-count argument against a pairwise interaction term (ten covariance parameters against four). And the note's reading of the thin-market absence is directional rather than agnostic: "everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
+PROPOSED REVISION STATED IN THE NOTE: Reframe the weighting function as a generalisation of FFORMA along one identified axis — exogenous measured market state at each step versus series properties computed once — rather than as new machinery. Pre-register the margin and the test that would count as beating equal weights, before the run. Expand the planned three-way comparison (equal / static learned / state-conditioned) to four-way by adding a discounted inverse-MSE arm, and add an oracle-weight arm fitted on the test window to separate "conditioning is wrong" from "estimation is too noisy". Add a Stock–Watson k-sweep. Run the weighting comparison on the index series rather than the per-counter panel, on the power argument. Fit the parametric agents against the combined objective rather than their own local losses, as the partial version of one-step joint estimation. Present the abstention channel as time-varying subset selection with a threshold, and shrink the abstaining agent's weight toward a floor rather than to exactly zero. Measure pool diversity as error correlation before claiming heterogeneity. Keep a separate note for the Frazier et al. working paper and check its publication status before citing it as anything other than a working paper. State explicitly in the write-up why there is no pairwise interaction term. And carry the warning that standard errors on a combined forecast are nontrivial because the weights are random and correlated with the forecasts — which matches the pattern where "the economic result and the formal test diverged" in the DRL global-equity portfolio note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="409.6" customHeight="1">
+      <c r="A57" s="29" t="inlineStr">
+        <is>
+          <t>P56</t>
+        </is>
+      </c>
+      <c r="B57" s="30" t="inlineStr">
+        <is>
+          <t>Gibbs, I. and Candès, E. (2021). Adaptive Conformal Inference Under Distribution Shift. Available from https://doi.org/10.48550/ARXIV.2106.00170 [Accessed 4 October 2026]. Citekey gibbsAdaptiveConformalInference2021. Authors: Isaac Gibbs and Emmanuel Candès, both in Stanford statistics, Candès also in mathematics. Venue per frontmatter: arXiv; the note's body records it as NeurIPS 2021. DOI: 10.48550/ARXIV.2106.00170. Zotero item: zotero://select/library/items/KZFWZYSI. Volume/pages: Not recorded in the note. Reference implementation in R at github.com/isgibbs/AdaptiveConformal.</t>
+        </is>
+      </c>
+      <c r="C57" s="30" t="inlineStr">
+        <is>
+          <t>2021 (frontmatter year, and the note's body dates it to NeurIPS 2021).</t>
+        </is>
+      </c>
+      <c r="D57" s="30" t="inlineStr">
+        <is>
+          <t>arXiv in the frontmatter; the note's body states "NeurIPS 2021". Both are recorded in the note, so I record both.</t>
+        </is>
+      </c>
+      <c r="E57" s="30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/ARXIV.2106.00170 — code at github.com/isgibbs/AdaptiveConformal.</t>
+        </is>
+      </c>
+      <c r="F57" s="30" t="inlineStr">
+        <is>
+          <t>Distribution-free uncertainty quantification / conformal prediction under distribution shift. This is a statistics methods paper and explicitly tooling rather than a competitor architecture: in my own words from the note, "there are no agents here, nothing resembling an orchestrator and no trading decision anywhere in it". It is the paper that introduced adaptive conformal inference (ACI). I file it alongside [[Predict the Future from the Past, On the Temporal Data Distribution Shift in Financial Sentiment Classifications]] as "the other half of the shift problem, that note measuring how much a fitted model decays over time and this one giving a mechanism that stays calibrated while it does."</t>
+        </is>
+      </c>
+      <c r="G57" s="30" t="inlineStr">
+        <is>
+          <t>Standard conformal prediction wraps any black-box regressor in a prediction set with a marginal coverage guarantee, but that guarantee rests on the calibration data and the test point being exchangeable, "which no financial time series satisfies". The specific failure the authors name in finance is that market behaviour shifts in response to legislation or major world events, which breaks exchangeability "in exactly the periods where a coverage statement would matter most". The objective is to drop the exchangeability assumption by turning miscoverage into a control problem: carry a single scalar alpha_t, compare the realised coverage of yesterday's interval against the target, and nudge alpha_t up or down by a fixed step. The reframing that makes this tractable is that the shift becomes a one-dimensional learning problem: rather than modelling how P(X_t, Y_t) changes, "which is hopeless", they define the realised miscoverage M_t(alpha) := P(S_t(X_t,Y_t) &gt; Q_hat_t(1-alpha)) and the optimal alpha_t* := sup{beta in [0,1] : M_t(beta) &lt;= alpha}, then track alpha_t* online. "Everything about the data generating process is compressed into the movement of a single parameter, which is what makes the distribution-free result possible and is also... what the result is silent about."
+Positioning against the two prior treatments of shift, both of which handle a single train-to-test transition rather than a continuously moving target: Tibshirani et al. reweight the calibration data by the likelihood ratio P_1(X)/P_0(X), which requires Y | X to be constant between training and test and the ratio itself to be known or accurately estimated, "neither of which holds for a market regime change"; Cauchois et al. form sets valid whenever D_f(P_1 || P_0) &lt;= rho by fixing a conservative alpha_rho in advance. The two differences the authors draw are that they estimate the optimal alpha* satisfying M(alpha*) = alpha rather than fixing a conservative value, and that they work in a fully online setting where the distribution moves at every step.</t>
+        </is>
+      </c>
+      <c r="H57" s="30" t="inlineStr">
+        <is>
+          <t>Two demonstration domains, neither of them a trading system. (1) Daily GARCH volatility prediction for twelve US stocks and indices, inputs taken from publicly available WSJ daily open-price datasets. (2) County-level US election-night forecasting, replicating the Washington Post's 2020 model over roughly 3,111 matched US counties. No frontier or emerging market anywhere in the paper; no CSE data.</t>
+        </is>
+      </c>
+      <c r="I57" s="30" t="inlineStr">
+        <is>
+          <t>Volatility experiment (the one I would be reimplementing):
+- Target: realised volatility V_t = R_t^2, with R_t = (P_t - P_{t-1})/P_{t-1}.
+- Inputs: daily open prices from publicly available WSJ datasets.
+- Universe: 12 stocks and indices, 4 shown in the main figure and 8 more in the appendix. Named panels in the note: Fannie Mae, BlackBerry, AMD, Nvidia.
+- Refit window: trailing 1,250 trading days, roughly 5 years, refit at every t &gt; 1250. Calibration uses the same 1,250-day trailing window of conformity scores.
+- Coverage metric: localCov, the average coverage over the most recent 500 days, roughly two years.
+- Period: not given as explicit start/end dates in the note, but the trajectories span at least 2004 through 2017 (AMD over-covering excursion in 2004, troughs in 2016-2017 for AMD and Nvidia, the 2008-2009 crisis window), and my own transfer note describes their calibration as being to "fifteen-plus years of daily data".
+Election experiment: conformalised quantile regression over 3,111 matched US counties, predictions starting once 500 counties have reported, each step splitting observed data 75/25 into training and calibration and refitting a linear quantile regression. Counties are ordered by time zone, east coast first and Hawaii last, so the covariate distribution drifts monotonically rather than jumping — "the shift is manufactured but realistic".</t>
+        </is>
+      </c>
+      <c r="J57" s="30" t="inlineStr">
+        <is>
+          <t>Pure numeric price time series (daily open prices) in the volatility experiment, and tabular cross-sectional county covariates in the election experiment. No text, no filings, no order-book data, no alternative data of any kind. The single engineered quantity that carries the method is the conformity score. For volatility it is normalised by the predicted variance:
+S_t := |V_t - (sigma_hat_t^t)^2| / (sigma_hat_t^t)^2
+where the superscript is the re-fitting index, so (sigma_hat_t^t)^2 is the GARCH point prediction from a model fitted using only data in [t-1250, t), and "the score at each step has seen nothing after t-1". That normalisation choice "turns out to carry as much weight as the adaptation itself".</t>
+        </is>
+      </c>
+      <c r="K57" s="30" t="inlineStr">
+        <is>
+          <t>"There is no architecture, which is the point." ACI is a wrapper and the algorithm is one line. Define the miscoverage event err_t := 1{Y_t not in C_hat_t(alpha_t)}, then update:
+alpha_{t+1} := alpha_t + gamma(alpha - err_t)
+where alpha is the target miscoverage rate, err_t is the realised miscoverage at step t taking value 0 or 1, and gamma &gt; 0 is the step size. When the interval covered, alpha_{t+1} rises by gamma*alpha and the next interval narrows; when it missed, alpha_{t+1} falls by gamma(1-alpha) and the next interval widens. The appendix shows this is online gradient descent on the pinball loss rho_alpha(beta_t - alpha_t), though the authors note standard regret bounds don't capture what they want, "because regret is measured against a fixed comparator and alpha_t* is a moving target". A weighted variant replaces err_t with sum_s w_s err_s for weights w_s proportional to 0.95^{t-s}, producing almost identical trajectories, "only smoother".
+Underlying split-conformal construction: fit a score S(X,Y) on a training set, compute its 1-alpha empirical quantile Q_hat(1-alpha) on a held-out calibration set, return C_hat_t = {y : S(X_t, y) &lt;= Q_hat(1-alpha)}.
+Point predictor in the volatility experiment: GARCH(1,1), sigma_t^2 = omega + tau*V_{t-1} + beta*sigma_{t-1}^2. Target coverage 1 - alpha = 0.9, initialised alpha_1250 = 0.1, step size gamma = 0.005 fixed. Comparators: fixed alpha_t = alpha on the same rolling window, plus an i.i.d. Bernoulli(0.1) sequence.
+The guarantee that costs nothing — Proposition 4.1, which is the one I would cite — states that with probability one, for all T:
+|(1/T) sum_{t=1}^{T} err_t - alpha| &lt;= (max{alpha_1, 1-alpha_1} + gamma) / (T*gamma)
+where alpha_1 is the initialisation; it follows from Lemma 4.1, that alpha_t stays in [-gamma, 1+gamma] for all t. The proof is three lines of rearranging the recursion and places "no constraint whatsoever on the data generating distribution", which is a strong statement and also "a statement about the time average rather than about any single t". The long-run empirical coverage frequency therefore converges to the target for any data generating process whatsoever, with the finite-sample deviation bound distribution-free and shrinking as 1/T.
+The sharper results cost assumptions. Theorems 4.1 and 4.2 model the environment as a hidden Markov chain {A_t} with non-zero absolute spectral gap 1 - eta, assume (alpha_t, A_t) is stationary and that Q_hat_t(.) and S_t(.) don't depend on t, then give a Bernstein-type concentration bound on |T^{-1} sum err_t - alpha| and an L-Lipschitz bound on E[(M(alpha_t | A_t) - alpha)^2] of the form
+(L(1+gamma)/gamma) * E[|alpha*_{A_{t+1}} - alpha*_{A_t}|] + (L/2)*gamma
+The practically useful fallout is the step-size prescription: that bound is minimised at gamma = (2 E[|alpha*_{A_{t+1}} - alpha*_{A_t}|])^{1/2}, so gamma should scale with the square root of the typical one-step movement in the optimal miscoverage level, larger in more volatile environments.
+Output: a prediction interval per step at the target coverage, plus the adapted miscoverage level alpha_t as a by-product series.</t>
+        </is>
+      </c>
+      <c r="L57" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — this is a single-model statistical wrapper with no agents, no orchestrator and no decision layer. In the note's words, "there are no agents here, nothing resembling an orchestrator and no trading decision anywhere in it". What it supplies instead is a scalar state variable, alpha_t, that an orchestrator elsewhere could consume. The property I single out is that ACI "has the useful property of not being a detector at all: alpha_t moves continuously, so the shift measurement and the response to it are the same quantity, which is a better fit for a weighting function than a binary alarm."</t>
+        </is>
+      </c>
+      <c r="M57" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no text, no sentiment component anywhere in this paper. Sentiment is in any case out of scope for my project.</t>
+        </is>
+      </c>
+      <c r="N57" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no filings, no retrieval, no document processing of any kind. The paper's only connection to A_F in my design is by analogy: the scope revision gave a worked example of structural confidence for A_F (does the extracted program parse, does every argument trace to a retrieved figure) and left the other three agents open; ACI supplies the analogue for A_V.</t>
+        </is>
+      </c>
+      <c r="O57" s="30" t="inlineStr">
+        <is>
+          <t>This is the paper's headline empirical domain. The point predictor is GARCH(1,1) on realised volatility V_t = R_t^2, refit on a trailing 1,250-day window, with the conformity score normalised by the predicted variance. The adaptation is substantial rather than cosmetic: across the four main-figure stocks alpha_t ranges between about 0.035 and 0.17 against a target of 0.1, so "at its extremes the method is targeting 96.5% coverage in some periods and 83% in others to achieve 90% on average". The troughs line up with crises, Fannie Mae and BlackBerry both bottoming out near 0.035 through 2008 and 2009, "which is the method widening its intervals hard when the GARCH fit is worst". At gamma = 0.005 a single miss moves alpha_t by 0.0045, so these swings take hundreds of days to develop and the series is slow-moving by construction, "in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]". The alpha_t trajectories "read as a volatility-regime series in their own right".
+Critically, the risk quantity produced is a coverage statement and not a width statement: see LIMITATIONS. The paper never attaches an interval to a position size or any other risk-budgeting decision.</t>
+        </is>
+      </c>
+      <c r="P57" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no liquidity variables, no spreads, no turnover, no execution cost anywhere in the paper. The liquidity question enters only in my transfer analysis: on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade."</t>
+        </is>
+      </c>
+      <c r="Q57" s="30" t="inlineStr">
+        <is>
+          <t>No attribution or interpretability machinery, and none needed — the method is a single scalar recursion and is fully transparent by construction. The interpretable artefact it produces is the alpha_t trajectory itself, which can be read directly as how badly the fitted model is tracking the market at each date. The theory is reported honestly in a way that matters for interpretation: the appendix comparison shows the naive bound decays as O(1/(T sqrt(epsilon_1))) and therefore *increases* as the shift size epsilon_1 shrinks, which the authors call undesirable, while the HMM-based bound decreases with the shift, and "both are reported side by side rather than only the flattering one".</t>
+        </is>
+      </c>
+      <c r="R57" s="30" t="inlineStr">
+        <is>
+          <t>Baselines: fixed alpha_t = alpha on the same rolling window, and an i.i.d. Bernoulli(0.1) sequence. The Bernoulli comparator is the right benchmark and not a strawman: "A perfectly calibrated method still produces a random coverage sequence, so a local coverage curve that wanders around 0.9 is not evidence of failure. The grey line is the moving average of an i.i.d. Bernoulli(0.1) sequence and shows how much wandering is expected from a method that is correct by construction. The test is therefore whether the adaptive curve stays inside that band, not whether it sits on 0.9, a more honest bar than most calibration plots set."
+Metrics: localCov (average coverage over the most recent 500 days) and quantile loss. Those are the only two. There is no decision-level evaluation of any kind, no cost attached to an interval that is too wide, and no comparison against any recalibration scheme beyond fixed-alpha on the same rolling window.
+An ablation on the score design is run: the normalised score S_t is replaced with the unnormalised S_tilde_t := |V_t - sigma_hat_t^2|.</t>
+        </is>
+      </c>
+      <c r="S57" s="30" t="inlineStr">
+        <is>
+          <t>- The non-adaptive method fails visibly and the adaptive one stays inside the Bernoulli band on all twelve names, with 2008 producing the clearest separation. Fannie Mae: fixed-alpha local coverage falls to roughly 0.83 against a target of 0.9 and stays depressed for most of 2008 and 2009, while the adaptive curve dips and recovers within the Bernoulli range. BlackBerry shows the same shape in 2008. AMD shows a fixed-alpha trough near 0.835 around 2016 and an over-covering excursion to 0.96 in 2004. Nvidia shows a trough near 0.85 across 2016 and 2017. "The useful reading is that the failure is two-sided, the fixed method over-covers as often as it under-covers, so what's being fixed is calibration drift rather than a conservatism bug." Caveat I flag in the note: the four stocks shown were selected out of twelve because they showed a clear failure of the non-adaptive method, which the authors state plainly, "so the main figure is a demonstration of the failure mode rather than a sample of typical behaviour, and the eight appendix panels are the ones to read for that."
+- alpha_t moves across roughly a fourfold range, about 0.035 to 0.17 against a 0.1 target.
+- The theory splits cleanly: Proposition 4.1 holds for any data generating process and is shown to be approximately tight, in that replacing max{1-alpha_1, alpha_1} with |alpha_1 - alpha*| under a noiseless idealisation recovers nearly the same bound, "so it is simultaneously agnostic and close to the best possible given a bad initialisation". Everything sharper needs the stationary HMM.
+- The conformity score design controls the result about as much as the adaptation does. The unnormalised score produces much wider swings in local coverage around 0.9 for the adaptive method, visibly outside the Bernoulli band and dropping below 0.6 on AMD and Fannie Mae in the crisis windows, against the normalised version which stays within a few percentage points throughout. The authors' explanation is that normalising by sigma_hat_t^2 is what makes the score approximately stationary, and they note the issue can be partially mitigated by a larger gamma. "So 'works with any black box' is true of the interface and not of the performance, and the real requirement is a score whose distribution moves slowly."
+- Election night: the fixed-alpha method incurs large troughs in local coverage at the time-zone changes, falling to about 0.825 and spending most of the sequence below 0.875, while the adaptive method holds near 0.9 with deviations comparable to the Bernoulli sequence. I rate this experiment as mattering more to me than the volatility panels, "because the shift is structural and predictable from the data ordering rather than driven by an exogenous shock, which is the shape of a cross-sectional screening problem."</t>
+        </is>
+      </c>
+      <c r="T57" s="30" t="inlineStr">
+        <is>
+          <t>- The guarantee is about coverage and says nothing about width, and no width or efficiency number appears anywhere in the paper. Proposition 4.1 is satisfied by a sequence that alternates between infinite and empty prediction sets in the right proportion, and the mechanism that makes it assumption-free is precisely the one that permits this: when alpha_t &lt; 0 the set is all of R and err_t = 0 by construction, which is how the proof of Lemma 4.1 gets its contradiction. "There is no table of average interval widths, no comparison of width against the fixed-alpha method, and no statement of how often alpha_t goes non-positive in the experiments." The alpha_t trajectories suggest it doesn't happen on these twelve stocks, the minimum sitting near 0.035, "but that's inference from a plot rather than a reported quantity, and a method sold on robustness to crises should report what its intervals cost in the crisis". I have not found that evaluation in the literature I have covered.
+- The results that hold at a single time step require a small shift, a stationary chain and a time-invariant quantile function, "which is close to the regime where I wouldn't need the method". Theorem 4.2 bounds the expected squared deviation of marginal coverage by a quantity proportional to E[|alpha*_{A_{t+1}} - alpha*_{A_t}|], which the authors interpret as a measurement of shift size, "so the bound is informative exactly when the shift is small and vacuous when it is large". The discussion concedes the fixed-Q_hat_t assumption directly and says it would be interesting to determine if similar results hold when Q_hat_t is fit online on recent data — which is what the volatility experiment actually does. "So the headline experiment sits outside the conditions of the sharper theory, and the only guarantee covering it is the long-run average one."
+- gamma = 0.005 is set once, justified in a sentence, and not varied anywhere in the paper. The stated reason is that it gave relatively stable trajectories while still allowing adaptation, "which is a reasonable thing to say and not a sensitivity analysis". The theory's prescription gamma proportional to sqrt(E|delta alpha*|) requires knowing the typical size of the shift in the optimal parameter, "which is the thing you are using the method to track", and the discussion names adaptive selection of gamma without prior knowledge as an open problem. "For a user with a short sample this is the live question, since the time to recover from a bad initialisation scales as 1/gamma."
+- Two domains, both with immediate feedback, and no decision-level evaluation of any kind. Y_t has to be revealed at every step for the update to run, and the discussion flags delayed or batched responses as outside the method. "Quantile loss and local coverage are the only metrics; there is no comparison against a simpler recalibration scheme beyond fixed-alpha on the same rolling window, no cost attached to an interval that's too wide, and nothing connecting calibration to a downstream decision. That's a fair scope for a statistics paper and a gap for anyone using it inside a trading system, where an interval has a position size attached."
+- The core modelling choice, adjusting the argument to Q_hat_t rather than Q_hat_t itself, is asserted as adequate rather than tested. The paper is explicit that in general both S_t(.) and Q_hat_t(.) should be re-estimated to track recent observations, and then proceeds to fix the quantile function and correct only alpha_t. The score-ablation result is the visible cost of that choice. "The design burden this pushes onto the user is real and under-acknowledged: picking a score that stays approximately stationary under regime change is a modelling problem of the same difficulty as the one the wrapper was meant to abstract away."
+- Data-depth constraint, flagged in the note as a hard constraint on transferring this and not a tuning detail: "Five years of daily data per counter is roughly thirteen times what my per-counter archive holds at 374 trading days, and the calibration set is drawn from the same window, so shrinking it degrades the GARCH fit and the empirical quantile simultaneously. The index track at ten years daily clears it comfortably; the per-counter track does not."</t>
+        </is>
+      </c>
+      <c r="U57" s="30" t="inlineStr">
+        <is>
+          <t>- The ACI update itself, as an adopted off-the-shelf component wrapping A_V's volatility forecast, with the normalised conformity score and the weighted variant (w_s proportional to 0.95^{t-s}) as the starting point rather than the plain update, because the weighted trajectories are smoother and my sample is short.
+- alpha_t as a candidate conditioning variable for the orchestrator: a continuous state variable rather than a binary alarm, running on the same daily index the orchestrator runs on, with no threshold to hand-tune. The concrete proposal recorded in the note is "to carry alpha_t as a candidate addition to the conditioning set and test it on the ablation protocol against the existing four terms rather than adopting it", a discipline [[Predicting financial market stress with machine learning]] makes the case for "after what 44 predictors on 84 observations did to that paper's out-of-sample performance."
+- A structural definition of C_{V,t}: wrap the FIGARCH or GJR-GARCH forecast in ACI with the normalised score, and let C_{V,t} be a function of the realised interval width at the target coverage, "so a volatility agent whose model has drifted reports wider intervals and is automatically down-weighted. That's a measured property of the output, which is precisely what the redefinition demanded."
+- A principled abstention trigger: "when alpha_t falls low enough that the interval at the target coverage spans the plausible range of next-day volatility, the agent has nothing to say, and the orchestrator should see that as absence rather than as a weak signal. This is the mechanism AlphaAgents lacked when a human deleted an agent by hand, expressed as a quantity that moves on its own."
+- The Bernoulli-band evaluation convention, as the honest way to judge a coverage curve.
+- A hard evaluation commitment carried over from the paper's own gap: "any calibration result reports average interval width alongside coverage, and reports both over quiet sub-periods separately from crisis windows, which is consistent with how the friction-aware evaluation already splits its reporting."
+- Two named experiments rather than design decisions: (a) a gamma sweep on the index track where I have the length to measure it, then carry the chosen value down to the counters; (b) testing whether a liquidity-adjusted volatility normaliser keeps the score stationary on a thin book, "using the same Amihud and turnover inputs already being computed for the cost model and for the composite liquidity state, so one measurement serves a third purpose."
+- The honesty discipline on claiming: "Claim this as an adopted component and not as a contribution, and say so before anyone asks."</t>
+        </is>
+      </c>
+      <c r="V57" s="30" t="inlineStr">
+        <is>
+          <t>- No link from calibration to a decision. The method stops at the interval. Nothing in the paper attaches an interval to a position size, a weight, or an abstention. "That's a fair scope for a statistics paper and a gap for anyone using it inside a trading system, where an interval has a position size attached."
+- No width accounting. Coverage is guaranteed, width is unreported and in principle unbounded. The failure mode this leaves open is exactly the one I have to avoid: "A volatility agent that achieves nominal coverage by widening its intervals during crises is well calibrated and useless for position sizing, which is the same failure as an orchestrator whose weights move impressively in the two or three most volatile CSE months and are inert otherwise."
+- No step-size selection procedure for short samples. gamma = 0.005 is calibrated to fifteen-plus years of daily data; the theoretical prescription is circular in practice; adaptive gamma selection is named by the authors as an open problem.
+- No guidance on score design for illiquid assets. Normalising by predicted variance works when the denominator is reliable; on a thin book with zero-return days and stale quotes it may not be, and that is left entirely to me.
+- No treatment of delayed or batched feedback, which the authors explicitly place outside the method.
+- No pooling-versus-per-unit guidance when the per-unit sample is too short for the refit window. The honest options I record are "a shorter joint window with the calibration degradation reported, or pooling scores across counters, which breaks the per-counter conditioning the method relies on."</t>
+        </is>
+      </c>
+      <c r="W57" s="30" t="inlineStr">
+        <is>
+          <t>[[Adaptive Conformal Inference Under Distribution Shift]]</t>
+        </is>
+      </c>
+      <c r="X57" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: C_{i,t} above all — specifically C_{V,t}, the confidence term for A_V — plus the abstention channel, the orchestrator's conditioning set (as a candidate fifth term), the distribution-shift item in the evaluation plan, and the data-depth discussion. It touches nothing in A_T, A_F or A_L directly, and it is tooling rather than a competing architecture, so it cannot close or threaten the orchestration claim in either direction.
+EFFECT ON MAIN GAP: It strengthens the main gap in two distinct ways and leaves the claim itself untouched. First, it closes a specification hole inside my own design rather than outside it. The scope revision redefined C_{i,t} as a structural property of an agent's output rather than a self-report, and gave a worked example only for A_F (does the extracted program parse, does every argument trace to a retrieved figure), leaving the other three agents open. ACI supplies the analogue for A_V: "the calibrated interval width is the structural confidence term the scope revision asked for, and it arrives measured rather than self-reported". The recipe is concrete — wrap the FIGARCH or GJR-GARCH forecast in ACI with the normalised score S_t = |V_t - sigma_hat^2| / sigma_hat^2, and let C_{V,t} be a function of the realised interval width at the target coverage, so a volatility agent whose model has drifted reports wider intervals and is automatically down-weighted. That is a measured property of the output, which is exactly what the redefinition demanded.
+Second, it converts the abstention channel from a hand-set threshold into a quantity that moves on its own. The design already treats abstention as structural because A_F is expected to be unusable more than half the time on CSE filings; the same machinery now works for a price-derived agent. "When alpha_t falls low enough that the interval at the target coverage spans the plausible range of next-day volatility, the agent has nothing to say, and the orchestrator should see that as absence rather than as a weak signal. This is the mechanism AlphaAgents lacked when a human deleted an agent by hand, expressed as a quantity that moves on its own."
+The boundary of the contribution needs stating plainly and early, which is why the note ends where it does: "ACI is an off-the-shelf wrapper with a public R implementation, four years old and widely cited, and there is nothing novel in applying it to a GARCH forecast since that is the paper's own worked example. What would be a candidate technical contribution not identified in the literature I have covered is using the adapted miscoverage level as an input to a weighting function over heterogeneous agents, which is a different claim and a much narrower one, and it needs validating against recent work before it goes anywhere near the novelty statement." So: adopt ACI as a component, claim only the orchestration use of alpha_t, and validate that narrower claim before it enters the novelty statement.
+EFFECT ON SUB-GAP 1: Mostly indirect, and it creates one new liquidity dependency rather than resolving anything. The paper has no liquidity content at all — no spreads, no turnover, no execution cost. But the score-design finding pushes liquidity into the calibration layer, which I had not anticipated. Normalising the conformity score by predicted variance is what made their score approximately stationary; on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade." The candidate fix is to normalise by a liquidity-adjusted volatility estimate "using the same Amihud and turnover inputs already being computed for the cost model and for the composite liquidity state, so one measurement serves a third purpose." That is a reuse of L_t inside the machinery that produces C_{V,t}, which is a genuine coupling between the liquidity state and the reliability of a price-derived agent — the second half of Sub-gap 1's statement, that liquidity simultaneously conditions the reliability of price-derived agents. It is recorded as "a named experiment, not a design decision", so it is a hypothesis I owe a test, not a finding I can lean on.
+EFFECT ON SUB-GAP 2: Substantial, and in a way that is adjacent to rather than inside Sub-gap 2. Sub-gap 2 is about volatility PERSISTENCE and specifically about replacing an EWMA half-life, which assumes exponential decay, with a persistence-aware decay schedule. ACI does not estimate persistence and does not propose a decay schedule, so it does not close the sub-gap. What it does is supply a second, independent slow-moving state series over the same volatility object: at gamma = 0.005 a single miss moves alpha_t by 0.0045, "so these swings take hundreds of days to develop, and the series is slow-moving by construction in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]." The alpha_t trajectories "read as a volatility-regime series in their own right", ranging about 0.035 to 0.17 and bottoming out in 2008-2009 when the GARCH fit is worst. That is a measurement of how badly a fitted volatility model is tracking the market, which is a different quantity from P_t but lives on the same timescale and is produced by the same agent — so the discipline required is to test whether alpha_t adds anything over the existing four conditioning terms, not to assume it does. Hence the note's framing: carry it "as a candidate addition to the conditioning set and test it on the ablation protocol against the existing four terms rather than adopting it."
+The sharper transfer finding is that ACI's own step size has the same structural problem Sub-gap 2 identifies in the EWMA half-life. gamma is a fixed decay rate on a non-stationary target, set once, never varied, and justified in a sentence; the theory's own prescription gamma proportional to sqrt(E|delta alpha*|) says gamma should be larger in more volatile environments, which is a persistence-type statement the paper does not operationalise. So ACI imports the exact defect Sub-gap 2 exists to correct, one level up. That is useful: it means the persistence argument generalises beyond the volatility scaler, and it also means I cannot adopt gamma = 0.005 and stop thinking. "On 374 observations a step that small means alpha_t barely leaves its initialisation, so the sample would be spent in the transient the theory warns about, and the prescription gamma proportional to sqrt(E|delta alpha*|) points the same way given the CSE's crisis sequence. The experiment is a gamma sweep on the index track where I have the length to measure it, then carry the chosen value down to the counters."
+CSE DATA EVIDENCE: The paper contains none — twelve US names and 3,111 US counties. The CSE evidence in this cell is my own data-depth accounting, and it is the sharpest constraint in the note: "The 1250-day refit window is the sharpest data-depth constraint I've hit in a review and it splits my two tracks. Five years of daily data per counter, with the calibration scores drawn from the same window, against 374 trading days per counter in the archive. On the index track at ten years daily the recipe transfers as written; on the per-counter track it does not, and the honest options are a shorter joint window with the calibration degradation reported, or pooling scores across counters, which breaks the per-counter conditioning the method relies on. This belongs in the data-depth discussion as a named requirement with a number attached, not as a general concern." Five years per counter is roughly thirteen times the per-counter archive. Note also that shrinking the window degrades the GARCH fit and the empirical quantile simultaneously, because the calibration scores come from the same window — the two failures are not independent.
+PROPOSED REVISION STATED IN THE NOTE: Several, all recorded as candidates or experiments rather than adopted design:
+1. Define C_{V,t} as a function of the ACI-calibrated interval width at the target coverage, wrapping the FIGARCH or GJR-GARCH forecast with the normalised conformity score.
+2. Trigger A_V abstention when alpha_t falls low enough that the target-coverage interval spans the plausible range of next-day volatility, and have the orchestrator read that as absence rather than as a weak signal.
+3. Carry alpha_t as a candidate fifth conditioning term and test it on the ablation protocol against L_t, V_t, P_t and C_{i,t} rather than adopting it.
+4. Attach ACI to the pre-registered distribution-shift item as its method, on the grounds that "alpha_t is a continuous state variable rather than an alarm" and so needs no threshold.
+5. Run a gamma sweep on the ten-year index track and carry the chosen value down to the counters; start from the weighted update (w_s proportional to 0.95^{t-s}) rather than the plain one.
+6. Test a liquidity-adjusted volatility normaliser for the conformity score on thin counters, reusing the Amihud and turnover inputs already computed for the cost model and the composite liquidity state.
+7. Record the 1,250-day refit requirement in the data-depth discussion as a named number that splits the index track from the per-counter track.
+8. Commit the evaluation to reporting average interval width alongside coverage, split between quiet sub-periods and crisis windows.
+9. Claim ACI as an adopted component, not a contribution; the only candidate contribution is using the adapted miscoverage level as an input to a weighting function over heterogeneous agents, and that needs validating against recent work first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="409.6" customHeight="1">
+      <c r="A58" s="29" t="inlineStr">
+        <is>
+          <t>P57</t>
+        </is>
+      </c>
+      <c r="B58" s="30" t="inlineStr">
+        <is>
+          <t>Gu, Kelly and Xiu. Empirical Asset Pricing via Machine Learning. Citekey guEmpiricalAssetPricing2018. Affiliations recorded in the note: Chicago Booth and Yale. The note's frontmatter gives year 2018 and the body dates the version read as the "November 2018 working version". The body also states this is "of what became the *Review of Financial Studies* paper that everything in this area now cites" — so the journal is the Review of Financial Studies, but the note does not record the RFS publication year, volume, pages or DOI. First names, DOI, arXiv ID and link: Not recorded in the note.
+TO BE EXPLICIT ABOUT WHICH IS WHICH: 2018 is the working-paper year from the note's frontmatter and is the version the note was written against; the Review of Financial Studies is the eventual journal of record, and its publication year is Not recorded in the note.</t>
+        </is>
+      </c>
+      <c r="C58" s="30" t="inlineStr">
+        <is>
+          <t>2020 (Review of Financial Studies 33(5)). The note's frontmatter carries 2018, the working-paper year; 2020 is the journal of record.</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="inlineStr">
+        <is>
+          <t>Working paper in the version read (November 2018); published subsequently in the *Review of Financial Studies*, which the note describes as "the paper that everything in this area now cites". Volume and pages: Not recorded in the note.</t>
+        </is>
+      </c>
+      <c r="E58" s="30" t="inlineStr">
+        <is>
+          <t>Not recorded in the note.</t>
+        </is>
+      </c>
+      <c r="F58" s="30" t="inlineStr">
+        <is>
+          <t>Empirical asset pricing / machine learning for cross-sectional return prediction. A comparative horse race of thirteen prediction methods on a single shared problem. The note is emphatic that this is not a competitor architecture and is not being read as one: "there are no agents here and no orchestration problem". It earns a full note for four reasons recorded verbatim in the note: it is "the best available calibration of what a well-specified return predictor actually achieves, and the number is small enough that it should reset my expectations for the technical agent before I build it"; "the signal families it ranks at the top are price trend, liquidity and volatility, which is independent large-sample evidence for two of the three state variables my orchestrator conditions on"; "its feature construction is the single-model version of conditioning on market state, every characteristic interacted with every macro variable, which is structurally the thing I am proposing to do one level up"; and "it is a clean, well-documented instance of the failure mode my cost sub-gap exists to address, reporting 113% monthly turnover and an annualised Sharpe of 2.35 in the same table without deducting a basis point."</t>
+        </is>
+      </c>
+      <c r="G58" s="30" t="inlineStr">
+        <is>
+          <t>Two literatures had accumulated hundreds of predictors and no way to evaluate them jointly. The cross-sectional strand regresses future returns on a few lagged characteristics; the time-series strand regresses aggregate returns on a few macro variables. The authors note the profession has accumulated "a staggering list of candidates", with Green et al. counting 330 stock-level signals, Harvey et al. 316 factors, and Welch and Goyal nearly 20 aggregate predictors. The stated problem is "how to assess the incremental content of a newly proposed predictor while jointly controlling for the gamut of extant signals, which is the multiple-comparisons problem dressed as an estimation problem."
+Three properties of the setting are argued to suit machine learning, and the note rates the argument as careful: risk-premium measurement is a conditional expectation, so it is a prediction problem rather than an inference problem; the predictor count approaches the observation count and the predictors are close cousins, "which is where OLS breaks"; and theory gives essentially no guidance on functional form, "so the search over specifications has to be mechanical."
+The framing is explicitly measurement, not mechanism, and the authors say so. Section 1.6 concedes that improved predictions are only measurements, that they do not identify deep associations between prices and conditioning variables, and that recovering mechanisms requires the economist to impose structure. The note calls this "the most honest paragraph in the paper and worth keeping in view, because the variable importance results later on are routinely cited as if they were economic findings."</t>
+        </is>
+      </c>
+      <c r="H58" s="30" t="inlineStr">
+        <is>
+          <t>US equities — every firm on NYSE, AMEX and NASDAQ. A deep, liquid, developed market, sixty years of it. No emerging or frontier market content. The note draws the implication in the opposite direction: "the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."</t>
+        </is>
+      </c>
+      <c r="I58" s="30" t="inlineStr">
+        <is>
+          <t>CRSP monthly total returns for every firm on NYSE, AMEX and NASDAQ, March 1957 to December 2016, with the Treasury bill rate used to form excess returns.
+- Universe: ~30,000 stocks, average &gt;6,200 per month.
+- Period: March 1957 to December 2016, 60 years.
+- Split: 18 years train (1957-1974), 12 validation (1975-1986), 30 test (1987-2016).
+- Features: 94 characteristics x (8 macro + 1) + 74 industry dummies = 920.
+- Characteristic frequency: 61 annual, 13 quarterly, 20 monthly.
+- Target: one-month-ahead individual excess return, pooled panel.
+- Refit: recursive, once per year, training window grows by one year each time.
+- Validation: fixed-size, rolled forward twelve months per refit.
+- Primary metric: R^2_oos benchmarked against zero, not the historical mean.
+Four choices the note flags as mattering more than they look: the sample is deliberately unfiltered — stocks below $5, share codes beyond 10 and 11, and financial firms all retained — "which I note here because the economic results later depend on the small end of the universe"; publication lags are imposed explicitly, monthly characteristics delayed at most one month, quarterly at least four, annual at least six; missing characteristics are replaced with the cross-sectional median for that month; and there is no cross-validation anywhere, by design, to preserve temporal ordering.</t>
+        </is>
+      </c>
+      <c r="J58" s="30" t="inlineStr">
+        <is>
+          <t>Purely numeric panel data: firm characteristics, aggregate macro series, and industry dummies. No text, no filings text, no alternative data.
+The over-arching feature construction is the part the note cares most about. Rather than feeding characteristics and macro variables in side by side, they take the Kronecker product, so every characteristic appears once on its own and once interacted with each of the eight macro state variables:
+z_{i,t} = x_t (kron) c_{i,t}
+where c_{i,t} is the P_c x 1 vector of stock i's characteristics at t, and x_t is the P_x x 1 vector of macroeconomic state variables, including a constant, common to all stocks.
+The motivation is the conditional beta-pricing identity E_t(r_{i,t+1}) = beta'_{i,t} lambda_t. If risk exposures are linear in characteristics, beta_{i,t} = theta_1 c_{i,t}, and the price of risk is linear in macro state, lambda_t = theta_2 x_t, then the model collapses exactly onto the interacted feature set:
+g*(z_{i,t}) = (x_t (kron) c_{i,t})' vec(theta_1' theta_2)
+"The interaction is not a convenience, it is where time variation in the signal's value enters the model."
+Dominant individual features by summed importance: short-term reversal, log market equity, twelve-month momentum, momentum change, recent maximum return, industry momentum, return volatility, dollar volume (top eight). Grouped families: price trend; liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread); risk (total and idiosyncratic volatility, beta, beta squared); valuation ratios a distant fourth.</t>
+        </is>
+      </c>
+      <c r="K58" s="30" t="inlineStr">
+        <is>
+          <t>Thirteen prediction methods, all on the same target and the same splits, differing only in how they constrain g(.): OLS on all 920 features, a three-characteristic OLS benchmark (OLS-3), PLS, PCR, elastic net, a spline generalized linear model with group lasso (GLM), random forest, gradient boosted regression trees (GBRT), and feed-forward networks at one through five hidden layers (NN1-NN5).
+- PCR and PLS both compress 920 features into K components, PCR maximising variance among the predictors and PLS maximising squared covariance with the target, "so PLS sacrifices fidelity to Z for predictive relevance".
+- GLM adds a second-order spline expansion per characteristic under a group lasso penalty, so a characteristic enters with all K of its spline terms or none, and critically it adds NO interactions — "which is what makes it the diagnostic model of the paper".
+- Networks are fixed at five architectures following the geometric pyramid rule, NN1 at 32 neurons through NN5 at 32-16-8-4-2, all ReLU, all fully connected, trained by SGD with Adam learning-rate shrinkage, l_1 penalisation, early stopping, batch normalisation, and seed ensembling.
+- Robust losses run throughout. The Huber objective replaces squared loss with absolute loss beyond a tuned threshold xi; the authors report the Huber variant for OLS, elastic net, GLM and GBRT because it performs better, and the Monte Carlo confirms it improves out-of-sample R^2 for every method it is applied to.
+Output: a one-month-ahead excess-return forecast per stock, aggregated into decile-spread portfolios and bottom-up S&amp;P 500 forecasts for the economic evaluation.</t>
+        </is>
+      </c>
+      <c r="L58" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — a single-estimator horse race with no agents, no orchestrator, no weighting of heterogeneous producers over a shared decision. What it does instead is the closest single-model analogue: the Kronecker construction makes every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator. The note draws the line precisely: "That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound. What it does not do is the thing I am claiming: the interaction weights are estimated once per annual refit, they are a function of macro variables rather than of any measured reliability of the signal, and no channel in their model can go absent, because a missing characteristic is median-imputed rather than down-weighted. The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line."</t>
+        </is>
+      </c>
+      <c r="M58" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — no sentiment data, no text, no news or social signal anywhere in the paper. Sentiment is out of scope for my project in any case.</t>
+        </is>
+      </c>
+      <c r="N58" s="30" t="inlineStr">
+        <is>
+          <t>No retrieval, no documents, no RAG — accounting characteristics enter as pre-constructed numeric features from CRSP/Compustat-style panels, not as parsed filings. What the paper contributes to A_F is a horizon and lag discipline rather than a pipeline. Accounting characteristics cluster at the bottom of the importance ranking, and the authors attribute this partly to their low update frequency, noting that at the annual horizon price-trend variables lose ground to liquidity and risk measures while industry becomes substantially predictive. The publication-lag structure is explicit — monthly characteristics delayed at most one month, quarterly at least four, annual at least six — and the note treats this as the specification to write down for A_F "before touching any filing data, since CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."</t>
+        </is>
+      </c>
+      <c r="O58" s="30" t="inlineStr">
+        <is>
+          <t>Volatility enters as a predictor family rather than as a modelled process. The "risk" group — total volatility, idiosyncratic volatility, beta, beta squared — is one of the three dominant families across every method. The marginal-relationship plots show trees and networks finding large sensitivity to volatility where penalized linear models find none: a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return under GBRT or NN3 (and the companion size effect: a firm falling from median size to the 20th percentile gains roughly 2.4% in annualised expected return). On the macro side, market-level stock variance gets little weight anywhere and essentially none from the networks.
+No conditional volatility model, no GARCH, no persistence estimate, no volatility targeting, no risk scaling of positions. Portfolio construction is decile sorts, equal- and value-weighted, with Sharpe reported but no volatility budget.</t>
+        </is>
+      </c>
+      <c r="P58" s="30" t="inlineStr">
+        <is>
+          <t>Liquidity appears as a predictor family and is absent as a friction, and the gap between those two facts is what the note exploits. The liquidity group (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) is one of the three dominant families across every method. But: "There are no transaction costs anywhere in the paper, and the turnover figures make that decisive rather than cosmetic." The best strategy, an equal-weighted decile spread on NN4 forecasts, returns 3.3% per month, 39.0% annualised, at an out-of-sample Sharpe of 2.35, with monthly turnover of 114.08%. Networks run 110.87% to 114.08%, elastic net 143.61% and OLS-3 156.78%, against 22.87% for a size decile spread. The authors note that high turnover is unsurprising given the dominance of price-trend predictors, "and then stop."
+Two things in their own results indicate the size of what is left out. Value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, "so the gap between the paper's two weighting schemes is larger than the gap between most of its methods." And the universe retains sub-$5 stocks by explicit choice. The paper offers the higher top-1,000 R^2, 0.72% against 0.46%, as reassurance that machine learning is not merely picking up small-scale inefficiencies driven by illiquidity, "but the result carrying the economic claim is an equal-weighted spread over the whole board, and both cannot be load-bearing at once."</t>
+        </is>
+      </c>
+      <c r="Q58" s="30" t="inlineStr">
+        <is>
+          <t>Variable importance is defined as the reduction in predictive R^2 from setting one predictor to zero with all other estimates held fixed. Marginal-relationship plots show each model's fitted sensitivity to individual characteristics. A placebo test adds five simulated noise characteristics and they rank low, which the note credits as a real check. The paper also reports model complexity over time (Figure 3): elastic net selecting fewer than five features in the first decade of the test sample and 20 to 40 after 2000, PCR using 20 to 40 components, GBRT moving from roughly 20 features to 30.
+The note's reading of the attribution machinery is sceptical — see LIMITATIONS — and it re-flags Section 1.6's own concession that these are measurements rather than mechanisms.</t>
+        </is>
+      </c>
+      <c r="R58" s="30" t="inlineStr">
+        <is>
+          <t>Baselines: OLS on all 920 features, OLS-3 (three characteristics), PLS, PCR, elastic net, GLM, random forest, GBRT, NN1-NN5. A Monte Carlo with 100 repetitions under both a sparse linear and a nonlinear interacted data generating process, with an oracle for reference.
+Primary metric:
+R^2_oos = 1 - [ sum_{(i,t) in T_3} (r_{i,t+1} - r_hat_{i,t+1})^2 ] / [ sum_{(i,t) in T_3} r_{i,t+1}^2 ]
+The denominator is the sum of squared excess returns WITHOUT demeaning, so the benchmark is a forecast of zero rather than the historical mean. The authors justify this on the grounds that the historical mean stock return is so noisy it artificially lowers the bar, and they quantify the difference: benchmarking against historical means raises every method's monthly R^2 by roughly three percentage points, with OLS-3 going to 3.74% per month. The note calls this "a decision that changes every number in the paper".
+For pairwise comparison they adapt Diebold-Mariano, which in its standard form assumes weak error dependence that cross-sectional return data violates. Their fix collapses the panel to one time series of cross-sectional average squared-error differences before testing:
+d_{12,t+1} = (1/n_3) sum_{i=1}^{n_3} [ (e_hat^{(1)}_{i,t+1})^2 - (e_hat^{(2)}_{i,t+1})^2 ],   DM_12 = d_bar_12 / sigma_hat_{d_bar_12}
+with sigma_hat a Newey-West standard error.
+Economic evaluation: decile-spread portfolios (equal- and value-weighted) with out-of-sample Sharpe and monthly turnover; bottom-up S&amp;P 500 forecasts; and the Campbell and Thompson mapping from predictive R^2 to Sharpe ratio, SR* = sqrt((SR^2 + R^2)/(1 - R^2)).</t>
+        </is>
+      </c>
+      <c r="S58" s="30" t="inlineStr">
+        <is>
+          <t>- Absolute numbers are tiny and the spread across methods is narrower than the narrative suggests. Monthly stock-level R^2_oos: OLS on all 920 features -4.60% (worse than forecasting zero); OLS-3 0.16%; elastic net 0.09%; PLS 0.18%; PCR 0.28%; GLM 0.19%; random forest 0.27%; GBRT 0.30%; networks 0.35% (NN1) to a peak of 0.39% (NN3). "So the entire distance from the three-characteristic benchmark to the best model in the paper is 23 basis points of monthly R^2." Size split: NN3 reaches 0.72% on the top 1,000 stocks by market value against 0.46% on the bottom 1,000. At the annual horizon everything scales up roughly an order of magnitude, NN4 at 3.60% and NN3 at 3.40% across all stocks.
+- The Diebold-Mariano table does not support the method ranking the abstract implies, and the paper is upfront about this itself. Differences among all the regularized linear models are insignificant — OLS-3, PLS, PCR, elastic net and GLM are statistically indistinguishable from each other. Trees improve on linear models but the improvements are described as at best marginally significant. Neural networks are the only class producing large significant gains over linear and generalized linear models, NN3 against OLS-3 at 3.01, and their improvement over trees is not significant. Among the networks themselves nothing clears: NN3 against NN5 reaching -1.92 and NN3 against NN4 only -1.03. "On this evidence the defensible claim is narrower than 'trees and neural nets are the best performing methods': it is that networks beat linear specifications, and that everything else in the ranking is suggestive."
+- Interactions, not nonlinearity, are the mechanism, and the GLM is the clean evidence. The GLM applies spline expansions to every individual characteristic and reaches 0.19%, no better than the linear specifications, despite selecting more features than elastic net. Since the only thing it lacks relative to trees and networks is multi-way interaction, the authors read the gap as attributable to interactions specifically rather than to curvature. The note rates this "the most convincing single inference in the paper because it is a genuine ablation rather than a comparison across unrelated model families." Marginal-relationship plots corroborate: penalized linear models find no association at all between returns and either size or volatility while trees and networks find large sensitivity to both.
+- Shallow beats deep, and the simulation says why. Performance peaks at three hidden layers and declines at four and five; random forests settle on trees of one to five layers on average; GBRT selects fewer than six leaves. The authors attribute this to "the comparative dearth of data and the low signal-to-noise ratio relative to settings like computer vision where deep learning thrives." The Monte Carlo makes the trade-off concrete: under a sparse linear DGP the nonlinear methods lose very little — ENet+H at 4.27% out-of-sample against NN1 at 4.42% and RF at 3.37% — but under a nonlinear interacted process the ordering becomes decisive, GBRT+H and NN2 both at 3.12% against ENet+H at 0.59% and GLM+H at 1.27%, with the oracle at 5.40%. "The asymmetry is the useful part: flexible methods cost almost nothing when the truth is linear and gain a great deal when it is not."
+- Aggregation into portfolios multiplies the measurable signal and is where linear methods fail outright. Bottom-up S&amp;P 500 forecasts give monthly R^2_oos of -0.11% for OLS-3 and -2.62% for PCR, against 0.86% for GLM and 1.80% for NN3, rising to 15.68% at the annual horizon. The explanation offered is that individual stock returns behave erratically for the smallest and least liquid names, so averaging into portfolios cancels idiosyncratic noise while preserving the signal. Running the Campbell-Thompson mapping, the S&amp;P 500 buy-and-hold Sharpe of 0.42 becomes 0.63 for an investor timing on NN3 forecasts.
+- Every method converges on the same three signal families. Top eight characteristics by summed importance across all eleven models: short-term reversal, log market equity, twelve-month momentum, momentum change, recent maximum return, industry momentum, return volatility, dollar volume. Grouped: price trend, liquidity, risk, with valuation ratios a distant fourth. Linear and dimension-reduction models concentrate importance heavily on momentum and reversal; trees and networks spread it more evenly. On the macro side every method treats aggregate book-to-market as a critical predictor — the single highest-weighted macro variable for the networks and the penalized linear models at 28.57% for NN1 and 43.46% for GLM — while stock variance gets little weight anywhere. The split between families is sharper than the consensus: linear models load overwhelmingly on default spread and the Treasury rate (42.13% on default spread for elastic net) while the networks put essentially nothing there (0.06% for NN3) and load instead on term spread and net equity issuance.
+- Economic results: best strategy is an equal-weighted decile spread on NN4 forecasts returning 3.3% per month, 39.0% annualised, out-of-sample Sharpe 2.35, monthly turnover 114.08%, with no costs deducted. Value weighting drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27.</t>
+        </is>
+      </c>
+      <c r="T58" s="30" t="inlineStr">
+        <is>
+          <t>- No transaction costs anywhere, and the turnover figures make that decisive rather than cosmetic (figures above). The authors note high turnover is unsurprising given the dominance of price-trend predictors and then stop. The value-weighted Sharpe collapse is "itself a partial, unacknowledged cost estimate". The top-1,000 reassurance and the equal-weighted headline "both cannot be load-bearing at once."
+- The Monte Carlo summary does not match its own table in the linear case. The text states that for the sparse linear model Lasso and ENet deliver the best and almost identical out-of-sample R^2, and that RF, NN and GBRT tend to overfit so their performance is slightly worse. Table A.1 shows NN1 at 4.42% and NN2 at 4.40% against ENet+H at 4.27% when P_c = 50, and 4.31% and 4.30% against 4.26% when P_c = 100, "so the networks are ahead in both panels. The trees do underperform as described, and the substantive conclusion about the nonlinear process is untouched, but the specific claim that penalized linear methods win when the truth is linear is contradicted by the numbers printed beneath it." That sentence is where the "match the method to the process" reading comes from.
+- Variable importance by zeroing a predictor is not clean attribution when the predictors are this correlated. Six of the top eight characteristics are versions of the same price-trend quantity measured over different windows, and setting one to zero leaves its correlates free to absorb the signal, "which understates each and leaves the group's total importance unallocated. The agreement across models that the paper highlights is therefore partly agreement about the correlation structure of the feature set rather than independent discovery." A second issue is specific to trees, where zeroing a characteristic sends observations to partitions the model never saw during training, "so the measured drop mixes the variable's contribution with an off-distribution evaluation." The placebo test passes but "establishes that irrelevant variables rank low, not that the ranking among relevant and correlated variables is meaningful."
+- Complexity is shown to drift over the test period and the drift is explained rather than tested, and no empirical table carries uncertainty. Figure 3's drift is attributed to a growing cross section and improving data coverage: "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." Models are refit once a year with the five architectures fixed throughout, a concession to compute the authors acknowledge. There are no confidence intervals or seed variation on Tables 1, 2, 5, 7, 8 or 9, only on the 100-repetition simulations. "The 60-year sample compounds this, since a model refit annually from 1957 through 2016 averages over an enormous range of market structures, and the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."
+- Framing limitation conceded by the authors themselves in Section 1.6: improved predictions are only measurements, they do not identify deep associations between prices and conditioning variables, and recovering mechanisms requires the economist to impose structure.</t>
+        </is>
+      </c>
+      <c r="U58" s="30" t="inlineStr">
+        <is>
+          <t>- A ceiling and an expectation band for A_T. Thirty thousand stocks, sixty years, 920 engineered features, eleven method families and a thirty-year test window produce 0.39% monthly R^2_oos at the stock level. Against that, my confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information", so "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result." This sits alongside the 0.54 to 0.58 directional-accuracy band from [[Extending machine learning prediction capabilities by explainable AI in financial time series prediction]] and the 54.3% out-of-sample figure in [[Deep Learning with Long Short-Term Memory Networks for Financial Market Predictions]], "and the three together are now a defensible prior rather than one paper's number."
+- Model sizing: "Size the technical agent at NN1 or NN2 scale and stop treating depth as a dial." Performance peaks at three hidden layers on sixty years of data and declines beyond it, with data scarcity and low signal-to-noise named as the cause; on a dataset smaller by orders of magnitude the implied architecture is one or two hidden layers, or a regularized tree ensemble, "and the depth sweep that would be routine elsewhere is not worth the compute here. The same reasoning applies to feature count, since every method in the paper selected far fewer features than it was offered."
+- Huber loss as a default, not a refinement — it improves out-of-sample performance for every method in the simulation and for four of the methods in the empirical work, "and CSE daily returns are heavier-tailed than US monthly returns, so the case is stronger here than there."
+- The publication-lag discipline as the A_F specification to write down before touching filing data: monthly delayed one month, quarterly four, annual six.
+- The evaluation protocol in full: "Recursive expanding training window, fixed-size rolling validation, annual refit, no cross-validation, modified Diebold-Mariano on cross-sectionally averaged error differences with Newey-West standard errors, and R^2_oos benchmarked against zero with the choice stated." Plus the Campbell-Thompson Sharpe mapping reported alongside the R^2, "cheap and converts a statistical number into the economic one the evaluation actually cares about, with the caveat that it assumes costless timing and will therefore be optimistic on a thin book."
+- Independent large-sample evidence for two of my three state variables (liquidity and risk/volatility), and for the macro rejection.
+- The cost sub-gap's reference case: a 113-114% monthly turnover strategy at Sharpe 2.35 with no cost deducted.</t>
+        </is>
+      </c>
+      <c r="V58" s="30" t="inlineStr">
+        <is>
+          <t>- No costs, no participation-rate analysis, no execution model. The paper reports turnover and stops. That is the whole of Sub-gap 1's motivation stated by a canonical paper without being addressed.
+- No reliability weighting and no absence channel. Conditioning on state happens through fixed, annually-refit interaction coefficients on macro variables; a missing input is median-imputed, never down-weighted, and nothing can go absent.
+- No test of whether the set of features carrying signal is itself regime-dependent — the drift in Figure 3 is explained rather than tested, and the note names this as "the hypothesis my orchestrator rests on and the one this paper was best placed to check."
+- No uncertainty on the empirical tables and no seed variation outside the simulations.
+- No volatility persistence content at all: volatility is a predictor, never a modelled process with a decay structure.
+- Nothing about frontier-market conditions; the paper's own size/liquidity result says its methods work least well there.
+- One open challenge to my macro rejection: aggregate book-to-market, which every model treats as critical and which tops the macro ranking for the networks and the penalized linear models.</t>
+        </is>
+      </c>
+      <c r="W58" s="30" t="inlineStr">
+        <is>
+          <t>[[Empirical Asset Pricing via Machine Learning]]</t>
+        </is>
+      </c>
+      <c r="X58" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: A_T first (expectation band, architecture sizing, loss function, feature count), then the orchestrator's conditioning set (independent large-sample evidence for L_t and V_t, and the Kronecker construction as the single-model analogue of the orchestration claim), then the evaluation layer (benchmark choice, DM test, recursive protocol, Campbell-Thompson mapping), then A_F (horizon and lag discipline, and an argument for a low baseline weight plus explicit abstention), and finally Sub-gap 1, for which this paper is the cleanest reference case in the set.
+EFFECT ON MAIN GAP: It strengthens the premise and sharpens the claim without threatening either. The Kronecker construction is the single-model version of what I am proposing one level up: "Gu et al. make every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator, and the beta-pricing derivation is a principled reason to do it. That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound." That matters because it means the idea that a signal's value varies with market state is not something I have to argue for from scratch — it is derivable from E_t(r_{i,t+1}) = beta'_{i,t} lambda_t with beta_{i,t} = theta_1 c_{i,t} and lambda_t = theta_2 x_t, and it is the standard specification in the most-cited paper in the area.
+Then the line. Three differences separate their construction from mine, and all three are in w(i,t) = f(L_t, V_t, P_t, C_{i,t}): their interaction weights are estimated once per annual refit, so they do not vary with measured market state at decision time, only with the value of the macro variable plugged into a fixed coefficient; they are a function of macro variables rather than of any measured reliability of the signal, so there is no C_{i,t} analogue anywhere in the model; and no channel can go absent, "because a missing characteristic is median-imputed rather than down-weighted". The note puts the whole claim on that last point: "The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line." Median imputation is the exact anti-pattern my abstention channel exists to replace — it substitutes a plausible value for a missing one and the downstream model cannot tell the difference, whereas abstention makes absence visible to the aggregator.
+It also supplies the evidence base for two of the four conditioning terms. Liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) and risk (total volatility, idiosyncratic volatility, beta, beta squared) are two of the three dominant families across every one of eleven method families on a ~30,000-stock, 60-year panel. "That is a far larger evidence base for those two conditioning inputs than the CSE-specific work in [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] or the Granger result at p = 0.0041 from volume to ASPI, and it composes with both." The macro rejection also survives: market-level stock variance is given little weight by any method and essentially none by the networks, consistent with the thin ARDL result in [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]] that already got the macro block rejected. The one live challenge is aggregate book-to-market — critical for every model, 28.57% for NN1 and 43.46% for GLM — and the honest response recorded in the note is to "test it against an ASPI-level valuation ratio rather than dismiss it on the strength of a rejection aimed at different variables."
+One further point that bears directly on the main gap and that the paper declined to test: Figure 3 shows model complexity drifting across the test period — elastic net selecting fewer than five features in the first decade and 20 to 40 after 2000, GBRT moving from roughly 20 features to 30 — and the authors explain it by a growing cross section and improving data coverage. "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." So the paper leaves my central hypothesis open on evidence it had in hand, which is a better position for me than either confirming or refuting it would have been.
+EFFECT ON SUB-GAP 1: This is the strongest available illustration of why cost belongs inside the objective rather than after it, and I would cite it as the reference case. "A strategy turning over 113% of its book monthly, concentrated in price-trend signals, on a universe that deliberately includes the smallest and least liquid names, reported at Sharpe 2.35 with no cost deduction and no participation-rate analysis, is the reference case for my cost sub-gap." Two details make it sharper than a generic "they ignored costs" complaint. First, the value-weighted collapse — NN3 from 2.32 to 1.25, OLS-3 from 0.89 to 0.27 — "is itself a partial, unacknowledged cost estimate and I should cite it that way": moving weight away from the small end halves the Sharpe before a single basis point of spread is charged, which is a lower bound on what liquidity is doing to the result. Second, the internal tension: the paper offers the top-1,000 R^2 of 0.72% against 0.46% on the bottom 1,000 as reassurance that the result is not driven by small-cap illiquidity, while the headline economic result is an equal-weighted spread over the whole board — "both cannot be load-bearing at once."
+Applied to the CSE this is not implementable at any size. "On the CSE, where Dissanayake and Nanayakkara find unexpected illiquidity shocks depressing returns by -0.084 to -0.097 and small caps more than large, that turnover is not implementable at any size, which is the concrete argument for sweeping participation rate against daily volume rather than charging a flat spread, as [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] both do in their different ways." So the paper does not close any part of Sub-gap 1 — it has no friction model at all — but it supplies the clearest demonstration of the failure the sub-gap names, from a source that is hard to dismiss.
+EFFECT ON SUB-GAP 2: Limited, and I should not overclaim it. The paper has no volatility process, no persistence estimate, no decay schedule and no volatility targeting; volatility enters only as a cross-sectional predictor. So it neither closes nor narrows Sub-gap 2. What it contributes is one piece of supporting evidence and one adjacent warning. The evidence: the risk family (total volatility, idiosyncratic volatility, beta, beta squared) is one of the three dominant predictor families across all eleven methods, and the GBRT/NN3 marginal relationship is economically large — a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return — which supports keeping V_t in the conditioning set but says nothing about P_t. The warning is the complexity-drift result again: the paper observed a time-varying structure in its own fitted models and explained it away rather than testing it, which is the same category of move as assuming a fixed exponential decay rate and never checking.
+CSE DATA EVIDENCE: None in the paper — US only. The CSE content in this cell is my own transfer accounting. My confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information" than 30,000 stocks over 60 years with 920 features. The direct consequence is a leakage tripwire: "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result", which composes with the 0.54-0.58 directional-accuracy band and the 54.3% out-of-sample figure from the two other notes into "a defensible prior rather than one paper's number". The second consequence is the architecture ceiling: if three hidden layers is already past the optimum on sixty years of US monthly data, one or two layers or a regularized tree ensemble is the ceiling on 374 trading days. The third is that the benchmark choice has to be stated every time, because "the three-percentage-point inflation from benchmarking against the historical mean is larger than any effect I am likely to measure, so a CSE result reported without naming its benchmark is uninterpretable." And the fourth is the frontier-market reading of their own size result: machine learning works least well in the conditions the CSE presents continuously.
+PROPOSED REVISION STATED IN THE NOTE:
+1. Reset the expectation band for A_T to a few tenths of a percent of monthly stock-level R^2 and treat anything materially above it as a leakage signal rather than a result.
+2. Size A_T at NN1 or NN2 scale (one or two hidden layers) or a regularized tree ensemble; drop the depth sweep; keep the feature count small, since every method in the paper selected far fewer features than it was offered.
+3. Adopt the Huber objective as a default across the technical agent, not as a refinement.
+4. Write down the publication-lag structure for A_F before touching any filing data — monthly delayed one month, quarterly four, annual six — because "CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."
+5. Copy the evaluation protocol in full: recursive expanding training window, fixed-size rolling validation, annual refit, no cross-validation, modified Diebold-Mariano on cross-sectionally averaged error differences with Newey-West standard errors, R^2_oos benchmarked against zero with the choice named explicitly every time, and the Campbell-Thompson mapping SR* = sqrt((SR^2 + R^2)/(1 - R^2)) reported alongside — with its costless-timing caveat flagged on a thin book.
+6. Give A_F a low baseline weight with an explicit abstention path rather than a weight that happens to fall to zero: "the fundamental agent is not a timing input and should not be asked for one, it is a slow-moving tilt whose natural horizon is quarters, and an orchestrator that weights it on a daily decision will be weighting noise most of the time", combined with the working assumption that the channel is unusable more than half the time on the CSE.
+7. Test aggregate book-to-market against an ASPI-level valuation ratio rather than dismissing it under the existing macro rejection.
+8. Sweep participation rate against daily volume rather than charging a flat spread, and cite the value-weighted Sharpe collapse (2.32 to 1.25 for NN3, 0.89 to 0.27 for OLS-3) as a partial, unacknowledged cost estimate when making the case.
+9. Draw the orchestration line at median imputation versus down-weighting, and use this paper as the place to draw it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="409.6" customHeight="1">
+      <c r="A59" s="29" t="inlineStr">
+        <is>
+          <t>P58</t>
+        </is>
+      </c>
+      <c r="B59" s="30" t="inlineStr">
+        <is>
+          <t>Jayarangi, W.C. and Buddhika, H.J.R. (2025). The Impact of Firm-Specific Factors on Share Prices of Diversified Financial Companies: Evidence from the Colombo Stock Exchange. South Asian Journal of Finance, Vol. 5 No. 1, pp. 67–83. DOI 10.4038/sajf.v5i1.113. Both authors are at the Department of Finance, Faculty of Commerce and Management Studies, University of Kelaniya. Received November 2024, accepted June 2025. Citekey jayarangiImpactFirmSpecificFactors2025.</t>
+        </is>
+      </c>
+      <c r="C59" s="30" t="inlineStr">
+        <is>
+          <t>2025.</t>
+        </is>
+      </c>
+      <c r="D59" s="30" t="inlineStr">
+        <is>
+          <t>South Asian Journal of Finance, Vol. 5 No. 1, pp. 67–83.</t>
+        </is>
+      </c>
+      <c r="E59" s="30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4038/sajf.v5i1.113 (accessed 4 October 2026). Zotero: zotero://select/library/items/4Y76RTSM.</t>
+        </is>
+      </c>
+      <c r="F59" s="30" t="inlineStr">
+        <is>
+          <t>Fundamentals. Firm-specific determinants of share price; local CSE empirical econometrics. The note's frontmatter records stream: fundamentals, market: CSE, status: reviewed.</t>
+        </is>
+      </c>
+      <c r="G59" s="30" t="inlineStr">
+        <is>
+          <t>The paper asks "whether five firm-specific accounting ratios, return on equity, dividend per share, earnings per share, the price to earnings ratio and debt to total assets, explain the share prices of Diversified Financial companies listed on the Colombo Stock Exchange". The gap it claims is threefold in my note. First, "the firm-specific determinants literature is developed-market and the Sri Lankan slice of it is thin and dated" — the authors anchor on Kumar (2017) for Indian autos, Nasif and Sharif (2010) for Amman commercial banks, Iqbal et al. (2016) for Kenyan energy and Sharif et al. (2014) for Bahrain, and cite Dissanayake and Herath (2016) and Pandigamage and Ranaweera (2023) as "near enough the whole local set". Second, and this is what I recorded as "their sharpest framing point", the only prior study of firm-specific factors on CSE diversified financials is a 2016 Central Bank staff study reporting percentage increments only, and "its results may no longer hold after the political and economic changes from 2020". I added my own qualification there: "I'd put this more strongly than they do, since their own sample runs straight through the same break and is estimated as one pooled regime." Third, the sector choice is a sampling rationale rather than a hypothesis — "Diversified Financials is picked for growth, not for theory", justified by earnings growing 43% and revenues 31% annually over 2021 to 2023 and the sector being roughly 20% of total market capitalisation per the Central Bank's 2023 industry analysis, which "means the sector was selected on the outcome variable's recent behaviour".</t>
+        </is>
+      </c>
+      <c r="H59" s="30" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange, Diversified Financials sector only. Twenty companies, "selected as the highest market capitalisation 20 of the 43 Diversified Financial firms listed on the CSE, LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b".</t>
+        </is>
+      </c>
+      <c r="I59" s="30" t="inlineStr">
+        <is>
+          <t>200 firm-year observations, 2013 to 2023 (eleven years), 20 firms, random effects panel estimated in STATA. Data is hand-collected from the CSE website and from company annual reports. I flagged the arithmetic directly: "Eleven years across twenty firms is 220 firm-years and every table reports 200, which is not explained anywhere in the paper."</t>
+        </is>
+      </c>
+      <c r="J59" s="30" t="inlineStr">
+        <is>
+          <t>Annual accounting data from filings plus monthly-averaged price. Dependent variable: share price measured as the average share price of the month, in nominal rupees, undifferenced and untransformed. Regressors: return on equity (net income over average shareholders' equity), dividend per share (annual dividend over the weighted average share count), earnings per share (net profit over the same denominator), price to earnings (market value per share over earnings per share), debt to total assets (total liabilities over total assets). Sole control: firm size as the natural logarithm of total assets — "the only variable entering in logs". The operationalisation table sources each measure to prior local work: Biyiri and Dissanayaka (2017), Irsath et al. (2015), Sritharan (2018) and Rajapaksha and Weerawickrama (2020).
+Descriptives (these are the distributional facts I care about): share price mean 262.078, standard deviation 458.181, range Rs. 0.50 to Rs. 1,950 — "the dependent variable is in nominal rupee levels and is dominated by a handful of high-priced counters". Price to earnings is worse: "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82", which I read as "what happens when a ratio with earnings in the denominator is computed on firm-years where earnings are near zero or negative, and the EPS minimum of −21.65 confirms loss-making years are in the sample". Neither variable is winsorised, trimmed or transformed. EPS mean 17.239, standard deviation 53.818; DPS mean 4.66; ROE mean 14.237%; DTA mean 57.277%; log total assets 20.041.
+Correlations with price: DPS 0.535, EPS 0.509, PE 0.319, DTA −0.502, firm size −0.404, ROE −0.160. Among regressors: "dividend per share and earnings per share correlate at 0.757 and debt to assets correlates with firm size at 0.726", which I noted is "the structure that decides how the insignificant coefficients below should be read". Mean VIF 2.23, maximum 2.81, "and the paper treats that as settling the question".</t>
+        </is>
+      </c>
+      <c r="K59" s="30" t="inlineStr">
+        <is>
+          <t>One pooled panel specification, random effects after a Hausman test, share price in levels as the dependent variable:
+SP_it = β0 + β1 ROE_it + β2 DPS_it + β3 EPS_it + β4 PE_it + β5 DTA_it + β6 log(SIZE_it) + ε_it
+with SP_it the average monthly share price of firm i in year t in nominal rupees, PE_it the price to earnings ratio, DTA_it total liabilities over total assets, log(SIZE_it) the natural log of total assets. "There are no year effects, no industry effects and no lagged dependent variable, and no standard error clustering is reported."
+The endogeneity-by-construction problem, which I set out as its own equation because it is the thing I take forward:
+PE_it = SP_it / EPS_it  ⟹  SP_it = β0 + … + β4 (SP_it / EPS_it) + … + ε_it
+My reading: "This is not an omitted control or a specification preference, it is an accounting identity relating two of the variables in the regression, and nothing in the paper acknowledges it. Whatever β4 is estimating, it is not the independent contribution of a valuation multiple to price."
+The within/between decomposition, which is the single most useful piece of the paper for me:
+R²_within = corr²(ŷ_it − ȳ̂_i, y_it − ȳ_i),   R²_between = corr²(ȳ̂_i, ȳ_i)
+"A model that separates expensive firms from cheap ones but says nothing about a given firm's path through time produces exactly the pattern reported here, high between and near-zero within."
+Output: in-sample coefficients and significance only. No forecast, no holdout, no agent.</t>
+        </is>
+      </c>
+      <c r="L59" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — this is a single-equation panel econometrics paper with no agents, no orchestration and no decision layer. As I put it in the note, "there is no forecast, no holdout and no agent anywhere in it, and I'm reading it the same way I read the other local empirical work, as evidence about what the fundamental channel on this market can and cannot carry." What it supplies instead is (a) a measured, published feature set for A_F on this exact market and sector, (b) the within-vs-between split that tells me what role A_F should play in the weighting function, and (c) a weak but real published baseline for the fundamental channel.</t>
+        </is>
+      </c>
+      <c r="M59" s="30" t="inlineStr">
+        <is>
+          <t>Not recorded in the note. (The paper is an accounting-ratio panel regression; no sentiment variable appears anywhere in my note.)</t>
+        </is>
+      </c>
+      <c r="N59" s="30" t="inlineStr">
+        <is>
+          <t>This is the paper's entire content and it is the row that matters most for A_F. The fundamental variables with measured CSE association are earnings per share (coefficient 1.887, standard error 0.501, t = 3.76, p = 0.000) and debt to total assets (−0.530, standard error 0.167, p = 0.002); firm size enters at −1.136 and is insignificant at p = 0.262; return on equity (−0.142, p = 0.575) and dividend per share (2.102, p = 0.248) do not clear. My own summary: "Earnings per share, leverage and firm size are the fundamental features with measured CSE association, and this is my citation for selecting them, scoped to cross-section… both are extractable from the income statement and balance sheet of any annual report. That is enough to justify the fundamental agent's feature set to a supervisor without my having to derive it from first principles, provided I say in the same sentence what the evidence is cross-sectional about."
+On update frequency and extraction cost, the note is explicit: all data is "hand-collected from the CSE website and from company annual reports", and "Twenty firms over eleven years, hand-collected from annual reports, is another data point on what fundamental extraction costs on this market. Two authors with institutional access pulled six variables for 200 firm-years by hand, which is the same message the Fernando note delivers from 167 firms, and it is why the retrieval pipeline over CSE filings is the component I expect to be the bottleneck rather than any model." I link that to structure-aware chunking of the kind in [[Financial Report Chunking for Effective Retrieval Augmented Generation]], which "reduces that cost without removing it".
+On feature construction for the RAG side, the price-to-earnings identity is a direct constraint I recorded: "Any ratio with price in the numerator fed into a model whose target is price or return carries a mechanical link to the label, and on a thin market where the denominator goes near zero it also carries a variance of the kind that produced a standard deviation of 1069.92 here. The fundamental agent's inputs should be restricted to quantities computed from the filings alone, with price-derived multiples either excluded or constructed against a lagged price and reported as such."</t>
+        </is>
+      </c>
+      <c r="O59" s="30" t="inlineStr">
+        <is>
+          <t>No volatility modelling of any kind — there is no variance model, no GARCH, no risk measure in the specification. The only risk content is interpretive: the authors read the negative debt-to-assets coefficient "as investors discounting financial risk". The regime instability content is relevant to V_t and P_t indirectly: the window "contains the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation peaking above 50%, and the dependent variable is an unadjusted nominal price with no year effects, no inflation adjustment and no regime split."</t>
+        </is>
+      </c>
+      <c r="P59" s="30" t="inlineStr">
+        <is>
+          <t>Not recorded in the note — there is no liquidity variable, no turnover screen, no trading-frequency filter and no transaction cost anywhere in this paper. The closest adjacent fact is the sample construction: the 20 largest of 43 sector firms by terminal market capitalisation, LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b, which is implicitly a size-and-prominence selection and is why the survivorship point below matters.</t>
+        </is>
+      </c>
+      <c r="Q59" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable in the ML sense. The model is a linear panel regression, so coefficients are the explanation by construction. I would note that the interpretability is undermined by the paper's own misreading of its coefficients: "it describes this as the effect of a 1% increase, but nothing except firm size is in logs, so the coefficient is the effect of one more rupee of EPS, which is Rs. 1.887 of price."</t>
+        </is>
+      </c>
+      <c r="R59" s="30" t="inlineStr">
+        <is>
+          <t>In-sample fit only. Overall R² 0.576, chi-square 64.394, Prob &gt; chi2 = 0.000, reported by the text as "the R square value lies at 58%" and "the overall model is significant". The same model summary table reports R² within of 0.090 and R² between of 0.709. There is "no train and test split, no holdout year, no rolling estimation and no forecast error reported anywhere". Comparison is to prior literature by sign agreement only: EPS "is consistent with Sharif et al. (2015), Su (2002) and Zhu (2003)", and the ROE null is placed "alongside Badruzaman (2020) and Zaman (2021) who also find negative or negligible ROE effects on price".</t>
+        </is>
+      </c>
+      <c r="S59" s="30" t="inlineStr">
+        <is>
+          <t>1. EPS is the strongest and most robust result: 1.887, standard error 0.501, t = 3.76, p = 0.000. "It is the only regressor whose univariate correlation with price (0.509), significance and sign all point the same way." But the magnitude is odd: "That is an implied marginal multiple of 1.887 against a sample where mean price over mean EPS is about 15.2", so "the levels regression is attributing almost all of the cross-sectional price level to something other than earnings, and reading the coefficient as a valuation multiple would understate the market's actual pricing by an order of magnitude."
+2. Debt to total assets is negative and significant at −0.530, standard error 0.167, p = 0.002 — one percentage point more leverage associates with Rs. 0.53 less price. Hedge carried through: DTA correlates 0.726 with firm size, firm size enters at −1.136 and is insignificant at p = 0.262, and both have sizeable negative univariate correlations with price (−0.502 and −0.404), so "the leverage coefficient and the size coefficient are competing to explain the same cross-sectional variation and the design has no way to separate them."
+3. Price to earnings is positive and significant at 0.673, p = 0.022, and "it is the one I would not cite" — given the identity and a regressor standard deviation of 1069.92, "I read this as a mechanical artefact rather than evidence about valuation multiples, and the fact that it reaches significance while dividend per share does not is a feature of the arithmetic rather than of the market."
+4. ROE (−0.142, p = 0.575) and DPS (2.102, p = 0.248) both fail; H1 and H2 are rejected "after a literature review spending four subsections on bird-in-hand, residual dividend policy, agency cost theory and dividend irrelevance". Important hedge: DPS has the highest univariate correlation with price in the whole matrix at 0.535 and correlates 0.757 with EPS, so "what the regression shows is that dividends add nothing beyond earnings in this specification, not that dividends are unrelated to price. The conclusion states the second."
+5. The fit split is the headline for me: "Nine percent of the year-to-year movement in a given company's share price is explained, against seventy-one percent of the differences between companies", so "the model is a cross-sectional pricing description that has very little to say about time."</t>
+        </is>
+      </c>
+      <c r="T59" s="30" t="inlineStr">
+        <is>
+          <t>I recorded a standing warning on this paper: two of its own diagnostic tables contradict the text that reports them. "The normality section states that the Skewness/Kurtosis p-values are above 0.05 when the table it points at shows 0.000 in every cell, and the Hausman test is reported with a chi-square statistic of −1489.934, which is not a value the statistic can take. The random effects choice that produces every coefficient below rests on that second one."
+- Normality: the text claims all six variables are normally distributed "because the p-values for the Skewness and Kurtosis tests are greater than 0.05", while Table 4 reports 0.000 for skewness and kurtosis on every variable and adjusted chi-square p-values of 0.000 or 0.001 throughout, which rejects normality for all of them. The same paragraph then says the chi-square p-values being below 0.05 confirms the assumption is met, so the two sentences contradict each other as well as the table. A dependent variable ranging from Rs. 0.50 to Rs. 1,950 with a standard deviation 1.75 times its mean "is visibly non-normal, and no transform is applied in response."
+- Hausman: "A chi-square test value of −1489.934 with a p-value of 1 is the standard symptom of the asymptotic assumptions failing, and STATA's own guidance is to re-run under a common variance assumption or use an overidentification test rather than to read the p-value. The paper reads the p-value, concludes random effects, and reports every coefficient from that estimator." Random effects also requires firm effects uncorrelated with the regressors, "which is hard to believe when two of the regressors are leverage and firm size".
+- Survivorship and look-ahead: "Selecting on terminal market capitalisation and then estimating on 2013 onwards keeps every firm that grew into the top twenty and drops every firm that fell out of it or delisted, which is survivorship combined with look-ahead selection." The missing 20 firm-years out of the expected 220 are never accounted for, and "the model summary's mean dependent variable of 83.107 with a standard deviation of 63.883 cannot be reconciled with the share price mean of 262.078 and standard deviation of 458.181 in the descriptives, so the two tables appear to come from different runs or different transformations of the dependent variable."
+- Regime pooling: "Eleven years of nominal rupee prices are pooled as one regime across a currency collapse." A rupee of EPS in 2014 and in 2023 "are not the same quantity, so part of what the coefficients are fitting is the unit of measurement changing underneath the panel." The paper frames this as an omitted-macro-variable issue "when the sharper problem is comparability of the dependent variable across the sample."
+- No out-of-sample evaluation despite forecasting claims: the abstract says the factors "can be used to make accurate future share price estimates" and the recommendations tell investors to monitor these ratios to "facilitate accurate forecasts of future share prices", while "an in-sample R² of 0.576 on a cross-section, with a within R² of 0.090, supports neither sentence." I noted this is "the gap I actually care about rather than a complaint about this paper specifically, since it is the standard shape of the local empirical literature."
+- Write-up slips: variable definitions render DPS as "Dep_osit" and EPS as "Esp_rit", every marginal effect is described as the response to a 1% change when only firm size is logged, the conclusion mentions a panel unit root test finding "at least one panel had a unit root" that appears nowhere in the results, and Table 10 duplicates the p-values already in Table 9. "None of these change a coefficient, and together they mean I should treat the figures as needing verification rather than as a clean reference."</t>
+        </is>
+      </c>
+      <c r="U59" s="30" t="inlineStr">
+        <is>
+          <t>- A measured, citable feature set for A_F on CSE: EPS and debt-to-assets as the two that clear at p = 0.000 and p = 0.002, with firm size as a control, all extractable from income statement and balance sheet alone — scoped explicitly to the cross-section.
+- The within R² of 0.090 against between R² of 0.709 as the number that fixes A_F's architectural role: "Fundamentals on this market separate counters from each other far better than they explain any one counter's path, so the fundamental channel should produce a slowly-updating relative view across the universe rather than a timing signal, with the technical channel carrying the short horizon and the orchestrator capping how much the fundamental weight is allowed to move between reporting dates."
+- A hard constraint on feature construction: exclude price-derived multiples from A_F, or build them against a lagged price and say so.
+- Point-in-time universe construction as a non-negotiable, with this paper as the worked counter-example.
+- A published, weak, in-sample baseline for the fundamental channel on CSE diversified financials to beat out of sample.</t>
+        </is>
+      </c>
+      <c r="V59" s="30" t="inlineStr">
+        <is>
+          <t>- No out-of-sample evaluation at all. "A linear six-variable model on CSE diversified financials with an in-sample overall R² of 0.576 and a within R² of 0.090 is a reference point my fundamental agent should beat out of sample, and since the paper reports no out-of-sample result at all, establishing one on a comparable universe is a contribution I can state plainly in the proposal rather than having to argue for."
+- No time-varying or state-conditional structure: one pooled regime over 2013–2023 with no year effects, no regime split and no inflation adjustment, across a window containing the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation above 50%. Nothing in the design lets the fundamental relationship's strength vary with market state, which is exactly what w(i,t) = f(L_t, V_t, P_t, C_i,t) is for.
+- No abstention channel: the specification forces a fitted value for every firm-year. "A fundamental agent that must emit a directional view on every counter at every step will manufacture signal out of exactly these variables" (ROE and DPS, which fail to clear). "Letting the channel return no view when its inputs are collinear or missing is the design consequence."
+- No liquidity or friction content whatsoever, so nothing here constrains SUB-GAP 1 directly; it leaves that side open.
+- No volatility persistence content, so nothing here constrains SUB-GAP 2 directly.</t>
+        </is>
+      </c>
+      <c r="W59" s="30" t="inlineStr">
+        <is>
+          <t>[[The Impact of Firm-Specific Factors on Share Prices of Diversified Financial Companies, Evidence from the Colombo Stock Exchange]]</t>
+        </is>
+      </c>
+      <c r="X59" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: A_F (the fundamental agent) — feature selection, update frequency and architectural role; the abstention channel; universe construction and point-in-time screening; and the local-evidence justification for using the CSE. It is the most recent published statement I have of which accounting ratios associate with price on CSE financials, over a window that overlaps mine almost exactly.
+EFFECT ON MAIN GAP: Strongly supportive, and in a very specific way. The within/between split — 0.090 within against 0.709 between — is a direct, locally measured statement that the fundamental channel's reliability is horizon-dependent on this market: it prices counters against each other well and says almost nothing about when a given counter moves. That is precisely the kind of structural property the weighting function w(i,t) = f(L_t, V_t, P_t, C_i,t) is meant to exploit, and it gives me a published, CSE-specific number for why the fundamental agent's weight should be capped and slow-moving between reporting dates rather than allowed to drive entry and exit. It also supports the C_i,t component being a structural property of the output rather than a self-report: ROE and DPS fail to clear not because they are irrelevant but because they are collinear with EPS (DPS–EPS at 0.757), so a channel whose inputs are collinear or missing should be detectable from the structure of its inputs and allowed to abstain. "Letting the channel return no view when its inputs are collinear or missing is the design consequence, and it is the same abstention argument the liquidity screen produces for the technical channel." Finally, the paper's pooling of eleven years containing a currency collapse as one regime is my clearest local illustration of what a fixed, non-state-conditional combination rule costs: "This is now the third CSE result pointing the same way, alongside the macro linkages breaking over 2014 to 2022 in [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] and the 2021 extension halving the investment-risk coefficient in the Fernando note."
+EFFECT ON SUB-GAP 1: Indirect and mostly cautionary. The paper has no liquidity variable, no turnover screen and no execution cost, so it offers no positive evidence on state-dependent execution friction. What it does supply is the mechanism by which thin trading corrupts a price-derived fundamental input: "on a thin market where the denominator goes near zero it also carries a variance of the kind that produced a standard deviation of 1069.92 here." That is the PE ratio blowing up to a range of −1471.22 to 2292.82 because earnings pass through zero, and it is a concrete local instance of the broader claim in SUB-GAP 1 that market conditions condition the reliability of price-derived quantities. It also gives me a worked example of a universe screen done wrong — top-20 by terminal capitalisation backfilled to 2013 — which is "the exact failure my own screen could reproduce if the liquidity filter is computed once over the full history rather than as of each rebalance date."
+EFFECT ON SUB-GAP 2: Indirect. There is no volatility persistence content in this paper — no variance model, no long-memory estimate. The only contribution is negative evidence about regime stability: eleven years pooled across the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation above 50%, with no year effects and no regime split, producing coefficients that partly fit a changing unit of measurement. That is an argument for conditioning on measured state, but it does not operationalise persistence, which remains mine to do.
+CSE DATA EVIDENCE: This is the richest part of the row for the justification rewrite, and it is all local and measured.
+- Universe depth and concentration: the Diversified Financials sector has 43 listed firms, of which the study could only work with the top 20 by capitalisation, spanning LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b — a roughly 60-fold spread in capitalisation inside a single sector of a single market. That is firm heterogeneity on this market stated in rupees.
+- Price-level heterogeneity: share price mean 262.078 against a standard deviation of 458.181, range Rs. 0.50 to Rs. 1,950, with the dependent variable "dominated by a handful of high-priced counters". A standard deviation 1.75 times the mean inside one sector is a quantified statement of cross-sectional dispersion.
+- Earnings heterogeneity and loss-making counters: EPS mean 17.239 with a standard deviation of 53.818 and a minimum of −21.65 — loss-making firm-years are present in the sample. This is why the PE ratio has "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82". That dispersion is the direct, local, empirical reason a price-derived multiple is not a safe input on this market.
+- Leverage: debt to total assets averages 57.277% across the sector, and one percentage point more leverage associates with Rs. 0.53 less price (p = 0.002).
+- Which fundamentals transmit to price here: EPS at 1.887 (p = 0.000) and leverage at −0.530 (p = 0.002) clear; ROE (p = 0.575) and DPS (p = 0.248) do not, with DPS's failure attributable to its 0.757 correlation with EPS rather than to irrelevance. Firm size enters negatively at −1.136 but is insignificant (p = 0.262), and its 0.726 correlation with leverage means the design cannot separate the two.
+- Transmission is cross-sectional, not temporal: R² within 0.090 against R² between 0.709. Fundamentals explain roughly nine percent of a given CSE counter's year-to-year price movement and roughly seventy-one percent of the differences between counters.
+- Fundamental data cost and update frequency: six variables for 200 firm-years were hand-collected from the CSE website and company annual reports by two authors with institutional access. Fundamentals on this market update at annual reporting frequency and are extracted from PDF filings by hand in the published literature — "it is why the retrieval pipeline over CSE filings is the component I expect to be the bottleneck rather than any model."
+- Regime instability in local fundamentals: "The window contains the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation peaking above 50%." The authors themselves argue that pre-2020 results "may no longer hold after the political and economic changes from 2020". This is local evidence that CSE relationships are not stationary across my own index track of 1 July 2014 to 30 June 2024.
+- Methodological fragility of the local literature as a whole: a 2025 journal paper in this space carries a Hausman statistic of −1489.934, a normality section contradicting its own table, two tables whose dependent-variable moments cannot be reconciled (mean 83.107 / sd 63.883 against mean 262.078 / sd 458.181), and forecasting recommendations with no holdout anywhere. I recorded explicitly that the absent out-of-sample evaluation "is the standard shape of the local empirical literature". I have not found that evaluation in the literature I have covered.
+PROPOSED REVISION STATED IN THE NOTE: The note states several design revisions driven by this paper. (1) A_F is to produce "a slowly-updating relative view across the universe rather than a timing signal", with the technical channel carrying the short horizon and "the orchestrator capping how much the fundamental weight is allowed to move between reporting dates". (2) A_F's inputs are "restricted to quantities computed from the filings alone, with price-derived multiples either excluded or constructed against a lagged price and reported as such". (3) The liquidity screen and universe construction must be computed "as of each rebalance date" and not once over the full history; the note records that "Taken with the delisting control in [[Relationship between firm-level investment, idiosyncratic risk and ownership, an emerging market perspective]], which does retain delisted firms, I now have both the right and the wrong version of this decision documented on the same market." (4) Targets should be returns and features should be deflated or expressed as ratios, "not merely to add controls", because of the nominal-price problem across 2020 to 2023. (5) A_F gets an abstention output rather than being forced to emit a directional view on every counter at every step. (6) The paper is adopted as "a usable published baseline for the fundamental channel, and a weak one, which is what makes it useful" — an in-sample overall R² of 0.576 and within R² of 0.090 to be beaten out of sample on a comparable universe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="409.6" customHeight="1">
+      <c r="A60" s="29" t="inlineStr">
+        <is>
+          <t>P59</t>
+        </is>
+      </c>
+      <c r="B60" s="30" t="inlineStr">
+        <is>
+          <t>Fernando, A.D., Nimal, P.D. and Abeysekera, A. (2026). Relationship between firm-level investment, idiosyncratic risk and ownership: an emerging market perspective. Managerial Finance, Vol. 52 No. 3, pp. 517–539. DOI 10.1108/MF-10-2024-0791. Affiliations: Abehitha Dinethri Fernando (University of Oklahoma), Pulukkuttige Don Nimal (University of Sri Jayewardenepura), Amal Abeysekera (Hofstra). Received October 2024, accepted June 2025. Citekey fernandoRelationshipFirmlevelInvestment2026.</t>
+        </is>
+      </c>
+      <c r="C60" s="30" t="inlineStr">
+        <is>
+          <t>2026.</t>
+        </is>
+      </c>
+      <c r="D60" s="30" t="inlineStr">
+        <is>
+          <t>Managerial Finance, Vol. 52 No. 3, pp. 517–539.</t>
+        </is>
+      </c>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/MF-10-2024-0791. Zotero: zotero://select/library/items/K3N7LZ4S.</t>
+        </is>
+      </c>
+      <c r="F60" s="30" t="inlineStr">
+        <is>
+          <t>Market structure. Corporate finance / firm-level investment under idiosyncratic risk, with ownership moderation; local CSE empirical econometrics. The note's frontmatter records stream: market-structure, market: CSE, status: reviewed.</t>
+        </is>
+      </c>
+      <c r="G60" s="30" t="inlineStr">
+        <is>
+          <t>The paper asks "whether firms listed on the Colombo Stock Exchange cut capital investment when their idiosyncratic risk rises, and whether insider and institutional ownership moderate that sensitivity". The gap it addresses, as I recorded it: (1) "The investment-risk sensitivity literature is almost entirely developed-market" — Panousi and Papanikolaou (2012) in the Journal of Finance is the anchor (risk-averse managers underinvest when firm-specific risk rises), with follow-on work (Glover and Levine, 2017; Liu and Wang, 2021; Florackis et al., 2019) staying in US and UK data; "The authors' claim is not that the mechanism is absent elsewhere, it's that the sign of the ownership moderation has no reason to carry over, because the agency environment that produces it is different." (2) "The alignment against entrenchment question is genuinely open in emerging markets" — higher insider ownership can tie managerial wealth to firm growth and push toward long-horizon investment (alignment, Ang et al., 2000) or concentrate undiversified personal wealth and raise risk aversion (entrenchment, Fahlenbrach and Stulz, 2009); the paper argues weaker legal protection and weaker formal governance in emerging markets (La Porta et al., 1998; Khanna and Palepu, 2002) raise the marginal value of insider ownership as a substitute governance mechanism, tilting toward alignment. "That is a testable framing and it is the paper's actual contribution." (3) The authors claim coverage of this relationship in South Asia, "which I can't independently verify but which is consistent with what I found when I went looking for CSE firm-level risk studies."</t>
+        </is>
+      </c>
+      <c r="H60" s="30" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange, non-financial listed firms. The sample excludes financials and heavily state-regulated sectors (utilities, energy, telecoms), firm-years with missing key variables, and negative book values.</t>
+        </is>
+      </c>
+      <c r="I60" s="30" t="inlineStr">
+        <is>
+          <t>1,226 firm-year observations covering 167 unique CSE firms from 2010 to 2018, with firm and year fixed effects and standard errors clustered at the firm level. "Both listed and delisted firms are retained, which is a deliberate survivorship-bias control and more than most of the local literature does." Ownership data is only available from 2011, and the sub-samples are much smaller: "the insider ownership sub-sample is 59 firms and the institutional sub-sample 54 firms", which produces the 297 and 278 observation counts in the moderation tables; after propensity score matching, "64 and 76 observations respectively". A robustness extension runs the sample three years further to 2021.</t>
+        </is>
+      </c>
+      <c r="J60" s="30" t="inlineStr">
+        <is>
+          <t>Annual accounting data plus weekly price series. "All accounting and insider ownership data is hand-collected from annual reports published by the CSE", prices and the index come from the CSE data libraries, and Treasury bill rates from the Central Bank of Sri Lanka.
+Idiosyncratic risk is built as the residual standard deviation from a Fama–French three-factor regression on weekly excess returns over 52 trading weeks:
+r_{i,t} − r_{f,t} = α_i + β_i^MKT MKT_t + β_i^SMB SMB_t + β_i^HML HML_t + ε_{i,t},   σ_i^idi = sd(ε̂_{i,t})_{t=1..52}
+where r_{i,t} is the weekly return adjusted for cash dividends, stock splits, scrip dividends, bonus issues and rights issues; the market proxy is "the percentage change in the All Share Total Return Index (ASTRI), not the ASPI, which is the right choice since it is total return rather than price only"; r_{f,t} is a weekly rate derived from the yield on 91-day Treasury bills; and "weekly returns exceeding +50% or falling below −50% are dropped as outliers, following Abeysekera and Nimal (2017)".
+Systematic risk is backed out of the decomposition rather than estimated separately: σ^sys = sqrt(σ^tot² − σ^idi²), with total risk the standard deviation of weekly returns.
+Ownership: insider ownership is the share of total outstanding shares held by executive directors on the board at year end; institutional ownership is the share held by pension funds, investment banks, mutual funds and companies holding more than 3% (both following Farwis and Azeez, 2019). Controls are cash flow over lagged PPE, firm size as the firm's PPE relative to total sample PPE that year, and leverage as total debt over total assets.
+Descriptives I keep returning to: mean idiosyncratic risk "0.221 with a standard deviation of only 0.050 and a full range of 0.117 to 0.315"; "insider and institutional ownership correlate at −0.703"; mean insider ownership 5.7% against mean institutional ownership 66.1%, "so this is a market of institutionally held firms with thin executive stakes". Sample mean investment rate is 11.60%, with a minimum in Table 2 of −0.082.</t>
+        </is>
+      </c>
+      <c r="K60" s="30" t="inlineStr">
+        <is>
+          <t>Three nested fixed-effect panel specifications, investment rate as dependent variable, firm-clustered standard errors.
+Model 1 (baseline):
+(I_{i,t}/K_{i,t−1}) = β0 + β1 log(σ^idi_{i,t−1}) + β2 log(σ^sys_{i,t−1}) + β3 (CF_t/K_{t−1})_{i,t−1} + β4 log(K̂_{i,t−1}) + β5 log(D_{i,t−1}/A_{i,t−1}) + η_i + g_t + ν_{i,t}
+where I_{i,t} is the change in net PPE in year t and K_{i,t−1} is lagged net PPE "so the dependent variable is an investment rate rather than a level"; η_i and g_t are firm and year fixed effects; "risk, size and leverage all enter in logs, following Panousi and Papanikolaou (2012)"; β1 is the coefficient of interest.
+Model 2 (the design I find most transferable): "rather than interacting risk with continuous ownership it sorts firms each year into two equally sized groups on the previous year's insider ownership relative to the annual median, and interacts risk with each group dummy, omitting the intercept to avoid the dummy trap":
+(I_{i,t}/K_{i,t−1}) = β1 log(σ^idi_{i,t−1}) × INSD_L + β2 log(σ^idi_{i,t−1}) × INSD_H + β3 log(σ^sys_{i,t−1}) + controls + INSD_L + INSD_H + η_i + g_t + ν_{i,t}
+Model 3 extends to a 2×2 grid, sorting first on institutional ownership then on insider ownership within each institutional group, yielding four interaction terms, to ask whether institutional monitoring substitutes for insider alignment. My note on the design choice: "splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it is close to the structure I'd want for ablating state inputs one at a time."
+Output: in-sample panel coefficients. "There are no agents, no forecasts and no out-of-sample period anywhere in it."</t>
+        </is>
+      </c>
+      <c r="L60" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable — this is a corporate finance panel econometrics paper with no agents, no orchestration, no decision layer and no forecast. As I put it: "Nothing in this paper is a methodological template for what I'm building… so I'm reading it as market-structure evidence rather than as a design precedent." What it supplies instead is (a) three conceded facts about CSE data depth that constrain the technical, volatility and fundamental channels respectively, (b) a reusable idiosyncratic risk estimator for A_V's cross-sectional input, and (c) a conditioning design — annual median splits with group-specific slopes — that is "close to the structure I'd want for ablating state inputs one at a time", i.e. a template for ablating L_t, V_t, P_t and C_i,t individually in the orchestrator.</t>
+        </is>
+      </c>
+      <c r="M60" s="30" t="inlineStr">
+        <is>
+          <t>Not recorded in the note. (No sentiment variable appears anywhere in this paper.)</t>
+        </is>
+      </c>
+      <c r="N60" s="30" t="inlineStr">
+        <is>
+          <t>Substantial, and it is where my A_F extraction-cost argument gets its strongest local evidence. All accounting and insider ownership data is hand-collected from annual reports published by the CSE. My note: "167 firms with usable accounting data and 59 with usable ownership data, all of it hand-collected from annual report PDFs, is the data-depth constraint arriving from a direction I hadn't checked. My liquidity screen question has been how many counters trade often enough to model, and this adds a second filter underneath it, how many have fundamentals complete enough to extract, with the answer coming from three authors who had institutional access, every incentive to keep the sample large, and who still spent the effort to pull accounting figures, insider stakes, board composition, CEO duality and family-firm status out of CSE filings by hand over nine years. That prices the extraction problem and explains why the retrieval pipeline over those filings is the component most likely to be the bottleneck, which is the case the structure-aware chunking work in [[Financial Report Chunking for Effective Retrieval Augmented Generation]] addresses and reduces rather than removes. It is also why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence."
+There is also a documented accounting break in the fundamentals: "SLFRS 16 in 2019 is a documented structural break in CSE fundamentals sitting in the middle of my training window. My index track runs 1 July 2014 to 30 June 2024, so any PPE-derived or lease-sensitive fundamental feature is not comparable across the 2019 boundary, and the fix is either a feature set that avoids the affected line items or an explicit break control with the choice stated in the methodology."
+Fundamental update frequency here is annual (annual reports, year-end ownership stakes, lagged-one-year risk and controls).</t>
+        </is>
+      </c>
+      <c r="O60" s="30" t="inlineStr">
+        <is>
+          <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama–French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
+What I would add: "the non-synchronous trading correction and a reported correlation between the risk estimate and turnover, because if those two move together on my sample then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it."
+Magnitude prior for A_V: "Mean idiosyncratic risk of 0.221 with a standard deviation of 0.050 sets a realistic prior on how much cross-sectional signal the volatility channel can carry. That is a narrow spread, and a one standard deviation move being worth 2.02 percentage points of investment is a real-economy effect rather than a trading one, so I should not expect the cross-sectional volatility ranking on CSE counters to separate firms as cleanly as it does on a US sample."</t>
+        </is>
+      </c>
+      <c r="P60" s="30" t="inlineStr">
+        <is>
+          <t>The paper has no liquidity variable, no turnover screen and no execution cost model, but it makes two liquidity-relevant concessions that I treat as primary evidence.
+First, the frequency concession, which I flagged as an important callout: "Weekly, not daily, and the paper says why in one sentence: 'since most stocks are not traded daily, we use weekly stock returns.' That is a finance journal on my exact market conceding the non-synchronous trading problem in the data section rather than the limitations section. Every frequency decision I make downstream has to answer to it."
+Second, the free-float consequence: "Mean institutional ownership of 66.1% against insider ownership of 5.7% is a free-float fact with a liquidity consequence. Two thirds of shares held by institutions means the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding. This is cheap to check on my own data and I should check it before setting the sweep range."
+Third, the untreated bias: "Weekly returns reduce the problem relative to daily but they do not eliminate it on a market where the paper itself says most stocks don't trade daily, and stale prices bias the residual standard deviation downward for exactly the thinnest counters. There is no Dimson or Scholes-Williams correction, no reported trading-frequency screen, and no check of whether the idiosyncratic risk measure correlates with turnover." The ±50% weekly return trim "is a sensible outlier rule and it is also a reminder of what the raw series looks like."</t>
+        </is>
+      </c>
+      <c r="Q60" s="30" t="inlineStr">
+        <is>
+          <t>Not applicable in the ML sense — coefficients and group-specific slopes are the explanation by construction. Figure 1 is the paper's clearest visual statement: "the low-ownership line falls from roughly 0.23 to 0.055 across the plotted range of log lagged idiosyncratic risk while the high-ownership line is flat and very slightly positive." I would note that the paper's headline mechanism is inferred rather than observed — see limitations.</t>
+        </is>
+      </c>
+      <c r="R60" s="30" t="inlineStr">
+        <is>
+          <t>In-sample panel estimation only; no holdout, no out-of-sample window, no forecast error. Adjusted R² moves from 0.029 to 0.206 across the three baseline columns, "so most of the explanatory power is coming from the fixed effects and controls rather than from risk, which is normal in this literature and worth remembering before reading the coefficient as a forecast." Baselines are prior literature by sign comparison: the result contradicts Panousi and Papanikolaou (2012) directly; the institutional substitution reading is consistent with Shleifer and Vishny (1986) and Gillan and Starks (2000); the governance null echoes Caixe et al. (2019) finding no governance mitigation in Brazil.
+Robustness battery, which I described as "unusually thorough and mostly holds": industry fixed effects and industry-by-year fixed effects leave the pattern intact; propensity score matched samples reproduce it; family firms (33% of firm-years, identified by hand from annual reports and executive biographies following Anderson and Reeb, 2003) show no differential sensitivity across five alternative family-ownership measures; adding independent board fraction and CEO duality changes nothing. Plus a sample extension to 2021.</t>
+        </is>
+      </c>
+      <c r="S60" s="30" t="inlineStr">
+        <is>
+          <t>1. Idiosyncratic risk is negatively and significantly related to firm-level investment across every specification: "−0.165* in the year-fixed-effects-only column rising to −0.232* with full controls and firm fixed effects, and −0.199 once a lagged dependent variable is added." Economic size: "a one standard deviation rise in idiosyncratic risk cuts the investment rate by 2.02 percentage points against a sample mean of 11.60%, a 17.48% decline."
+2. "The negative sensitivity is concentrated entirely in low-insider-ownership firms, and that is the opposite of the US result." Risk × low insider dummy is −0.435* with year effects only and −0.599 with the full specification; the high insider dummy interaction "is statistically indistinguishable from zero throughout (0.035, standard error 0.180)". The authors read this as alignment dominating entrenchment, contradicting Panousi and Papanikolaou (2012).
+3. Institutional ownership substitutes for insider alignment: in the 2×2 design "the only significantly negative cell is low institutional combined with low insider ownership, at −0.566* and then −0.985 with full controls, while the high-institutional-low-insider cell is insignificant at −0.392 (standard error 0.276)." My hedge, carried through: "I'd hold it a little more loosely than they do because the insignificance could be power rather than absence given the cell counts."
+4. The extension result, which I rate as the most useful finding in the paper for me: "Extending the sample three years to 2021 weakens the baseline result from −0.232* to −0.123*, and the paper calls this 'largely consistent'." The ownership results survive better — "low insider at −0.407 and low-institutional-low-insider at −0.787, and the high-institutional-low-insider cell now turns significant at −0.433." My reading: "I read the halving of the main coefficient and the loss of two significance stars as the more informative result here, and it is the single most useful thing in the paper for my own period argument." Note the surviving 2021 baseline is significant only at the 10% level (−0.123*).</t>
+        </is>
+      </c>
+      <c r="T60" s="30" t="inlineStr">
+        <is>
+          <t>- "The moderation results, which are the paper's contribution, rest on very few firms." 59 unique firms and 297 firm-years for insider tests, 54 firms and 278 for institutional tests, and after propensity score matching "64 and 76 observations respectively, all of this carrying firm fixed effects, year fixed effects and category dummies. At those sample sizes firm fixed effects consume a large share of the degrees of freedom and the matched-sample estimates in particular are being asked to do more than the data can support. The authors are not hiding any of this, the counts are in every table, but the write-up treats the matched results as confirmation when at 64 observations they are closer to a consistency check."
+- "The −0.703 correlation between insider and institutional ownership makes the 2×2 grid structurally unbalanced, and the insignificant cells are where that bites. Two variables correlating that strongly cannot produce four well-populated quadrants from 278 observations, so the high-insider-high-institutional cell is thin by construction, and every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one. The substitution story the paper tells could be right, but the evidence for it is one significant cell and three insignificant ones, and the design can't separate a genuine null from low power."
+- "Non-synchronous trading is handled by moving to weekly data and then not mentioned again… stale prices bias the residual standard deviation downward for exactly the thinnest counters. There is no Dimson or Scholes-Williams correction, no reported trading-frequency screen, and no check of whether the idiosyncratic risk measure correlates with turnover. That matters because firm size is a control and size correlates with liquidity, so part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant."
+- "The investment measure is a net quantity doing the work of a gross one. The change in net PPE nets out depreciation and disposals, so a firm that holds capex constant while an existing asset base ages records a falling investment rate, and a firm that sells a property records a negative one, which is why the minimum in Table 2 is −0.082. Capex is reported separately in Sri Lankan annual reports and the paper hand-collects everything else, so this is a choice rather than a constraint, inherited from Panousi and Papanikolaou for comparability, and it leaves the dependent variable noisier than the framing suggests."
+- "Alignment against entrenchment is inferred from a sign pattern rather than tested. Nothing in the design observes managerial risk preference, wealth concentration or the project set, so the mechanism is read off the direction of an interaction coefficient… which is a reasonable inference and not a test. The authors say as much in their conclusion, where they note the underlying mechanisms warrant further exploration."
+- "The 2018 cutoff is well-argued and the extension quietly undercuts the argument for it. SLFRS 16 changing lease recognition in 2019 genuinely contaminates PPE, and that justifies the main sample. But the extended analysis to 2021 then runs straight through SLFRS 16, the Easter attacks and COVID with no adjustment to the PPE measure and no regime split, and reports the result as consistent, so the paper ends up both claiming the break is serious enough to truncate the sample and treating a sample that spans it as corroborating evidence."</t>
+        </is>
+      </c>
+      <c r="U60" s="30" t="inlineStr">
+        <is>
+          <t>- The citation for why A_T cannot assume a daily price series on CSE: a finance journal estimating a factor model on CSE firms moves to weekly because most stocks don't trade daily. "That is a stronger warrant than anything I could get from the ML literature."
+- The idiosyncratic risk estimator for A_V's cross-sectional input — residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free — plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk–turnover correlation).
+- A realistic prior on how much cross-sectional signal A_V can carry: mean idiosyncratic risk 0.221, standard deviation only 0.050, range 0.117 to 0.315.
+- A mechanism-level argument for volatility persistence that is independent of the statistical long-memory literature.
+- The free-float fact (66.1% institutional, 5.7% insider) as a calibration input for the execution-cost participation-rate sweep.
+- SLFRS 16 (2019) as a documented structural break inside my training window.
+- The annual-median-split, group-specific-slope design as a template for ablating state inputs one at a time.
+- Retention of delisted firms as the correct survivorship control, and the correct counterpart to the wrong version documented in [[The Impact of Firm-Specific Factors on Share Prices of Diversified Financial Companies, Evidence from the Colombo Stock Exchange]].</t>
+        </is>
+      </c>
+      <c r="V60" s="30" t="inlineStr">
+        <is>
+          <t>- The non-synchronous trading problem is conceded and then left untreated: no Dimson or Scholes–Williams correction, no trading-frequency screen, no check of whether the risk measure correlates with turnover. That correction, and the reported risk–turnover correlation, is work I have to do, and it is exactly the boundary between A_V and A_L.
+- No out-of-sample period, no forecast, no decision objective — so nothing here tells me how a risk estimate should be weighted in a live allocation, only how it relates contemporaneously to corporate investment.
+- No execution cost model, no order size, no depth — the free-float fact implies the friction problem but the paper does not model it.
+- No persistence modelling. The paper gives a mechanism for slow decay but estimates no persistence parameter, no long-memory d and no regime structure.
+- No state-conditional combination of any channel; the conditioning is on ownership, a firm attribute, not on market state L_t, V_t or P_t.</t>
+        </is>
+      </c>
+      <c r="W60" s="30" t="inlineStr">
+        <is>
+          <t>[[Relationship between firm-level investment, idiosyncratic risk and ownership, an emerging market perspective]]</t>
+        </is>
+      </c>
+      <c r="X60" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk–turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
+EFFECT ON MAIN GAP: Strongly supportive on two fronts. First, regime instability: "The 2021 extension weakening the main coefficient from −0.232* to −0.123* is corroboration that CSE relationships estimated pre-2020 do not survive the crisis window intact. Taken with [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] finding the traditional macro linkages broken over 2014 to 2022, that is now two independent CSE results pointing at regime instability across exactly the period a static system would be evaluated on, which is the clearest empirical case I have for an orchestrator that conditions on measured state rather than a fixed combination rule." Note the surviving coefficient is significant only at 10%.
+Second, the C_i,t component and abstention. The frequency concession forces an abstention design on A_T: "It doesn't mean I build at weekly frequency, the index track is liquid enough for daily, it means the per-counter liquidity screen has to come before any cross-sectional feature is computed and counters that fail it have to produce an abstention rather than a stale-price signal. This is the same structural failure [[AlphaAgents, Large Language Model Based Multi-Agents for Equity Portfolio Constructions]] fixed by deleting an agent by hand." And the data-depth fact forces the same on A_F: "it is why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence." Both of these are structural properties of the input and output, not self-reports, which is exactly what C_i,t is meant to be.
+Third, a methodological warning for the state vector itself: if the volatility estimate and the liquidity estimate co-move on my sample, "then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it." That is a concrete pre-registration task for the main gap, and the paper's own −0.703 insider/institutional correlation is the worked example of what unmanaged collinearity does to a conditioning design: "every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one."
+Fourth, Model 2's design is a usable template: "splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it is close to the structure I'd want for ablating state inputs one at a time."
+EFFECT ON SUB-GAP 1: This is the strongest row in the note for state-dependent execution friction and for liquidity conditioning the reliability of price-derived agents. The reliability half is stated by the paper itself: "since most stocks are not traded daily, we use weekly stock returns" — a published finance journal on my exact market changing its estimation frequency because of thin trading. That is local empirical evidence that price-derived quantities on CSE degrade with liquidity, and it is the warrant for L_t conditioning A_T's and A_V's weights rather than being a separate add-on signal. The untreated residual is my opening: stale prices "bias the residual standard deviation downward for exactly the thinnest counters", with no Dimson or Scholes–Williams correction, no trading-frequency screen and no risk–turnover check anywhere in the paper, and "part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant." The execution-cost half comes from the ownership structure: institutional ownership averaging 66.1% against insider 5.7% means "the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding."
+EFFECT ON SUB-GAP 2: Supportive at the mechanism level, which is more than a statistical citation gives me. "The investment channel is the mechanism-level argument for pairing forecast variance with persistence rather than treating volatility as a point-in-time cap. If elevated idiosyncratic risk causes firms to cut capital spending by 17.48% of the mean investment rate, then a volatility shock on this market propagates into fundamentals with a lag measured in reporting periods, not days, and the real activity it suppresses takes just as long to come back. That is a fundamental reason to expect slow decay, independent of the statistical long-memory evidence in [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] and [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], and it is a better sentence for the proposal than another citation of a d estimate." The paper itself estimates no persistence parameter, so operationalising P_t remains entirely mine.
+CSE DATA EVIDENCE: This is the single densest source of local empirical evidence I have for the justification rewrite, and the fact that it comes from authors with no stake in making a data-depth argument is what makes it usable.
+- Thin trading, conceded in the data section: "since most stocks are not traded daily, we use weekly stock returns." Three authors with institutional access, publishing in Managerial Finance, could not estimate a factor model at daily frequency on this market. That is direct local evidence of liquidity constraint, and it is stated as a design constraint rather than as a limitation.
+- Heterogeneous trading activity: the ±50% weekly return trim following Abeysekera and Nimal (2017) is itself "a reminder of what the raw series looks like" — a market where weekly moves beyond ±50% occur often enough to need a documented rule.
+- Universe depth: 167 unique firms with usable accounting data, 1,226 firm-years over 2010–2018, after excluding financials, utilities, energy and telecoms, firm-years with missing variables, and negative book values. Ownership data available only from 2011 and only for 59 firms (insider) and 54 firms (institutional) — "usable ownership data exists for roughly a third of the firms that have usable accounting data". After propensity score matching, 64 and 76 observations.
+- Ownership concentration and free float: mean institutional ownership 66.1%, mean insider ownership 5.7%, correlating at −0.703. "This is a market of institutionally held firms with thin executive stakes." Two thirds of shares in institutional hands is a free-float constraint with a direct depth consequence.
+- Family control: family firms are 33% of firm-years, identified by hand from annual reports and executive biographies following Anderson and Reeb (2003).
+- Idiosyncratic risk levels: mean 0.221, standard deviation 0.050, range 0.117 to 0.315 — "the cross-sectional spread in firm-specific risk on this market is narrow". This is a quantified statement of how much, and how little, firm-level risk varies across CSE counters.
+- Firm fundamentals respond to firm risk: a one standard deviation rise in idiosyncratic risk cuts the investment rate by 2.02 percentage points against a sample mean of 11.60%, a 17.48% decline. Baseline coefficient −0.232* with full controls and firm fixed effects; −0.199 with a lagged dependent variable.
+- Governance heterogeneity in the transmission: the sensitivity is concentrated entirely in low-insider-ownership firms (−0.599 full specification) while high-insider firms are indistinguishable from zero (0.035, standard error 0.180), and in the 2×2 grid only the low-institutional/low-insider cell is significantly negative (−0.566*, then −0.985 with full controls). Hedge: the insignificant cells may be low power rather than genuine nulls given cell counts and the −0.703 correlation.
+- Regime instability: extending the sample three years to 2021 halves the baseline coefficient from −0.232* to −0.123*, significant only at 10%. The window crosses SLFRS 16 (2019), the Easter attacks and COVID.
+- Documented accounting break: SLFRS 16 changed lease recognition in 2019 and contaminates PPE — a structural break in CSE fundamentals sitting inside my 1 July 2014 to 30 June 2024 index track.
+- Fundamental extraction cost: all accounting figures, insider stakes, board composition, CEO duality and family-firm status were pulled out of CSE annual report PDFs by hand over nine years, by authors with institutional access and every incentive to keep the sample large.
+- Correct survivorship handling exists in the local literature: "Both listed and delisted firms are retained, which is a deliberate survivorship-bias control and more than most of the local literature does."
+PROPOSED REVISION STATED IN THE NOTE: (1) A per-counter liquidity screen must run before any cross-sectional feature is computed, and counters failing it must emit an abstention rather than a stale-price signal — A_T does not get to assume a daily series on this market. (2) A_V reuses this idiosyncratic risk construction (residual standard deviation from a local factor model over a rolling window, ASTRI market proxy, 91-day Treasury bill risk-free, with Abeysekera and Nimal (2017) as a four-factor local alternative) but adds the non-synchronous trading correction they skip and reports the correlation between the risk estimate and turnover, to establish whether A_V and A_L are partly measuring the same thing before any weighting is set on them. (3) The cross-sectional volatility ranking's expected separating power on CSE counters should be "pinned down on my own data before the agent's influence weight is allowed to swing much on it", given the 0.221/0.050 spread. (4) Any PPE-derived or lease-sensitive fundamental feature must either avoid the affected line items or carry an explicit SLFRS 16 break control, "with the choice stated in the methodology — I'd rather find this now than discover it in an ablation". (5) The execution-cost participation-rate sweep must be calibrated against free float rather than shares outstanding, and this is to be checked on my own data "before setting the sweep range". (6) A_F is designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence. (7) The volatility-persistence argument in the proposal is to be made at the mechanism level — investment suppression propagating through reporting periods — rather than by another citation of a long-memory d estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="409.6" customHeight="1">
+      <c r="A61" s="29" t="inlineStr">
+        <is>
+          <t>P60</t>
+        </is>
+      </c>
+      <c r="B61" s="30" t="inlineStr">
+        <is>
+          <t>Pavithya, M.B.D., Perera, G.S.D., Munasinghe, S.L. and Karunarathna, S.N. (2021). Quantitative Analysis and Sentiment Analysis for Stock Price Forecast: The Case of Colombo Stock Exchange. 2021 10th International Conference on Information and Automation for Sustainability (ICIAfS), August 2021, pp. 512-517. DOI: 10.1109/ICIAfS52090.2021.9606034. Citekey: pavithyaQuantitativeAnalysisSentiment2021. Affiliation as recorded in my note: all authors out of the Department of Computer Engineering at the University of Peradeniya.</t>
+        </is>
+      </c>
+      <c r="C61" s="30" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D61" s="30" t="inlineStr">
+        <is>
+          <t>2021 10th International Conference on Information and Automation for Sustainability (ICIAfS), pp. 512-517. Conference paper.</t>
+        </is>
+      </c>
+      <c r="E61" s="30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ICIAfS52090.2021.9606034 (accessed 4 October 2026). Zotero: zotero://select/library/items/XMAIQR9E</t>
+        </is>
+      </c>
+      <c r="F61" s="30" t="inlineStr">
+        <is>
+          <t>Orchestration (stream field in the note frontmatter). Market: CSE. In my own framing this is the CSE-local instance of the fixed-influence combination problem: two methodologically heterogeneous forecasting models merged into a single binary decision by a constant weight pair. As I put it in the note, "This is the closest thing in my CSE set to the shape of what I'm building, and it runs aground in exactly the place my main gap sits."</t>
+        </is>
+      </c>
+      <c r="G61" s="30" t="inlineStr">
+        <is>
+          <t>Forecast the next trading day's up/down direction for CSE counters by building a quantitative price model and a text model separately and then merging them with a fixed weighted vote. Three motivating gaps as I recorded them:
+- Forecasting models validated on deep markets are not guaranteed to transfer to a disrupted one. The abstract is explicit that prior work is built on well established exchanges and that such models are not guaranteed to capture the trends of exchanges showing high disruptive behaviour like the CSE, "where some indexes have no trades on some days and the data is therefore incomplete." My note's judgement: "That is the right motivation and it is close to my own, and it is also the thing the methodology then fails to act on."
+- Combining a price model with a text model rather than running either alone. The surveyed work in Table I is mostly one channel or the other, and where both appear the integration is a single joint model rather than two models with an explicit combination step. "Building two and then asking how to merge them is the genuinely interesting decision in this paper, and it is the one that receives the least analysis."
+- The CSE text channel had not been established as usable at all. The authors tried the exchange's own announcement feed first and abandoned it, "which is itself the finding."</t>
+        </is>
+      </c>
+      <c r="H61" s="30" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange, Sri Lanka. Three counters: John Keells Holdings (JKH), Ceylon Tobacco Corporation (CTC) and Agalawatte Plantations PLC (AGAL). Daily frequency, single-market, frontier market.</t>
+        </is>
+      </c>
+      <c r="I61" s="30" t="inlineStr">
+        <is>
+          <t>CSE trade information for the past eight years, one file per index, for JKH, CTC and AGAL. The authors stress this is real exchange data rather than a downloadable synthetic set, which they argue makes the results more realistic for automated trading on the CSE. Split: six years training, one year validation, one year testing, with the training partition expanding on each iteration because of the walk-forward scheme.
+Text corpus: the CSE announcement data obtained from the exchange was not rich enough to train a usable classifier, so news was scraped from a public economic-news blog with a pagination loop, giving over 4,000 articles from 2012 to 2019. Roughly 4,000 articles across eight years is about two per trading day (my arithmetic in the note, not the paper's).</t>
+        </is>
+      </c>
+      <c r="J61" s="30" t="inlineStr">
+        <is>
+          <t>Two modalities, price/volume and news text.
+Price side: missing values were handled and the data normalised, except for CTC, which was trained unnormalised with a different parameter set and is therefore not comparable with the other two. PCA was applied for dimension reduction and then dropped as unsuitable, after which feature selection was done on correlation and autocorrelation instead: previous-day close, high, low and open plus volume correlated best, and the previous seven days of prices showed higher autocorrelation than days further back. Day of the week was added on the observation that Mondays and Fridays behave differently from the three mid-week days, which is what makes the multivariate variant multivariate. Seasonality and trend removal was attempted and abandoned because the model did not perform well on the stationarised series, "reported plainly as a pitfall rather than buried."
+Text side: CountVectorizer n-gram range, stop-word removal and TfidfTransformer settings tuned. Labels were not annotated, they were derived mechanically: each article was joined to the quantitative data by publication date under the assumption that news published on one day moves the trend on the next, and inherited that next day's up or down label.</t>
+        </is>
+      </c>
+      <c r="K61" s="30" t="inlineStr">
+        <is>
+          <t>Univariate and multivariate LSTMs over eight years of CSE trade data for three counters, plus a Multinomial Naive Bayes classifier over roughly 4,000 scraped economic news articles, combined by a fixed weighted vote into a single up or down call for the next trading day.
+Final LSTM: four layers of 128, 64, 16 and 1 units, dropout 0.5 on the first two layers, an L1L2 bias regulariser at l1 = l2 = 0.001, batch size 10, Adam optimiser. Depth, width, epochs, dropout, optimiser and learning rate searched using a Hyperas wrapper and grid search.
+Text model selection: Decision Tree, Naive Bayes, SVM, Random Forest and a simple ANN compared. Multinomial Naive Bayes selected on 10-fold cross-validation accuracy: Naive Bayes 0.95 (+/-0.02) and SVM 0.95 (+/-0.03) against Decision Tree and Random Forest at 0.88.
+The combination rule, which is the mechanism I care about:
+Trend_t = ( w_V * V_t + w_P * sum_{k=1}^{n_t} P_{k,t-1} ) / ( w_V + n_t * w_P )
+where:
+- V_t is the single up or down prediction from the quantitative model, fed four days of past prices, trend details and day of the week
+- P_{k,t-1} is the text model's prediction for the k-th of the n_t articles published on the previous day
+- w_V : w_P = 1:3 in the finalised model, after the authors tried several ratios and kept the one with the highest holdout accuracy
+- both w_V and w_P carry no time index, "which is the whole point of the note"
+Reported evaluation metric alongside accuracy, the Matthews correlation coefficient:
+MCC = (TP*TN - FP*FN) / sqrt( (TP+FP)(TP+FN)(TN+FP)(TN+FN) )
+Output: a single binary up/down trend call for the next trading day.</t>
+        </is>
+      </c>
+      <c r="L61" s="30" t="inlineStr">
+        <is>
+          <t>No agents in the LLM sense, but there is an explicit two-channel combination with a stated weight vector, which is why I treat it as an orchestration-stream paper. The orchestration is a constant: two methodologically heterogeneous models, one shared binary decision, and "a combination rule that is a pair of constants found by trying a few values and keeping the best. No conditioning on market state, no per-day reweighting, no handling of a channel whose input is absent that day."
+My central structural finding on the mechanism, recorded in the note as a warning callout: the stated 1:3 weight ratio is not what actually decides the trend, the article count is. The combining rule sums one prediction from the quantitative model against one prediction per news article and divides by total weight, so with n_t articles the text channel holds n_t*w_P / (w_V + n_t*w_P) of the decision. At the reported 1:3 ratio a single article already gives text 75%, two give it 86%, and roughly 4,000 articles across eight years is about two per trading day. "The LSTM, which is the better-validated of the two components, is therefore carrying something near 14% of a typical day's decision, and moving from equal weights to 1:3 only shifts the text share from about 67% to about 86%. That is the real reason the weight axis buys so little, 2.15 accuracy points, and the paper never states the quantity."
+There is an accidental abstention behaviour: when no article appears the text term vanishes and the decision falls back entirely to the quantitative model. This is arrived at "by accident rather than design," and as implemented "the system cannot tell a confident abstention from a quiet news day."</t>
+        </is>
+      </c>
+      <c r="M61" s="30" t="inlineStr">
+        <is>
+          <t>What the paper did: news was scraped from a public economic-news blog with a pagination loop after the CSE's own announcement feed was found not rich enough to train a usable classifier, giving over 4,000 articles from 2012 to 2019. Labels were derived mechanically rather than annotated: each article was joined to the quantitative data by publication date under the assumption that news published on day t-1 moves the trend on day t, and inherited that next day's up or down label. Five classifiers were compared (Decision Tree, Naive Bayes, SVM, Random Forest, a simple ANN), tuned over CountVectorizer n-gram range, stop-word removal and TfidfTransformer settings, and Multinomial Naive Bayes was selected on 10-fold cross-validation accuracy of 0.95 (+/-0.02), tied with SVM at 0.95 (+/-0.03) against Decision Tree and Random Forest at 0.88. The text predictions then enter the weighted vote one term per article.
+My reading of that 0.95: it "is not evidence of predictive skill, and the hybrid result demonstrates that. Those labels were assigned mechanically from the next day's price direction, and 10-fold CV shuffles articles that are temporally adjacent and frequently cover the same event, so articles sharing a day share a label and overlapping vocabulary and the classifier can recover the day rather than the direction. The test that matters is the one the paper itself runs: a component scoring 0.95 in isolation contributes about four accuracy points to a joint decision in which it holds most of the weight. Those two numbers cannot both be measuring the same thing."
+Scope statement: this component is out of scope for my project. The sentiment agent was removed from my architecture by the supervisor's scope decision (see [[Scope sentiment analysis dropped]]), and my note states the consequence directly: "the only reading available to me since sentiment is out of scope and the text half is not something I'll rebuild." This row is retained in the matrix as evidence about the CSE and about fixed-weight combination, not as a design input. Per the scope rules the text channel is cited as a fixed-influence failure case, not as a component to rebuild.</t>
+        </is>
+      </c>
+      <c r="N61" s="30" t="inlineStr">
+        <is>
+          <t>No fundamental agent and no retrieval architecture in the paper. The relevant transferable finding is about document availability rather than retrieval method: the CSE announcement data obtained from the exchange was not rich enough to train a usable classifier, so the authors abandoned the exchange's own feed for a scraped economic-news blog. I read that as direct evidence for how I scope A_F: "The authors had the exchange's own data and had to abandon it for scraped material, the same thin-channel failure AlphaAgents hit with news on fifteen US megacaps, and it is why I expect the fundamental channel to be unusable a large fraction of the time. The binding constraint on structure-aware retrieval over CSE filings is document availability per counter per period, so that count is worth establishing before the retrieval design is settled."</t>
+        </is>
+      </c>
+      <c r="O61" s="30" t="inlineStr">
+        <is>
+          <t>Not recorded in the note as a modelled component. There is no volatility model, no risk term and no position sizing in the paper. The nearest related observation in my note is a failure mode rather than a risk treatment: "Since seasonality and trend removal were abandoned, the network is fitting levels rather than changes, which is the condition under which that failure mode is expected" (the failure mode being that the LSTM reproduces the shape of the series with a lag and smooths away the local swings).</t>
+        </is>
+      </c>
+      <c r="P61" s="30" t="inlineStr">
+        <is>
+          <t>None implemented, and this is a load-bearing omission. The disrupted-data problem that motivates the paper is never handled in the methodology: non-trading days on thin counters are named in the abstract as the reason a CSE-specific model is needed, and then "the only treatment is a general statement that missing values in the raw data were handled. Nothing says whether an absent day was dropped, forward-filled or zero-filled, and on a lookback of four days the difference between those choices changes what the window contains. AGAL is a plantation counter and the most likely of the three to have gaps, which makes the omission load-bearing rather than cosmetic."
+No liquidity screen on counter selection either: JKH, CTC and AGAL "are described as powerful counters without a stated selection criterion, and they differ sharply in how actively they trade."
+No friction accounting at all: "There is also no position, no fee, no spread and no return, so the claim that at 58% accuracy 'the users will always receive an overall gain' does not follow from anything in the paper." My note sets that against the local evidence: "on a market where [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] measures unexpected illiquidity shocks depressing returns by 8 to 10 basis points, a near-coin-flip signal traded daily is the case where costs decide the outcome."</t>
+        </is>
+      </c>
+      <c r="Q61" s="30" t="inlineStr">
+        <is>
+          <t>Not recorded in the note as an explicit contribution. The nearest thing is the reporting of the weight ratio itself, which my note credits as the one advantage this paper has over the LLM systems for gap-argument purposes: "the contrast is cleaner here than in any of the LLM systems, because this paper does at least have an explicit weight vector to point at." The paper does not report the realised per-day share each channel held, which is the quantity my note reconstructs and criticises it for omitting.</t>
+        </is>
+      </c>
+      <c r="R61" s="30" t="inlineStr">
+        <is>
+          <t>Protocol, which is the part my note credits: the authors reject k-fold cross validation explicitly, on the grounds that it assumes instances are independent and therefore ignores the temporal component, and use walk-forward validation instead, where real data for a batch is added back and the model retrained before predicting the next batch. My note positions that against the local set: "That puts this paper ahead of [[Machine Learning-Driven Sri Lankan Stock Market Prediction, Harnessing Economic Indicators and Sentiment Analysis]], which treats shuffling the series before splitting as a design improvement, and ahead of [[ARIMA and ANN Approach for forecasting daily stock price fluctuations of industries in Colombo Stock Exchange]], which selects a neural architecture with no validation partition at all."
+Metrics: an undefined "error score" on normalised data for the lookback sweep; accuracy, sensitivity, specificity, precision and Matthews correlation coefficient for the trend classification; 10-fold cross-validation accuracy for text-classifier selection.
+Baselines: none. "For a binary direction task the relevant floors are the majority-class rate and a persistence call, neither of which is computed, and the class balance needed to work out the first is not reported." No backtest, no position, no fee, no spread, no return. The only internal comparison is equal weights against the finalised 1:3 weights, and that comparison is contaminated (see LIMITATIONS).</t>
+        </is>
+      </c>
+      <c r="S61" s="30" t="inlineStr">
+        <is>
+          <t>- Headline: the combination lifts trend accuracy from 54% to 58%, and a 1:3 weight ratio favouring the text model beat equal weighting on the holdout set.
+- Precisely: accuracy moves from 0.5622 to 0.5837 and the Matthews correlation from 0.0966 to 0.1493. My reading: "Accuracy on a binary task whose class balance is never reported is close to uninformative... At 0.1493 the finalised model has some directional signal and not much, and the gap between an accuracy that sounds like 58% and an MCC that sits at 0.15 is the whole story of the result."
+- Lookback sweep on CTC, leading days 1 to 10: the one-day-ahead error score falls from 0.0436 at one day to 0.0189 at four and 0.0177 at five, then rises again to 0.0267 at six and 0.0280 at ten. The same shape holds across the two- and three-day prediction columns. The authors' reading, that four or five previous days beats both shorter and longer windows, is supported by the table. Two caveats I recorded: the correlation analysis had pointed at seven days and the final architecture diagram says four, "so the empirical sweep overrode the feature-selection step and the paper doesn't remark on it"; and the metric itself is never defined, reported only as "error score" on normalised data, "so the shape of the curve is usable to me and the levels are not."
+- Class bias: sensitivity 0.6232 against specificity 0.4737 under equal weights, so the down class is being called worse than a coin flip while the headline accuracy still reads 0.5622. The finalised weights narrow it to 0.6391 against 0.5100, "which is the more meaningful of the two improvements since it is specificity rather than accuracy that moved, but precision barely shifts at all, 0.6324 to 0.6343. The honest summary is that the weight change mostly bought a less lopsided classifier rather than a better one."
+- Text classifier 10-fold CV: Naive Bayes 0.95 (+/-0.02), SVM 0.95 (+/-0.03), Decision Tree and Random Forest 0.88.
+- Qualitative LSTM behaviour on CTC: the predicted line tracks the fall from roughly 1,350 to 1,290 and then flattens where the actual flattens, "but it cuts the amplitude of nearly every local swing and misses the terminal drop to about 1,203 entirely. The authors describe this as having predicted the basic behaviour with less fluctuations, which is accurate, and it is also the signature of a network leaning heavily on the most recent close."</t>
+        </is>
+      </c>
+      <c r="T61" s="30" t="inlineStr">
+        <is>
+          <t>- The weights were selected on the data the result is reported on. Table IV is headed as a holdout measurement and reports both the equal-weight and finalised instances on it, and the finalised ratio was found by changing the weights until performance was at its best. There is no third partition separating weight selection from reporting, so 0.5837 is an in-sample figure for the one parameter the paper's contribution turns on. "The 54% to 58% improvement is therefore not independently evidenced, and with the walk-forward machinery already built, holding out a separate window for the combination step would have cost very little."
+- The disrupted-data problem that motivates the paper is never handled in the methodology. Non-trading days on thin counters are named in the abstract as the reason a CSE-specific model is needed, then treated only by a general statement that missing values were handled. On a lookback of four days the choice between dropping, forward-filling and zero-filling changes what the window contains. AGAL is the counter most likely to have gaps, "which makes the omission load-bearing rather than cosmetic."
+- No baseline of any kind, and no backtest. Majority-class rate and persistence are not computed and class balance is not reported. No position, fee, spread or return, so the claim that at 58% accuracy "the users will always receive an overall gain" does not follow.
+- Three counters, one of them trained differently, and no liquidity screen. JKH, CTC and AGAL described as powerful counters with no stated selection criterion. CTC was trained unnormalised with a different parameter set, "so cross-counter comparison is not available even in principle, and the trend-classification result in Table IV is reported as a single number without saying which counter or counters produced it."
+- The label construction fixes a one-day news-to-price lag by assumption, and the conclusion concedes it is wrong. The authors acknowledge that this is not the real scenario since any news or event can affect the stock at the moment it is published. "Both legs of the hybrid are consequently trained against the same label stream under an assumption the paper itself disowns, and the proposed fix, real-time news acquisition, is listed as future work rather than tested."
+- The stated weight ratio is not the realised weighting (my own finding, above): the article count sets the effective share and the paper never states that quantity.
+- The 0.95 text-classifier CV score is not evidence of predictive skill, because the labels were derived from the target and 10-fold CV shuffles temporally adjacent articles covering the same event.</t>
+        </is>
+      </c>
+      <c r="U61" s="30" t="inlineStr">
+        <is>
+          <t>- Walk-forward with retraining as the protocol, with this paper as the local precedent I cite for it. Expanding training window, retrain on each batch, evaluate on the next, with the horizon and the refit policy stated as columns in every results table. My note's broader observation: "That is three CSE papers now where the modelling is ordinary and the evaluation is what separates them, which keeps pointing at the same thing: on this market the contribution worth making is evaluation that survives being checked."
+- A four to five day lookback as the starting point for the technical agent A_T, not thirty. "The error sweep here is the only direct evidence I have on window length for CSE counters and it says short beats long, with the curve turning sharply after five days. On a per-counter archive of 374 trading days a five-day lookback yields far more usable sequences than a thirty-day one, so this cuts in the same direction as the data-depth constraint, and window length goes into the ablation set rather than being inherited."
+- The rule that component-level accuracy is not a basis for setting an agent's weight. "The text model was given three times the influence because it scored higher in individual testing, and that individual score was measuring a different and much easier task than the one it was being weighted for. So the weight my orchestrator assigns A_T, A_F, A_V or A_L has to come from each agent's measured marginal contribution to the joint decision, computed by ablation on held-out windows, and never from how well an agent does on its own in-domain metric. That is a direct argument for the ablation design already in the evaluation plan."
+- The rule that influence has to be normalised explicitly, or input volume sets it accidentally. "My orchestrator emits a weight vector that sums to one over agents, one scalar per agent regardless of how many documents, bars or signals that agent consumed, and the effective share each agent held gets logged per day so the realised weighting can be audited against the intended one."
+- The abstention design lesson. "When no article appears the text term vanishes and the decision falls back entirely to the quantitative model, which is the behaviour I want from A_F on a counter whose last filing is stale, arrived at here by accident rather than design. The lesson is that fallback has to be an explicit state with the remaining weights renormalised and the event recorded, not a side effect of a denominator, because as implemented here the system cannot tell a confident abstention from a quiet news day."
+- The reporting rule: MCC alongside accuracy for every directional result, and a return alongside both. "Any directional number my system reports carries the class balance, the Matthews correlation and the cost-adjusted return on the same row."
+- The 2021 data point on how thin the CSE's own announcement channel is, as a scoping input for A_F.</t>
+        </is>
+      </c>
+      <c r="V61" s="30" t="inlineStr">
+        <is>
+          <t>The combination weights are constants, chosen once by a small search and never conditioned on anything. There is no per-day reweighting, no conditioning on liquidity, volatility level or volatility persistence, no agent confidence term, and no designed abstention channel. The realised per-day influence is set by how many articles happened to be published, which is an availability-weighted scheme that was neither designed nor analysed as such, and the paper never states that quantity. The disrupted-data behaviour that motivates the paper, non-trading days on thin counters, is named and then not acted on in the methodology, so there is no treatment of what an absent observation does to a short lookback window. There is no execution-cost model, no spread, no fee and no return, so nothing here tells me whether a near-coin-flip directional signal survives CSE friction. Weight selection and result reporting share a partition, so even the one combination result is not independently evidenced. That is the opening my orchestrator sits in: replacing the constant with w(i,t) = f(L_t, V_t, P_t, C_{i,t}), with an explicit abstention state, with per-agent weights that sum to one independent of input volume, with the realised share logged, and with the combination step selected on a partition separate from the one it is reported on.</t>
+        </is>
+      </c>
+      <c r="W61" s="30" t="inlineStr">
+        <is>
+          <t>[[Quantitative Analysis and Sentiment Analysis for Stock Price Forecast, The Case of Colombo Stock Exchange]]</t>
+        </is>
+      </c>
+      <c r="X61" s="30" t="inlineStr">
+        <is>
+          <t>SPEAKS TO: The main gap, directly and locally; the evaluation protocol; the scoping of A_F; the window length for A_T; and the abstention channel. This is the CSE-local instance of the fixed-influence failure, and in my note it "belongs in the gap argument beside FinAgent and AlphaAgents." It is also retained evidence under the exception the supervisor granted for sentiment papers: the scope decision of 20 September 2026 (status Final) removed the sentiment component from my architecture, not the sentiment papers from my literature review.
+EFFECT ON MAIN GAP: Strengthens it, and strengthens it more cleanly than the LLM systems do, because there is an explicit numeric weight vector to point at. Two heterogeneous models, one shared decision, and the combination rule is a constant chosen once by trying a few values and keeping the best. What I am building replaces the constant with a function of measured state, Decision_t = sum_i w_{i,t} A_{i,t} with w_{i,t} = f(L_t, V_t, P_t, C_{i,t}). Three specific consequences for the design of f. First, C_{i,t} cannot be an in-domain self-score: this paper gave the text model three times the influence because it scored 0.95 in isolation, on a task that was mechanically easier than the one it was being weighted for, and the joint result then contributed about four accuracy points. That is the concrete argument for treating confidence as a structural property of the output and for setting weights from measured marginal contribution via ablation on held-out windows. Second, the weight vector must be normalised over agents explicitly, one scalar per agent regardless of how many documents, bars or signals that agent consumed, because here the denominator let input volume set the realised share; at the stated 1:3 ratio one article gives the text channel 75% and two give it 86%, so the LSTM carried roughly 14% of a typical day's decision while the paper reported the ratio as 1:3. The realised share per agent per day goes into my logs so the intended weighting can be audited against the realised one. Third, the abstention channel gets a positive design here by negative example: when no article appeared the text term simply vanished and the decision fell back to the quantitative model, which is the behaviour I want from A_F on a counter whose last filing is stale, but it has to be an explicit state with the remaining weights renormalised and the event recorded, because as implemented the system cannot tell a confident abstention from a quiet news day.
+EFFECT ON SUB-GAP 1: Supports it by omission, and the omission is unusually well documented. The paper's own motivation is that the CSE shows high disruptive behaviour, that some indexes have no trades on some days and the data is therefore incomplete, and then nothing in the methodology acts on it beyond a general statement that missing values were handled. There is no statement of whether an absent day was dropped, forward-filled or zero-filled, which on a four-day lookback changes what the window contains; AGAL is the counter most likely to have gaps. There is no liquidity screen on counter selection, and the three counters differ sharply in how actively they trade. There is no position, fee, spread or return anywhere, so the paper's claim that at 58% accuracy "the users will always receive an overall gain" rests on nothing, and against the local measurement of unexpected illiquidity shocks depressing returns by 8 to 10 basis points, a near-coin-flip signal traded daily is exactly the case where costs decide the outcome. So: expected execution cost entering the decision objective, and liquidity conditioning the reliability of the price-derived agents, are both untouched here.
+EFFECT ON SUB-GAP 2: Essentially none, and that absence is itself informative. There is no volatility model, no volatility level term, no persistence term and no regime notion of any kind. The only time-structure finding is the lookback sweep, which says four to five previous days beats both shorter and longer windows on these counters, and that is about predictive window length rather than about persistence. Seasonality and trend removal were attempted and abandoned, which leaves the network fitting levels rather than changes. I have not found an operationalisation of volatility persistence in this paper.
+CSE DATA EVIDENCE: Several usable facts, all from 2021. The exchange's own announcement feed was not rich enough to train a usable classifier and had to be abandoned for a scraped economic-news blog, which is direct evidence on the thinness of the CSE's own document channel and a scoping input for A_F; the binding constraint on structure-aware retrieval over CSE filings is document availability per counter per period, so that count is worth establishing before the retrieval design is settled. Eight years of real exchange trade data for JKH, CTC and AGAL was obtainable, one file per index, with a six/one/one year train/validation/test split. The scraped corpus was over 4,000 articles from 2012 to 2019, about two per trading day. Feature selection on CSE data found previous-day close, high, low, open and volume correlated best and the previous seven days showed higher autocorrelation than days further back, while the empirical sweep settled on four to five days. Day-of-week effects were observed, Mondays and Fridays behaving differently from the three mid-week days. Stationarising the series hurt performance and was abandoned. Non-trading days on thin counters are acknowledged by the authors as a real property of CSE data. On the quantitative side the LSTM fitted levels with a lag and smoothed away local swings on CTC, tracking a fall from roughly 1,350 to 1,290 but missing the terminal drop to about 1,203.
+PROPOSED REVISION STATED IN THE NOTE: Cite this as the CSE-local instance of fixed-influence combination in the gap argument, alongside FinAgent and AlphaAgents, rather than as a pipeline to extend. Per the scope rules the text channel is cited as a fixed-influence failure case, not as a component to rebuild; sentiment is out of scope per [[Scope sentiment analysis dropped]] and the text half is not something I will rebuild. Adopt walk-forward with retraining as the evaluation protocol and cite this paper as the local precedent, stating horizon and refit policy as columns in every results table. Put a four to five day lookback in as the starting point for A_T and into the ablation set rather than inheriting it. Set agent weights from measured marginal contribution by ablation on held-out windows, never from in-domain component scores. Emit a weight vector that sums to one over agents independent of input volume, and log the realised per-agent share per day. Make abstention an explicit state with renormalisation and an event record. Report class balance, MCC and cost-adjusted return on the same row as any directional accuracy figure. Separate the partition used to select combination parameters from the partition used to report them.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-08 11:07:46
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -712,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X61"/>
+  <dimension ref="A1:X60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7423,173 +7423,49 @@
       </c>
     </row>
     <row r="54" ht="409.6" customHeight="1">
-      <c r="A54" s="32" t="inlineStr">
-        <is>
-          <t>P53</t>
-        </is>
-      </c>
-      <c r="B54" s="33" t="inlineStr">
-        <is>
-          <t>Smart Trading Rule: A Modular Machine Learning Framework for Portfolio Optimization with Transaction Costs. Journal of Financial Data Science 8(2), 2026. Bibliographic details recovered from the Research Papers Grid entry 42; the paper itself is paywalled and has not been obtained.</t>
-        </is>
-      </c>
-      <c r="C54" s="33" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D54" s="33" t="inlineStr">
-        <is>
-          <t>Journal of Financial Data Science 8(2)</t>
-        </is>
-      </c>
-      <c r="E54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="F54" s="33" t="inlineStr">
-        <is>
-          <t>Portfolio optimisation with transaction costs</t>
-        </is>
-      </c>
-      <c r="G54" s="33" t="inlineStr">
-        <is>
-          <t>NOT YET REVIEWED - the vault note is an empty file.</t>
-        </is>
-      </c>
-      <c r="H54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="I54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="J54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="K54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="L54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="M54" s="33" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="N54" s="33" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="O54" s="33" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="P54" s="33" t="inlineStr">
-        <is>
-          <t>Likely relevant to Sub-gap 1 given the title, but nothing is recorded.</t>
-        </is>
-      </c>
-      <c r="Q54" s="33" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="R54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="S54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="T54" s="33" t="inlineStr">
-        <is>
-          <t>Not recorded.</t>
-        </is>
-      </c>
-      <c r="U54" s="33" t="inlineStr">
-        <is>
-          <t>NOT YET REVIEWED. The note file is empty. On the title alone this is likely to bear on Sub-gap 1, the modular framework for portfolio optimisation with transaction costs, so it should be read before Sub-gap 1 is defended.</t>
-        </is>
-      </c>
-      <c r="V54" s="33" t="inlineStr">
-        <is>
-          <t>Unknown until read.</t>
-        </is>
-      </c>
-      <c r="W54" s="33" t="inlineStr">
-        <is>
-          <t>[[Smart Trading Rule, A Modular Machine Learning Framework for Portfolio Optimization with Transaction Costs]] - EMPTY FILE</t>
-        </is>
-      </c>
-      <c r="X54" s="33" t="inlineStr">
-        <is>
-          <t>SPEAKS TO: probably A_T and the friction-aware evaluation layer, on the title alone.
-NOT YET REVIEWED, AND BLOCKED ON ACCESS RATHER THAN ON EFFORT. The paper is paywalled. Routes to try, in order: institutional access, interlibrary loan, or emailing the authors for a copy.
-WHY IT MATTERS: on its title it is a modular framework for portfolio optimisation WITH TRANSACTION COSTS, which is exactly Sub-gap 1's territory, and it may narrow that sub-gap further. Sub-gap 1 should not be presented as final until this has been read.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="409.6" customHeight="1">
-      <c r="A55" s="29" t="inlineStr">
+      <c r="A54" s="29" t="inlineStr">
         <is>
           <t>P54</t>
         </is>
       </c>
-      <c r="B55" s="30" t="inlineStr">
+      <c r="B54" s="30" t="inlineStr">
         <is>
           <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid–ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
         </is>
       </c>
-      <c r="C55" s="30" t="inlineStr">
+      <c r="C54" s="30" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D55" s="30" t="inlineStr">
+      <c r="D54" s="30" t="inlineStr">
         <is>
           <t>Journal of Financial Economics (JFE), volume 161, article 103916.</t>
         </is>
       </c>
-      <c r="E55" s="30" t="inlineStr">
+      <c r="E54" s="30" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jfineco.2024.103916 — accessed 4 October 2026. Code and data: github.com/eguidotti/bidask.</t>
         </is>
       </c>
-      <c r="F55" s="30" t="inlineStr">
+      <c r="F54" s="30" t="inlineStr">
         <is>
           <t>Low-frequency microstructure econometrics — estimation of the effective bid–ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin–Schultz (2012) / Abdi–Ranaldo (2017) lineage.</t>
         </is>
       </c>
-      <c r="G55" s="30" t="inlineStr">
+      <c r="G54" s="30" t="inlineStr">
         <is>
           <t>Produce an estimator of the effective bid–ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
 The object being estimated is the effective spread, not the quoted spread. The quoted spread is the posted distance between best bid and best ask; the effective spread is the realised distance between the transaction price and the unobserved fundamental price, S = 2D(P − P̃)/P̃, with D = +1 for buyer-initiated and −1 for seller-initiated trades. They differ because dealers often execute inside the quotes, and "one of this paper's headline empirical results is that the end-of-day quoted spread overstates the effective spread by up to 100%." For a cost model the effective spread is the right object and the harder one, since P̃ is never observed.
 The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid–ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed — Roll additionally required equally likely buys and sells; Corwin–Schultz and Abdi–Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
         </is>
       </c>
-      <c r="H55" s="30" t="inlineStr">
+      <c r="H54" s="30" t="inlineStr">
         <is>
           <t>US equities (NYSE / AMEX / NASDAQ) as the main empirical setting, plus a cryptocurrency application on Binance. No emerging or frontier market anywhere in the paper. The note records: "Emerging and thin markets" are represented only by the crypto section, which "is the closest thing here to an illiquid non-US market" and "has no benchmark whatsoever".</t>
         </is>
       </c>
-      <c r="I55" s="30" t="inlineStr">
+      <c r="I54" s="30" t="inlineStr">
         <is>
           <t>Two evaluations (a simulation and a CRSP–TAQ empirical study) plus three applications.
 Simulation: Corwin and Schultz (2012) design as reused by Abdi and Ranaldo (2017). 10,000 months, each 21 trading days, each day 390 minutes. Fundamental price P̃_m = P̃_{m−1}e^{σz}, P̃_0 = 1, z standard Gaussian. Daily sd 3%, per-minute sd 3%/√390. Trade prices are P̃_m times one minus (plus) half the spread, 50% chance of a bid (ask). Trade probability varied so expected trades per day runs from 1 to 390. On no-trade days the previous day's close is forward-filled into all four prices. Spreads tested: 0.50%, 1.00%, 2.00% through 8.00%.
@@ -7597,12 +7473,12 @@
 Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high–low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
         </is>
       </c>
-      <c r="J55" s="30" t="inlineStr">
+      <c r="J54" s="30" t="inlineStr">
         <is>
           <t>Daily (or intraday) open, high, low and close prices and nothing else. No quote feed, no trade-by-trade data, no vendor dependency. The derived quantities are: o_t, h_t, l_t, c_t as log-prices; η_t = (h_t + l_t)/2 the mid log-price; and the indicator τ_t that flags whether the high, the low and the previous close all coincide. The note flags the τ_t indicator as itself a usable feature — "the fraction of days on which the open or close coincides with the high or low, which falls out of the EDGE computation at no extra cost".</t>
         </is>
       </c>
-      <c r="K55" s="30" t="inlineStr">
+      <c r="K54" s="30" t="inlineStr">
         <is>
           <t>"There is no architecture, this is an estimator, and the whole mechanism rests on one indicator variable."
 τ_t = 0 if h_t = l_t = c_{t−1}, and 1 otherwise.
@@ -7621,47 +7497,47 @@
 Output: an effective spread in basis points per asset per period, from OHLC alone.</t>
         </is>
       </c>
-      <c r="L55" s="30" t="inlineStr">
+      <c r="L54" s="30" t="inlineStr">
         <is>
           <t>Not applicable — this is a closed-form econometric estimator with no agents, no decision and no orchestration. The note states it plainly: "This is tooling, not a competitor architecture, there is no agent in it and no trading decision, but it goes at the part of my design that is currently weakest."</t>
         </is>
       </c>
-      <c r="M55" s="30" t="inlineStr">
+      <c r="M54" s="30" t="inlineStr">
         <is>
           <t>Not applicable — the paper uses only OHLC prices and contains no textual or sentiment component. (Sentiment is out of scope for this project in any case, per the supervisor decision.)</t>
         </is>
       </c>
-      <c r="N55" s="30" t="inlineStr">
+      <c r="N54" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no disclosures, filings, retrieval or text of any kind. The only inputs are the four daily prices.</t>
         </is>
       </c>
-      <c r="O55" s="30" t="inlineStr">
+      <c r="O54" s="30" t="inlineStr">
         <is>
           <t>No volatility model is estimated, but volatility enters the paper twice as a nuisance that drives the estimator's error. First, through the truncation channel: because Ŝ² can come out negative in small samples, standard practice is to reset negatives to zero, and Jahan-Parvar and Zikes (2023) show this introduces a strong upward bias that does not decline with sample size, "with volatility as its primary driver". Second, through the spread-to-volatility ratio: the degradation of correlation with the TAQ benchmark over time is attributed by the authors to spreads shrinking relative to volatility, consistent with the spread-quintile table where correlation runs 17.84% in the narrowest quintile against 71.38% in the widest.
 The note also flags a tension with the volatility side of the project's own literature: Assumption 1 rules out serially correlated fundamental returns, "which sits uneasily beside the long-memory results on the ASPI and SL20 in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], though that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it."
 Estimation variance is roughly proportional to σ₁⁴/N for N observations at per-period volatility σ₁, so the standard error scales with σ₁²/√N — which is the formula behind the frequency result below.</t>
         </is>
       </c>
-      <c r="P55" s="30" t="inlineStr">
+      <c r="P54" s="30" t="inlineStr">
         <is>
           <t>This is the whole paper. EDGE measures the effective spread — the realised cost of a marginal trade — directly, in basis points, from OHLC. The discreteness correction is explicitly a function of how thinly the asset trades: the probability that the open or close coincides with the high or low is "a direct consequence of too few trades per period", running from about 25% for large-cap US stocks to 75% for small-caps over 1926–2021, peaking in the 1930s and 1940s, collapsing after 2000 with electronification to roughly 2–5% for large-caps while small-caps still sit near 15% at the end of the sample. The authors' own reading is that "the correction is less significant for recent samples and becomes essential for small stocks and for older periods, and crucially that it also depends on sampling frequency, since going from daily to intraday prices reduces the trades observed per interval and pushes the probability back up."
 What the paper does NOT handle: order size. "There is no order size anywhere in the model, so what EDGE measures is the cost of a marginal trade." The effective spread is computed from the transaction prices that happened, at whatever sizes they happened in, and the estimator has no mechanism for saying what a larger order would have paid.</t>
         </is>
       </c>
-      <c r="Q55" s="30" t="inlineStr">
+      <c r="Q54" s="30" t="inlineStr">
         <is>
           <t>Not applicable in the ML sense — there is no black box. The estimator is closed-form, every term is interpretable, and the discreteness correction has a direct structural reading (the denominator is one under continuous observation and shrinks in proportion to how often the price failed to move). Reproducibility is strong: implementations in several languages, the computed spread data, and a Harvard Dataverse replication package.</t>
         </is>
       </c>
-      <c r="R55" s="30" t="inlineStr">
+      <c r="R54" s="30" t="inlineStr">
         <is>
           <t>Baselines: ROLL (Roll 1984), CS (Corwin and Schultz 2012), AR (Abdi and Ranaldo 2017), plus the paper's own intermediate estimators OHLC and CHL. Benchmark truth is the Holden and Jacobsen (2014) TAQ-based effective spread, May 1993 – December 2021.
 Evaluation axes: (i) simulation bias as a function of expected trades per day from 390 down to 1; (ii) simulation mean and standard deviation across true spreads 0.50%–8.00%; (iii) empirical Pearson and Spearman correlation, MAPE, RMSE and fraction of non-positive estimates on 1,637,621 merged stock-months, cut by market venue, sub-period, size quintile and decile, spread quintile and trading-frequency quintile; (iv) daily versus minute sampling on 711,161 stock-months; (v) the Binance crypto application across daily / hourly / minute, which has no benchmark.
 The note records a caveat on the empirical comparison: "The comparison is descriptive throughout, no standard errors on the differences and no formal test, which at this sample size is defensible but means the quintile tables are read by eye."</t>
         </is>
       </c>
-      <c r="S55" s="30" t="inlineStr">
+      <c r="S54" s="30" t="inlineStr">
         <is>
           <t>1. Infrequent trading breaks the alternatives and not EDGE. At 390 trades per day all estimators are unbiased and recover the 1% simulated spread. By 100 trades per day CS estimates 0.75%; by around twenty trades per day it has fallen to 0.1%; and below roughly thirteen trades per day CS returns exactly zero. AR degrades more gracefully but is still biased down to about 0.30% at one trade per day and 0.62% at roughly two. EDGE tracks 1.00% across the entire range, including simulations where only a single trade per period is expected on average. The note: "This is the single most transferable result in the paper for my purposes and I report it as the paper's evidence rather than as a general claim, since the simulation's price process is a geometric Brownian motion and its no-trade handling is forward-filling rather than genuine absence."
 2. Variance. Under infrequent trading, mean estimate with sd in parentheses against the true spread:
@@ -7676,7 +7552,7 @@
 5. The discreteness term is itself a market-structure measurement: the coincidence probability ranges from ~25% (US large-cap) to 75% (small-cap) over 1926–2021, peaking in the 1930s–40s, collapsing after 2000 to 2–5% for large-caps with small-caps still near 15%.</t>
         </is>
       </c>
-      <c r="T55" s="30" t="inlineStr">
+      <c r="T54" s="30" t="inlineStr">
         <is>
           <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% — "a bias roughly seven times the quantity being measured" — and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
 2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid–ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information — Chen et al. (2017) being their example — is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
@@ -7687,7 +7563,7 @@
 7. A premise doing quiet work throughout: that the effective spread is the whole of the transaction cost, since nothing in the model has an order size in it. The paper never claims otherwise and the title is honest about scope.</t>
         </is>
       </c>
-      <c r="U55" s="30" t="inlineStr">
+      <c r="U54" s="30" t="inlineStr">
         <is>
           <t>- EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC — the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
 - The infrequent-trading bias result as external evidence that thin-book calibration is a real problem, not a rhetorical one: below roughly thirteen trades per day CS returns exactly zero and AR is biased down by about a third at a few trades per day, "which means any cost model built on those estimators would charge approximately nothing for trading the least liquid counters on the CSE. That is backwards in the most expensive possible direction." Worth citing directly in the proposal when defending the thin-book calibration item.
@@ -7697,7 +7573,7 @@
 - A positioning rule. EDGE is a 2024 JFE paper with public implementations, open spread data and a replication package, "so there is no contribution in running it on a new market and no reason to imply one." The defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered, and that the contribution is what an orchestrator does with a cost term that varies by counter and date rather than the estimator that produces it. "One sentence, offered before anyone asks."</t>
         </is>
       </c>
-      <c r="V55" s="30" t="inlineStr">
+      <c r="V54" s="30" t="inlineStr">
         <is>
           <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
 Second, the small-count regime is untested: the estimator is defined with three usable observations but the paper never characterises its behaviour there, and that is exactly the regime a CSE counter with five trading days in a month occupies.
@@ -7705,12 +7581,12 @@
 Fourth, no validation against a quote-based benchmark in an emerging or frontier market: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."</t>
         </is>
       </c>
-      <c r="W55" s="30" t="inlineStr">
+      <c r="W54" s="30" t="inlineStr">
         <is>
           <t>[[Efficient estimation of bid–ask spreads from open, high, low, and close prices]]</t>
         </is>
       </c>
-      <c r="X55" s="30" t="inlineStr">
+      <c r="X54" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_L above all — this is the measurement instrument the liquidity agent currently lacks — plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
 EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency — "all proxies for illiquidity rather than measurements of what a trade pays" — and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade — "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren–Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
@@ -7722,39 +7598,39 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="409.6" customHeight="1">
-      <c r="A56" s="29" t="inlineStr">
+    <row r="55" ht="409.6" customHeight="1">
+      <c r="A55" s="29" t="inlineStr">
         <is>
           <t>P55</t>
         </is>
       </c>
-      <c r="B56" s="30" t="inlineStr">
+      <c r="B55" s="30" t="inlineStr">
         <is>
           <t>Wang, X., Hyndman, R.J., Li, F. and Kang, Y. (2023). Forecast combinations: An over 50-year review. International Journal of Forecasting, 39(4), 1518–1547. DOI: 10.1016/j.ijforecast.2022.11.005. arXiv version 2205.04216v2 dated 26 September 2022. Affiliations: Xiaoqian Wang and Yanfei Kang at Beihang, Rob J Hyndman at Monash, Feng Li at the Central University of Finance and Economics — "about as authoritative an author list as this particular topic has". Citekey: wangForecastCombinations50year2023.</t>
         </is>
       </c>
-      <c r="C56" s="30" t="inlineStr">
+      <c r="C55" s="30" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="D56" s="30" t="inlineStr">
+      <c r="D55" s="30" t="inlineStr">
         <is>
           <t>International Journal of Forecasting, 39(4), 1518–1547.</t>
         </is>
       </c>
-      <c r="E56" s="30" t="inlineStr">
+      <c r="E55" s="30" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ijforecast.2022.11.005 (arXiv 2205.04216v2).</t>
         </is>
       </c>
-      <c r="F56" s="30" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>Forecast combination / forecast pooling — a narrative review of over fifty years of work on combining multiple forecasts of the same quantity, from Bates and Granger (1969) (and behind that Galton's 1906 ox-weight competition, where the average of 787 estimates came close to the animal's actual weight) through to the feature-based cross-learning methods that placed in M4. Organising split: point forecast combinations (section 2), probabilistic forecast combinations (section 3), eight open problems in closing, with a running commentary on which R and Python packages implement what.
 This is the most direct body of prior art on the orchestration half of my design. As the note puts it: "My orchestrator computes w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) over four heterogeneous agent outputs, and that object is a time-varying, feature-conditioned linear combination, which is a named construct in this literature with five decades of results attached to it, a good number of them inconvenient." It belongs next to the RL-in-quant-finance survey as the other half of the prior art: "that one establishes that coordination protocols among heterogeneous agents are underexplored in RL, this one establishes what fifty years of statistics already knows about combining their outputs once they exist."</t>
         </is>
       </c>
-      <c r="G56" s="30" t="inlineStr">
+      <c r="G55" s="30" t="inlineStr">
         <is>
           <t>Update the field's standing reviews — Clemen (1989) and Timmermann (2006) — and, structurally, set point and probabilistic combination side by side for the first time in a single survey. Three gaps motivate it:
 1. Both standing reviews predate the entire cross-learning and meta-learning strand, the M4 and M5 competitions, most of the probabilistic combination work, and the open-source tooling that now carries these methods into practice. The authors' Web of Science count puts combination papers at "13.80% of all published forecasting papers in 2021", up from roughly 1% in 1969, "so the case for an update is quantitative rather than rhetorical."
@@ -7764,22 +7640,22 @@
 SCOPE BOUND (the note flags this as bounding everything else): the authors take the individual forecasts "as given", do not discuss how they are generated, and restrict attention to forecasts derived from separate and non-interfering models for a single target series. Two adjacent literatures are named and excluded: manipulating one series into many and combining the results (Petropoulos and Spiliotis' "wisdom of the data", covering theta, bagging and temporal aggregation), and forecast reconciliation for hierarchical series following Hyndman et al. (2011). The target is always a realised value of one series and the loss is almost always quadratic. "There are no portfolios, no transaction costs, no execution, and no decisions. So this is prior art on the weighting mechanism and on the evidence about weighting, not on anything downstream of it, and the non-interfering assumption in particular is one my design may violate."</t>
         </is>
       </c>
-      <c r="H56" s="30" t="inlineStr">
+      <c r="H55" s="30" t="inlineStr">
         <is>
           <t>General forecasting, not finance-specific. Named application areas are retail, energy, economics, epidemiology and meteorology; the financial examples are macroeconomic series such as inflation and GDP growth. Competition datasets are M3, M4 (100,000 series), M5 and FRED. "Emerging and thin markets are absent from the entire paper."</t>
         </is>
       </c>
-      <c r="I56" s="30" t="inlineStr">
+      <c r="I55" s="30" t="inlineStr">
         <is>
           <t>No dataset of its own — the authors run no experiment. The evidence base is other people's results on M-competition data (M3, M4 at 100,000 series, M5), FRED, and individual case studies. Coverage spans 1969 to roughly 2022, with the Web of Science publication-share chart (Figure 1) the only quantitative artefact the authors produce. "There is no protocol, no screening count, and no stated inclusion criterion anywhere in the paper."</t>
         </is>
       </c>
-      <c r="J56" s="30" t="inlineStr">
+      <c r="J55" s="30" t="inlineStr">
         <is>
           <t>Univariate time series forecasts (point and probabilistic) as the inputs to be combined. The feature strand is the one that matters: FFORMA (Montero-Manso et al., 2020) extracts 42 statistical features of the series with the tsfeatures package and maps them to weights via an XGBoost meta-model. Collopy and Armstrong (1992) is the ancestor — a hand-built rule base of 99 rules over 18 time series features and four statistical models — and "the line from there to XGBoost over 42 features is the clearest trajectory in the paper." The feature pool has itself become a research object: Lemke and Gabrys (2010) add six features measuring diversity of the method pool rather than properties of the series, and Kang et al. (2021) build a combination model from a diversity matrix alone.</t>
         </is>
       </c>
-      <c r="K56" s="30" t="inlineStr">
+      <c r="K55" s="30" t="inlineStr">
         <is>
           <t>Not an architecture — a taxonomy of weighting schemes. The framing holding section 2 together is a one-dimensional aggregator over an N-vector of h-step-ahead forecasts:
 ỹ_{T+h|T} = C(ŷ_{T+h|T}; w_{T+h|T}), linear case ỹ_{T+h|T} = w'_{T+h|T} ŷ_{T+h|T}
@@ -7810,46 +7686,46 @@
 Quantile combination (Vincentization, after Vincent 1912): Q̃_{T+h|T}(τ) = Σ w_{T+h|T,i} Q_{T+h|T,i}(τ) for 0 &lt; τ ≤ 1. The geometric statement, which the note calls "the clearest sentence in section 3": "quantile combination averages the individuals' cdfs horizontally while linear pooling averages them vertically." If components are in the same location-scale family the quantile average stays in it, so averaging normals gives a normal and is always unimodal, where linear pooling can be multimodal. Both share the same mean. Quantile averaging is sharper because it does not absorb disagreement in location as extra spread — Lichtendahl et al. (2013) and Busetti (2017) both come down on its side, the former arguing the average probability forecast is generally under-confident while the average quantile forecast is always sharper.</t>
         </is>
       </c>
-      <c r="L56" s="30" t="inlineStr">
+      <c r="L55" s="30" t="inlineStr">
         <is>
           <t>Not applicable as implemented — "a paper with no architecture in it, no trading decision anywhere, and nothing resembling an agent". But this is the closest named prior art to my orchestrator: combination weights over heterogeneous producers are exactly the orchestration object, and the survey supplies the ladder from equal weights to feature-conditioned meta-learned weights.
 CRITICAL CONSTRAINT: the non-interfering assumption. "The components here are separate models that do not see each other's outputs. Every LLM multi-agent trading system in my reading violates that: [[TradingAgents, Multi-Agents LLM Financial Trading Framework]] has agents debating, [[HedgeAgents, A Balanced-aware Multi-agent Financial Trading System]] runs conferences, and even the ones that do not communicate share the same underlying price history and the same disclosures. So the clean statistical properties derived here, the unbiasedness of the combination and the variance bound, hold under an assumption my pool does not satisfy. My four agents read overlapping data by construction, and the paper's own observation that component forecasts trained on overlapping information sets produce highly correlated errors is the mechanism by which that bites."
 Subset selection is named as prior art for an abstention channel: the paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme, citing Li et al. (2022).</t>
         </is>
       </c>
-      <c r="M56" s="30" t="inlineStr">
+      <c r="M55" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no textual or sentiment component anywhere; the inputs are numerical forecasts of a single target series. (Sentiment is out of scope for this project regardless, per the supervisor decision of 20 September 2026, status Final.)</t>
         </is>
       </c>
-      <c r="N56" s="30" t="inlineStr">
+      <c r="N55" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no documents, filings, retrieval or text. The only relevance is structural: the abstention channel exists because my fundamental agent will have no disclosure to work from "more than half the time", and the paper supplies the vocabulary (time-varying subset selection) for that.</t>
         </is>
       </c>
-      <c r="O56" s="30" t="inlineStr">
+      <c r="O55" s="30" t="inlineStr">
         <is>
           <t>No volatility modelling. One result touches the high-volatility regime: Zischke et al. (2022) report that when forecasting during high-volatility periods, weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample — which the note reads as "a result about choosing what to score rather than about how elaborate the pooling function is". This is the single exception in section 3 where sophistication earned its keep, and it is region-specific.
 Second-order relevance: the probabilistic variance decomposition means a deliberately heterogeneous pool produces an under-confident interval, which bears on any risk interval the orchestrator might emit.</t>
         </is>
       </c>
-      <c r="P56" s="30" t="inlineStr">
+      <c r="P55" s="30" t="inlineStr">
         <is>
           <t>Not applicable — "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages."</t>
         </is>
       </c>
-      <c r="Q56" s="30" t="inlineStr">
+      <c r="Q55" s="30" t="inlineStr">
         <is>
           <t>Interpreting combination weights is one of the paper's eight stated future directions — in the authors' words, "discussing if, how, and when it is helpful to interpret combination weights", prompted by the observation that some schemes drive poor forecasts to zero asymptotically while individually bad forecasts can still be useful. The paper also flags in future directions that "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts", which the note treats as a direct warning about significance testing on a weighted output.</t>
         </is>
       </c>
-      <c r="R56" s="30" t="inlineStr">
+      <c r="R55" s="30" t="inlineStr">
         <is>
           <t>The paper runs no evaluation of its own. "The authors run no experiment of their own and aggregate no results from the papers they cover, so there is no table anywhere comparing two weighting schemes on shared data. Every performance claim in the paper is a report of a single study's finding, which means I can cite this for the existence and the lineage of a method but never for its relative performance."
 The de facto benchmark throughout is the equally weighted average, and the evidence base is M-competition results plus individual case studies.</t>
         </is>
       </c>
-      <c r="S56" s="30" t="inlineStr">
+      <c r="S55" s="30" t="inlineStr">
         <is>
           <t>1. THE FORECAST COMBINATION PUZZLE — the field's central empirical result, fifty years old and still open. Stock and Watson (2004) named it: theoretically sophisticated weighting schemes should dominate the simple average, and empirically the simple average dominates them. Evidence runs from Makridakis et al. (1982) in the original M-competition through to M4, where "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) is the most recent restatement across M3, M4, M5 and FRED, finding that the winning combination method differs by data source while simple averaging shows, on average, more gain than complex methods. The explanations all centre on estimation error: Timmermann (2006) attributes it to parameter estimation error that simple schemes avoid entirely; Smith and Wallis (2009) to finite-sample estimation effects; Claeskens et al. (2016) prove that treating the weights as random rather than fixed can introduce bias into combinations of unbiased components and inflate the combination's variance past the fixed-weight case; Blanc and Setzer (2020) frame it as a bias-variance tradeoff where equal weights underfit and estimated weights carry estimation variance; Elliott (2011) bounds the available gain from optimal over equal weights and finds it is usually too small to pay for the estimation.
 2. CORRELATIONS AMONG FORECAST ERRORS SHOULD BE IGNORED RATHER THAN ESTIMATED — an empirical finding, not a convenience. Bates and Granger argued correlations are poorly estimated in practice and should be left out; Newbold and Granger (1974) and Winkler and Makridakis (1983) tested that over more series, methods and horizons and concluded that "combinations ignoring correlations are more successful than those attempting to account for them". The mechanism is visible in the optimal-weight formula: the full covariance matrix needs N(N+1)/2 parameters from the same short error history that a diagonal treatment needs N from, and with highly correlated forecast errors the sample estimator of Σ is unstable. Chan et al. (1999) add that OLS combination performs very poorly when N is large, which pushes the literature toward principal components regression and clustering.
@@ -7860,7 +7736,7 @@
 7. NONLINEAR COMBINATION OF POINT FORECASTS IS A THIN LITERATURE AND THE AUTHORS SAY SO PLAINLY. Two forms: a neural network over the individual forecasts (Donaldson and Kamstra, 1996), with purely linear and purely nonlinear specifications as special cases; and an additive pairwise term Σ_{i&lt;j} π_{ij} v_{ij} where v_{ij} is a nonlinear function of forecasts i and j. Reported results generally dominate simple averaging, OLS weights and performance-based weights, but the authors' own assessment of that evidence is that it rests on "fewer than ten time series, possibly hand-picked", alongside neglect of error correlations, unstable parameter estimation and multicollinearity from overlapping information sets.</t>
         </is>
       </c>
-      <c r="T56" s="30" t="inlineStr">
+      <c r="T55" s="30" t="inlineStr">
         <is>
           <t>1. Narrative review with no protocol, no screening counts and no meta-analysis, "so it establishes what exists and not what works." The Web of Science query is given in full but only for the Figure 1 publication-share chart, not for the review's own selection. Nothing states how papers were found, how many were screened, or what put one in or out. The authors run no experiment and aggregate no results, so there is no table anywhere comparing two weighting schemes on shared data. "I can cite this for the existence and the lineage of a method but never for its relative performance. This is the same structural weakness I recorded against [[The Evolution of Reinforcement Learning in Quantitative Finance, A Survey]], and the two surveys share it for the same reason, that coverage and adjudication are different jobs."
 2. The puzzle is reported rather than resolved, and where the paper gestures at a contradiction there is not actually one. Claeskens et al. (2016) derive that random combination weights can introduce bias and inflate the variance of the combined forecast relative to fixed weights; Zischke et al. (2022) are quoted as finding the opposite, that weight estimation imparts no bias or variability at all, and the authors record the opposition in a single clause and move on. The note's own reading: the opposition is a compression rather than a real disagreement — "Claeskens is a finite-sample result about the MSE of the combined point forecast under unbiased components, Zischke is a first-order asymptotic result about the sampling variability of the out-of-sample expected score", so the two answer different questions about different objects and neither refutes the other. "The genuine limitation is that the review leaves the question my contribution turns on, whether estimated weights can be expected to beat fixed ones, standing open, while the work that takes it considerably further was already in circulation when the review went to press."
@@ -7871,7 +7747,7 @@
 7. (Recorded in the note as a WARNING against the paper, from work that postdates it.) The puzzle may be substantially a testing artefact. Frazier, Covey, Martin and Poskitt, "Solving the Forecast Combination Puzzle", Monash EBS working paper 18/2023 and arXiv:2308.05263, subsumes both positions above, characterising Claeskens as "more general than but ultimately commensurate with Smith and Wallis (2009)", i.e. one context-specific explanation among several rather than the general one. Their argument is that the puzzle is a consequence of the two-step estimation methodology itself: because estimated weights impart no first-order sampling variability into the usual predictive-accuracy statistic, that statistic converges to a non-standard generalised chi-squared rather than a normal, and their Theorem 1 states that when two weight vectors lie within O(T^{−1/4−ε}) of each other "the test has no power to distinguish them at all". An underpowered test defaults to the naive approach, which is the puzzle. Their remedy is one-step joint estimation of the constituent parameters and the combination weights against the final loss, which their Theorem 2 shows restores power. The note is explicit that this "needs a note of its own, and its publication status needs checking before it is cited as anything other than a working paper."</t>
         </is>
       </c>
-      <c r="U56" s="30" t="inlineStr">
+      <c r="U55" s="30" t="inlineStr">
         <is>
           <t>- A lineage and a precise statement of what is new, which the note judges "a stronger framing than novelty". My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) is a time-varying feature-conditioned linear combination, and the paper contains both halves separately: time-varying weights through the Kalman-filter and smooth-transition line, feature-conditioned weights through FFORMA. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That reads as a generalisation along an identified axis rather than new machinery. It also tells me what the honest comparison is: FFORMA's structure — a gradient-boosted meta-model mapping features to a weight simplex — is available to me as an implementation choice, "and if I use something simpler I should say why rather than let it look like I did not know."
 - The hardest possible equal-weight baseline, plus a falsification condition to pre-register.
@@ -7884,7 +7760,7 @@
 - A warning on inference: "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts."</t>
         </is>
       </c>
-      <c r="V56" s="30" t="inlineStr">
+      <c r="V55" s="30" t="inlineStr">
         <is>
           <t>The review contains weights that change over time and weights that change as a regression function of covariates, "and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state." The two nearest things are Deutsch et al.'s smooth transition specification, where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step. That is the axis along which my weighting function generalises existing work.
 Second, the review leaves standing open the question my contribution turns on — whether estimated weights can be expected to beat fixed ones — and its own two guidelines on the matter cut in opposite directions, with the paper clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature.
@@ -7893,12 +7769,12 @@
 Fifth, subset selection has, in the paper's own assessment, "received scant attention, is mainly trimming on expertise alone", and "most existing algorithms are ad hoc and lack statistical rationale" — so a principled selection rule driven by a structural property of the output is defensible ground.</t>
         </is>
       </c>
-      <c r="W56" s="30" t="inlineStr">
+      <c r="W55" s="30" t="inlineStr">
         <is>
           <t>[[Forecast combinations, An over 50-year review]]</t>
         </is>
       </c>
-      <c r="X56" s="30" t="inlineStr">
+      <c r="X55" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: The orchestrator above everything else — this is the prior art for the weighting function itself, and the note is blunt that it is being written up precisely because "it is the most direct body of prior art on the half of my design I have covered least". Also the abstention channel (named here as time-varying subset selection), the confidence term C_{i,t} (via quantile averaging and calibrated intervals), the agent pool design (diversity as a measurable quantity rather than an asserted one), the explainability claim, and — most consequentially — the entire evaluation design.
 EFFECT ON MAIN GAP: THIS IS THE PAPER THAT BOTH LEGITIMISES AND THREATENS THE MAIN GAP, AND BOTH HALVES HAVE TO BE CARRIED THROUGH HONESTLY.
@@ -7920,49 +7796,49 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="409.6" customHeight="1">
-      <c r="A57" s="29" t="inlineStr">
+    <row r="56" ht="409.6" customHeight="1">
+      <c r="A56" s="29" t="inlineStr">
         <is>
           <t>P56</t>
         </is>
       </c>
-      <c r="B57" s="30" t="inlineStr">
+      <c r="B56" s="30" t="inlineStr">
         <is>
           <t>Gibbs, I. and Candès, E. (2021). Adaptive Conformal Inference Under Distribution Shift. Available from https://doi.org/10.48550/ARXIV.2106.00170 [Accessed 4 October 2026]. Citekey gibbsAdaptiveConformalInference2021. Authors: Isaac Gibbs and Emmanuel Candès, both in Stanford statistics, Candès also in mathematics. Venue per frontmatter: arXiv; the note's body records it as NeurIPS 2021. DOI: 10.48550/ARXIV.2106.00170. Zotero item: zotero://select/library/items/KZFWZYSI. Volume/pages: Not recorded in the note. Reference implementation in R at github.com/isgibbs/AdaptiveConformal.</t>
         </is>
       </c>
-      <c r="C57" s="30" t="inlineStr">
+      <c r="C56" s="30" t="inlineStr">
         <is>
           <t>2021 (frontmatter year, and the note's body dates it to NeurIPS 2021).</t>
         </is>
       </c>
-      <c r="D57" s="30" t="inlineStr">
+      <c r="D56" s="30" t="inlineStr">
         <is>
           <t>arXiv in the frontmatter; the note's body states "NeurIPS 2021". Both are recorded in the note, so I record both.</t>
         </is>
       </c>
-      <c r="E57" s="30" t="inlineStr">
+      <c r="E56" s="30" t="inlineStr">
         <is>
           <t>https://doi.org/10.48550/ARXIV.2106.00170 — code at github.com/isgibbs/AdaptiveConformal.</t>
         </is>
       </c>
-      <c r="F57" s="30" t="inlineStr">
+      <c r="F56" s="30" t="inlineStr">
         <is>
           <t>Distribution-free uncertainty quantification / conformal prediction under distribution shift. This is a statistics methods paper and explicitly tooling rather than a competitor architecture: in my own words from the note, "there are no agents here, nothing resembling an orchestrator and no trading decision anywhere in it". It is the paper that introduced adaptive conformal inference (ACI). I file it alongside [[Predict the Future from the Past, On the Temporal Data Distribution Shift in Financial Sentiment Classifications]] as "the other half of the shift problem, that note measuring how much a fitted model decays over time and this one giving a mechanism that stays calibrated while it does."</t>
         </is>
       </c>
-      <c r="G57" s="30" t="inlineStr">
+      <c r="G56" s="30" t="inlineStr">
         <is>
           <t>Standard conformal prediction wraps any black-box regressor in a prediction set with a marginal coverage guarantee, but that guarantee rests on the calibration data and the test point being exchangeable, "which no financial time series satisfies". The specific failure the authors name in finance is that market behaviour shifts in response to legislation or major world events, which breaks exchangeability "in exactly the periods where a coverage statement would matter most". The objective is to drop the exchangeability assumption by turning miscoverage into a control problem: carry a single scalar alpha_t, compare the realised coverage of yesterday's interval against the target, and nudge alpha_t up or down by a fixed step. The reframing that makes this tractable is that the shift becomes a one-dimensional learning problem: rather than modelling how P(X_t, Y_t) changes, "which is hopeless", they define the realised miscoverage M_t(alpha) := P(S_t(X_t,Y_t) &gt; Q_hat_t(1-alpha)) and the optimal alpha_t* := sup{beta in [0,1] : M_t(beta) &lt;= alpha}, then track alpha_t* online. "Everything about the data generating process is compressed into the movement of a single parameter, which is what makes the distribution-free result possible and is also... what the result is silent about."
 Positioning against the two prior treatments of shift, both of which handle a single train-to-test transition rather than a continuously moving target: Tibshirani et al. reweight the calibration data by the likelihood ratio P_1(X)/P_0(X), which requires Y | X to be constant between training and test and the ratio itself to be known or accurately estimated, "neither of which holds for a market regime change"; Cauchois et al. form sets valid whenever D_f(P_1 || P_0) &lt;= rho by fixing a conservative alpha_rho in advance. The two differences the authors draw are that they estimate the optimal alpha* satisfying M(alpha*) = alpha rather than fixing a conservative value, and that they work in a fully online setting where the distribution moves at every step.</t>
         </is>
       </c>
-      <c r="H57" s="30" t="inlineStr">
+      <c r="H56" s="30" t="inlineStr">
         <is>
           <t>Two demonstration domains, neither of them a trading system. (1) Daily GARCH volatility prediction for twelve US stocks and indices, inputs taken from publicly available WSJ daily open-price datasets. (2) County-level US election-night forecasting, replicating the Washington Post's 2020 model over roughly 3,111 matched US counties. No frontier or emerging market anywhere in the paper; no CSE data.</t>
         </is>
       </c>
-      <c r="I57" s="30" t="inlineStr">
+      <c r="I56" s="30" t="inlineStr">
         <is>
           <t>Volatility experiment (the one I would be reimplementing):
 - Target: realised volatility V_t = R_t^2, with R_t = (P_t - P_{t-1})/P_{t-1}.
@@ -7974,14 +7850,14 @@
 Election experiment: conformalised quantile regression over 3,111 matched US counties, predictions starting once 500 counties have reported, each step splitting observed data 75/25 into training and calibration and refitting a linear quantile regression. Counties are ordered by time zone, east coast first and Hawaii last, so the covariate distribution drifts monotonically rather than jumping — "the shift is manufactured but realistic".</t>
         </is>
       </c>
-      <c r="J57" s="30" t="inlineStr">
+      <c r="J56" s="30" t="inlineStr">
         <is>
           <t>Pure numeric price time series (daily open prices) in the volatility experiment, and tabular cross-sectional county covariates in the election experiment. No text, no filings, no order-book data, no alternative data of any kind. The single engineered quantity that carries the method is the conformity score. For volatility it is normalised by the predicted variance:
 S_t := |V_t - (sigma_hat_t^t)^2| / (sigma_hat_t^t)^2
 where the superscript is the re-fitting index, so (sigma_hat_t^t)^2 is the GARCH point prediction from a model fitted using only data in [t-1250, t), and "the score at each step has seen nothing after t-1". That normalisation choice "turns out to carry as much weight as the adaptation itself".</t>
         </is>
       </c>
-      <c r="K57" s="30" t="inlineStr">
+      <c r="K56" s="30" t="inlineStr">
         <is>
           <t>"There is no architecture, which is the point." ACI is a wrapper and the algorithm is one line. Define the miscoverage event err_t := 1{Y_t not in C_hat_t(alpha_t)}, then update:
 alpha_{t+1} := alpha_t + gamma(alpha - err_t)
@@ -7997,45 +7873,45 @@
 Output: a prediction interval per step at the target coverage, plus the adapted miscoverage level alpha_t as a by-product series.</t>
         </is>
       </c>
-      <c r="L57" s="30" t="inlineStr">
+      <c r="L56" s="30" t="inlineStr">
         <is>
           <t>Not applicable — this is a single-model statistical wrapper with no agents, no orchestrator and no decision layer. In the note's words, "there are no agents here, nothing resembling an orchestrator and no trading decision anywhere in it". What it supplies instead is a scalar state variable, alpha_t, that an orchestrator elsewhere could consume. The property I single out is that ACI "has the useful property of not being a detector at all: alpha_t moves continuously, so the shift measurement and the response to it are the same quantity, which is a better fit for a weighting function than a binary alarm."</t>
         </is>
       </c>
-      <c r="M57" s="30" t="inlineStr">
+      <c r="M56" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no text, no sentiment component anywhere in this paper. Sentiment is in any case out of scope for my project.</t>
         </is>
       </c>
-      <c r="N57" s="30" t="inlineStr">
+      <c r="N56" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no filings, no retrieval, no document processing of any kind. The paper's only connection to A_F in my design is by analogy: the scope revision gave a worked example of structural confidence for A_F (does the extracted program parse, does every argument trace to a retrieved figure) and left the other three agents open; ACI supplies the analogue for A_V.</t>
         </is>
       </c>
-      <c r="O57" s="30" t="inlineStr">
+      <c r="O56" s="30" t="inlineStr">
         <is>
           <t>This is the paper's headline empirical domain. The point predictor is GARCH(1,1) on realised volatility V_t = R_t^2, refit on a trailing 1,250-day window, with the conformity score normalised by the predicted variance. The adaptation is substantial rather than cosmetic: across the four main-figure stocks alpha_t ranges between about 0.035 and 0.17 against a target of 0.1, so "at its extremes the method is targeting 96.5% coverage in some periods and 83% in others to achieve 90% on average". The troughs line up with crises, Fannie Mae and BlackBerry both bottoming out near 0.035 through 2008 and 2009, "which is the method widening its intervals hard when the GARCH fit is worst". At gamma = 0.005 a single miss moves alpha_t by 0.0045, so these swings take hundreds of days to develop and the series is slow-moving by construction, "in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]". The alpha_t trajectories "read as a volatility-regime series in their own right".
 Critically, the risk quantity produced is a coverage statement and not a width statement: see LIMITATIONS. The paper never attaches an interval to a position size or any other risk-budgeting decision.</t>
         </is>
       </c>
-      <c r="P57" s="30" t="inlineStr">
+      <c r="P56" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no liquidity variables, no spreads, no turnover, no execution cost anywhere in the paper. The liquidity question enters only in my transfer analysis: on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade."</t>
         </is>
       </c>
-      <c r="Q57" s="30" t="inlineStr">
+      <c r="Q56" s="30" t="inlineStr">
         <is>
           <t>No attribution or interpretability machinery, and none needed — the method is a single scalar recursion and is fully transparent by construction. The interpretable artefact it produces is the alpha_t trajectory itself, which can be read directly as how badly the fitted model is tracking the market at each date. The theory is reported honestly in a way that matters for interpretation: the appendix comparison shows the naive bound decays as O(1/(T sqrt(epsilon_1))) and therefore *increases* as the shift size epsilon_1 shrinks, which the authors call undesirable, while the HMM-based bound decreases with the shift, and "both are reported side by side rather than only the flattering one".</t>
         </is>
       </c>
-      <c r="R57" s="30" t="inlineStr">
+      <c r="R56" s="30" t="inlineStr">
         <is>
           <t>Baselines: fixed alpha_t = alpha on the same rolling window, and an i.i.d. Bernoulli(0.1) sequence. The Bernoulli comparator is the right benchmark and not a strawman: "A perfectly calibrated method still produces a random coverage sequence, so a local coverage curve that wanders around 0.9 is not evidence of failure. The grey line is the moving average of an i.i.d. Bernoulli(0.1) sequence and shows how much wandering is expected from a method that is correct by construction. The test is therefore whether the adaptive curve stays inside that band, not whether it sits on 0.9, a more honest bar than most calibration plots set."
 Metrics: localCov (average coverage over the most recent 500 days) and quantile loss. Those are the only two. There is no decision-level evaluation of any kind, no cost attached to an interval that is too wide, and no comparison against any recalibration scheme beyond fixed-alpha on the same rolling window.
 An ablation on the score design is run: the normalised score S_t is replaced with the unnormalised S_tilde_t := |V_t - sigma_hat_t^2|.</t>
         </is>
       </c>
-      <c r="S57" s="30" t="inlineStr">
+      <c r="S56" s="30" t="inlineStr">
         <is>
           <t>- The non-adaptive method fails visibly and the adaptive one stays inside the Bernoulli band on all twelve names, with 2008 producing the clearest separation. Fannie Mae: fixed-alpha local coverage falls to roughly 0.83 against a target of 0.9 and stays depressed for most of 2008 and 2009, while the adaptive curve dips and recovers within the Bernoulli range. BlackBerry shows the same shape in 2008. AMD shows a fixed-alpha trough near 0.835 around 2016 and an over-covering excursion to 0.96 in 2004. Nvidia shows a trough near 0.85 across 2016 and 2017. "The useful reading is that the failure is two-sided, the fixed method over-covers as often as it under-covers, so what's being fixed is calibration drift rather than a conservatism bug." Caveat I flag in the note: the four stocks shown were selected out of twelve because they showed a clear failure of the non-adaptive method, which the authors state plainly, "so the main figure is a demonstration of the failure mode rather than a sample of typical behaviour, and the eight appendix panels are the ones to read for that."
 - alpha_t moves across roughly a fourfold range, about 0.035 to 0.17 against a 0.1 target.
@@ -8044,7 +7920,7 @@
 - Election night: the fixed-alpha method incurs large troughs in local coverage at the time-zone changes, falling to about 0.825 and spending most of the sequence below 0.875, while the adaptive method holds near 0.9 with deviations comparable to the Bernoulli sequence. I rate this experiment as mattering more to me than the volatility panels, "because the shift is structural and predictable from the data ordering rather than driven by an exogenous shock, which is the shape of a cross-sectional screening problem."</t>
         </is>
       </c>
-      <c r="T57" s="30" t="inlineStr">
+      <c r="T56" s="30" t="inlineStr">
         <is>
           <t>- The guarantee is about coverage and says nothing about width, and no width or efficiency number appears anywhere in the paper. Proposition 4.1 is satisfied by a sequence that alternates between infinite and empty prediction sets in the right proportion, and the mechanism that makes it assumption-free is precisely the one that permits this: when alpha_t &lt; 0 the set is all of R and err_t = 0 by construction, which is how the proof of Lemma 4.1 gets its contradiction. "There is no table of average interval widths, no comparison of width against the fixed-alpha method, and no statement of how often alpha_t goes non-positive in the experiments." The alpha_t trajectories suggest it doesn't happen on these twelve stocks, the minimum sitting near 0.035, "but that's inference from a plot rather than a reported quantity, and a method sold on robustness to crises should report what its intervals cost in the crisis". I have not found that evaluation in the literature I have covered.
 - The results that hold at a single time step require a small shift, a stationary chain and a time-invariant quantile function, "which is close to the regime where I wouldn't need the method". Theorem 4.2 bounds the expected squared deviation of marginal coverage by a quantity proportional to E[|alpha*_{A_{t+1}} - alpha*_{A_t}|], which the authors interpret as a measurement of shift size, "so the bound is informative exactly when the shift is small and vacuous when it is large". The discussion concedes the fixed-Q_hat_t assumption directly and says it would be interesting to determine if similar results hold when Q_hat_t is fit online on recent data — which is what the volatility experiment actually does. "So the headline experiment sits outside the conditions of the sharper theory, and the only guarantee covering it is the long-run average one."
@@ -8054,7 +7930,7 @@
 - Data-depth constraint, flagged in the note as a hard constraint on transferring this and not a tuning detail: "Five years of daily data per counter is roughly thirteen times what my per-counter archive holds at 374 trading days, and the calibration set is drawn from the same window, so shrinking it degrades the GARCH fit and the empirical quantile simultaneously. The index track at ten years daily clears it comfortably; the per-counter track does not."</t>
         </is>
       </c>
-      <c r="U57" s="30" t="inlineStr">
+      <c r="U56" s="30" t="inlineStr">
         <is>
           <t>- The ACI update itself, as an adopted off-the-shelf component wrapping A_V's volatility forecast, with the normalised conformity score and the weighted variant (w_s proportional to 0.95^{t-s}) as the starting point rather than the plain update, because the weighted trajectories are smoother and my sample is short.
 - alpha_t as a candidate conditioning variable for the orchestrator: a continuous state variable rather than a binary alarm, running on the same daily index the orchestrator runs on, with no threshold to hand-tune. The concrete proposal recorded in the note is "to carry alpha_t as a candidate addition to the conditioning set and test it on the ablation protocol against the existing four terms rather than adopting it", a discipline [[Predicting financial market stress with machine learning]] makes the case for "after what 44 predictors on 84 observations did to that paper's out-of-sample performance."
@@ -8066,7 +7942,7 @@
 - The honesty discipline on claiming: "Claim this as an adopted component and not as a contribution, and say so before anyone asks."</t>
         </is>
       </c>
-      <c r="V57" s="30" t="inlineStr">
+      <c r="V56" s="30" t="inlineStr">
         <is>
           <t>- No link from calibration to a decision. The method stops at the interval. Nothing in the paper attaches an interval to a position size, a weight, or an abstention. "That's a fair scope for a statistics paper and a gap for anyone using it inside a trading system, where an interval has a position size attached."
 - No width accounting. Coverage is guaranteed, width is unreported and in principle unbounded. The failure mode this leaves open is exactly the one I have to avoid: "A volatility agent that achieves nominal coverage by widening its intervals during crises is well calibrated and useless for position sizing, which is the same failure as an orchestrator whose weights move impressively in the two or three most volatile CSE months and are inert otherwise."
@@ -8076,12 +7952,12 @@
 - No pooling-versus-per-unit guidance when the per-unit sample is too short for the refit window. The honest options I record are "a shorter joint window with the calibration degradation reported, or pooling scores across counters, which breaks the per-counter conditioning the method relies on."</t>
         </is>
       </c>
-      <c r="W57" s="30" t="inlineStr">
+      <c r="W56" s="30" t="inlineStr">
         <is>
           <t>[[Adaptive Conformal Inference Under Distribution Shift]]</t>
         </is>
       </c>
-      <c r="X57" s="30" t="inlineStr">
+      <c r="X56" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: C_{i,t} above all — specifically C_{V,t}, the confidence term for A_V — plus the abstention channel, the orchestrator's conditioning set (as a candidate fifth term), the distribution-shift item in the evaluation plan, and the data-depth discussion. It touches nothing in A_T, A_F or A_L directly, and it is tooling rather than a competing architecture, so it cannot close or threaten the orchestration claim in either direction.
 EFFECT ON MAIN GAP: It strengthens the main gap in two distinct ways and leaves the claim itself untouched. First, it closes a specification hole inside my own design rather than outside it. The scope revision redefined C_{i,t} as a structural property of an agent's output rather than a self-report, and gave a worked example only for A_F (does the extracted program parse, does every argument trace to a retrieved figure), leaving the other three agents open. ACI supplies the analogue for A_V: "the calibrated interval width is the structural confidence term the scope revision asked for, and it arrives measured rather than self-reported". The recipe is concrete — wrap the FIGARCH or GJR-GARCH forecast in ACI with the normalised score S_t = |V_t - sigma_hat^2| / sigma_hat^2, and let C_{V,t} be a function of the realised interval width at the target coverage, so a volatility agent whose model has drifted reports wider intervals and is automatically down-weighted. That is a measured property of the output, which is exactly what the redefinition demanded.
@@ -8104,51 +7980,51 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="409.6" customHeight="1">
-      <c r="A58" s="29" t="inlineStr">
+    <row r="57" ht="409.6" customHeight="1">
+      <c r="A57" s="29" t="inlineStr">
         <is>
           <t>P57</t>
         </is>
       </c>
-      <c r="B58" s="30" t="inlineStr">
+      <c r="B57" s="30" t="inlineStr">
         <is>
           <t>Gu, Kelly and Xiu. Empirical Asset Pricing via Machine Learning. Citekey guEmpiricalAssetPricing2018. Affiliations recorded in the note: Chicago Booth and Yale. The note's frontmatter gives year 2018 and the body dates the version read as the "November 2018 working version". The body also states this is "of what became the *Review of Financial Studies* paper that everything in this area now cites" — so the journal is the Review of Financial Studies, but the note does not record the RFS publication year, volume, pages or DOI. First names, DOI, arXiv ID and link: Not recorded in the note.
 TO BE EXPLICIT ABOUT WHICH IS WHICH: 2018 is the working-paper year from the note's frontmatter and is the version the note was written against; the Review of Financial Studies is the eventual journal of record, and its publication year is Not recorded in the note.</t>
         </is>
       </c>
-      <c r="C58" s="30" t="inlineStr">
+      <c r="C57" s="30" t="inlineStr">
         <is>
           <t>2020 (Review of Financial Studies 33(5)). The note's frontmatter carries 2018, the working-paper year; 2020 is the journal of record.</t>
         </is>
       </c>
-      <c r="D58" s="30" t="inlineStr">
+      <c r="D57" s="30" t="inlineStr">
         <is>
           <t>Working paper in the version read (November 2018); published subsequently in the *Review of Financial Studies*, which the note describes as "the paper that everything in this area now cites". Volume and pages: Not recorded in the note.</t>
         </is>
       </c>
-      <c r="E58" s="30" t="inlineStr">
+      <c r="E57" s="30" t="inlineStr">
         <is>
           <t>Not recorded in the note.</t>
         </is>
       </c>
-      <c r="F58" s="30" t="inlineStr">
+      <c r="F57" s="30" t="inlineStr">
         <is>
           <t>Empirical asset pricing / machine learning for cross-sectional return prediction. A comparative horse race of thirteen prediction methods on a single shared problem. The note is emphatic that this is not a competitor architecture and is not being read as one: "there are no agents here and no orchestration problem". It earns a full note for four reasons recorded verbatim in the note: it is "the best available calibration of what a well-specified return predictor actually achieves, and the number is small enough that it should reset my expectations for the technical agent before I build it"; "the signal families it ranks at the top are price trend, liquidity and volatility, which is independent large-sample evidence for two of the three state variables my orchestrator conditions on"; "its feature construction is the single-model version of conditioning on market state, every characteristic interacted with every macro variable, which is structurally the thing I am proposing to do one level up"; and "it is a clean, well-documented instance of the failure mode my cost sub-gap exists to address, reporting 113% monthly turnover and an annualised Sharpe of 2.35 in the same table without deducting a basis point."</t>
         </is>
       </c>
-      <c r="G58" s="30" t="inlineStr">
+      <c r="G57" s="30" t="inlineStr">
         <is>
           <t>Two literatures had accumulated hundreds of predictors and no way to evaluate them jointly. The cross-sectional strand regresses future returns on a few lagged characteristics; the time-series strand regresses aggregate returns on a few macro variables. The authors note the profession has accumulated "a staggering list of candidates", with Green et al. counting 330 stock-level signals, Harvey et al. 316 factors, and Welch and Goyal nearly 20 aggregate predictors. The stated problem is "how to assess the incremental content of a newly proposed predictor while jointly controlling for the gamut of extant signals, which is the multiple-comparisons problem dressed as an estimation problem."
 Three properties of the setting are argued to suit machine learning, and the note rates the argument as careful: risk-premium measurement is a conditional expectation, so it is a prediction problem rather than an inference problem; the predictor count approaches the observation count and the predictors are close cousins, "which is where OLS breaks"; and theory gives essentially no guidance on functional form, "so the search over specifications has to be mechanical."
 The framing is explicitly measurement, not mechanism, and the authors say so. Section 1.6 concedes that improved predictions are only measurements, that they do not identify deep associations between prices and conditioning variables, and that recovering mechanisms requires the economist to impose structure. The note calls this "the most honest paragraph in the paper and worth keeping in view, because the variable importance results later on are routinely cited as if they were economic findings."</t>
         </is>
       </c>
-      <c r="H58" s="30" t="inlineStr">
+      <c r="H57" s="30" t="inlineStr">
         <is>
           <t>US equities — every firm on NYSE, AMEX and NASDAQ. A deep, liquid, developed market, sixty years of it. No emerging or frontier market content. The note draws the implication in the opposite direction: "the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."</t>
         </is>
       </c>
-      <c r="I58" s="30" t="inlineStr">
+      <c r="I57" s="30" t="inlineStr">
         <is>
           <t>CRSP monthly total returns for every firm on NYSE, AMEX and NASDAQ, March 1957 to December 2016, with the Treasury bill rate used to form excess returns.
 - Universe: ~30,000 stocks, average &gt;6,200 per month.
@@ -8163,7 +8039,7 @@
 Four choices the note flags as mattering more than they look: the sample is deliberately unfiltered — stocks below $5, share codes beyond 10 and 11, and financial firms all retained — "which I note here because the economic results later depend on the small end of the universe"; publication lags are imposed explicitly, monthly characteristics delayed at most one month, quarterly at least four, annual at least six; missing characteristics are replaced with the cross-sectional median for that month; and there is no cross-validation anywhere, by design, to preserve temporal ordering.</t>
         </is>
       </c>
-      <c r="J58" s="30" t="inlineStr">
+      <c r="J57" s="30" t="inlineStr">
         <is>
           <t>Purely numeric panel data: firm characteristics, aggregate macro series, and industry dummies. No text, no filings text, no alternative data.
 The over-arching feature construction is the part the note cares most about. Rather than feeding characteristics and macro variables in side by side, they take the Kronecker product, so every characteristic appears once on its own and once interacted with each of the eight macro state variables:
@@ -8175,7 +8051,7 @@
 Dominant individual features by summed importance: short-term reversal, log market equity, twelve-month momentum, momentum change, recent maximum return, industry momentum, return volatility, dollar volume (top eight). Grouped families: price trend; liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread); risk (total and idiosyncratic volatility, beta, beta squared); valuation ratios a distant fourth.</t>
         </is>
       </c>
-      <c r="K58" s="30" t="inlineStr">
+      <c r="K57" s="30" t="inlineStr">
         <is>
           <t>Thirteen prediction methods, all on the same target and the same splits, differing only in how they constrain g(.): OLS on all 920 features, a three-characteristic OLS benchmark (OLS-3), PLS, PCR, elastic net, a spline generalized linear model with group lasso (GLM), random forest, gradient boosted regression trees (GBRT), and feed-forward networks at one through five hidden layers (NN1-NN5).
 - PCR and PLS both compress 920 features into K components, PCR maximising variance among the predictors and PLS maximising squared covariance with the target, "so PLS sacrifices fidelity to Z for predictive relevance".
@@ -8185,40 +8061,40 @@
 Output: a one-month-ahead excess-return forecast per stock, aggregated into decile-spread portfolios and bottom-up S&amp;P 500 forecasts for the economic evaluation.</t>
         </is>
       </c>
-      <c r="L58" s="30" t="inlineStr">
+      <c r="L57" s="30" t="inlineStr">
         <is>
           <t>Not applicable — a single-estimator horse race with no agents, no orchestrator, no weighting of heterogeneous producers over a shared decision. What it does instead is the closest single-model analogue: the Kronecker construction makes every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator. The note draws the line precisely: "That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound. What it does not do is the thing I am claiming: the interaction weights are estimated once per annual refit, they are a function of macro variables rather than of any measured reliability of the signal, and no channel in their model can go absent, because a missing characteristic is median-imputed rather than down-weighted. The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line."</t>
         </is>
       </c>
-      <c r="M58" s="30" t="inlineStr">
+      <c r="M57" s="30" t="inlineStr">
         <is>
           <t>Not applicable — no sentiment data, no text, no news or social signal anywhere in the paper. Sentiment is out of scope for my project in any case.</t>
         </is>
       </c>
-      <c r="N58" s="30" t="inlineStr">
+      <c r="N57" s="30" t="inlineStr">
         <is>
           <t>No retrieval, no documents, no RAG — accounting characteristics enter as pre-constructed numeric features from CRSP/Compustat-style panels, not as parsed filings. What the paper contributes to A_F is a horizon and lag discipline rather than a pipeline. Accounting characteristics cluster at the bottom of the importance ranking, and the authors attribute this partly to their low update frequency, noting that at the annual horizon price-trend variables lose ground to liquidity and risk measures while industry becomes substantially predictive. The publication-lag structure is explicit — monthly characteristics delayed at most one month, quarterly at least four, annual at least six — and the note treats this as the specification to write down for A_F "before touching any filing data, since CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."</t>
         </is>
       </c>
-      <c r="O58" s="30" t="inlineStr">
+      <c r="O57" s="30" t="inlineStr">
         <is>
           <t>Volatility enters as a predictor family rather than as a modelled process. The "risk" group — total volatility, idiosyncratic volatility, beta, beta squared — is one of the three dominant families across every method. The marginal-relationship plots show trees and networks finding large sensitivity to volatility where penalized linear models find none: a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return under GBRT or NN3 (and the companion size effect: a firm falling from median size to the 20th percentile gains roughly 2.4% in annualised expected return). On the macro side, market-level stock variance gets little weight anywhere and essentially none from the networks.
 No conditional volatility model, no GARCH, no persistence estimate, no volatility targeting, no risk scaling of positions. Portfolio construction is decile sorts, equal- and value-weighted, with Sharpe reported but no volatility budget.</t>
         </is>
       </c>
-      <c r="P58" s="30" t="inlineStr">
+      <c r="P57" s="30" t="inlineStr">
         <is>
           <t>Liquidity appears as a predictor family and is absent as a friction, and the gap between those two facts is what the note exploits. The liquidity group (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) is one of the three dominant families across every method. But: "There are no transaction costs anywhere in the paper, and the turnover figures make that decisive rather than cosmetic." The best strategy, an equal-weighted decile spread on NN4 forecasts, returns 3.3% per month, 39.0% annualised, at an out-of-sample Sharpe of 2.35, with monthly turnover of 114.08%. Networks run 110.87% to 114.08%, elastic net 143.61% and OLS-3 156.78%, against 22.87% for a size decile spread. The authors note that high turnover is unsurprising given the dominance of price-trend predictors, "and then stop."
 Two things in their own results indicate the size of what is left out. Value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, "so the gap between the paper's two weighting schemes is larger than the gap between most of its methods." And the universe retains sub-$5 stocks by explicit choice. The paper offers the higher top-1,000 R^2, 0.72% against 0.46%, as reassurance that machine learning is not merely picking up small-scale inefficiencies driven by illiquidity, "but the result carrying the economic claim is an equal-weighted spread over the whole board, and both cannot be load-bearing at once."</t>
         </is>
       </c>
-      <c r="Q58" s="30" t="inlineStr">
+      <c r="Q57" s="30" t="inlineStr">
         <is>
           <t>Variable importance is defined as the reduction in predictive R^2 from setting one predictor to zero with all other estimates held fixed. Marginal-relationship plots show each model's fitted sensitivity to individual characteristics. A placebo test adds five simulated noise characteristics and they rank low, which the note credits as a real check. The paper also reports model complexity over time (Figure 3): elastic net selecting fewer than five features in the first decade of the test sample and 20 to 40 after 2000, PCR using 20 to 40 components, GBRT moving from roughly 20 features to 30.
 The note's reading of the attribution machinery is sceptical — see LIMITATIONS — and it re-flags Section 1.6's own concession that these are measurements rather than mechanisms.</t>
         </is>
       </c>
-      <c r="R58" s="30" t="inlineStr">
+      <c r="R57" s="30" t="inlineStr">
         <is>
           <t>Baselines: OLS on all 920 features, OLS-3 (three characteristics), PLS, PCR, elastic net, GLM, random forest, GBRT, NN1-NN5. A Monte Carlo with 100 repetitions under both a sparse linear and a nonlinear interacted data generating process, with an oracle for reference.
 Primary metric:
@@ -8230,7 +8106,7 @@
 Economic evaluation: decile-spread portfolios (equal- and value-weighted) with out-of-sample Sharpe and monthly turnover; bottom-up S&amp;P 500 forecasts; and the Campbell and Thompson mapping from predictive R^2 to Sharpe ratio, SR* = sqrt((SR^2 + R^2)/(1 - R^2)).</t>
         </is>
       </c>
-      <c r="S58" s="30" t="inlineStr">
+      <c r="S57" s="30" t="inlineStr">
         <is>
           <t>- Absolute numbers are tiny and the spread across methods is narrower than the narrative suggests. Monthly stock-level R^2_oos: OLS on all 920 features -4.60% (worse than forecasting zero); OLS-3 0.16%; elastic net 0.09%; PLS 0.18%; PCR 0.28%; GLM 0.19%; random forest 0.27%; GBRT 0.30%; networks 0.35% (NN1) to a peak of 0.39% (NN3). "So the entire distance from the three-characteristic benchmark to the best model in the paper is 23 basis points of monthly R^2." Size split: NN3 reaches 0.72% on the top 1,000 stocks by market value against 0.46% on the bottom 1,000. At the annual horizon everything scales up roughly an order of magnitude, NN4 at 3.60% and NN3 at 3.40% across all stocks.
 - The Diebold-Mariano table does not support the method ranking the abstract implies, and the paper is upfront about this itself. Differences among all the regularized linear models are insignificant — OLS-3, PLS, PCR, elastic net and GLM are statistically indistinguishable from each other. Trees improve on linear models but the improvements are described as at best marginally significant. Neural networks are the only class producing large significant gains over linear and generalized linear models, NN3 against OLS-3 at 3.01, and their improvement over trees is not significant. Among the networks themselves nothing clears: NN3 against NN5 reaching -1.92 and NN3 against NN4 only -1.03. "On this evidence the defensible claim is narrower than 'trees and neural nets are the best performing methods': it is that networks beat linear specifications, and that everything else in the ranking is suggestive."
@@ -8241,7 +8117,7 @@
 - Economic results: best strategy is an equal-weighted decile spread on NN4 forecasts returning 3.3% per month, 39.0% annualised, out-of-sample Sharpe 2.35, monthly turnover 114.08%, with no costs deducted. Value weighting drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27.</t>
         </is>
       </c>
-      <c r="T58" s="30" t="inlineStr">
+      <c r="T57" s="30" t="inlineStr">
         <is>
           <t>- No transaction costs anywhere, and the turnover figures make that decisive rather than cosmetic (figures above). The authors note high turnover is unsurprising given the dominance of price-trend predictors and then stop. The value-weighted Sharpe collapse is "itself a partial, unacknowledged cost estimate". The top-1,000 reassurance and the equal-weighted headline "both cannot be load-bearing at once."
 - The Monte Carlo summary does not match its own table in the linear case. The text states that for the sparse linear model Lasso and ENet deliver the best and almost identical out-of-sample R^2, and that RF, NN and GBRT tend to overfit so their performance is slightly worse. Table A.1 shows NN1 at 4.42% and NN2 at 4.40% against ENet+H at 4.27% when P_c = 50, and 4.31% and 4.30% against 4.26% when P_c = 100, "so the networks are ahead in both panels. The trees do underperform as described, and the substantive conclusion about the nonlinear process is untouched, but the specific claim that penalized linear methods win when the truth is linear is contradicted by the numbers printed beneath it." That sentence is where the "match the method to the process" reading comes from.
@@ -8250,7 +8126,7 @@
 - Framing limitation conceded by the authors themselves in Section 1.6: improved predictions are only measurements, they do not identify deep associations between prices and conditioning variables, and recovering mechanisms requires the economist to impose structure.</t>
         </is>
       </c>
-      <c r="U58" s="30" t="inlineStr">
+      <c r="U57" s="30" t="inlineStr">
         <is>
           <t>- A ceiling and an expectation band for A_T. Thirty thousand stocks, sixty years, 920 engineered features, eleven method families and a thirty-year test window produce 0.39% monthly R^2_oos at the stock level. Against that, my confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information", so "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result." This sits alongside the 0.54 to 0.58 directional-accuracy band from [[Extending machine learning prediction capabilities by explainable AI in financial time series prediction]] and the 54.3% out-of-sample figure in [[Deep Learning with Long Short-Term Memory Networks for Financial Market Predictions]], "and the three together are now a defensible prior rather than one paper's number."
 - Model sizing: "Size the technical agent at NN1 or NN2 scale and stop treating depth as a dial." Performance peaks at three hidden layers on sixty years of data and declines beyond it, with data scarcity and low signal-to-noise named as the cause; on a dataset smaller by orders of magnitude the implied architecture is one or two hidden layers, or a regularized tree ensemble, "and the depth sweep that would be routine elsewhere is not worth the compute here. The same reasoning applies to feature count, since every method in the paper selected far fewer features than it was offered."
@@ -8261,7 +8137,7 @@
 - The cost sub-gap's reference case: a 113-114% monthly turnover strategy at Sharpe 2.35 with no cost deducted.</t>
         </is>
       </c>
-      <c r="V58" s="30" t="inlineStr">
+      <c r="V57" s="30" t="inlineStr">
         <is>
           <t>- No costs, no participation-rate analysis, no execution model. The paper reports turnover and stops. That is the whole of Sub-gap 1's motivation stated by a canonical paper without being addressed.
 - No reliability weighting and no absence channel. Conditioning on state happens through fixed, annually-refit interaction coefficients on macro variables; a missing input is median-imputed, never down-weighted, and nothing can go absent.
@@ -8272,12 +8148,12 @@
 - One open challenge to my macro rejection: aggregate book-to-market, which every model treats as critical and which tops the macro ranking for the networks and the penalized linear models.</t>
         </is>
       </c>
-      <c r="W58" s="30" t="inlineStr">
+      <c r="W57" s="30" t="inlineStr">
         <is>
           <t>[[Empirical Asset Pricing via Machine Learning]]</t>
         </is>
       </c>
-      <c r="X58" s="30" t="inlineStr">
+      <c r="X57" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T first (expectation band, architecture sizing, loss function, feature count), then the orchestrator's conditioning set (independent large-sample evidence for L_t and V_t, and the Kronecker construction as the single-model analogue of the orchestration claim), then the evaluation layer (benchmark choice, DM test, recursive protocol, Campbell-Thompson mapping), then A_F (horizon and lag discipline, and an argument for a low baseline weight plus explicit abstention), and finally Sub-gap 1, for which this paper is the cleanest reference case in the set.
 EFFECT ON MAIN GAP: It strengthens the premise and sharpens the claim without threatening either. The Kronecker construction is the single-model version of what I am proposing one level up: "Gu et al. make every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator, and the beta-pricing derivation is a principled reason to do it. That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound." That matters because it means the idea that a signal's value varies with market state is not something I have to argue for from scratch — it is derivable from E_t(r_{i,t+1}) = beta'_{i,t} lambda_t with beta_{i,t} = theta_1 c_{i,t} and lambda_t = theta_2 x_t, and it is the standard specification in the most-cited paper in the area.
@@ -8301,60 +8177,60 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="409.6" customHeight="1">
-      <c r="A59" s="29" t="inlineStr">
+    <row r="58" ht="409.6" customHeight="1">
+      <c r="A58" s="29" t="inlineStr">
         <is>
           <t>P58</t>
         </is>
       </c>
-      <c r="B59" s="30" t="inlineStr">
+      <c r="B58" s="30" t="inlineStr">
         <is>
           <t>Jayarangi, W.C. and Buddhika, H.J.R. (2025). The Impact of Firm-Specific Factors on Share Prices of Diversified Financial Companies: Evidence from the Colombo Stock Exchange. South Asian Journal of Finance, Vol. 5 No. 1, pp. 67–83. DOI 10.4038/sajf.v5i1.113. Both authors are at the Department of Finance, Faculty of Commerce and Management Studies, University of Kelaniya. Received November 2024, accepted June 2025. Citekey jayarangiImpactFirmSpecificFactors2025.</t>
         </is>
       </c>
-      <c r="C59" s="30" t="inlineStr">
+      <c r="C58" s="30" t="inlineStr">
         <is>
           <t>2025.</t>
         </is>
       </c>
-      <c r="D59" s="30" t="inlineStr">
+      <c r="D58" s="30" t="inlineStr">
         <is>
           <t>South Asian Journal of Finance, Vol. 5 No. 1, pp. 67–83.</t>
         </is>
       </c>
-      <c r="E59" s="30" t="inlineStr">
+      <c r="E58" s="30" t="inlineStr">
         <is>
           <t>https://doi.org/10.4038/sajf.v5i1.113 (accessed 4 October 2026). Zotero: zotero://select/library/items/4Y76RTSM.</t>
         </is>
       </c>
-      <c r="F59" s="30" t="inlineStr">
+      <c r="F58" s="30" t="inlineStr">
         <is>
           <t>Fundamentals. Firm-specific determinants of share price; local CSE empirical econometrics. The note's frontmatter records stream: fundamentals, market: CSE, status: reviewed.</t>
         </is>
       </c>
-      <c r="G59" s="30" t="inlineStr">
+      <c r="G58" s="30" t="inlineStr">
         <is>
           <t>The paper asks "whether five firm-specific accounting ratios, return on equity, dividend per share, earnings per share, the price to earnings ratio and debt to total assets, explain the share prices of Diversified Financial companies listed on the Colombo Stock Exchange". The gap it claims is threefold in my note. First, "the firm-specific determinants literature is developed-market and the Sri Lankan slice of it is thin and dated" — the authors anchor on Kumar (2017) for Indian autos, Nasif and Sharif (2010) for Amman commercial banks, Iqbal et al. (2016) for Kenyan energy and Sharif et al. (2014) for Bahrain, and cite Dissanayake and Herath (2016) and Pandigamage and Ranaweera (2023) as "near enough the whole local set". Second, and this is what I recorded as "their sharpest framing point", the only prior study of firm-specific factors on CSE diversified financials is a 2016 Central Bank staff study reporting percentage increments only, and "its results may no longer hold after the political and economic changes from 2020". I added my own qualification there: "I'd put this more strongly than they do, since their own sample runs straight through the same break and is estimated as one pooled regime." Third, the sector choice is a sampling rationale rather than a hypothesis — "Diversified Financials is picked for growth, not for theory", justified by earnings growing 43% and revenues 31% annually over 2021 to 2023 and the sector being roughly 20% of total market capitalisation per the Central Bank's 2023 industry analysis, which "means the sector was selected on the outcome variable's recent behaviour".</t>
         </is>
       </c>
-      <c r="H59" s="30" t="inlineStr">
+      <c r="H58" s="30" t="inlineStr">
         <is>
           <t>Colombo Stock Exchange, Diversified Financials sector only. Twenty companies, "selected as the highest market capitalisation 20 of the 43 Diversified Financial firms listed on the CSE, LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b".</t>
         </is>
       </c>
-      <c r="I59" s="30" t="inlineStr">
+      <c r="I58" s="30" t="inlineStr">
         <is>
           <t>200 firm-year observations, 2013 to 2023 (eleven years), 20 firms, random effects panel estimated in STATA. Data is hand-collected from the CSE website and from company annual reports. I flagged the arithmetic directly: "Eleven years across twenty firms is 220 firm-years and every table reports 200, which is not explained anywhere in the paper."</t>
         </is>
       </c>
-      <c r="J59" s="30" t="inlineStr">
+      <c r="J58" s="30" t="inlineStr">
         <is>
           <t>Annual accounting data from filings plus monthly-averaged price. Dependent variable: share price measured as the average share price of the month, in nominal rupees, undifferenced and untransformed. Regressors: return on equity (net income over average shareholders' equity), dividend per share (annual dividend over the weighted average share count), earnings per share (net profit over the same denominator), price to earnings (market value per share over earnings per share), debt to total assets (total liabilities over total assets). Sole control: firm size as the natural logarithm of total assets — "the only variable entering in logs". The operationalisation table sources each measure to prior local work: Biyiri and Dissanayaka (2017), Irsath et al. (2015), Sritharan (2018) and Rajapaksha and Weerawickrama (2020).
 Descriptives (these are the distributional facts I care about): share price mean 262.078, standard deviation 458.181, range Rs. 0.50 to Rs. 1,950 — "the dependent variable is in nominal rupee levels and is dominated by a handful of high-priced counters". Price to earnings is worse: "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82", which I read as "what happens when a ratio with earnings in the denominator is computed on firm-years where earnings are near zero or negative, and the EPS minimum of −21.65 confirms loss-making years are in the sample". Neither variable is winsorised, trimmed or transformed. EPS mean 17.239, standard deviation 53.818; DPS mean 4.66; ROE mean 14.237%; DTA mean 57.277%; log total assets 20.041.
 Correlations with price: DPS 0.535, EPS 0.509, PE 0.319, DTA −0.502, firm size −0.404, ROE −0.160. Among regressors: "dividend per share and earnings per share correlate at 0.757 and debt to assets correlates with firm size at 0.726", which I noted is "the structure that decides how the insignificant coefficients below should be read". Mean VIF 2.23, maximum 2.81, "and the paper treats that as settling the question".</t>
         </is>
       </c>
-      <c r="K59" s="30" t="inlineStr">
+      <c r="K58" s="30" t="inlineStr">
         <is>
           <t>One pooled panel specification, random effects after a Hausman test, share price in levels as the dependent variable:
 SP_it = β0 + β1 ROE_it + β2 DPS_it + β3 EPS_it + β4 PE_it + β5 DTA_it + β6 log(SIZE_it) + ε_it
@@ -8368,44 +8244,44 @@
 Output: in-sample coefficients and significance only. No forecast, no holdout, no agent.</t>
         </is>
       </c>
-      <c r="L59" s="30" t="inlineStr">
+      <c r="L58" s="30" t="inlineStr">
         <is>
           <t>Not applicable — this is a single-equation panel econometrics paper with no agents, no orchestration and no decision layer. As I put it in the note, "there is no forecast, no holdout and no agent anywhere in it, and I'm reading it the same way I read the other local empirical work, as evidence about what the fundamental channel on this market can and cannot carry." What it supplies instead is (a) a measured, published feature set for A_F on this exact market and sector, (b) the within-vs-between split that tells me what role A_F should play in the weighting function, and (c) a weak but real published baseline for the fundamental channel.</t>
         </is>
       </c>
-      <c r="M59" s="30" t="inlineStr">
+      <c r="M58" s="30" t="inlineStr">
         <is>
           <t>Not recorded in the note. (The paper is an accounting-ratio panel regression; no sentiment variable appears anywhere in my note.)</t>
         </is>
       </c>
-      <c r="N59" s="30" t="inlineStr">
+      <c r="N58" s="30" t="inlineStr">
         <is>
           <t>This is the paper's entire content and it is the row that matters most for A_F. The fundamental variables with measured CSE association are earnings per share (coefficient 1.887, standard error 0.501, t = 3.76, p = 0.000) and debt to total assets (−0.530, standard error 0.167, p = 0.002); firm size enters at −1.136 and is insignificant at p = 0.262; return on equity (−0.142, p = 0.575) and dividend per share (2.102, p = 0.248) do not clear. My own summary: "Earnings per share, leverage and firm size are the fundamental features with measured CSE association, and this is my citation for selecting them, scoped to cross-section… both are extractable from the income statement and balance sheet of any annual report. That is enough to justify the fundamental agent's feature set to a supervisor without my having to derive it from first principles, provided I say in the same sentence what the evidence is cross-sectional about."
 On update frequency and extraction cost, the note is explicit: all data is "hand-collected from the CSE website and from company annual reports", and "Twenty firms over eleven years, hand-collected from annual reports, is another data point on what fundamental extraction costs on this market. Two authors with institutional access pulled six variables for 200 firm-years by hand, which is the same message the Fernando note delivers from 167 firms, and it is why the retrieval pipeline over CSE filings is the component I expect to be the bottleneck rather than any model." I link that to structure-aware chunking of the kind in [[Financial Report Chunking for Effective Retrieval Augmented Generation]], which "reduces that cost without removing it".
 On feature construction for the RAG side, the price-to-earnings identity is a direct constraint I recorded: "Any ratio with price in the numerator fed into a model whose target is price or return carries a mechanical link to the label, and on a thin market where the denominator goes near zero it also carries a variance of the kind that produced a standard deviation of 1069.92 here. The fundamental agent's inputs should be restricted to quantities computed from the filings alone, with price-derived multiples either excluded or constructed against a lagged price and reported as such."</t>
         </is>
       </c>
-      <c r="O59" s="30" t="inlineStr">
+      <c r="O58" s="30" t="inlineStr">
         <is>
           <t>No volatility modelling of any kind — there is no variance model, no GARCH, no risk measure in the specification. The only risk content is interpretive: the authors read the negative debt-to-assets coefficient "as investors discounting financial risk". The regime instability content is relevant to V_t and P_t indirectly: the window "contains the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation peaking above 50%, and the dependent variable is an unadjusted nominal price with no year effects, no inflation adjustment and no regime split."</t>
         </is>
       </c>
-      <c r="P59" s="30" t="inlineStr">
+      <c r="P58" s="30" t="inlineStr">
         <is>
           <t>Not recorded in the note — there is no liquidity variable, no turnover screen, no trading-frequency filter and no transaction cost anywhere in this paper. The closest adjacent fact is the sample construction: the 20 largest of 43 sector firms by terminal market capitalisation, LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b, which is implicitly a size-and-prominence selection and is why the survivorship point below matters.</t>
         </is>
       </c>
-      <c r="Q59" s="30" t="inlineStr">
+      <c r="Q58" s="30" t="inlineStr">
         <is>
           <t>Not applicable in the ML sense. The model is a linear panel regression, so coefficients are the explanation by construction. I would note that the interpretability is undermined by the paper's own misreading of its coefficients: "it describes this as the effect of a 1% increase, but nothing except firm size is in logs, so the coefficient is the effect of one more rupee of EPS, which is Rs. 1.887 of price."</t>
         </is>
       </c>
-      <c r="R59" s="30" t="inlineStr">
+      <c r="R58" s="30" t="inlineStr">
         <is>
           <t>In-sample fit only. Overall R² 0.576, chi-square 64.394, Prob &gt; chi2 = 0.000, reported by the text as "the R square value lies at 58%" and "the overall model is significant". The same model summary table reports R² within of 0.090 and R² between of 0.709. There is "no train and test split, no holdout year, no rolling estimation and no forecast error reported anywhere". Comparison is to prior literature by sign agreement only: EPS "is consistent with Sharif et al. (2015), Su (2002) and Zhu (2003)", and the ROE null is placed "alongside Badruzaman (2020) and Zaman (2021) who also find negative or negligible ROE effects on price".</t>
         </is>
       </c>
-      <c r="S59" s="30" t="inlineStr">
+      <c r="S58" s="30" t="inlineStr">
         <is>
           <t>1. EPS is the strongest and most robust result: 1.887, standard error 0.501, t = 3.76, p = 0.000. "It is the only regressor whose univariate correlation with price (0.509), significance and sign all point the same way." But the magnitude is odd: "That is an implied marginal multiple of 1.887 against a sample where mean price over mean EPS is about 15.2", so "the levels regression is attributing almost all of the cross-sectional price level to something other than earnings, and reading the coefficient as a valuation multiple would understate the market's actual pricing by an order of magnitude."
 2. Debt to total assets is negative and significant at −0.530, standard error 0.167, p = 0.002 — one percentage point more leverage associates with Rs. 0.53 less price. Hedge carried through: DTA correlates 0.726 with firm size, firm size enters at −1.136 and is insignificant at p = 0.262, and both have sizeable negative univariate correlations with price (−0.502 and −0.404), so "the leverage coefficient and the size coefficient are competing to explain the same cross-sectional variation and the design has no way to separate them."
@@ -8414,7 +8290,7 @@
 5. The fit split is the headline for me: "Nine percent of the year-to-year movement in a given company's share price is explained, against seventy-one percent of the differences between companies", so "the model is a cross-sectional pricing description that has very little to say about time."</t>
         </is>
       </c>
-      <c r="T59" s="30" t="inlineStr">
+      <c r="T58" s="30" t="inlineStr">
         <is>
           <t>I recorded a standing warning on this paper: two of its own diagnostic tables contradict the text that reports them. "The normality section states that the Skewness/Kurtosis p-values are above 0.05 when the table it points at shows 0.000 in every cell, and the Hausman test is reported with a chi-square statistic of −1489.934, which is not a value the statistic can take. The random effects choice that produces every coefficient below rests on that second one."
 - Normality: the text claims all six variables are normally distributed "because the p-values for the Skewness and Kurtosis tests are greater than 0.05", while Table 4 reports 0.000 for skewness and kurtosis on every variable and adjusted chi-square p-values of 0.000 or 0.001 throughout, which rejects normality for all of them. The same paragraph then says the chi-square p-values being below 0.05 confirms the assumption is met, so the two sentences contradict each other as well as the table. A dependent variable ranging from Rs. 0.50 to Rs. 1,950 with a standard deviation 1.75 times its mean "is visibly non-normal, and no transform is applied in response."
@@ -8425,7 +8301,7 @@
 - Write-up slips: variable definitions render DPS as "Dep_osit" and EPS as "Esp_rit", every marginal effect is described as the response to a 1% change when only firm size is logged, the conclusion mentions a panel unit root test finding "at least one panel had a unit root" that appears nowhere in the results, and Table 10 duplicates the p-values already in Table 9. "None of these change a coefficient, and together they mean I should treat the figures as needing verification rather than as a clean reference."</t>
         </is>
       </c>
-      <c r="U59" s="30" t="inlineStr">
+      <c r="U58" s="30" t="inlineStr">
         <is>
           <t>- A measured, citable feature set for A_F on CSE: EPS and debt-to-assets as the two that clear at p = 0.000 and p = 0.002, with firm size as a control, all extractable from income statement and balance sheet alone — scoped explicitly to the cross-section.
 - The within R² of 0.090 against between R² of 0.709 as the number that fixes A_F's architectural role: "Fundamentals on this market separate counters from each other far better than they explain any one counter's path, so the fundamental channel should produce a slowly-updating relative view across the universe rather than a timing signal, with the technical channel carrying the short horizon and the orchestrator capping how much the fundamental weight is allowed to move between reporting dates."
@@ -8434,7 +8310,7 @@
 - A published, weak, in-sample baseline for the fundamental channel on CSE diversified financials to beat out of sample.</t>
         </is>
       </c>
-      <c r="V59" s="30" t="inlineStr">
+      <c r="V58" s="30" t="inlineStr">
         <is>
           <t>- No out-of-sample evaluation at all. "A linear six-variable model on CSE diversified financials with an in-sample overall R² of 0.576 and a within R² of 0.090 is a reference point my fundamental agent should beat out of sample, and since the paper reports no out-of-sample result at all, establishing one on a comparable universe is a contribution I can state plainly in the proposal rather than having to argue for."
 - No time-varying or state-conditional structure: one pooled regime over 2013–2023 with no year effects, no regime split and no inflation adjustment, across a window containing the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation above 50%. Nothing in the design lets the fundamental relationship's strength vary with market state, which is exactly what w(i,t) = f(L_t, V_t, P_t, C_i,t) is for.
@@ -8443,12 +8319,12 @@
 - No volatility persistence content, so nothing here constrains SUB-GAP 2 directly.</t>
         </is>
       </c>
-      <c r="W59" s="30" t="inlineStr">
+      <c r="W58" s="30" t="inlineStr">
         <is>
           <t>[[The Impact of Firm-Specific Factors on Share Prices of Diversified Financial Companies, Evidence from the Colombo Stock Exchange]]</t>
         </is>
       </c>
-      <c r="X59" s="30" t="inlineStr">
+      <c r="X58" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_F (the fundamental agent) — feature selection, update frequency and architectural role; the abstention channel; universe construction and point-in-time screening; and the local-evidence justification for using the CSE. It is the most recent published statement I have of which accounting ratios associate with price on CSE financials, over a window that overlaps mine almost exactly.
 EFFECT ON MAIN GAP: Strongly supportive, and in a very specific way. The within/between split — 0.090 within against 0.709 between — is a direct, locally measured statement that the fundamental channel's reliability is horizon-dependent on this market: it prices counters against each other well and says almost nothing about when a given counter moves. That is precisely the kind of structural property the weighting function w(i,t) = f(L_t, V_t, P_t, C_i,t) is meant to exploit, and it gives me a published, CSE-specific number for why the fundamental agent's weight should be capped and slow-moving between reporting dates rather than allowed to drive entry and exit. It also supports the C_i,t component being a structural property of the output rather than a self-report: ROE and DPS fail to clear not because they are irrelevant but because they are collinear with EPS (DPS–EPS at 0.757), so a channel whose inputs are collinear or missing should be detectable from the structure of its inputs and allowed to abstain. "Letting the channel return no view when its inputs are collinear or missing is the design consequence, and it is the same abstention argument the liquidity screen produces for the technical channel." Finally, the paper's pooling of eleven years containing a currency collapse as one regime is my clearest local illustration of what a fixed, non-state-conditional combination rule costs: "This is now the third CSE result pointing the same way, alongside the macro linkages breaking over 2014 to 2022 in [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] and the 2021 extension halving the investment-risk coefficient in the Fernando note."
@@ -8468,53 +8344,53 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="409.6" customHeight="1">
-      <c r="A60" s="29" t="inlineStr">
+    <row r="59" ht="409.6" customHeight="1">
+      <c r="A59" s="29" t="inlineStr">
         <is>
           <t>P59</t>
         </is>
       </c>
-      <c r="B60" s="30" t="inlineStr">
+      <c r="B59" s="30" t="inlineStr">
         <is>
           <t>Fernando, A.D., Nimal, P.D. and Abeysekera, A. (2026). Relationship between firm-level investment, idiosyncratic risk and ownership: an emerging market perspective. Managerial Finance, Vol. 52 No. 3, pp. 517–539. DOI 10.1108/MF-10-2024-0791. Affiliations: Abehitha Dinethri Fernando (University of Oklahoma), Pulukkuttige Don Nimal (University of Sri Jayewardenepura), Amal Abeysekera (Hofstra). Received October 2024, accepted June 2025. Citekey fernandoRelationshipFirmlevelInvestment2026.</t>
         </is>
       </c>
-      <c r="C60" s="30" t="inlineStr">
+      <c r="C59" s="30" t="inlineStr">
         <is>
           <t>2026.</t>
         </is>
       </c>
-      <c r="D60" s="30" t="inlineStr">
+      <c r="D59" s="30" t="inlineStr">
         <is>
           <t>Managerial Finance, Vol. 52 No. 3, pp. 517–539.</t>
         </is>
       </c>
-      <c r="E60" s="30" t="inlineStr">
+      <c r="E59" s="30" t="inlineStr">
         <is>
           <t>https://doi.org/10.1108/MF-10-2024-0791. Zotero: zotero://select/library/items/K3N7LZ4S.</t>
         </is>
       </c>
-      <c r="F60" s="30" t="inlineStr">
+      <c r="F59" s="30" t="inlineStr">
         <is>
           <t>Market structure. Corporate finance / firm-level investment under idiosyncratic risk, with ownership moderation; local CSE empirical econometrics. The note's frontmatter records stream: market-structure, market: CSE, status: reviewed.</t>
         </is>
       </c>
-      <c r="G60" s="30" t="inlineStr">
+      <c r="G59" s="30" t="inlineStr">
         <is>
           <t>The paper asks "whether firms listed on the Colombo Stock Exchange cut capital investment when their idiosyncratic risk rises, and whether insider and institutional ownership moderate that sensitivity". The gap it addresses, as I recorded it: (1) "The investment-risk sensitivity literature is almost entirely developed-market" — Panousi and Papanikolaou (2012) in the Journal of Finance is the anchor (risk-averse managers underinvest when firm-specific risk rises), with follow-on work (Glover and Levine, 2017; Liu and Wang, 2021; Florackis et al., 2019) staying in US and UK data; "The authors' claim is not that the mechanism is absent elsewhere, it's that the sign of the ownership moderation has no reason to carry over, because the agency environment that produces it is different." (2) "The alignment against entrenchment question is genuinely open in emerging markets" — higher insider ownership can tie managerial wealth to firm growth and push toward long-horizon investment (alignment, Ang et al., 2000) or concentrate undiversified personal wealth and raise risk aversion (entrenchment, Fahlenbrach and Stulz, 2009); the paper argues weaker legal protection and weaker formal governance in emerging markets (La Porta et al., 1998; Khanna and Palepu, 2002) raise the marginal value of insider ownership as a substitute governance mechanism, tilting toward alignment. "That is a testable framing and it is the paper's actual contribution." (3) The authors claim coverage of this relationship in South Asia, "which I can't independently verify but which is consistent with what I found when I went looking for CSE firm-level risk studies."</t>
         </is>
       </c>
-      <c r="H60" s="30" t="inlineStr">
+      <c r="H59" s="30" t="inlineStr">
         <is>
           <t>Colombo Stock Exchange, non-financial listed firms. The sample excludes financials and heavily state-regulated sectors (utilities, energy, telecoms), firm-years with missing key variables, and negative book values.</t>
         </is>
       </c>
-      <c r="I60" s="30" t="inlineStr">
+      <c r="I59" s="30" t="inlineStr">
         <is>
           <t>1,226 firm-year observations covering 167 unique CSE firms from 2010 to 2018, with firm and year fixed effects and standard errors clustered at the firm level. "Both listed and delisted firms are retained, which is a deliberate survivorship-bias control and more than most of the local literature does." Ownership data is only available from 2011, and the sub-samples are much smaller: "the insider ownership sub-sample is 59 firms and the institutional sub-sample 54 firms", which produces the 297 and 278 observation counts in the moderation tables; after propensity score matching, "64 and 76 observations respectively". A robustness extension runs the sample three years further to 2021.</t>
         </is>
       </c>
-      <c r="J60" s="30" t="inlineStr">
+      <c r="J59" s="30" t="inlineStr">
         <is>
           <t>Annual accounting data plus weekly price series. "All accounting and insider ownership data is hand-collected from annual reports published by the CSE", prices and the index come from the CSE data libraries, and Treasury bill rates from the Central Bank of Sri Lanka.
 Idiosyncratic risk is built as the residual standard deviation from a Fama–French three-factor regression on weekly excess returns over 52 trading weeks:
@@ -8525,7 +8401,7 @@
 Descriptives I keep returning to: mean idiosyncratic risk "0.221 with a standard deviation of only 0.050 and a full range of 0.117 to 0.315"; "insider and institutional ownership correlate at −0.703"; mean insider ownership 5.7% against mean institutional ownership 66.1%, "so this is a market of institutionally held firms with thin executive stakes". Sample mean investment rate is 11.60%, with a minimum in Table 2 of −0.082.</t>
         </is>
       </c>
-      <c r="K60" s="30" t="inlineStr">
+      <c r="K59" s="30" t="inlineStr">
         <is>
           <t>Three nested fixed-effect panel specifications, investment rate as dependent variable, firm-clustered standard errors.
 Model 1 (baseline):
@@ -8537,31 +8413,31 @@
 Output: in-sample panel coefficients. "There are no agents, no forecasts and no out-of-sample period anywhere in it."</t>
         </is>
       </c>
-      <c r="L60" s="30" t="inlineStr">
+      <c r="L59" s="30" t="inlineStr">
         <is>
           <t>Not applicable — this is a corporate finance panel econometrics paper with no agents, no orchestration, no decision layer and no forecast. As I put it: "Nothing in this paper is a methodological template for what I'm building… so I'm reading it as market-structure evidence rather than as a design precedent." What it supplies instead is (a) three conceded facts about CSE data depth that constrain the technical, volatility and fundamental channels respectively, (b) a reusable idiosyncratic risk estimator for A_V's cross-sectional input, and (c) a conditioning design — annual median splits with group-specific slopes — that is "close to the structure I'd want for ablating state inputs one at a time", i.e. a template for ablating L_t, V_t, P_t and C_i,t individually in the orchestrator.</t>
         </is>
       </c>
-      <c r="M60" s="30" t="inlineStr">
+      <c r="M59" s="30" t="inlineStr">
         <is>
           <t>Not recorded in the note. (No sentiment variable appears anywhere in this paper.)</t>
         </is>
       </c>
-      <c r="N60" s="30" t="inlineStr">
+      <c r="N59" s="30" t="inlineStr">
         <is>
           <t>Substantial, and it is where my A_F extraction-cost argument gets its strongest local evidence. All accounting and insider ownership data is hand-collected from annual reports published by the CSE. My note: "167 firms with usable accounting data and 59 with usable ownership data, all of it hand-collected from annual report PDFs, is the data-depth constraint arriving from a direction I hadn't checked. My liquidity screen question has been how many counters trade often enough to model, and this adds a second filter underneath it, how many have fundamentals complete enough to extract, with the answer coming from three authors who had institutional access, every incentive to keep the sample large, and who still spent the effort to pull accounting figures, insider stakes, board composition, CEO duality and family-firm status out of CSE filings by hand over nine years. That prices the extraction problem and explains why the retrieval pipeline over those filings is the component most likely to be the bottleneck, which is the case the structure-aware chunking work in [[Financial Report Chunking for Effective Retrieval Augmented Generation]] addresses and reduces rather than removes. It is also why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence."
 There is also a documented accounting break in the fundamentals: "SLFRS 16 in 2019 is a documented structural break in CSE fundamentals sitting in the middle of my training window. My index track runs 1 July 2014 to 30 June 2024, so any PPE-derived or lease-sensitive fundamental feature is not comparable across the 2019 boundary, and the fix is either a feature set that avoids the affected line items or an explicit break control with the choice stated in the methodology."
 Fundamental update frequency here is annual (annual reports, year-end ownership stakes, lagged-one-year risk and controls).</t>
         </is>
       </c>
-      <c r="O60" s="30" t="inlineStr">
+      <c r="O59" s="30" t="inlineStr">
         <is>
           <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama–French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
 What I would add: "the non-synchronous trading correction and a reported correlation between the risk estimate and turnover, because if those two move together on my sample then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it."
 Magnitude prior for A_V: "Mean idiosyncratic risk of 0.221 with a standard deviation of 0.050 sets a realistic prior on how much cross-sectional signal the volatility channel can carry. That is a narrow spread, and a one standard deviation move being worth 2.02 percentage points of investment is a real-economy effect rather than a trading one, so I should not expect the cross-sectional volatility ranking on CSE counters to separate firms as cleanly as it does on a US sample."</t>
         </is>
       </c>
-      <c r="P60" s="30" t="inlineStr">
+      <c r="P59" s="30" t="inlineStr">
         <is>
           <t>The paper has no liquidity variable, no turnover screen and no execution cost model, but it makes two liquidity-relevant concessions that I treat as primary evidence.
 First, the frequency concession, which I flagged as an important callout: "Weekly, not daily, and the paper says why in one sentence: 'since most stocks are not traded daily, we use weekly stock returns.' That is a finance journal on my exact market conceding the non-synchronous trading problem in the data section rather than the limitations section. Every frequency decision I make downstream has to answer to it."
@@ -8569,18 +8445,18 @@
 Third, the untreated bias: "Weekly returns reduce the problem relative to daily but they do not eliminate it on a market where the paper itself says most stocks don't trade daily, and stale prices bias the residual standard deviation downward for exactly the thinnest counters. There is no Dimson or Scholes-Williams correction, no reported trading-frequency screen, and no check of whether the idiosyncratic risk measure correlates with turnover." The ±50% weekly return trim "is a sensible outlier rule and it is also a reminder of what the raw series looks like."</t>
         </is>
       </c>
-      <c r="Q60" s="30" t="inlineStr">
+      <c r="Q59" s="30" t="inlineStr">
         <is>
           <t>Not applicable in the ML sense — coefficients and group-specific slopes are the explanation by construction. Figure 1 is the paper's clearest visual statement: "the low-ownership line falls from roughly 0.23 to 0.055 across the plotted range of log lagged idiosyncratic risk while the high-ownership line is flat and very slightly positive." I would note that the paper's headline mechanism is inferred rather than observed — see limitations.</t>
         </is>
       </c>
-      <c r="R60" s="30" t="inlineStr">
+      <c r="R59" s="30" t="inlineStr">
         <is>
           <t>In-sample panel estimation only; no holdout, no out-of-sample window, no forecast error. Adjusted R² moves from 0.029 to 0.206 across the three baseline columns, "so most of the explanatory power is coming from the fixed effects and controls rather than from risk, which is normal in this literature and worth remembering before reading the coefficient as a forecast." Baselines are prior literature by sign comparison: the result contradicts Panousi and Papanikolaou (2012) directly; the institutional substitution reading is consistent with Shleifer and Vishny (1986) and Gillan and Starks (2000); the governance null echoes Caixe et al. (2019) finding no governance mitigation in Brazil.
 Robustness battery, which I described as "unusually thorough and mostly holds": industry fixed effects and industry-by-year fixed effects leave the pattern intact; propensity score matched samples reproduce it; family firms (33% of firm-years, identified by hand from annual reports and executive biographies following Anderson and Reeb, 2003) show no differential sensitivity across five alternative family-ownership measures; adding independent board fraction and CEO duality changes nothing. Plus a sample extension to 2021.</t>
         </is>
       </c>
-      <c r="S60" s="30" t="inlineStr">
+      <c r="S59" s="30" t="inlineStr">
         <is>
           <t>1. Idiosyncratic risk is negatively and significantly related to firm-level investment across every specification: "−0.165* in the year-fixed-effects-only column rising to −0.232* with full controls and firm fixed effects, and −0.199 once a lagged dependent variable is added." Economic size: "a one standard deviation rise in idiosyncratic risk cuts the investment rate by 2.02 percentage points against a sample mean of 11.60%, a 17.48% decline."
 2. "The negative sensitivity is concentrated entirely in low-insider-ownership firms, and that is the opposite of the US result." Risk × low insider dummy is −0.435* with year effects only and −0.599 with the full specification; the high insider dummy interaction "is statistically indistinguishable from zero throughout (0.035, standard error 0.180)". The authors read this as alignment dominating entrenchment, contradicting Panousi and Papanikolaou (2012).
@@ -8588,7 +8464,7 @@
 4. The extension result, which I rate as the most useful finding in the paper for me: "Extending the sample three years to 2021 weakens the baseline result from −0.232* to −0.123*, and the paper calls this 'largely consistent'." The ownership results survive better — "low insider at −0.407 and low-institutional-low-insider at −0.787, and the high-institutional-low-insider cell now turns significant at −0.433." My reading: "I read the halving of the main coefficient and the loss of two significance stars as the more informative result here, and it is the single most useful thing in the paper for my own period argument." Note the surviving 2021 baseline is significant only at the 10% level (−0.123*).</t>
         </is>
       </c>
-      <c r="T60" s="30" t="inlineStr">
+      <c r="T59" s="30" t="inlineStr">
         <is>
           <t>- "The moderation results, which are the paper's contribution, rest on very few firms." 59 unique firms and 297 firm-years for insider tests, 54 firms and 278 for institutional tests, and after propensity score matching "64 and 76 observations respectively, all of this carrying firm fixed effects, year fixed effects and category dummies. At those sample sizes firm fixed effects consume a large share of the degrees of freedom and the matched-sample estimates in particular are being asked to do more than the data can support. The authors are not hiding any of this, the counts are in every table, but the write-up treats the matched results as confirmation when at 64 observations they are closer to a consistency check."
 - "The −0.703 correlation between insider and institutional ownership makes the 2×2 grid structurally unbalanced, and the insignificant cells are where that bites. Two variables correlating that strongly cannot produce four well-populated quadrants from 278 observations, so the high-insider-high-institutional cell is thin by construction, and every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one. The substitution story the paper tells could be right, but the evidence for it is one significant cell and three insignificant ones, and the design can't separate a genuine null from low power."
@@ -8598,7 +8474,7 @@
 - "The 2018 cutoff is well-argued and the extension quietly undercuts the argument for it. SLFRS 16 changing lease recognition in 2019 genuinely contaminates PPE, and that justifies the main sample. But the extended analysis to 2021 then runs straight through SLFRS 16, the Easter attacks and COVID with no adjustment to the PPE measure and no regime split, and reports the result as consistent, so the paper ends up both claiming the break is serious enough to truncate the sample and treating a sample that spans it as corroborating evidence."</t>
         </is>
       </c>
-      <c r="U60" s="30" t="inlineStr">
+      <c r="U59" s="30" t="inlineStr">
         <is>
           <t>- The citation for why A_T cannot assume a daily price series on CSE: a finance journal estimating a factor model on CSE firms moves to weekly because most stocks don't trade daily. "That is a stronger warrant than anything I could get from the ML literature."
 - The idiosyncratic risk estimator for A_V's cross-sectional input — residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free — plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk–turnover correlation).
@@ -8610,7 +8486,7 @@
 - Retention of delisted firms as the correct survivorship control, and the correct counterpart to the wrong version documented in [[The Impact of Firm-Specific Factors on Share Prices of Diversified Financial Companies, Evidence from the Colombo Stock Exchange]].</t>
         </is>
       </c>
-      <c r="V60" s="30" t="inlineStr">
+      <c r="V59" s="30" t="inlineStr">
         <is>
           <t>- The non-synchronous trading problem is conceded and then left untreated: no Dimson or Scholes–Williams correction, no trading-frequency screen, no check of whether the risk measure correlates with turnover. That correction, and the reported risk–turnover correlation, is work I have to do, and it is exactly the boundary between A_V and A_L.
 - No out-of-sample period, no forecast, no decision objective — so nothing here tells me how a risk estimate should be weighted in a live allocation, only how it relates contemporaneously to corporate investment.
@@ -8619,12 +8495,12 @@
 - No state-conditional combination of any channel; the conditioning is on ownership, a firm attribute, not on market state L_t, V_t or P_t.</t>
         </is>
       </c>
-      <c r="W60" s="30" t="inlineStr">
+      <c r="W59" s="30" t="inlineStr">
         <is>
           <t>[[Relationship between firm-level investment, idiosyncratic risk and ownership, an emerging market perspective]]</t>
         </is>
       </c>
-      <c r="X60" s="30" t="inlineStr">
+      <c r="X59" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk–turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
 EFFECT ON MAIN GAP: Strongly supportive on two fronts. First, regime instability: "The 2021 extension weakening the main coefficient from −0.232* to −0.123* is corroboration that CSE relationships estimated pre-2020 do not survive the crisis window intact. Taken with [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] finding the traditional macro linkages broken over 2014 to 2022, that is now two independent CSE results pointing at regime instability across exactly the period a static system would be evaluated on, which is the clearest empirical case I have for an orchestrator that conditions on measured state rather than a fixed combination rule." Note the surviving coefficient is significant only at 10%.
@@ -8650,38 +8526,38 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="409.6" customHeight="1">
-      <c r="A61" s="29" t="inlineStr">
+    <row r="60" ht="409.6" customHeight="1">
+      <c r="A60" s="29" t="inlineStr">
         <is>
           <t>P60</t>
         </is>
       </c>
-      <c r="B61" s="30" t="inlineStr">
+      <c r="B60" s="30" t="inlineStr">
         <is>
           <t>Pavithya, M.B.D., Perera, G.S.D., Munasinghe, S.L. and Karunarathna, S.N. (2021). Quantitative Analysis and Sentiment Analysis for Stock Price Forecast: The Case of Colombo Stock Exchange. 2021 10th International Conference on Information and Automation for Sustainability (ICIAfS), August 2021, pp. 512-517. DOI: 10.1109/ICIAfS52090.2021.9606034. Citekey: pavithyaQuantitativeAnalysisSentiment2021. Affiliation as recorded in my note: all authors out of the Department of Computer Engineering at the University of Peradeniya.</t>
         </is>
       </c>
-      <c r="C61" s="30" t="inlineStr">
+      <c r="C60" s="30" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="D61" s="30" t="inlineStr">
+      <c r="D60" s="30" t="inlineStr">
         <is>
           <t>2021 10th International Conference on Information and Automation for Sustainability (ICIAfS), pp. 512-517. Conference paper.</t>
         </is>
       </c>
-      <c r="E61" s="30" t="inlineStr">
+      <c r="E60" s="30" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/ICIAfS52090.2021.9606034 (accessed 4 October 2026). Zotero: zotero://select/library/items/XMAIQR9E</t>
         </is>
       </c>
-      <c r="F61" s="30" t="inlineStr">
+      <c r="F60" s="30" t="inlineStr">
         <is>
           <t>Orchestration (stream field in the note frontmatter). Market: CSE. In my own framing this is the CSE-local instance of the fixed-influence combination problem: two methodologically heterogeneous forecasting models merged into a single binary decision by a constant weight pair. As I put it in the note, "This is the closest thing in my CSE set to the shape of what I'm building, and it runs aground in exactly the place my main gap sits."</t>
         </is>
       </c>
-      <c r="G61" s="30" t="inlineStr">
+      <c r="G60" s="30" t="inlineStr">
         <is>
           <t>Forecast the next trading day's up/down direction for CSE counters by building a quantitative price model and a text model separately and then merging them with a fixed weighted vote. Three motivating gaps as I recorded them:
 - Forecasting models validated on deep markets are not guaranteed to transfer to a disrupted one. The abstract is explicit that prior work is built on well established exchanges and that such models are not guaranteed to capture the trends of exchanges showing high disruptive behaviour like the CSE, "where some indexes have no trades on some days and the data is therefore incomplete." My note's judgement: "That is the right motivation and it is close to my own, and it is also the thing the methodology then fails to act on."
@@ -8689,25 +8565,25 @@
 - The CSE text channel had not been established as usable at all. The authors tried the exchange's own announcement feed first and abandoned it, "which is itself the finding."</t>
         </is>
       </c>
-      <c r="H61" s="30" t="inlineStr">
+      <c r="H60" s="30" t="inlineStr">
         <is>
           <t>Colombo Stock Exchange, Sri Lanka. Three counters: John Keells Holdings (JKH), Ceylon Tobacco Corporation (CTC) and Agalawatte Plantations PLC (AGAL). Daily frequency, single-market, frontier market.</t>
         </is>
       </c>
-      <c r="I61" s="30" t="inlineStr">
+      <c r="I60" s="30" t="inlineStr">
         <is>
           <t>CSE trade information for the past eight years, one file per index, for JKH, CTC and AGAL. The authors stress this is real exchange data rather than a downloadable synthetic set, which they argue makes the results more realistic for automated trading on the CSE. Split: six years training, one year validation, one year testing, with the training partition expanding on each iteration because of the walk-forward scheme.
 Text corpus: the CSE announcement data obtained from the exchange was not rich enough to train a usable classifier, so news was scraped from a public economic-news blog with a pagination loop, giving over 4,000 articles from 2012 to 2019. Roughly 4,000 articles across eight years is about two per trading day (my arithmetic in the note, not the paper's).</t>
         </is>
       </c>
-      <c r="J61" s="30" t="inlineStr">
+      <c r="J60" s="30" t="inlineStr">
         <is>
           <t>Two modalities, price/volume and news text.
 Price side: missing values were handled and the data normalised, except for CTC, which was trained unnormalised with a different parameter set and is therefore not comparable with the other two. PCA was applied for dimension reduction and then dropped as unsuitable, after which feature selection was done on correlation and autocorrelation instead: previous-day close, high, low and open plus volume correlated best, and the previous seven days of prices showed higher autocorrelation than days further back. Day of the week was added on the observation that Mondays and Fridays behave differently from the three mid-week days, which is what makes the multivariate variant multivariate. Seasonality and trend removal was attempted and abandoned because the model did not perform well on the stationarised series, "reported plainly as a pitfall rather than buried."
 Text side: CountVectorizer n-gram range, stop-word removal and TfidfTransformer settings tuned. Labels were not annotated, they were derived mechanically: each article was joined to the quantitative data by publication date under the assumption that news published on one day moves the trend on the next, and inherited that next day's up or down label.</t>
         </is>
       </c>
-      <c r="K61" s="30" t="inlineStr">
+      <c r="K60" s="30" t="inlineStr">
         <is>
           <t>Univariate and multivariate LSTMs over eight years of CSE trade data for three counters, plus a Multinomial Naive Bayes classifier over roughly 4,000 scraped economic news articles, combined by a fixed weighted vote into a single up or down call for the next trading day.
 Final LSTM: four layers of 128, 64, 16 and 1 units, dropout 0.5 on the first two layers, an L1L2 bias regulariser at l1 = l2 = 0.001, batch size 10, Adam optimiser. Depth, width, epochs, dropout, optimiser and learning rate searched using a Hyperas wrapper and grid search.
@@ -8724,50 +8600,50 @@
 Output: a single binary up/down trend call for the next trading day.</t>
         </is>
       </c>
-      <c r="L61" s="30" t="inlineStr">
+      <c r="L60" s="30" t="inlineStr">
         <is>
           <t>No agents in the LLM sense, but there is an explicit two-channel combination with a stated weight vector, which is why I treat it as an orchestration-stream paper. The orchestration is a constant: two methodologically heterogeneous models, one shared binary decision, and "a combination rule that is a pair of constants found by trying a few values and keeping the best. No conditioning on market state, no per-day reweighting, no handling of a channel whose input is absent that day."
 My central structural finding on the mechanism, recorded in the note as a warning callout: the stated 1:3 weight ratio is not what actually decides the trend, the article count is. The combining rule sums one prediction from the quantitative model against one prediction per news article and divides by total weight, so with n_t articles the text channel holds n_t*w_P / (w_V + n_t*w_P) of the decision. At the reported 1:3 ratio a single article already gives text 75%, two give it 86%, and roughly 4,000 articles across eight years is about two per trading day. "The LSTM, which is the better-validated of the two components, is therefore carrying something near 14% of a typical day's decision, and moving from equal weights to 1:3 only shifts the text share from about 67% to about 86%. That is the real reason the weight axis buys so little, 2.15 accuracy points, and the paper never states the quantity."
 There is an accidental abstention behaviour: when no article appears the text term vanishes and the decision falls back entirely to the quantitative model. This is arrived at "by accident rather than design," and as implemented "the system cannot tell a confident abstention from a quiet news day."</t>
         </is>
       </c>
-      <c r="M61" s="30" t="inlineStr">
+      <c r="M60" s="30" t="inlineStr">
         <is>
           <t>What the paper did: news was scraped from a public economic-news blog with a pagination loop after the CSE's own announcement feed was found not rich enough to train a usable classifier, giving over 4,000 articles from 2012 to 2019. Labels were derived mechanically rather than annotated: each article was joined to the quantitative data by publication date under the assumption that news published on day t-1 moves the trend on day t, and inherited that next day's up or down label. Five classifiers were compared (Decision Tree, Naive Bayes, SVM, Random Forest, a simple ANN), tuned over CountVectorizer n-gram range, stop-word removal and TfidfTransformer settings, and Multinomial Naive Bayes was selected on 10-fold cross-validation accuracy of 0.95 (+/-0.02), tied with SVM at 0.95 (+/-0.03) against Decision Tree and Random Forest at 0.88. The text predictions then enter the weighted vote one term per article.
 My reading of that 0.95: it "is not evidence of predictive skill, and the hybrid result demonstrates that. Those labels were assigned mechanically from the next day's price direction, and 10-fold CV shuffles articles that are temporally adjacent and frequently cover the same event, so articles sharing a day share a label and overlapping vocabulary and the classifier can recover the day rather than the direction. The test that matters is the one the paper itself runs: a component scoring 0.95 in isolation contributes about four accuracy points to a joint decision in which it holds most of the weight. Those two numbers cannot both be measuring the same thing."
 Scope statement: this component is out of scope for my project. The sentiment agent was removed from my architecture by the supervisor's scope decision (see [[Scope sentiment analysis dropped]]), and my note states the consequence directly: "the only reading available to me since sentiment is out of scope and the text half is not something I'll rebuild." This row is retained in the matrix as evidence about the CSE and about fixed-weight combination, not as a design input. Per the scope rules the text channel is cited as a fixed-influence failure case, not as a component to rebuild.</t>
         </is>
       </c>
-      <c r="N61" s="30" t="inlineStr">
+      <c r="N60" s="30" t="inlineStr">
         <is>
           <t>No fundamental agent and no retrieval architecture in the paper. The relevant transferable finding is about document availability rather than retrieval method: the CSE announcement data obtained from the exchange was not rich enough to train a usable classifier, so the authors abandoned the exchange's own feed for a scraped economic-news blog. I read that as direct evidence for how I scope A_F: "The authors had the exchange's own data and had to abandon it for scraped material, the same thin-channel failure AlphaAgents hit with news on fifteen US megacaps, and it is why I expect the fundamental channel to be unusable a large fraction of the time. The binding constraint on structure-aware retrieval over CSE filings is document availability per counter per period, so that count is worth establishing before the retrieval design is settled."</t>
         </is>
       </c>
-      <c r="O61" s="30" t="inlineStr">
+      <c r="O60" s="30" t="inlineStr">
         <is>
           <t>Not recorded in the note as a modelled component. There is no volatility model, no risk term and no position sizing in the paper. The nearest related observation in my note is a failure mode rather than a risk treatment: "Since seasonality and trend removal were abandoned, the network is fitting levels rather than changes, which is the condition under which that failure mode is expected" (the failure mode being that the LSTM reproduces the shape of the series with a lag and smooths away the local swings).</t>
         </is>
       </c>
-      <c r="P61" s="30" t="inlineStr">
+      <c r="P60" s="30" t="inlineStr">
         <is>
           <t>None implemented, and this is a load-bearing omission. The disrupted-data problem that motivates the paper is never handled in the methodology: non-trading days on thin counters are named in the abstract as the reason a CSE-specific model is needed, and then "the only treatment is a general statement that missing values in the raw data were handled. Nothing says whether an absent day was dropped, forward-filled or zero-filled, and on a lookback of four days the difference between those choices changes what the window contains. AGAL is a plantation counter and the most likely of the three to have gaps, which makes the omission load-bearing rather than cosmetic."
 No liquidity screen on counter selection either: JKH, CTC and AGAL "are described as powerful counters without a stated selection criterion, and they differ sharply in how actively they trade."
 No friction accounting at all: "There is also no position, no fee, no spread and no return, so the claim that at 58% accuracy 'the users will always receive an overall gain' does not follow from anything in the paper." My note sets that against the local evidence: "on a market where [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] measures unexpected illiquidity shocks depressing returns by 8 to 10 basis points, a near-coin-flip signal traded daily is the case where costs decide the outcome."</t>
         </is>
       </c>
-      <c r="Q61" s="30" t="inlineStr">
+      <c r="Q60" s="30" t="inlineStr">
         <is>
           <t>Not recorded in the note as an explicit contribution. The nearest thing is the reporting of the weight ratio itself, which my note credits as the one advantage this paper has over the LLM systems for gap-argument purposes: "the contrast is cleaner here than in any of the LLM systems, because this paper does at least have an explicit weight vector to point at." The paper does not report the realised per-day share each channel held, which is the quantity my note reconstructs and criticises it for omitting.</t>
         </is>
       </c>
-      <c r="R61" s="30" t="inlineStr">
+      <c r="R60" s="30" t="inlineStr">
         <is>
           <t>Protocol, which is the part my note credits: the authors reject k-fold cross validation explicitly, on the grounds that it assumes instances are independent and therefore ignores the temporal component, and use walk-forward validation instead, where real data for a batch is added back and the model retrained before predicting the next batch. My note positions that against the local set: "That puts this paper ahead of [[Machine Learning-Driven Sri Lankan Stock Market Prediction, Harnessing Economic Indicators and Sentiment Analysis]], which treats shuffling the series before splitting as a design improvement, and ahead of [[ARIMA and ANN Approach for forecasting daily stock price fluctuations of industries in Colombo Stock Exchange]], which selects a neural architecture with no validation partition at all."
 Metrics: an undefined "error score" on normalised data for the lookback sweep; accuracy, sensitivity, specificity, precision and Matthews correlation coefficient for the trend classification; 10-fold cross-validation accuracy for text-classifier selection.
 Baselines: none. "For a binary direction task the relevant floors are the majority-class rate and a persistence call, neither of which is computed, and the class balance needed to work out the first is not reported." No backtest, no position, no fee, no spread, no return. The only internal comparison is equal weights against the finalised 1:3 weights, and that comparison is contaminated (see LIMITATIONS).</t>
         </is>
       </c>
-      <c r="S61" s="30" t="inlineStr">
+      <c r="S60" s="30" t="inlineStr">
         <is>
           <t>- Headline: the combination lifts trend accuracy from 54% to 58%, and a 1:3 weight ratio favouring the text model beat equal weighting on the holdout set.
 - Precisely: accuracy moves from 0.5622 to 0.5837 and the Matthews correlation from 0.0966 to 0.1493. My reading: "Accuracy on a binary task whose class balance is never reported is close to uninformative... At 0.1493 the finalised model has some directional signal and not much, and the gap between an accuracy that sounds like 58% and an MCC that sits at 0.15 is the whole story of the result."
@@ -8777,7 +8653,7 @@
 - Qualitative LSTM behaviour on CTC: the predicted line tracks the fall from roughly 1,350 to 1,290 and then flattens where the actual flattens, "but it cuts the amplitude of nearly every local swing and misses the terminal drop to about 1,203 entirely. The authors describe this as having predicted the basic behaviour with less fluctuations, which is accurate, and it is also the signature of a network leaning heavily on the most recent close."</t>
         </is>
       </c>
-      <c r="T61" s="30" t="inlineStr">
+      <c r="T60" s="30" t="inlineStr">
         <is>
           <t>- The weights were selected on the data the result is reported on. Table IV is headed as a holdout measurement and reports both the equal-weight and finalised instances on it, and the finalised ratio was found by changing the weights until performance was at its best. There is no third partition separating weight selection from reporting, so 0.5837 is an in-sample figure for the one parameter the paper's contribution turns on. "The 54% to 58% improvement is therefore not independently evidenced, and with the walk-forward machinery already built, holding out a separate window for the combination step would have cost very little."
 - The disrupted-data problem that motivates the paper is never handled in the methodology. Non-trading days on thin counters are named in the abstract as the reason a CSE-specific model is needed, then treated only by a general statement that missing values were handled. On a lookback of four days the choice between dropping, forward-filling and zero-filling changes what the window contains. AGAL is the counter most likely to have gaps, "which makes the omission load-bearing rather than cosmetic."
@@ -8788,7 +8664,7 @@
 - The 0.95 text-classifier CV score is not evidence of predictive skill, because the labels were derived from the target and 10-fold CV shuffles temporally adjacent articles covering the same event.</t>
         </is>
       </c>
-      <c r="U61" s="30" t="inlineStr">
+      <c r="U60" s="30" t="inlineStr">
         <is>
           <t>- Walk-forward with retraining as the protocol, with this paper as the local precedent I cite for it. Expanding training window, retrain on each batch, evaluate on the next, with the horizon and the refit policy stated as columns in every results table. My note's broader observation: "That is three CSE papers now where the modelling is ordinary and the evaluation is what separates them, which keeps pointing at the same thing: on this market the contribution worth making is evaluation that survives being checked."
 - A four to five day lookback as the starting point for the technical agent A_T, not thirty. "The error sweep here is the only direct evidence I have on window length for CSE counters and it says short beats long, with the curve turning sharply after five days. On a per-counter archive of 374 trading days a five-day lookback yields far more usable sequences than a thirty-day one, so this cuts in the same direction as the data-depth constraint, and window length goes into the ablation set rather than being inherited."
@@ -8799,17 +8675,17 @@
 - The 2021 data point on how thin the CSE's own announcement channel is, as a scoping input for A_F.</t>
         </is>
       </c>
-      <c r="V61" s="30" t="inlineStr">
+      <c r="V60" s="30" t="inlineStr">
         <is>
           <t>The combination weights are constants, chosen once by a small search and never conditioned on anything. There is no per-day reweighting, no conditioning on liquidity, volatility level or volatility persistence, no agent confidence term, and no designed abstention channel. The realised per-day influence is set by how many articles happened to be published, which is an availability-weighted scheme that was neither designed nor analysed as such, and the paper never states that quantity. The disrupted-data behaviour that motivates the paper, non-trading days on thin counters, is named and then not acted on in the methodology, so there is no treatment of what an absent observation does to a short lookback window. There is no execution-cost model, no spread, no fee and no return, so nothing here tells me whether a near-coin-flip directional signal survives CSE friction. Weight selection and result reporting share a partition, so even the one combination result is not independently evidenced. That is the opening my orchestrator sits in: replacing the constant with w(i,t) = f(L_t, V_t, P_t, C_{i,t}), with an explicit abstention state, with per-agent weights that sum to one independent of input volume, with the realised share logged, and with the combination step selected on a partition separate from the one it is reported on.</t>
         </is>
       </c>
-      <c r="W61" s="30" t="inlineStr">
+      <c r="W60" s="30" t="inlineStr">
         <is>
           <t>[[Quantitative Analysis and Sentiment Analysis for Stock Price Forecast, The Case of Colombo Stock Exchange]]</t>
         </is>
       </c>
-      <c r="X61" s="30" t="inlineStr">
+      <c r="X60" s="30" t="inlineStr">
         <is>
           <t>SPEAKS TO: The main gap, directly and locally; the evaluation protocol; the scoping of A_F; the window length for A_T; and the abstention channel. This is the CSE-local instance of the fixed-influence failure, and in my note it "belongs in the gap argument beside FinAgent and AlphaAgents." It is also retained evidence under the exception the supervisor granted for sentiment papers: the scope decision of 20 September 2026 (status Final) removed the sentiment component from my architecture, not the sentiment papers from my literature review.
 EFFECT ON MAIN GAP: Strengthens it, and strengthens it more cleanly than the LLM systems do, because there is an explicit numeric weight vector to point at. Two heterogeneous models, one shared decision, and the combination rule is a constant chosen once by trying a few values and keeping the best. What I am building replaces the constant with a function of measured state, Decision_t = sum_i w_{i,t} A_{i,t} with w_{i,t} = f(L_t, V_t, P_t, C_{i,t}). Three specific consequences for the design of f. First, C_{i,t} cannot be an in-domain self-score: this paper gave the text model three times the influence because it scored 0.95 in isolation, on a task that was mechanically easier than the one it was being weighted for, and the joint result then contributed about four accuracy points. That is the concrete argument for treating confidence as a structural property of the output and for setting weights from measured marginal contribution via ablation on held-out windows. Second, the weight vector must be normalised over agents explicitly, one scalar per agent regardless of how many documents, bars or signals that agent consumed, because here the denominator let input volume set the realised share; at the stated 1:3 ratio one article gives the text channel 75% and two give it 86%, so the LSTM carried roughly 14% of a typical day's decision while the paper reported the ratio as 1:3. The realised share per agent per day goes into my logs so the intended weighting can be audited against the realised one. Third, the abstention channel gets a positive design here by negative example: when no article appeared the text term simply vanished and the decision fell back to the quantitative model, which is the behaviour I want from A_F on a counter whose last filing is stale, but it has to be an explicit state with the remaining weights renormalised and the event recorded, because as implemented the system cannot tell a confident abstention from a quiet news day.
@@ -8820,6 +8696,7 @@
         </is>
       </c>
     </row>
+    <row r="61" ht="409.6" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-11 18:09:18
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -214,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -313,6 +313,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7423,49 +7429,49 @@
       </c>
     </row>
     <row r="54" ht="409.6" customHeight="1">
-      <c r="A54" s="29" t="inlineStr">
+      <c r="A54" s="34" t="inlineStr">
         <is>
           <t>P54</t>
         </is>
       </c>
-      <c r="B54" s="30" t="inlineStr">
+      <c r="B54" s="35" t="inlineStr">
         <is>
           <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid–ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
         </is>
       </c>
-      <c r="C54" s="30" t="inlineStr">
+      <c r="C54" s="35" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D54" s="30" t="inlineStr">
+      <c r="D54" s="35" t="inlineStr">
         <is>
           <t>Journal of Financial Economics (JFE), volume 161, article 103916.</t>
         </is>
       </c>
-      <c r="E54" s="30" t="inlineStr">
+      <c r="E54" s="35" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jfineco.2024.103916 — accessed 4 October 2026. Code and data: github.com/eguidotti/bidask.</t>
         </is>
       </c>
-      <c r="F54" s="30" t="inlineStr">
+      <c r="F54" s="35" t="inlineStr">
         <is>
           <t>Low-frequency microstructure econometrics — estimation of the effective bid–ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin–Schultz (2012) / Abdi–Ranaldo (2017) lineage.</t>
         </is>
       </c>
-      <c r="G54" s="30" t="inlineStr">
+      <c r="G54" s="35" t="inlineStr">
         <is>
           <t>Produce an estimator of the effective bid–ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
 The object being estimated is the effective spread, not the quoted spread. The quoted spread is the posted distance between best bid and best ask; the effective spread is the realised distance between the transaction price and the unobserved fundamental price, S = 2D(P − P̃)/P̃, with D = +1 for buyer-initiated and −1 for seller-initiated trades. They differ because dealers often execute inside the quotes, and "one of this paper's headline empirical results is that the end-of-day quoted spread overstates the effective spread by up to 100%." For a cost model the effective spread is the right object and the harder one, since P̃ is never observed.
 The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid–ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed — Roll additionally required equally likely buys and sells; Corwin–Schultz and Abdi–Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
         </is>
       </c>
-      <c r="H54" s="30" t="inlineStr">
+      <c r="H54" s="35" t="inlineStr">
         <is>
           <t>US equities (NYSE / AMEX / NASDAQ) as the main empirical setting, plus a cryptocurrency application on Binance. No emerging or frontier market anywhere in the paper. The note records: "Emerging and thin markets" are represented only by the crypto section, which "is the closest thing here to an illiquid non-US market" and "has no benchmark whatsoever".</t>
         </is>
       </c>
-      <c r="I54" s="30" t="inlineStr">
+      <c r="I54" s="35" t="inlineStr">
         <is>
           <t>Two evaluations (a simulation and a CRSP–TAQ empirical study) plus three applications.
 Simulation: Corwin and Schultz (2012) design as reused by Abdi and Ranaldo (2017). 10,000 months, each 21 trading days, each day 390 minutes. Fundamental price P̃_m = P̃_{m−1}e^{σz}, P̃_0 = 1, z standard Gaussian. Daily sd 3%, per-minute sd 3%/√390. Trade prices are P̃_m times one minus (plus) half the spread, 50% chance of a bid (ask). Trade probability varied so expected trades per day runs from 1 to 390. On no-trade days the previous day's close is forward-filled into all four prices. Spreads tested: 0.50%, 1.00%, 2.00% through 8.00%.
@@ -7473,12 +7479,12 @@
 Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high–low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
         </is>
       </c>
-      <c r="J54" s="30" t="inlineStr">
+      <c r="J54" s="35" t="inlineStr">
         <is>
           <t>Daily (or intraday) open, high, low and close prices and nothing else. No quote feed, no trade-by-trade data, no vendor dependency. The derived quantities are: o_t, h_t, l_t, c_t as log-prices; η_t = (h_t + l_t)/2 the mid log-price; and the indicator τ_t that flags whether the high, the low and the previous close all coincide. The note flags the τ_t indicator as itself a usable feature — "the fraction of days on which the open or close coincides with the high or low, which falls out of the EDGE computation at no extra cost".</t>
         </is>
       </c>
-      <c r="K54" s="30" t="inlineStr">
+      <c r="K54" s="35" t="inlineStr">
         <is>
           <t>"There is no architecture, this is an estimator, and the whole mechanism rests on one indicator variable."
 τ_t = 0 if h_t = l_t = c_{t−1}, and 1 otherwise.
@@ -7497,47 +7503,47 @@
 Output: an effective spread in basis points per asset per period, from OHLC alone.</t>
         </is>
       </c>
-      <c r="L54" s="30" t="inlineStr">
+      <c r="L54" s="35" t="inlineStr">
         <is>
           <t>Not applicable — this is a closed-form econometric estimator with no agents, no decision and no orchestration. The note states it plainly: "This is tooling, not a competitor architecture, there is no agent in it and no trading decision, but it goes at the part of my design that is currently weakest."</t>
         </is>
       </c>
-      <c r="M54" s="30" t="inlineStr">
+      <c r="M54" s="35" t="inlineStr">
         <is>
           <t>Not applicable — the paper uses only OHLC prices and contains no textual or sentiment component. (Sentiment is out of scope for this project in any case, per the supervisor decision.)</t>
         </is>
       </c>
-      <c r="N54" s="30" t="inlineStr">
+      <c r="N54" s="35" t="inlineStr">
         <is>
           <t>Not applicable — no disclosures, filings, retrieval or text of any kind. The only inputs are the four daily prices.</t>
         </is>
       </c>
-      <c r="O54" s="30" t="inlineStr">
+      <c r="O54" s="35" t="inlineStr">
         <is>
           <t>No volatility model is estimated, but volatility enters the paper twice as a nuisance that drives the estimator's error. First, through the truncation channel: because Ŝ² can come out negative in small samples, standard practice is to reset negatives to zero, and Jahan-Parvar and Zikes (2023) show this introduces a strong upward bias that does not decline with sample size, "with volatility as its primary driver". Second, through the spread-to-volatility ratio: the degradation of correlation with the TAQ benchmark over time is attributed by the authors to spreads shrinking relative to volatility, consistent with the spread-quintile table where correlation runs 17.84% in the narrowest quintile against 71.38% in the widest.
 The note also flags a tension with the volatility side of the project's own literature: Assumption 1 rules out serially correlated fundamental returns, "which sits uneasily beside the long-memory results on the ASPI and SL20 in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], though that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it."
 Estimation variance is roughly proportional to σ₁⁴/N for N observations at per-period volatility σ₁, so the standard error scales with σ₁²/√N — which is the formula behind the frequency result below.</t>
         </is>
       </c>
-      <c r="P54" s="30" t="inlineStr">
+      <c r="P54" s="35" t="inlineStr">
         <is>
           <t>This is the whole paper. EDGE measures the effective spread — the realised cost of a marginal trade — directly, in basis points, from OHLC. The discreteness correction is explicitly a function of how thinly the asset trades: the probability that the open or close coincides with the high or low is "a direct consequence of too few trades per period", running from about 25% for large-cap US stocks to 75% for small-caps over 1926–2021, peaking in the 1930s and 1940s, collapsing after 2000 with electronification to roughly 2–5% for large-caps while small-caps still sit near 15% at the end of the sample. The authors' own reading is that "the correction is less significant for recent samples and becomes essential for small stocks and for older periods, and crucially that it also depends on sampling frequency, since going from daily to intraday prices reduces the trades observed per interval and pushes the probability back up."
 What the paper does NOT handle: order size. "There is no order size anywhere in the model, so what EDGE measures is the cost of a marginal trade." The effective spread is computed from the transaction prices that happened, at whatever sizes they happened in, and the estimator has no mechanism for saying what a larger order would have paid.</t>
         </is>
       </c>
-      <c r="Q54" s="30" t="inlineStr">
+      <c r="Q54" s="35" t="inlineStr">
         <is>
           <t>Not applicable in the ML sense — there is no black box. The estimator is closed-form, every term is interpretable, and the discreteness correction has a direct structural reading (the denominator is one under continuous observation and shrinks in proportion to how often the price failed to move). Reproducibility is strong: implementations in several languages, the computed spread data, and a Harvard Dataverse replication package.</t>
         </is>
       </c>
-      <c r="R54" s="30" t="inlineStr">
+      <c r="R54" s="35" t="inlineStr">
         <is>
           <t>Baselines: ROLL (Roll 1984), CS (Corwin and Schultz 2012), AR (Abdi and Ranaldo 2017), plus the paper's own intermediate estimators OHLC and CHL. Benchmark truth is the Holden and Jacobsen (2014) TAQ-based effective spread, May 1993 – December 2021.
 Evaluation axes: (i) simulation bias as a function of expected trades per day from 390 down to 1; (ii) simulation mean and standard deviation across true spreads 0.50%–8.00%; (iii) empirical Pearson and Spearman correlation, MAPE, RMSE and fraction of non-positive estimates on 1,637,621 merged stock-months, cut by market venue, sub-period, size quintile and decile, spread quintile and trading-frequency quintile; (iv) daily versus minute sampling on 711,161 stock-months; (v) the Binance crypto application across daily / hourly / minute, which has no benchmark.
 The note records a caveat on the empirical comparison: "The comparison is descriptive throughout, no standard errors on the differences and no formal test, which at this sample size is defensible but means the quintile tables are read by eye."</t>
         </is>
       </c>
-      <c r="S54" s="30" t="inlineStr">
+      <c r="S54" s="35" t="inlineStr">
         <is>
           <t>1. Infrequent trading breaks the alternatives and not EDGE. At 390 trades per day all estimators are unbiased and recover the 1% simulated spread. By 100 trades per day CS estimates 0.75%; by around twenty trades per day it has fallen to 0.1%; and below roughly thirteen trades per day CS returns exactly zero. AR degrades more gracefully but is still biased down to about 0.30% at one trade per day and 0.62% at roughly two. EDGE tracks 1.00% across the entire range, including simulations where only a single trade per period is expected on average. The note: "This is the single most transferable result in the paper for my purposes and I report it as the paper's evidence rather than as a general claim, since the simulation's price process is a geometric Brownian motion and its no-trade handling is forward-filling rather than genuine absence."
 2. Variance. Under infrequent trading, mean estimate with sd in parentheses against the true spread:
@@ -7552,7 +7558,7 @@
 5. The discreteness term is itself a market-structure measurement: the coincidence probability ranges from ~25% (US large-cap) to 75% (small-cap) over 1926–2021, peaking in the 1930s–40s, collapsing after 2000 to 2–5% for large-caps with small-caps still near 15%.</t>
         </is>
       </c>
-      <c r="T54" s="30" t="inlineStr">
+      <c r="T54" s="35" t="inlineStr">
         <is>
           <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% — "a bias roughly seven times the quantity being measured" — and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
 2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid–ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information — Chen et al. (2017) being their example — is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
@@ -7563,9 +7569,22 @@
 7. A premise doing quiet work throughout: that the effective spread is the whole of the transaction cost, since nothing in the model has an order size in it. The paper never claims otherwise and the title is honest about scope.</t>
         </is>
       </c>
-      <c r="U54" s="30" t="inlineStr">
-        <is>
-          <t>- EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC — the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
+      <c r="U54" s="35" t="inlineStr">
+        <is>
+          <t>STATUS, 11 OCTOBER 2026 - DEMOTED TO LAST RESORT, AND MAY NEVER BE USED AT ALL. EDGE is held as a contingency measurement route, not as a component of the design, and nothing load-bearing may rest on it.
+THE REASON IS THAT IT IS UNVALIDATED ON THIN AND FRONTIER MARKETS. The paper's empirical work is CRSP-TAQ US equities plus a Binance cryptocurrency section that carries no quote benchmark at all - the authors state plainly that trade and quote data were unavailable to them - so there is no emerging or frontier market anywhere in it. Its own numbers put the estimator at its weakest precisely where the CSE sits: 25.63% of estimates from daily prices are non-positive, 41% of large-cap stock-months come out negative before truncation, and the thinnest simulated panel is roughly four expected trades per day with no-trade days forward-filled, against CSE counters that can go whole days without trading at all. A monthly window on the per-counter archive gives about 21 observations, squarely inside that regime.
+THE CONSEQUENCE. Applying it to the CSE would mean defending a number produced in the regime the paper never validates, on a market that has no quote data to check it against - so the estimate could not be falsified even in principle. If EDGE is computed at all it is a sensitivity check reported alongside the proxies, never the spread term behind a headline result. The cost term stays on the proxies already in the conditioning set: Amihud, turnover, zero-return frequency and the high-low range.
+The text below is retained as the record of the evaluation that produced this decision, in the same way the Dataset sheet keeps its excluded rows rather than deleting them. Read it as superseded.
+WHAT SURVIVES THE DEMOTION, because it costs nothing and requires no EDGE computation:
+- The infrequent-trading bias result as external evidence that thin-book calibration is a real problem and not a rhetorical one: below roughly thirteen trades per day Corwin-Schultz returns exactly zero and Abdi-Ranaldo is biased down by about a third, so any cost model built on those estimators would charge approximately nothing for trading the least liquid counters. Citable directly in the proposal; it is a statement about other estimators, not an output of this one.
+- The frequency result as a data-priority argument: a month of minute prices gives a standard error 7702 times smaller than a month of daily prices, where a year of daily prices gives only 3.5 times. That is a reason to ask the supervisor about any intraday CSE feed regardless of what is done with EDGE, and it is the same question as the volatility-estimator one.
+- The positioning rule, inverted. v5 held that there is no contribution in running a published 2024 JFE estimator on a new market. That still holds, and now cuts the other way too: there is also no cost in not running it.
+WHAT IS WITHDRAWN WITH THE DEMOTION:
+- EDGE itself as the measurement half of the cost model. Withdrawn. The cost term reverts to the proxies already in L_t until real quotes arrive.
+- The two candidate L_t inputs, the measured spread and the tau_t staleness indicator. Both fall out of an EDGE computation and are therefore not computed. L_t stays on Amihud, turnover, zero-return frequency and the high-low range.
+- The forced window decision (quarterly per-counter, monthly index-track, non-positive fraction reported alongside every series). Moot unless EDGE is revived, and retained below only as the specification to follow if it ever is.
+--- RETAINED AS RECORD, SUPERSEDED ---
+- EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC — the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
 - The infrequent-trading bias result as external evidence that thin-book calibration is a real problem, not a rhetorical one: below roughly thirteen trades per day CS returns exactly zero and AR is biased down by about a third at a few trades per day, "which means any cost model built on those estimators would charge approximately nothing for trading the least liquid counters on the CSE. That is backwards in the most expensive possible direction." Worth citing directly in the proposal when defending the thin-book calibration item.
 - Two new candidate inputs to the liquidity state L_t. (a) The measured spread itself, which unlike Amihud (price impact per unit volume), turnover (activity) and zero-return frequency (staleness) "is denominated in the same units as the objective". (b) The τ_t indicator — the fraction of days on which the open or close coincides with the high or low — which "falls out of the EDGE computation at no extra cost" and is a candidate staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both go into the ablation protocol "as additions to test rather than adopt".
 - A forced window decision. Given 25.63% non-positive daily-price estimates on CRSP and 41% negative for large-caps, and a monthly estimate from the per-counter archive being roughly 21 observations — "squarely in that regime" — the decision is a quarterly window on the per-counter track, accepting a cost term that cannot move within a quarter, and monthly on the index track where ten years of daily data supports it, "with the fraction of non-positive estimates reported alongside every spread series in both cases. Reporting that fraction is not optional here, it is the only visible signal that the truncation is distorting the number."
@@ -7573,22 +7592,30 @@
 - A positioning rule. EDGE is a 2024 JFE paper with public implementations, open spread data and a replication package, "so there is no contribution in running it on a new market and no reason to imply one." The defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered, and that the contribution is what an orchestrator does with a cost term that varies by counter and date rather than the estimator that produces it. "One sentence, offered before anyone asks."</t>
         </is>
       </c>
-      <c r="V54" s="30" t="inlineStr">
+      <c r="V54" s="35" t="inlineStr">
         <is>
           <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
 Second, the small-count regime is untested: the estimator is defined with three usable observations but the paper never characterises its behaviour there, and that is exactly the regime a CSE counter with five trading days in a month occupies.
 Third, the paper measures a spread; it never puts that spread inside a decision objective. "It sits alongside [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] as the measurement layer those papers assume and never supply." The claim that cost belongs inside the objective rather than deducted afterwards is still mine to make — and now has two separately validated pieces behind the cost term.
-Fourth, no validation against a quote-based benchmark in an emerging or frontier market: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."</t>
-        </is>
-      </c>
-      <c r="W54" s="30" t="inlineStr">
-        <is>
-          <t>[[Efficient estimation of bid–ask spreads from open, high, low, and close prices]]</t>
-        </is>
-      </c>
-      <c r="X54" s="30" t="inlineStr">
-        <is>
-          <t>SPEAKS TO: A_L above all — this is the measurement instrument the liquidity agent currently lacks — plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
+Fourth, no validation against a quote-based benchmark in an emerging or frontier market: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
+AMENDED 11 OCTOBER 2026: with EDGE demoted to last resort, the INTERCEPT of the cost function is open as well, not only the slope. The whole cost term now rests on proxies until real CSE quotes are obtained, which makes the CSE request for bid/ask and depth materially more important than v5 recorded - it is no longer a validation step for an estimator already built, it is the only route to a measured spread.</t>
+        </is>
+      </c>
+      <c r="W54" s="35" t="inlineStr">
+        <is>
+          <t>[[Efficient estimation of bid–ask spreads from open, high, low, and close prices]]
+DEMOTED TO LAST RESORT, 11 Oct 2026 - may never be used. See Speaks To / Effect on the Gaps.</t>
+        </is>
+      </c>
+      <c r="X54" s="35" t="inlineStr">
+        <is>
+          <t>STATUS, 11 OCTOBER 2026 - DEMOTED TO LAST RESORT, AND MAY NEVER BE USED AT ALL. EDGE is held as a contingency measurement route, not as a component of the design, and nothing load-bearing may rest on it.
+THE REASON IS THAT IT IS UNVALIDATED ON THIN AND FRONTIER MARKETS. The paper's empirical work is CRSP-TAQ US equities plus a Binance cryptocurrency section that carries no quote benchmark at all - the authors state plainly that trade and quote data were unavailable to them - so there is no emerging or frontier market anywhere in it. Its own numbers put the estimator at its weakest precisely where the CSE sits: 25.63% of estimates from daily prices are non-positive, 41% of large-cap stock-months come out negative before truncation, and the thinnest simulated panel is roughly four expected trades per day with no-trade days forward-filled, against CSE counters that can go whole days without trading at all. A monthly window on the per-counter archive gives about 21 observations, squarely inside that regime.
+THE CONSEQUENCE. Applying it to the CSE would mean defending a number produced in the regime the paper never validates, on a market that has no quote data to check it against - so the estimate could not be falsified even in principle. If EDGE is computed at all it is a sensitivity check reported alongside the proxies, never the spread term behind a headline result. The cost term stays on the proxies already in the conditioning set: Amihud, turnover, zero-return frequency and the high-low range.
+The text below is retained as the record of the evaluation that produced this decision, in the same way the Dataset sheet keeps its excluded rows rather than deleting them. Read it as superseded.
+AMENDED EFFECT ON SUB-GAP 1, 11 OCTOBER 2026: the claim below that this paper CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 is WITHDRAWN. With EDGE demoted, the measurement half is open again and the cost term stays on the existing proxies until real CSE quotes are obtained. Sub-gap 1 is therefore stated with two caveats rather than one: a potentially overlapping 2026 paper (Smart Trading Rule) was identified and could not be obtained, AND the proxy route that would have substituted for the missing quote data is not validated on any market resembling the CSE. That is a weaker position than v5 recorded and it should be stated as such rather than discovered in the viva.
+--- RETAINED AS RECORD, SUPERSEDED ---
+SPEAKS TO: A_L above all — this is the measurement instrument the liquidity agent currently lacks — plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
 EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency — "all proxies for illiquidity rather than measurements of what a trade pays" — and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade — "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren–Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
 The second half of Sub-gap 1 — that liquidity simultaneously conditions the reliability of price-derived agents — gets independent support from the paper's own mechanism rather than from my framing. The τ_t = 0 condition is literally the case where the price carries no information about the spread within the period, and the coincidence probability that drives the correction is "a direct consequence of too few trades per period". That is a measured, published statement that price-derived quantities degrade in a specific, quantifiable way as trading thins — which is precisely the premise under which L_t should down-weight A_T.
 EFFECT ON MAIN GAP: Indirect but real. The main gap is market-state-aware dynamic orchestration with w(i,t) = f(L_t, V_t, P_t, C_{i,t}), and the weakest-specified argument of that function is L_t. This paper contributes two candidate components to it that measure something the existing three proxies do not. The spread gives L_t a component denominated in the same units as the objective. The τ_t indicator gives a staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both enter the ablation protocol as additions to test rather than adopt, "which turns the question from whether liquidity matters into whether a measured spread and a measured staleness rate carry anything beyond the three proxies already there." That reframing is itself useful: it converts a soft claim about liquidity-awareness into a falsifiable ablation.

</xml_diff>

<commit_message>
vault backup: 2026-10-11 18:24:21
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -8899,75 +8899,77 @@
       </c>
     </row>
     <row r="3" ht="409.6" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Sub-gap 1
 (Former G1)</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="33" t="inlineStr">
         <is>
           <t>NARROWED IN V5. No reviewed work calibrates a nonlinear, depth-conditioned execution-cost function to a thin frontier order book, nor sweeps participation rate to establish the shape of that cost curve where a single order is a material fraction of resting depth; and no portfolio-allocation system embeds such a cost function inside its allocation objective rather than deducting a flat rate after the fact. This is a calibration-and-integration gap, not a modelling-form gap, and the change is deliberate.</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="33" t="inlineStr">
         <is>
           <t>Method-Integration + Domain</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="33" t="inlineStr">
         <is>
           <t>THE GENERIC CLAIM IS DEAD AND MUST NOT BE WRITTEN AGAIN. Two papers implement size-dependent execution cost directly. Chen et al. (ICAIF '22) build a queue-reactive LOB simulator where impact is fully endogenous, an order consumes queue, brings a level toward depletion and raises the probability of an adverse mid-price move, and they quantify the cost of ignoring it at 3.04 bps on seven liquid US names. Wang, Gao and Li (Finance and Stochastics 2026) implement Almgren-Chriss explicitly with linear permanent and temporary impact, solve it in closed form, and evaluate inside a LOBSTER historical-order-flow simulator with permanent book contamination. The allocation literature still leaves the assumption intact, Moallemi and Wang assume the order infinitesimal, Guo et al. use one scalar for all assets and sizes, HLOB has no cost model, and the RL survey confirms fixed costs and assumed execution certainty as the field convention with the one modelled form proportional to position change rather than to order size against depth. But that silence is now evidence of a division of labour between the execution and allocation literatures, not of an absence in the field.</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="33" t="inlineStr">
         <is>
           <t>Wang, Gao and Li IS the 2026 Almgren-Chriss market-impact work the supervisor cited and v4 carried as unverified, so open item 2 is closed and the supervisor's prediction was correct. Chen et al. is the queue-reactive equivalent. Four things survive them, and the notes state all four independently. (1) NONLINEARITY: every impact model in the set is linear or mechanistic-but-unswept, neither tests a square-root or concave form, and Potters-Bouchaud logarithmic impact appears once in the whole corpus as a future-work line. (2) NO ORDER-SIZE SWEEP ANYWHERE, and both execution notes say it in nearly the same words, Chen et al. running everything at one inventory and horizon and Wang et al. everything at 10% of ADTV, so the shape of the cost curve in order size is empirically untested across the entire set. (3) THIN-MARKET CALIBRATION: not one of the five calibrates to a market where a single order is a visible fraction of resting depth; universes are NASDAQ, IEX and LOBSTER large caps trading 2 to 115 million shares a day. (4) THE PASSIVE SIDE: all three execution papers are market-orders-only, no spread capture, no queue position, no partial fills, no cancellation, no fees. Guo et al. turns from foil into asset here, its transaction remainder factor with constant bounds is the container that lets a cost term stay inside a convex objective rather than sitting outside as a post-hoc deduction, and substituting a state-dependent cost into it is the constructive move.</t>
         </is>
       </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="F3" s="33" t="inlineStr">
         <is>
           <t>Unexpected illiquidity shocks depress contemporaneous CSE returns at -0.084 to -0.097, small caps more than large. The amplification argument is now explicit and is the load-bearing sentence: if ignoring impact costs about 3 bps on names trading two to a hundred and fifteen million shares a day, then on a counter where a single order is a visible fraction of resting depth the same neglect is not a small correction to a backtest, it is capable of reversing the sign of a reported edge. That is an argument by amplification rather than a calibrated result, and it should be stated as such.</t>
         </is>
       </c>
-      <c r="G3" s="16" t="inlineStr">
+      <c r="G3" s="33" t="inlineStr">
         <is>
           <t>Technical: a nonlinear, depth-conditioned cost function calibrated to a thin frontier book and embedded inside the allocation objective rather than deducted afterwards. Domain: a participation-rate sweep establishing the shape of the cost curve on a market where order size is material relative to depth, which is the cleanest remaining claim in the set and which no reviewed paper provides for any market.</t>
         </is>
       </c>
-      <c r="H3" s="16" t="inlineStr">
+      <c r="H3" s="33" t="inlineStr">
         <is>
           <t>Substitute a state-dependent cost into Guo et al.'s transaction remainder factor so it stays inside the convex objective. Sweep participation rate rather than fixing it. Prefer a LEARNED friction component over naive calibrate-then-plug-in, on Wang et al.'s own evidence that estimation error in the impact parameters is amplified through the closed-form control, their statistical calibration turning in -905.742 on AAPL at high risk aversion against the learned variant's +102.285, and on CSE data the estimation error would be strictly worse. Run the tick-size classification on CSE counters first, since it needs only best bid, best ask and the tick schedule, and if liquid CSE counters come out small-tick the microstructural route is ruled out at near-zero cost and the friction work is daily-bar-based by necessity rather than preference.</t>
         </is>
       </c>
-      <c r="I3" s="16" t="inlineStr">
-        <is>
-          <t>Per-counter CSE daily price and turnover for the volume profile and the Amihud measure. The data ladder is now explicit: level-III message data for the full queue-reactive route and almost certainly out of reach; multi-level depth snapshots for a weaker version; top-of-book only for the tick classification, which is decisive and nearly free and runs first; intraday trade-and-quote without depth for the five-scalar policy route, which is fittable on a short archive where a learned agent is not; and daily bars only for the fallback, turnover, traded value, zero-return frequency and Amihud-style measures.</t>
-        </is>
-      </c>
-      <c r="J3" s="16" t="inlineStr">
+      <c r="I3" s="33" t="inlineStr">
+        <is>
+          <t>Per-counter CSE daily price and turnover for the volume profile and the Amihud measure. The data ladder is now explicit: level-III message data for the full queue-reactive route and almost certainly out of reach; multi-level depth snapshots for a weaker version; top-of-book only for the tick classification, which is decisive and nearly free and runs first; intraday trade-and-quote without depth for the five-scalar policy route, which is fittable on a short archive where a learned agent is not; and daily bars only for the fallback, turnover, traded value, zero-return frequency and Amihud-style measures.
+AMENDED 11 OCTOBER 2026: the bottom rung of that ladder is where this now sits, and it has no spread measurement on it. The EDGE route that would have put a measured effective spread on the daily-bars rung is demoted to last resort and is not assumed available. This changes what the CSE request is for: bid/ask and depth are no longer a validation extra for an estimator already built, they are the only route to a measured spread, which moves them to the top of the request rather than the middle.</t>
+        </is>
+      </c>
+      <c r="J3" s="33" t="inlineStr">
         <is>
           <t>(a) Zero-cost execution. (b) Flat 2 bps. (c) FreQuant's solved fee fixed point with no impact term. (d) Naive full-size execution at close. (e) NEW, Almgren-Chriss at a fixed participation rate, which is now the strongest published treatment and therefore the baseline that actually matters. (f) NEW, the 19-strategy training-free OLPS family plus First All / Last All / TWAP / VWAP.</t>
         </is>
       </c>
-      <c r="K3" s="16" t="inlineStr">
+      <c r="K3" s="33" t="inlineStr">
         <is>
           <t>The framework under all cost regimes, plus the participation-rate sweep that is missing from the whole literature. TWO EXPERIMENTS ARE INDEPENDENT OF THE CSE DATA BLOCKER and both should run while the data request is outstanding: sweeping the cost parameter from 5 bps to north of 100 bps on Guo et al.'s own four datasets, which establishes where the crossover against simpler baselines sits and is directly the argument for why a frontier market needs different machinery; and the tick-size classification on CSE counters from top-of-book alone. Report the half-spread unit, average transaction cost in bps against the decision price, risk-adjusted PnL relative to TWAP, and round-trip practicability against action count, since the first two are pure cost measures indifferent between a reliable schedule and a volatile one.</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
+      <c r="L3" s="33" t="inlineStr">
         <is>
           <t>High for the daily-turnover version and for both blocker-independent experiments. Low for anything needing level-III messages or queue intensities, which the notes judge almost certainly out of reach. The evaluation layer and A_L are gated on exactly the same data, so whatever cannot be observed cannot be simulated either, and they should be treated as one workstream and one data request rather than two.</t>
         </is>
       </c>
-      <c r="M3" s="16" t="inlineStr">
-        <is>
-          <t>The novelty has genuinely narrowed and the rating moves with it rather than being defended at its old level. There is still no ground-truth execution data to validate a CSE simulator against, so simulated slippage is not measured slippage and must be presented that way. The tick-size classification may return small-tick, which would close the microstructural route entirely. And a reviewer who knows the execution literature will ask why the impact model is not simply Almgren-Chriss with CSE parameters, so the nonlinearity and the in-objective embedding have to be the argued contribution rather than the calibration alone.</t>
-        </is>
-      </c>
-      <c r="N3" s="16" t="inlineStr">
-        <is>
-          <t>RETAIN, NARROWED - generic claim withdrawn, calibration and in-objective embedding retained  |  Revised novelty 3 / 5</t>
+      <c r="M3" s="33" t="inlineStr">
+        <is>
+          <t>The novelty has genuinely narrowed and the rating moves with it rather than being defended at its old level. There is still no ground-truth execution data to validate a CSE simulator against, so simulated slippage is not measured slippage and must be presented that way. The tick-size classification may return small-tick, which would close the microstructural route entirely. And a reviewer who knows the execution literature will ask why the impact model is not simply Almgren-Chriss with CSE parameters, so the nonlinearity and the in-objective embedding have to be the argued contribution rather than the calibration alone.
+ADDED 11 OCTOBER 2026 - SUB-GAP 1 NOW CARRIES TWO CAVEATS AND THEY MUST BE STATED TOGETHER. (1) Smart Trading Rule (Journal of Financial Data Science 8(2), 2026) was identified, judged potentially overlapping on the modular transaction-cost layer, and could not be obtained because it is paywalled. Its contents are unknown to me, so this sub-gap is not presented as though the literature had been fully swept. (2) THE MEASUREMENT HALF IS OPEN AGAIN. P54, the EDGE estimator of effective spread from daily OHLC, was the route that would have substituted for the CSE's missing quote data, and on 11 October it was demoted to last resort because it is unvalidated on thin and frontier markets - no emerging or frontier market appears anywhere in that paper, its crypto section has no quote benchmark at all, and its own numbers put it at its weakest exactly where the CSE sits. With no CSE quote data to validate against, an EDGE spread here could not be falsified even in principle. So the cost term rests on proxies for illiquidity - Amihud, turnover, zero-return frequency and the high-low range - rather than on any measurement of what a trade actually pays. That is a weaker evidential base than v5 recorded and the write-up should say so rather than leave it to be found. The defensible form is that the cost function is calibrated on proxies because no validated spread measurement exists for this market, and that validating it is what the CSE data request is for.</t>
+        </is>
+      </c>
+      <c r="N3" s="33" t="inlineStr">
+        <is>
+          <t>RETAIN, NARROWED - generic claim withdrawn, calibration and in-objective embedding retained  |  Revised novelty 3 / 5  |  11 Oct 2026: unchanged in substance, but state it with BOTH caveats - the unobtainable Smart Trading Rule and the demoted EDGE proxy route.</t>
         </is>
       </c>
     </row>
@@ -12279,119 +12281,123 @@
       </c>
     </row>
     <row r="24" ht="409.6" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t>D23</t>
         </is>
       </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Effective bid-ask spread estimated from OHLC (derived)</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>Effective bid-ask spread estimated from OHLC (derived) - LAST RESORT, MAY NEVER BE COMPUTED</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>Derived dataset</t>
         </is>
       </c>
-      <c r="D24" s="30" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>Own computation over D22, following Ardia, Guidotti &amp; Kroencke, Journal of Financial Economics 2024</t>
         </is>
       </c>
-      <c r="E24" s="30" t="inlineStr">
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>Grid #61 in the Research Papers Grid; reference implementations are public</t>
         </is>
       </c>
-      <c r="F24" s="30" t="inlineStr">
+      <c r="F24" s="35" t="inlineStr">
         <is>
           <t>CSE, every security in D22 that survives the D17 screen.</t>
         </is>
       </c>
-      <c r="G24" s="30" t="inlineStr">
+      <c r="G24" s="35" t="inlineStr">
         <is>
           <t>Derived per-security daily spread estimate. The Level A proxy route for Sub-gap 1.</t>
         </is>
       </c>
-      <c r="H24" s="30" t="inlineStr">
+      <c r="H24" s="35" t="inlineStr">
         <is>
           <t>Same span as D22: 2012-01-02 to 2026-10-02.</t>
         </is>
       </c>
-      <c r="I24" s="30" t="inlineStr">
+      <c r="I24" s="35" t="inlineStr">
         <is>
           <t>Daily, per security.</t>
         </is>
       </c>
-      <c r="J24" s="30" t="inlineStr">
+      <c r="J24" s="35" t="inlineStr">
         <is>
           <t>Not yet computed. Upper bound is the D22 panel.</t>
         </is>
       </c>
-      <c r="K24" s="30" t="inlineStr">
+      <c r="K24" s="35" t="inlineStr">
         <is>
           <t>Estimated effective spread per security-day, from open, high, low and close.</t>
         </is>
       </c>
-      <c r="L24" s="30" t="inlineStr">
+      <c r="L24" s="35" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="M24" s="30" t="inlineStr">
+      <c r="M24" s="35" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="N24" s="30" t="inlineStr">
+      <c r="N24" s="35" t="inlineStr">
         <is>
           <t>One pass over data already held. No external dependency, no permission, no subscription.</t>
         </is>
       </c>
-      <c r="O24" s="30" t="inlineStr">
+      <c r="O24" s="35" t="inlineStr">
         <is>
           <t>n/a - derived. Inherits whatever terms attach to D22.</t>
         </is>
       </c>
-      <c r="P24" s="30" t="inlineStr">
-        <is>
-          <t>NOT YET COMPUTED. Three limits to state before relying on it. (1) It estimates the EFFECTIVE spread, not quoted spread and not depth, so it supports a cost model but not a queue-reactive one. (2) Accuracy is known to degrade in thin, frequently non-trading conditions - which is exactly the CSE case this is wanted for, so it must be reported by liquidity tier from D17 rather than pooled. (3) It is an estimate validated on other markets and not on the CSE; it needs checking against real quotes on whatever window can be obtained before any headline result rests on it.</t>
-        </is>
-      </c>
-      <c r="Q24" s="30" t="inlineStr">
-        <is>
-          <t>Method verified - peer-reviewed in the Journal of Financial Economics. The CSE estimates do not exist yet.</t>
-        </is>
-      </c>
-      <c r="R24" s="30" t="inlineStr">
-        <is>
-          <t>A_L and the friction-aware evaluation layer.</t>
-        </is>
-      </c>
-      <c r="S24" s="30" t="inlineStr">
-        <is>
-          <t>Converts the bid-ask gap from a blocker into a validation target. D22 carries open, high, low and close, which is exactly this estimator's input, so the Level A proxy route in the execution model can be built now rather than waiting on the CSE or on a MyCSE subscription. It also gives the CSE request a fallback: if bid/ask is refused, the sub-gap degrades to a proxy-based model with a published method behind it instead of collapsing.</t>
-        </is>
-      </c>
-      <c r="T24" s="30" t="inlineStr">
-        <is>
-          <t>An estimate, not an observation. Does not provide depth, so the microstructure route (D21) stays closed without real order-book data. Its weakest regime is the thin-counter case the research is most interested in.</t>
-        </is>
-      </c>
-      <c r="U24" s="30" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="V24" s="30" t="inlineStr">
-        <is>
-          <t>COMPUTE - after D17, before the CSE reply</t>
-        </is>
-      </c>
-      <c r="W24" s="30" t="inlineStr">
-        <is>
-          <t>Do not let this remove the CSE request. It changes what the request is FOR: real quotes become the validation set for an estimator that is already built, rather than the precondition for building one. That is a much better position to negotiate from, and it means a refusal costs the project a validation step instead of a component.</t>
+      <c r="P24" s="35" t="inlineStr">
+        <is>
+          <t>NOT YET COMPUTED. Three limits to state before relying on it. (1) It estimates the EFFECTIVE spread, not quoted spread and not depth, so it supports a cost model but not a queue-reactive one. (2) Accuracy is known to degrade in thin, frequently non-trading conditions - which is exactly the CSE case this is wanted for, so it must be reported by liquidity tier from D17 rather than pooled. (3) It is an estimate validated on other markets and not on the CSE; it needs checking against real quotes on whatever window can be obtained before any headline result rests on it.
+DECISION CHANGED 11 OCTOBER 2026 - the third limit below is now the governing one rather than one of three. The estimator is UNVALIDATED ON THIN AND FRONTIER MARKETS: the paper's empirical work is CRSP-TAQ US equities plus a Binance section carrying no quote benchmark at all, so no emerging or frontier market appears anywhere in it, and its own numbers put it at its weakest exactly where the CSE sits - 25.63% of daily-price estimates non-positive, 41% of large-cap stock-months negative before truncation, thinnest simulated panel roughly four expected trades per day with no-trade days forward-filled. A monthly window on D22 is about 21 observations, squarely inside that regime. The CSE has no quote data to check the output against, so an estimate produced here could not be falsified even in principle, which is a worse position than having no number because a number invites use.</t>
+        </is>
+      </c>
+      <c r="Q24" s="35" t="inlineStr">
+        <is>
+          <t>Method verified - peer-reviewed in the Journal of Financial Economics. NOT VERIFIABLE ON THIS MARKET: there is no CSE quote data to validate the estimates against, and that is the reason for the demotion rather than any doubt about the method. The CSE estimates do not exist and may never be computed.</t>
+        </is>
+      </c>
+      <c r="R24" s="35" t="inlineStr">
+        <is>
+          <t>NONE AS OF 11 OCTOBER 2026. Previously A_L and the friction-aware evaluation layer; both now run on the proxies (Amihud, turnover, zero-return frequency, high-low range). If EDGE is ever computed it feeds a sensitivity check, not a component.</t>
+        </is>
+      </c>
+      <c r="S24" s="35" t="inlineStr">
+        <is>
+          <t>Converts the bid-ask gap from a blocker into a validation target. D22 carries open, high, low and close, which is exactly this estimator's input, so the Level A proxy route in the execution model can be built now rather than waiting on the CSE or on a MyCSE subscription. It also gives the CSE request a fallback: if bid/ask is refused, the sub-gap degrades to a proxy-based model with a published method behind it instead of collapsing.
+SUPERSEDED 11 OCTOBER 2026. The argument above still describes what EDGE would give; it is retained as the record of the case for computing it. What it does not weigh is whether the resulting number could be defended, which is the question the demotion turns on.</t>
+        </is>
+      </c>
+      <c r="T24" s="35" t="inlineStr">
+        <is>
+          <t>An estimate, not an observation. Does not provide depth, so the microstructure route (D21) stays closed without real order-book data. Its weakest regime is the thin-counter case the research is most interested in.
+11 OCTOBER 2026: and the weakest regime is not merely the thin-counter case the research is most interested in, it is also the case the paper never validates and this market cannot validate. Those two facts together are what moved the decision.</t>
+        </is>
+      </c>
+      <c r="U24" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="V24" s="35" t="inlineStr">
+        <is>
+          <t>LAST RESORT - DO NOT COMPUTE AS A COMPONENT. May never be computed at all.</t>
+        </is>
+      </c>
+      <c r="W24" s="35" t="inlineStr">
+        <is>
+          <t>DEMOTED 11 OCTOBER 2026, and the demotion does not change what the CSE request is for - it raises its priority. Bid/ask and depth were previously the validation set for an estimator already built; they are now the ONLY route to a measured spread, because the proxy route is not defensible on this market. Until they arrive the cost model runs on proxies and the write-up says so.
+IF EDGE IS COMPUTED AT ALL it is a sensitivity check reported alongside the proxies, never the spread term behind a headline result, and the fraction of non-positive estimates and the per-counter observation count are reported with it every time, because those two numbers are the only visible signal that the estimate came from the regime the paper never validates.
+WHAT WOULD REVIVE IT, written down so the demotion is reversible on a stated condition: real CSE quotes for any window and any subset of counters, even a few weeks on the twenty most liquid names, would turn this from an unfalsifiable estimate into a validated one, and the computation is cheap once that exists. Failing that, a published validation of EDGE against a quote-based benchmark in a genuinely thin market by someone else.
+SUPERSEDED JUSTIFICATION, retained as the record: Do not let this remove the CSE request. It changes what the request is FOR: real quotes become the validation set for an estimator that is already built, rather than the precondition for building one. That is a much better position to negotiate from, and it means a refusal costs the project a validation step instead of a component.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 12:49:00
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>arXiv:2508.11152 | https://arxiv.org/abs/2508.11152</t>
+          <t>arXiv:2508.11152 | https://arxiv.org/abs/2508.11152 | DOI 10.48550/arXiv.2508.11152</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>MacroHFT | github.com/ZONG0004/MacroHFT</t>
+          <t>MacroHFT | github.com/ZONG0004/MacroHFT | DOI 10.1145/3637528.3672064</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="W21" s="14" t="inlineStr">
         <is>
-          <t>[[FinMe, A Performance-Enhanced LLM Trading Agent With Layered Memory and Character Design]]</t>
+          <t>[[FinMem, A Performance-Enhanced LLM Trading Agent With Layered Memory and Character Design]]</t>
         </is>
       </c>
       <c r="X21" s="14" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E27" s="28" t="inlineStr">
         <is>
-          <t>staged note only; no DOI/URL recorded in the note.</t>
+          <t>DOI 10.48550/ARXIV.2605.19337.</t>
         </is>
       </c>
       <c r="F27" s="28" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>journal article, open access; no URL in the note.</t>
+          <t>DOI 10.1016/j.iswa.2026.200653. journal article, open access</t>
         </is>
       </c>
       <c r="F29" s="20" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>no DOI/URL recorded in the note.</t>
+          <t>DOI 10.1016/j.ijforecast.2024.09.002.</t>
         </is>
       </c>
       <c r="F39" s="20" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>none recorded.</t>
+          <t>DOI 10.1109/ICITR51448.2020.9310826.</t>
         </is>
       </c>
       <c r="F42" s="20" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="E45" s="28" t="inlineStr">
         <is>
-          <t>none recorded. "No code release."</t>
+          <t>DOI 10.1016/j.ejor.2017.11.054. "No code release."</t>
         </is>
       </c>
       <c r="F45" s="28" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="E46" s="20" t="inlineStr">
         <is>
-          <t>no DOI recorded; "Code is on Code Ocean as a reproducible capsule, which is more than almost anything else in my set offers."</t>
+          <t>DOI 10.1016/j.asoc.2022.109876. "Code is on Code Ocean as a reproducible capsule, which is more than almost anything else in my set offers."</t>
         </is>
       </c>
       <c r="F46" s="20" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="W47" s="20" t="inlineStr">
         <is>
-          <t>[[Neo4j Graph-RAG for CSE]]</t>
+          <t>[[Neo4j-Powered Graph-RAG System for Financial Insights on the Colombo Stock Exchange]]</t>
         </is>
       </c>
       <c r="X47" s="20" t="inlineStr">
@@ -6952,7 +6952,7 @@
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>github.com/czyssrs/ConvFinQA — "built on top of FinQA and therefore on FinTabNet."</t>
+          <t>github.com/czyssrs/ConvFinQA — "built on top of FinQA and therefore on FinTabNet." | DOI 10.18653/v1/2022.emnlp-main.421</t>
         </is>
       </c>
       <c r="F50" s="20" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-10-18 19:07:28
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -14,6 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Survey'!$A$1:$X$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Research Gap Analysis'!$A$1:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Conditioning Set'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Reclassified Components'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -77,8 +80,14 @@
       <family val="2"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -155,6 +164,36 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -213,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -330,6 +369,33 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8752,95 +8818,95 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="17.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="8.77734375" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="30.21875" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="43.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="20.21875" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="19" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="23.21875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="13.44140625" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="18.5546875" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="22.6640625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="14" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="30" bestFit="1" customWidth="1" min="13" max="13"/>
-    <col width="8.77734375" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="16" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="62" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="72" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="82" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="52" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="50" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="60" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="46" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="52" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="62" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="42" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="62" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="34" bestFit="1" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="92.40000000000001" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="40" t="inlineStr">
         <is>
           <t>Gap ID &amp; Level</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="40" t="inlineStr">
         <is>
           <t>Reframed Research Gap</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="40" t="inlineStr">
         <is>
           <t>Gap Type</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="40" t="inlineStr">
         <is>
           <t>Literature Evidence &amp; Baseline Limitations</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="40" t="inlineStr">
         <is>
           <t>Nearest Prior Work &amp; Delta</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="40" t="inlineStr">
         <is>
           <t>Why CSE Exposes It</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="40" t="inlineStr">
         <is>
           <t>Contribution to Body of Knowledge</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="40" t="inlineStr">
         <is>
           <t>Proposed Technical Direction</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="40" t="inlineStr">
         <is>
           <t>Required Data</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="40" t="inlineStr">
         <is>
           <t>Baselines Required</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="40" t="inlineStr">
         <is>
           <t>Experiment &amp; Ablation</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="40" t="inlineStr">
         <is>
           <t>Feasibility</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="40" t="inlineStr">
         <is>
           <t>Risk &amp; Failure Mode</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="40" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="409.6" customHeight="1">
+    <row r="2" ht="549" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
           <t>MAIN GAP</t>
@@ -8858,12 +8924,14 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>The v4 framing was that existing systems weight agents badly. The reviews since have replaced it with a sharper and better-evidenced one: most existing systems have no quantity that could be weighted. TradingAgents runs seven roles through a hierarchy whose facilitator is described in a single sentence; FinVision concatenates four channels into one prompt; Park's anomaly framework summarises three experts into free text. The same absence stated three times across three unrelated designs is a property of the field rather than an artefact of any one architecture. External validation now exists for that reading: the ACM Computing Surveys review of 167 RL papers states that the establishment of coordination and communication protocols among different agents is underexplored. FinAgent still supplies the sharpest motivating failure, its auxiliary strategies returning 16% on ETHUSD against buy-and-hold's 29%, and there are now three such documented fixed-influence failures rather than one: Jung and Lee measure a 10.36-point total-return degradation from a text agent the architecture cannot notice, AlphaAgents deletes its sentiment agent by hand for thin coverage, and the temporal-shift work shows a sentiment channel decaying with nothing watching. PIXIU adds a fourth from the opposite direction, FinMA-7B-trade collapsing from 0.94 to 0.03 F1 on FPB after specialisation while gaining nothing on the task it was specialised for, which is the argument that the four agents must fail independently and that a shared backbone forbids exactly that.</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>MacroHFT is no longer the single opponent and the defence should be restructured as a five-way contrast, which is the most consequential change in v5. HEDGEAGENTS is now nearest on the orchestration-mechanism axis, the only paper where the orchestration layer is a solved constrained optimisation over an explicit weight vector with return, variance and CVaR terms, plus genuine state-triggered deliberation on a 5% daily / 10% three-day amplitude alarm across 36 emergency sessions in nine months. It is defeated on two grounds: the weights are over assets rather than agents and coincide only because the mapping is one-to-one, and the state-awareness lives in a hand-set threshold with the allocation between triggers never revisited. MACROHFT remains nearest on continuous state conditioning, defeated on homogeneity. JUNG AND LEE is nearest on the heterogeneous pool, technical / on-chain / macro / social / news with a meta-synthesiser, defeated by a fixed prompt template exactly where the weighting should be. TRIAG is nearest on the orchestrator as learned coordinator, with an explicit global/local reward split and a declared confidence field, defeated because its state vector has no environment block and the confidence field is never computed with. AUTOMATE STRATEGY FINDING is demoted from competitor to Baseline 2: the BlackRock survey nominates it as the field's one adaptive gating mechanism tuning signal influence in real time, and the primary paper does not do that, its adaptivity is at selection with weights carrying no time index. Two scoping riders are mandatory: the BlackRock survey has no review protocol so its empty cells evidence its own coverage rather than the field's, and the Agentic Trading snapshot closed 2026-03-09 with 18 of 19 primary studies from 2024 onward, so any statement about what the literature does not report carries that cutoff.</t>
+          <t>The v4 framing was that existing systems weight agents badly. The reviews since have replaced it with a sharper and better-evidenced one: most existing systems have no quantity that could be weighted. TradingAgents runs seven roles through a hierarchy whose facilitator is described in a single sentence; FinVision concatenates four channels into one prompt; Park's anomaly framework summarises three experts into free text. The same absence stated three times across three unrelated designs is a property of the field rather than an artefact of any one architecture. External validation now exists for that reading: the ACM Computing Surveys review of 167 RL papers states that the establishment of coordination and communication protocols among different agents is underexplored. FinAgent still supplies the sharpest motivating failure, its auxiliary strategies returning 16% on ETHUSD against buy-and-hold's 29%, and there are now three such documented fixed-influence failures rather than one: Jung and Lee measure a 10.36-point total-return degradation from a text agent the architecture cannot notice, AlphaAgents deletes its sentiment agent by hand for thin coverage, and the temporal-shift work shows a sentiment channel decaying with nothing watching. PIXIU adds a fourth from the opposite direction, FinMA-7B-trade collapsing from 0.94 to 0.03 F1 on FPB after specialisation while gaining nothing on the task it was specialised for, which is the argument that the four agents must fail independently and that a shared backbone forbids exactly that.
+ADDED IN V6, THE LINEAGE THE CLAIM SITS IN. The reviews behind v5 were agent-system papers almost without exception, which left the gap defended only against designs that have no weight object at all. The forecast combination review, covering over fifty years of work, is the prior art for the weighting function itself, and it changes the framing rather than the conclusion. That literature already contains weights that vary over time, through Kalman-filter and smooth-transition specifications, and weights that are a function of covariates, through FFORMA. What my note records it as not containing, anywhere in that review, is weights that are a function of measured exogenous market state. FFORMA is the nearest named ancestor and the difference is one sentence from the note: its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted. Separately, Gu, Kelly and Xiu give independent evidence that the premise is standard rather than speculative: their Kronecker construction interacts each of 94 characteristics with eight macro state variables inside one estimator, derived from the beta-pricing relation rather than asserted. Their interaction weights are re-estimated once per annual refit and so do not vary at decision time, which is where my construction differs from theirs.</t>
+        </is>
+      </c>
+      <c r="E2" s="41" t="inlineStr">
+        <is>
+          <t>MacroHFT is no longer the single opponent and the defence should be restructured as a five-way contrast, which is the most consequential change in v5. HEDGEAGENTS is now nearest on the orchestration-mechanism axis, the only paper where the orchestration layer is a solved constrained optimisation over an explicit weight vector with return, variance and CVaR terms, plus genuine state-triggered deliberation on a 5% daily / 10% three-day amplitude alarm across 36 emergency sessions in nine months. It is defeated on two grounds: the weights are over assets rather than agents and coincide only because the mapping is one-to-one, and the state-awareness lives in a hand-set threshold with the allocation between triggers never revisited. MACROHFT remains nearest on continuous state conditioning, defeated on homogeneity. JUNG AND LEE is nearest on the heterogeneous pool, technical / on-chain / macro / social / news with a meta-synthesiser, defeated by a fixed prompt template exactly where the weighting should be. TRIAG is nearest on the orchestrator as learned coordinator, with an explicit global/local reward split and a declared confidence field, defeated because its state vector has no environment block and the confidence field is never computed with. AUTOMATE STRATEGY FINDING is demoted from competitor to Baseline 2: the BlackRock survey nominates it as the field's one adaptive gating mechanism tuning signal influence in real time, and the primary paper does not do that, its adaptivity is at selection with weights carrying no time index. Two scoping riders are mandatory: the BlackRock survey has no review protocol so its empty cells evidence its own coverage rather than the field's, and the Agentic Trading snapshot closed 2026-03-09 with 18 of 19 primary studies from 2024 onward, so any statement about what the literature does not report carries that cutoff.
+SIXTH CONTRAST, ADDED IN V6, AND IT IS THE ONE AN EXAMINER FROM OUTSIDE THE AGENT LITERATURE WILL REACH FOR FIRST. FORECAST COMBINATION is nearest on the weighting function itself rather than on any architectural axis. It is defeated as prior art on one axis only, that its weights are functions of time or of properties of the series being forecast, not of measured exogenous market state; the two nearest things in it are Deutsch et al.'s smooth transition specification, whose transition variable could in principle be exogenous, and FFORMA, whose features are computed once from the history. That is a narrower and more honest delta than the agent-literature contrast gives, and the two should be stated together: the agent-system contrast establishes that the field I am building in has no quantity that could be weighted, and the forecast combination contrast establishes what is new about mine against a field that does.</t>
         </is>
       </c>
       <c r="F2" s="13" t="inlineStr">
@@ -8888,12 +8956,13 @@
       </c>
       <c r="J2" s="13" t="inlineStr">
         <is>
-          <t>(a) Equal weights. (b) STATIC LEARNED weight, and this now has a reference implementation to build against rather than being an abstraction, since Automate Strategy Finding is exactly that design. (c) Hard regime router. (d) MacroHFT's conditioning set, trend and realised volatility only, on CSE data. (e) FinMem's three-day return sign test. (f) NEW, a recency-weighted autoregression over past models that ignores market state entirely, a cheap control the conditioning set must beat. (g) NEW, state-conditional agent INCLUSION with static weights, to separate selection-adaptivity from weighting-adaptivity, because if selection recovers most of the benefit the contribution narrows to the weighting function specifically.</t>
+          <t>(a) EQUAL WEIGHTS, PROMOTED IN V6 FROM A LISTED BASELINE TO THE PRE-REGISTERED PRIMARY BENCHMARK. The forecast combination literature is fifty years of evidence that the equally weighted average is hard to beat and that estimated weights lose to estimation error, and the review reports that pattern independently for point and for probabilistic forecasting. The margin and the significance test that would count as beating it are to be written down before the run. (b) STATIC LEARNED weight, which now has a reference implementation to build against rather than being an abstraction, since Automate Strategy Finding is exactly that design. (c) Hard regime router. (d) MacroHFT's conditioning set, trend and realised volatility only, on CSE data. (e) FinMem's three-day return sign test. (f) A recency-weighted autoregression over past models that ignores market state entirely, a cheap control the conditioning set must beat. (g) State-conditional agent INCLUSION with static weights, to separate selection-adaptivity from weighting-adaptivity, because if selection recovers most of the benefit the contribution narrows to the weighting function specifically. (h) NEW IN V6, FFORMA's structure, a meta-model mapping features to a weight simplex, as the named implementation comparator; if I use something simpler I should say why rather than let it look like I did not know the construct existed.</t>
         </is>
       </c>
       <c r="K2" s="13" t="inlineStr">
         <is>
-          <t>Three weighting schemes, then each state input ablated alone. The Graph-RAG paper supplies the discipline requirement that protects this: its fatal flaw is that the proposed system got both the graph and the agent scaffolding while the baseline got neither, so Baseline 2 has to be identical to the proposed system in every respect except the weighting function, and the ablations move one input at a time. Pre-registered diagnostics: weight-distribution ENTROPY over time, plus a cross-play check. A_F on/off inside the full framework is now required rather than optional, on the precedent that a text channel bolted onto a working structured pipeline cost 10.36 points with nothing able to notice. Report behavioural-fidelity metrics beside returns, equalise trade counts before comparing, report exposure time, holding period and turnover, and commit to dispersion and a paired significance test before seeing numbers.</t>
+          <t>Three weighting schemes, then each state input ablated alone. The Graph-RAG paper supplies the discipline requirement that protects this: its fatal flaw is that the proposed system got both the graph and the agent scaffolding while the baseline got neither, so Baseline 2 has to be identical to the proposed system in every respect except the weighting function, and the ablations move one input at a time. Pre-registered diagnostics: weight-distribution ENTROPY over time, plus a cross-play check. A_F on/off inside the full framework is now required rather than optional, on the precedent that a text channel bolted onto a working structured pipeline cost 10.36 points with nothing able to notice. Report behavioural-fidelity metrics beside returns, equalise trade counts before comparing, report exposure time, holding period and turnover, and commit to dispersion and a paired significance test before seeing numbers.
+PRE-REGISTRATION, ADDED IN V6. Before the first run, record the margin over equal weights and the paired significance test that would count as the state-conditioned weighting having earned its place, together with the direction the forecast combination literature predicts. Both outcomes are reportable: the review states that comprehensive quantitative guidance on when estimated weights beat fixed ones does not yet exist in that literature, so a pre-registered answer on a thin frontier market is a contribution even if the answer is that equal weights win. Record also the absence of a pairwise interaction term as a deliberate choice rather than an oversight, since with four agents an interaction form is ten parameters against four on roughly 374 days, and the combination literature tried that first and moved away from it.</t>
         </is>
       </c>
       <c r="L2" s="13" t="inlineStr">
@@ -8903,91 +8972,94 @@
       </c>
       <c r="M2" s="13" t="inlineStr">
         <is>
-          <t>The entropy collapse risk stands and the pre-registered diagnostic stands with it. A second risk is now better defined: with A_F usable less than half the time, the orchestrator may learn to zero it permanently rather than conditionally, in which case the heterogeneity claim survives on paper while the system behaves as a three-agent one, and the weight trajectory around reporting dates is the natural test of whether the mechanism is conditional or merely selective. Third, the regularisation sign-flip observed on a larger dataset than the CSE offers means the orchestrator's own stability has to be swept and reported rather than tuned once. Fourth, the Agentic Trading cutoff means this gap statement has a shelf life and should be re-checked before submission.</t>
-        </is>
-      </c>
-      <c r="N2" s="13" t="inlineStr">
-        <is>
-          <t>RETAIN AS MAIN GAP - defend against the five-way contrast, not MacroHFT alone  |  Revised novelty 4 / 5</t>
+          <t>The entropy collapse risk stands and the pre-registered diagnostic stands with it. A second risk is now better defined: with A_F usable less than half the time, the orchestrator may learn to zero it permanently rather than conditionally, in which case the heterogeneity claim survives on paper while the system behaves as a three-agent one, and the weight trajectory around reporting dates is the natural test of whether the mechanism is conditional or merely selective. Third, the regularisation sign-flip observed on a larger dataset than the CSE offers means the orchestrator's own stability has to be swept and reported rather than tuned once. Fourth, the Agentic Trading cutoff means this gap statement has a shelf life and should be re-checked before submission.
+FIFTH, AND ADDED IN V6, THE FORECAST COMBINATION PUZZLE IS THE FIELD'S STANDING PRIOR AGAINST THIS DESIGN AND IT BELONGS IN THE WRITE-UP BEFORE THE RESULTS RATHER THAN AFTER THEM. Elliott bounds the available gain from optimal over equal weights as usually too small to pay for the estimation; Claeskens et al. show estimated weights can introduce bias into a combination of unbiased components and inflate variance past the fixed-weight case; and the probabilistic side reproduces the pattern independently. Everything that literature says about estimation error swamping the gains is worse in my setting, not better, because my components are themselves estimated on short, illiquid and intermittently traded series. The review's own two practical guidelines cut in opposite directions here: with limited historical data it recommends the simple average or weights that ignore covariances, which my roughly 374 trading days per counter argues for, while it also holds that structural change affects sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state. Which effect dominates on CSE data is the empirical question, and a failure to beat equal weights is the expected outcome under the field's prior rather than a surprise.</t>
+        </is>
+      </c>
+      <c r="N2" s="42" t="inlineStr">
+        <is>
+          <t>RETAIN AS MAIN GAP - defend against the five-way contrast, not MacroHFT alone  |  Revised novelty 4 / 5
+V6: defend on two fronts rather than one. The agent-system contrast for the absence of a weight object, and the forecast combination contrast for what is new about mine against a field that has one. Pre-register against equal weights. The novelty rating is unchanged at 4 / 5: the conditioning axis is still uncovered in both literatures, so the construct remains novel, and what the forecast combination evidence bounds is the expected SIZE of the gain, which is carried in Risk &amp; Failure Mode rather than in the rating.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="409.6" customHeight="1">
-      <c r="A3" s="25" t="inlineStr">
+    <row r="3" ht="451" customHeight="1">
+      <c r="A3" s="43" t="inlineStr">
         <is>
           <t>Sub-gap 1
 (Former G1)</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="41" t="inlineStr">
         <is>
           <t>NARROWED IN V5. No reviewed work calibrates a nonlinear, depth-conditioned execution-cost function to a thin frontier order book, nor sweeps participation rate to establish the shape of that cost curve where a single order is a material fraction of resting depth; and no portfolio-allocation system embeds such a cost function inside its allocation objective rather than deducting a flat rate after the fact. This is a calibration-and-integration gap, not a modelling-form gap, and the change is deliberate.</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
+      <c r="C3" s="41" t="inlineStr">
         <is>
           <t>Method-Integration + Domain</t>
         </is>
       </c>
-      <c r="D3" s="26" t="inlineStr">
-        <is>
-          <t>THE GENERIC CLAIM IS DEAD AND MUST NOT BE WRITTEN AGAIN. Two papers implement size-dependent execution cost directly. Chen et al. (ICAIF '22) build a queue-reactive LOB simulator where impact is fully endogenous, an order consumes queue, brings a level toward depletion and raises the probability of an adverse mid-price move, and they quantify the cost of ignoring it at 3.04 bps on seven liquid US names. Wang, Gao and Li (Finance and Stochastics 2026) implement Almgren-Chriss explicitly with linear permanent and temporary impact, solve it in closed form, and evaluate inside a LOBSTER historical-order-flow simulator with permanent book contamination. The allocation literature still leaves the assumption intact, Moallemi and Wang assume the order infinitesimal, Guo et al. use one scalar for all assets and sizes, HLOB has no cost model, and the RL survey confirms fixed costs and assumed execution certainty as the field convention with the one modelled form proportional to position change rather than to order size against depth. But that silence is now evidence of a division of labour between the execution and allocation literatures, not of an absence in the field.</t>
-        </is>
-      </c>
-      <c r="E3" s="26" t="inlineStr">
-        <is>
-          <t>Wang, Gao and Li IS the 2026 Almgren-Chriss market-impact work the supervisor cited and v4 carried as unverified, so open item 2 is closed and the supervisor's prediction was correct. Chen et al. is the queue-reactive equivalent. Four things survive them, and the notes state all four independently. (1) NONLINEARITY: every impact model in the set is linear or mechanistic-but-unswept, neither tests a square-root or concave form, and Potters-Bouchaud logarithmic impact appears once in the whole corpus as a future-work line. (2) NO ORDER-SIZE SWEEP ANYWHERE, and both execution notes say it in nearly the same words, Chen et al. running everything at one inventory and horizon and Wang et al. everything at 10% of ADTV, so the shape of the cost curve in order size is empirically untested across the entire set. (3) THIN-MARKET CALIBRATION: not one of the five calibrates to a market where a single order is a visible fraction of resting depth; universes are NASDAQ, IEX and LOBSTER large caps trading 2 to 115 million shares a day. (4) THE PASSIVE SIDE: all three execution papers are market-orders-only, no spread capture, no queue position, no partial fills, no cancellation, no fees. Guo et al. turns from foil into asset here, its transaction remainder factor with constant bounds is the container that lets a cost term stay inside a convex objective rather than sitting outside as a post-hoc deduction, and substituting a state-dependent cost into it is the constructive move.</t>
-        </is>
-      </c>
-      <c r="F3" s="26" t="inlineStr">
+      <c r="D3" s="41" t="inlineStr">
+        <is>
+          <t>THE GENERIC CLAIM IS DEAD AND MUST NOT BE WRITTEN AGAIN. Two papers implement size-dependent execution cost directly. Chen et al. (ICAIF '22) build a queue-reactive LOB simulator where impact is fully endogenous, an order consumes queue, brings a level toward depletion and raises the probability of an adverse mid-price move, and they quantify the cost of ignoring it at 3.04 bps on seven liquid US names. Wang, Gao and Li (Finance and Stochastics 2026) implement Almgren-Chriss explicitly with linear permanent and temporary impact, solve it in closed form, and evaluate inside a LOBSTER historical-order-flow simulator with permanent book contamination. The allocation literature still leaves the assumption intact, Moallemi and Wang assume the order infinitesimal, Guo et al. use one scalar for all assets and sizes, HLOB has no cost model, and the RL survey confirms fixed costs and assumed execution certainty as the field convention with the one modelled form proportional to position change rather than to order size against depth. But that silence is now evidence of a division of labour between the execution and allocation literatures, not of an absence in the field.
+ADDED IN V6. Gu, Kelly and Xiu are the cleanest reference case in the reviewed set for why this sub-gap exists, and my note records them as exactly that. Their best strategy is an equal-weighted decile spread on NN4 forecasts returning 3.3% per month, 39.0% annualised, at an out-of-sample Sharpe of 2.35 with monthly turnover of 114.08%, on a universe that retains sub-$5 stocks by explicit choice, and there are no transaction costs anywhere in the paper. Their own results bound what is being left out: value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, which is a partial and unacknowledged cost estimate and should be cited as one rather than as a weighting result. Liquidity appears there as a predictor family, one of the three dominant ones, and is absent as a friction, which is the division of labour this sub-gap sits inside.</t>
+        </is>
+      </c>
+      <c r="E3" s="41" t="inlineStr">
+        <is>
+          <t>Wang, Gao and Li IS the 2026 Almgren-Chriss market-impact work the supervisor cited and v4 carried as unverified, so open item 2 is closed and the supervisor's prediction was correct. Chen et al. is the queue-reactive equivalent. Four things survive them, and the notes state all four independently. (1) NONLINEARITY: every impact model in the set is linear or mechanistic-but-unswept, neither tests a square-root or concave form, and Potters-Bouchaud logarithmic impact appears once in the whole corpus as a future-work line. (2) NO ORDER-SIZE SWEEP IN THE REVIEWED SET, and both execution notes say it in nearly the same words, Chen et al. running everything at one inventory and horizon and Wang et al. everything at 10% of ADTV, so the shape of the cost curve in order size is empirically untested across the entire set. (3) THIN-MARKET CALIBRATION: not one of the five calibrates to a market where a single order is a visible fraction of resting depth; universes are NASDAQ, IEX and LOBSTER large caps trading 2 to 115 million shares a day. (4) THE PASSIVE SIDE: all three execution papers are market-orders-only, no spread capture, no queue position, no partial fills, no cancellation, no fees. Guo et al. turns from foil into asset here, its transaction remainder factor with constant bounds is the container that lets a cost term stay inside a convex objective rather than sitting outside as a post-hoc deduction, and substituting a state-dependent cost into it is the constructive move.</t>
+        </is>
+      </c>
+      <c r="F3" s="41" t="inlineStr">
         <is>
           <t>Unexpected illiquidity shocks depress contemporaneous CSE returns at -0.084 to -0.097, small caps more than large. The amplification argument is now explicit and is the load-bearing sentence: if ignoring impact costs about 3 bps on names trading two to a hundred and fifteen million shares a day, then on a counter where a single order is a visible fraction of resting depth the same neglect is not a small correction to a backtest, it is capable of reversing the sign of a reported edge. That is an argument by amplification rather than a calibrated result, and it should be stated as such.</t>
         </is>
       </c>
-      <c r="G3" s="26" t="inlineStr">
+      <c r="G3" s="41" t="inlineStr">
         <is>
           <t>Technical: a nonlinear, depth-conditioned cost function calibrated to a thin frontier book and embedded inside the allocation objective rather than deducted afterwards. Domain: a participation-rate sweep establishing the shape of the cost curve on a market where order size is material relative to depth, which is the cleanest remaining claim in the set and which no reviewed paper provides for any market.</t>
         </is>
       </c>
-      <c r="H3" s="26" t="inlineStr">
+      <c r="H3" s="41" t="inlineStr">
         <is>
           <t>Substitute a state-dependent cost into Guo et al.'s transaction remainder factor so it stays inside the convex objective. Sweep participation rate rather than fixing it. Prefer a LEARNED friction component over naive calibrate-then-plug-in, on Wang et al.'s own evidence that estimation error in the impact parameters is amplified through the closed-form control, their statistical calibration turning in -905.742 on AAPL at high risk aversion against the learned variant's +102.285, and on CSE data the estimation error would be strictly worse. Run the tick-size classification on CSE counters first, since it needs only best bid, best ask and the tick schedule, and if liquid CSE counters come out small-tick the microstructural route is ruled out at near-zero cost and the friction work is daily-bar-based by necessity rather than preference.</t>
         </is>
       </c>
-      <c r="I3" s="26" t="inlineStr">
+      <c r="I3" s="41" t="inlineStr">
         <is>
           <t>Per-counter CSE daily price and turnover for the volume profile and the Amihud measure. The data ladder is now explicit: level-III message data for the full queue-reactive route and almost certainly out of reach; multi-level depth snapshots for a weaker version; top-of-book only for the tick classification, which is decisive and nearly free and runs first; intraday trade-and-quote without depth for the five-scalar policy route, which is fittable on a short archive where a learned agent is not; and daily bars only for the fallback, turnover, traded value, zero-return frequency and Amihud-style measures.
 AMENDED 11 OCTOBER 2026: the bottom rung of that ladder is where this now sits, and it has no spread measurement on it. The EDGE route that would have put a measured effective spread on the daily-bars rung is demoted to last resort and is not assumed available. This changes what the CSE request is for: bid/ask and depth are no longer a validation extra for an estimator already built, they are the only route to a measured spread, which moves them to the top of the request rather than the middle.</t>
         </is>
       </c>
-      <c r="J3" s="26" t="inlineStr">
+      <c r="J3" s="41" t="inlineStr">
         <is>
           <t>(a) Zero-cost execution. (b) Flat 2 bps. (c) FreQuant's solved fee fixed point with no impact term. (d) Naive full-size execution at close. (e) NEW, Almgren-Chriss at a fixed participation rate, which is now the strongest published treatment and therefore the baseline that actually matters. (f) NEW, the 19-strategy training-free OLPS family plus First All / Last All / TWAP / VWAP.</t>
         </is>
       </c>
-      <c r="K3" s="26" t="inlineStr">
+      <c r="K3" s="41" t="inlineStr">
         <is>
           <t>The framework under all cost regimes, plus the participation-rate sweep that is missing from the whole literature. TWO EXPERIMENTS ARE INDEPENDENT OF THE CSE DATA BLOCKER and both should run while the data request is outstanding: sweeping the cost parameter from 5 bps to north of 100 bps on Guo et al.'s own four datasets, which establishes where the crossover against simpler baselines sits and is directly the argument for why a frontier market needs different machinery; and the tick-size classification on CSE counters from top-of-book alone. Report the half-spread unit, average transaction cost in bps against the decision price, risk-adjusted PnL relative to TWAP, and round-trip practicability against action count, since the first two are pure cost measures indifferent between a reliable schedule and a volatile one.</t>
         </is>
       </c>
-      <c r="L3" s="26" t="inlineStr">
+      <c r="L3" s="41" t="inlineStr">
         <is>
           <t>High for the daily-turnover version and for both blocker-independent experiments. Low for anything needing level-III messages or queue intensities, which the notes judge almost certainly out of reach. The evaluation layer and A_L are gated on exactly the same data, so whatever cannot be observed cannot be simulated either, and they should be treated as one workstream and one data request rather than two.</t>
         </is>
       </c>
-      <c r="M3" s="26" t="inlineStr">
+      <c r="M3" s="41" t="inlineStr">
         <is>
           <t>The novelty has genuinely narrowed and the rating moves with it rather than being defended at its old level. There is still no ground-truth execution data to validate a CSE simulator against, so simulated slippage is not measured slippage and must be presented that way. The tick-size classification may return small-tick, which would close the microstructural route entirely. And a reviewer who knows the execution literature will ask why the impact model is not simply Almgren-Chriss with CSE parameters, so the nonlinearity and the in-objective embedding have to be the argued contribution rather than the calibration alone.
 ADDED 11 OCTOBER 2026 - SUB-GAP 1 NOW CARRIES TWO CAVEATS AND THEY MUST BE STATED TOGETHER. (1) Smart Trading Rule (Journal of Financial Data Science 8(2), 2026) was identified, judged potentially overlapping on the modular transaction-cost layer, and could not be obtained because it is paywalled. Its contents are unknown to me, so this sub-gap is not presented as though the literature had been fully swept. (2) THE MEASUREMENT HALF IS OPEN AGAIN. P54, the EDGE estimator of effective spread from daily OHLC, was the route that would have substituted for the CSE's missing quote data, and on 11 October it was demoted to last resort because it is unvalidated on thin and frontier markets - no emerging or frontier market appears anywhere in that paper, its crypto section has no quote benchmark at all, and its own numbers put it at its weakest exactly where the CSE sits. With no CSE quote data to validate against, an EDGE spread here could not be falsified even in principle. So the cost term rests on proxies for illiquidity - Amihud, turnover, zero-return frequency and the high-low range - rather than on any measurement of what a trade actually pays. That is a weaker evidential base than v5 recorded and the write-up should say so rather than leave it to be found. The defensible form is that the cost function is calibrated on proxies because no validated spread measurement exists for this market, and that validating it is what the CSE data request is for.</t>
         </is>
       </c>
-      <c r="N3" s="26" t="inlineStr">
+      <c r="N3" s="41" t="inlineStr">
         <is>
           <t>RETAIN, NARROWED - generic claim withdrawn, calibration and in-objective embedding retained  |  Revised novelty 3 / 5  |  11 Oct 2026: unchanged in substance, but state it with BOTH caveats - the unobtainable Smart Trading Rule and the demoted EDGE proxy route.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.6" customHeight="1">
+    <row r="4" ht="220" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Sub-gap 2
@@ -8996,7 +9068,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>NARROWED AND SHARPENED IN V5. The level of volatility is routinely operationalised as an exposure scaler; the persistence of volatility is estimated descriptively and never used to set the schedule on which that exposure is restored after a shock. Stated against a specific named component rather than against the literature in general: the standard target-volatility scaler that multiplies each position by a volatility ratio built from an EWMA estimate.</t>
+          <t>NARROWED AND SHARPENED IN V5. The level of volatility is routinely operationalised as an exposure scaler; the persistence of volatility is estimated descriptively, and in the literature I have covered I have not found it used to set the schedule on which that exposure is restored after a shock. Stated against a specific named component rather than against the literature in general: the standard target-volatility scaler that multiplies each position by a volatility ratio built from an EWMA estimate.</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
@@ -9006,10 +9078,10 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>THE BROAD CLAIM IS NO LONGER SAFE. Deep Learning for Portfolio Optimization operationalises a volatility estimate into an allocation every single day through a target-volatility scaler, and the note shows empirically that this non-learned scaler rather than the learned policy does most of the risk work, lifting Sharpe from 0.929 to 1.526 on one allocation and 0.759 to 1.120 on mean-variance, with the COVID de-risking traceable to a spike in the volatility estimate rather than to any weight change. So nobody feeds a volatility estimate into an allocation is false and is withdrawn. Across all the volatility papers exactly one operationalises a level and none operationalises a decay rate. On the agent side the picture is unchanged: FinCon's backward-looking empirical CVaR, FinHEAR's sampled Beta, FinMem's three-day sign test, FinAgent reporting six risk metrics and feeding back none, AlphaAgents' prompt adjective.</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
+          <t>THE BROAD CLAIM IS NO LONGER SAFE. Deep Learning for Portfolio Optimization operationalises a volatility estimate into an allocation every single day through a target-volatility scaler, and the note shows empirically that this non-learned scaler rather than the learned policy does most of the risk work, lifting Sharpe from 0.929 to 1.526 on one allocation and 0.759 to 1.120 on mean-variance, with the COVID de-risking traceable to a spike in the volatility estimate rather than to any weight change. So the claim that a volatility estimate is never fed into an allocation is false and is withdrawn. Across all the volatility papers exactly one operationalises a level and none operationalises a decay rate. On the agent side the picture is unchanged: FinCon's backward-looking empirical CVaR, FinHEAR's sampled Beta, FinMem's three-day sign test, FinAgent reporting six risk metrics and feeding back none, AlphaAgents' prompt adjective.</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
         <is>
           <t>The nearest prior work is now that scaler, and the delta is a named mechanism rather than an absence. An EWMA estimator assumes shocks decay exponentially, which is precisely the assumption the CSE long-memory result contradicts, so after a shock the scaler re-levers on a schedule that is too fast and exposure returns while the shock is still decaying hyperbolically. The original authors concede the opening themselves, their conclusion notes the volatility estimates are lagged and do not necessarily represent current market volatilities and proposes inferring forward volatility inside the network as future work, so the contribution answers a stated future-work item rather than inventing a grievance. The state of the art in volatility forecasting confirms the persistence axis is untouched even there: in GNNHAR long memory appears only as a justification for the HAR lag structure, the cheapest way to reproduce long-memory decay without fitting a fractionally integrated model, absorbed into functional form and never estimated, never reported, never fed anywhere, and the paper ends at a loss ratio with no portfolio, no value-at-risk backtest and no cost-bearing application.</t>
         </is>
@@ -9054,13 +9126,14 @@
           <t>The honest check still cuts against the CSE-specific framing: return persistence is statistically indistinguishable between cryptocurrency and equity markets, so the case for CSE-specific modelling rests on liquidity and microstructure, and with sentiment out of scope that case is one leg thinner than in v3. Against that, P_t is now locally evidenced rather than imported: three CSE papers detect volatility clustering and discard it, residual bands widening by a factor of several across 2020 to 2022 under a constant-variance fit, ARCH statistics of 86.55 on the ASPI addressed only with robust standard errors, and a decade of daily data fitted with no variance modelling at all. That is the argument for P_t and it should be quoted directly. Technical risk unchanged: if the persistence-conditioned layer cannot beat a three-day sign test, the econometric layer is not earning its place and the ablation should say so.</t>
         </is>
       </c>
-      <c r="N4" s="13" t="inlineStr">
+      <c r="N4" s="42" t="inlineStr">
         <is>
           <t>RETAIN, SHARPENED - now targets a named component and runs before the CSE data arrives  |  Revised novelty 3.5 / 5</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -9074,52 +9147,53 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="76" customWidth="1" min="3" max="3"/>
+    <col width="66" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="6"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="92.40000000000001" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="40" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Status after 53 reviews</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="B1" s="40" t="inlineStr">
+        <is>
+          <t>Status after 59 reviews</t>
+        </is>
+      </c>
+      <c r="C1" s="40" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="40" t="inlineStr">
         <is>
           <t>How it is computed</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="40" t="inlineStr">
         <is>
           <t>What it does in the framework</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="40" t="inlineStr">
         <is>
           <t>Open question</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="409.6" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
           <t>L_t  liquidity state</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="44" t="inlineStr">
         <is>
           <t>KEEP - strongest positive result across the set, and the justification is now three-fold rather than one</t>
         </is>
@@ -9141,49 +9215,51 @@
       </c>
       <c r="F2" s="13" t="inlineStr">
         <is>
-          <t>Whether the monthly Granger result survives re-estimation at daily frequency with turnover and a spread proxy alongside. If it does not, the discrepancy is itself worth reporting.</t>
+          <t>Whether the monthly Granger result survives re-estimation at daily frequency with turnover and a spread proxy alongside. If it does not, the discrepancy is itself worth reporting.
+ADDED IN V6: see the V_t row. The risk-turnover correlation means L_t and V_t may not be independent inputs on this market, and the ablation has to be able to tell them apart.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="409.6" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="3" ht="159" customHeight="1">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>V_t  volatility level</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="44" t="inlineStr">
         <is>
           <t>KEEP, but specify the estimator and pin the window</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="46" t="inlineStr">
         <is>
           <t>Volatility level is the one quantity in the set that is already routinely operationalised, through the target-volatility scaler, and the scaler carries most of the risk work in the paper that uses it. So V_t is not in question; what it is computed from is.</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="46" t="inlineStr">
         <is>
           <t>Five-minute intraday realised volatility is confirmed unavailable on the CSE, so a daily range-based estimator, Parkinson or Garman-Klass. The calm/turbulent stratification from GNNHAR is a better regime template than volatility tertiles, with the caveat that its labelling is ex post at a full-sample quantile while a live indicator needs rolling estimates.</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>Sets the exposure level, conditions agent weights, and shares the deliberation trigger with L_t.</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>The minimum rolling window that yields a usable turbulence indicator on roughly 240 days. This is flagged twice in the notes and resolves in one experiment alongside the volatility-estimator window question.</t>
+      <c r="F3" s="46" t="inlineStr">
+        <is>
+          <t>The minimum rolling window that yields a usable turbulence indicator on roughly 240 days. This is flagged twice in the notes and resolves in one experiment alongside the volatility-estimator window question.
+ADDED IN V6: the CSE firm-level study reports a correlation between its risk estimate and turnover and does not treat it. If V_t and L_t move together on my sample then the volatility and liquidity agents are partly measuring the same thing and the conditioning set has a collinearity problem, which has to be checked on my own data before weights are allowed to swing much on either term.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.6" customHeight="1">
+    <row r="4" ht="146" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>P_t  volatility persistence</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>KEEP - was the weakest-supported term in v4 and is now locally evidenced</t>
         </is>
@@ -9209,53 +9285,58 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="409.6" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="5" ht="281" customHeight="1">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>C_i,t  agent confidence</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>KEEP, but REDEFINED - this is the largest single change in v5</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Four independent notes converge on the same pattern and one states it explicitly: confidence should be a STRUCTURAL PROPERTY OF THE OUTPUT rather than a self-reported score. The negative evidence is now strong enough to be an argument for the gap rather than a hole in it. TRIAG declares a confidence field in its protocol, puts it in a figure, and never computes with it, appearing in no reward term, no fusion rule, no state block and no experiment. HedgeAgents feeds three LLM-authored expected returns straight into an exact mean-variance-CVaR optimiser with no calibration and no realised-versus-predicted record, which is a well-specified objective over uncalibrated inputs inheriting the uncertainty of the inputs while hiding it behind the precision of the output.</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Per agent, from the output's own structure. A_F: whether generated queries validated, how many retries a sub-query needed, whether every claim traced to a retrieved chunk, and program step count as a calibrated difficulty proxy at 67.61 / 59.08 / 22.78 per cent for one, two and three-plus steps. A_V: a rolling loss ratio against a fixed benchmark, unit-free and computable for any component emitting a forecast of the same target. A_T: Theil's U2 against the random walk, which is also what decides whether the channel gets any weight at all that day; explicitly NOT a raw softmax, since a network whose edge is arbitraged away has no reason to become less confident. Across all four: the gap between fitted-period and next-period accuracy, computable without knowing how a component works, used jointly with the level rather than alone, since a gap metric on its own ranks a uniformly weak agent above a strong but drifting one.</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>KEEP, but REDEFINED - this is the largest single change in v5
+V6: five notes rather than four, and the A_V mechanism is now supplied rather than left open.</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>Four independent notes converge on the same pattern and one states it explicitly: confidence should be a STRUCTURAL PROPERTY OF THE OUTPUT rather than a self-reported score. The negative evidence is now strong enough to be an argument for the gap rather than a hole in it. TRIAG declares a confidence field in its protocol, puts it in a figure, and never computes with it, appearing in no reward term, no fusion rule, no state block and no experiment. HedgeAgents feeds three LLM-authored expected returns straight into an exact mean-variance-CVaR optimiser with no calibration and no realised-versus-predicted record, which is a well-specified objective over uncalibrated inputs inheriting the uncertainty of the inputs while hiding it behind the precision of the output.
+ADDED IN V6. Adaptive conformal inference closes the hole this row previously recorded. The v5 redefinition gave a worked mechanism only for A_F, whether the extracted program parses and whether every argument traces to a retrieved figure, and left A_T, A_V and A_L open. My note on the conformal work states the analogue for A_V directly: the calibrated interval width is the structural confidence term the scope revision asked for, and it arrives measured rather than self-reported. Separately, the CSE firm-level investment study supplies a locally measured reason to cap A_F rather than let it drive entry and exit: a within-firm coefficient of 0.090 against 0.709 between firms says the fundamental channel prices counters against each other well and says little about when a given counter moves.</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>Per agent, from the output's own structure. A_F: whether generated queries validated, how many retries a sub-query needed, whether every claim traced to a retrieved chunk, and program step count as a calibrated difficulty proxy at 67.61 / 59.08 / 22.78 per cent for one, two and three-plus steps. A_V: a rolling loss ratio against a fixed benchmark, unit-free and computable for any component emitting a forecast of the same target. A_T: Theil's U2 against the random walk, which is also what decides whether the channel gets any weight at all that day; explicitly NOT a raw softmax, since a network whose edge is arbitraged away has no reason to become less confident. Across all four: the gap between fitted-period and next-period accuracy, computable without knowing how a component works, used jointly with the level rather than alone, since a gap metric on its own ranks a uniformly weak agent above a strong but drifting one.
+A_V, ADDED IN V6: wrap the FIGARCH or GJR-GARCH forecast in adaptive conformal inference with the normalised score S_t = |V_t - sigma_hat^2| / sigma_hat^2, and let C_V,t be a function of the realised interval width at the target coverage, so an agent whose model has drifted reports wider intervals and is down-weighted without anyone intervening.</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>Enters the weighting function, and is calibrated per agent against realised hit rate on a held-out period so the orchestrator combines calibrated quantities rather than self-reports. Unparseable output is a fourth outcome state feeding a hard zero rather than a low value.</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>Whether these several backward-looking competence estimates can be made comparable across four architectures, or whether having several is progress on the problem rather than a solution to it. The notes say the latter, and writing it down as unresolved is more useful than picking one.</t>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>Whether these several backward-looking competence estimates can be made comparable across four architectures, or whether having several is progress on the problem rather than a solution to it. The notes say the latter, and writing it down as unresolved is more useful than picking one.
+V6: the conformal route is an off-the-shelf wrapper, so the contribution is the use rather than the method, and the note is explicit that this should be said early. Still open for A_T and A_L.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="409.6" customHeight="1">
+    <row r="6" ht="207" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>ABSTENTION channel
 (NEW, proposed)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>ADD - the one structural change to f() the reviews argue for</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>A_F is expected to be wrong or to abstain on more than half of computed questions over CSE filings, on two independent pipelines measuring 50% and 53.19%. A channel that is frequently unusable rather than occasionally imperfect needs an explicit zero, not a small number.</t>
+          <t>A_F is expected to be wrong or to abstain on more than half of computed questions over CSE filings, on two independent pipelines measuring 50% and 53.19%. A channel that is frequently unusable rather than occasionally imperfect needs an explicit zero, not a small number.
+ADDED IN V6, TWO STRENGTHENINGS. First, adaptive conformal inference converts abstention from a hand-set threshold into a quantity that moves on its own: when the interval at the target coverage spans the plausible range of next-day volatility the agent has nothing to say, and the orchestrator should read that as absence rather than as a weak signal. My note frames it as the mechanism AlphaAgents lacked when a human deleted an agent by hand, expressed as a quantity that moves on its own. Second, the CSE firm-level study forces an abstention design on A_T as well as A_F, since it uses weekly returns on the ground that most CSE stocks are not traded daily. Third, the forecast combination review names the same construct from the other side as time-varying subset selection, so abstention is not an invention either but a named option in that literature.</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
@@ -9274,47 +9355,47 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="409.6" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="45" t="inlineStr">
         <is>
           <t>Pairwise conflict score
 (CANDIDATE, pre-registered)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="43" t="inlineStr">
         <is>
           <t>TEST, do not adopt yet</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="46" t="inlineStr">
         <is>
           <t>The strongest candidate mechanism found for comparing heterogeneous producers: score the RELATIONSHIP between two agents' outputs externally on a fixed rubric rather than asking either agent to self-report, which sidesteps internal calibration and generalises to any pair that can emit text. Observed distributions in the source are conflict mean 0.42 median 0.30 with a cluster near 0.7, and actionability mean 0.55 median 0.60 max 0.90. Take the mechanism, not the validation: the published version is same-model-family self-grading and is never checked against outcomes, which the authors concede.</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="46" t="inlineStr">
         <is>
           <t>One scoring pass over agent pairs on CSE data, then a correlation check against realised next-period error or return before anything touches the orchestrator.</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>If conflict carries signal it is an information-state input no reviewed system uses. If not, the conditioning set falls back to market state alone.</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="46" t="inlineStr">
         <is>
           <t>Pre-registered either way, because both outcomes are reportable and the cost is one scoring pass.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="409.6" customHeight="1">
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Distribution-shift estimate
 (CANDIDATE, expected to fail)</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>TEST and expect to reject</t>
         </is>
@@ -9340,40 +9421,41 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="409.6" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="122" customHeight="1">
+      <c r="A9" s="45" t="inlineStr">
         <is>
           <t>MACRO block
 (rejected)</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>DO NOT ADD - two independent CSE results point the same way</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="46" t="inlineStr">
         <is>
           <t>The ARDL study puts five macro variables across a decade of CSE data and reaches R-squared 0.300153 falling to adjusted 0.189286 on 117 observations. The Granger study runs the horse race and macro loses outright, volume at p = 0.0041 against money supply and inflation reaching nothing. Two independent CSE results on how little a macro block buys.</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="46" t="inlineStr">
         <is>
           <t>N/A.</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="46" t="inlineStr">
         <is>
           <t>N/A. The defensible position is not that macro is useless on the CSE but that it operates at a frequency and horizon the orchestrator does not decide at, which is a scoping argument rather than a dismissal.</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="46" t="inlineStr">
         <is>
           <t>One honesty caveat: the Granger nulls may be underpowered rather than true, since lag one forecloses the lag structure other CSE evidence points at. And USD/LKR leads the index at a two-month lag, 0.583956 at p = 0.0015, so if any macro variable is carried it is that one as a slow lagged feature into A_F's context, not as a fifth agent. Complicated further by a reverse-causality finding, which is itself a small argument for the main gap since a regime-dependent sign is what a static feature set handles badly.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9387,66 +9469,71 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="30.21875" customWidth="1" min="4" max="5"/>
-    <col width="13" customWidth="1" min="6" max="10"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="5"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="76" customWidth="1" min="6" max="10"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="92.40000000000001" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="40" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="40" t="inlineStr">
         <is>
           <t>Original ID</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="40" t="inlineStr">
         <is>
           <t>Reclassified Role</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="40" t="inlineStr">
         <is>
           <t>Reframed Research Statement</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="40" t="inlineStr">
         <is>
           <t>Literature Grounding &amp; Baselines</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="40" t="inlineStr">
         <is>
           <t>Nearest Prior Work &amp; Delta</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="40" t="inlineStr">
         <is>
           <t>Required Data</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="40" t="inlineStr">
         <is>
           <t>Experiment &amp; Ablation</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="40" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="40" t="inlineStr">
         <is>
           <t>Decision &amp; Integration Plan</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="409.6" customHeight="1">
+    <row r="2" ht="171" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Input Agent Pipeline</t>
@@ -9472,7 +9559,7 @@
           <t>FinanceBench establishes the failure rate and the question taxonomy, element-based chunking establishes the structural approach, MultiFinRAG establishes modality-aware indexing, and the retrieval-quality and prompt-sensitivity bounds are established elsewhere. FinQA, TAT-QA and ConvFinQA collectively specify the numeric reasoning task. The planning band agreed across three independent papers is below 50% on computed quantities over CSE filings, nearer 40% than 60% on first build.</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="F2" s="41" t="inlineStr">
         <is>
           <t>CLOSED AND NOW VERIFIED. Shamila, Silva and Talagala, ERU Symposium 2025, DOI 10.31705/ERU.2025.35, University of Moratuwa, with a public GitHub repository. This is the paper v4 carried as an unverified supervisor-supplied citation and it is confirmed. Priority is priority, and the two-page-abstract weakness does not reopen it. THREE THINGS REMAIN FOR A_F and they are the only three defended: (1) NUMERIC STATEMENT EXTRACTION, since their graph captures governance and ownership and puts tabular financial data explicitly out of scope, so the differentiation is numeric rather than architectural; (2) POINT-IN-TIME CORRECTNESS, since their graph is a static snapshot with no as-of field, which is a lookahead hazard rather than an inconvenience in a backtest, and no paper in the set does this; (3) THE ORCHESTRATION THAT CONSUMES THE SIGNAL, since annual-report evidence refreshing once or twice a year beside daily-moving state is the fixed-influence failure mode by construction.</t>
         </is>
@@ -9492,65 +9579,65 @@
           <t>A_F is expected to be unusable more often than not, which is now a design constraint rather than a caveat. Citation tracing is also the only attribution path over text, so if the retrieval layer cites a chunk that did not drive the decision the explanation is wrong in the one place a reader will check it, and faithfulness has to be tested by perturbation rather than asserted.</t>
         </is>
       </c>
-      <c r="J2" s="13" t="inlineStr">
+      <c r="J2" s="42" t="inlineStr">
         <is>
           <t>SYSTEM COMPONENT BUILT ON PUBLISHED TASK DEFINITIONS, and the review chapter should say so. Adopt the Graph-RAG pipeline constants as defaults but not as validated settings. Prototype A_F first, because annual reports are not gated by the OHLCV depth blocker. Benchmarks are development artefacts only: FinQA is most usable and permissively licensed, ConvFinQA pairs with it as a probe corpus, TAT-QA supplies the scale taxonomy and is non-commercial use only. None is usable as a CSE evaluation set.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="409.6" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="3" ht="120" customHeight="1">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>System Requirement</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="45" t="inlineStr">
         <is>
           <t>Former G6</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="46" t="inlineStr">
         <is>
           <t>Architectural Design Requirement</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="46" t="inlineStr">
         <is>
           <t>Component-level attribution across modalities, because a generated rationale is not evidence of what caused the decision. A design requirement, not a novelty claim.</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>AlphaAgents remains the strongest existing instance. FinMem returns the IDs of the highest-influence events with every decision. FinAgent tags retrieved evidence with the intent that found it. The anomaly-detection work now supplies the Correct / Incorrect / Uncertain output contract, which the notes call the only concrete cross-agent output vocabulary found.</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="41" t="inlineStr">
         <is>
           <t>Explainable multi-agent trading is not unexplored and the claim is not reopened. What the orchestration design contributes at no extra cost is that the weight vector IS an explanation: a decision annotated with how much weight the liquidity state put on the retrieval agent that day is attributable without further instrumentation.</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="46" t="inlineStr">
         <is>
           <t>None additional. Instrumentation on components built for the main gap and the sub-gaps.</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="H3" s="46" t="inlineStr">
         <is>
           <t>Faithfulness by perturbation rather than assertion. Report MCC beside F1 with a no-skill reference line for every classification output, since F1 up to 1.00 at MCC exactly 0.00 is a model predicting one class for every row.</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="I3" s="46" t="inlineStr">
         <is>
           <t>Risk of becoming a checkbox. The sharper risk is that retrieval citation tracing is the only attribution path over text after the scope cut.</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J3" s="42" t="inlineStr">
         <is>
           <t>SYSTEM DESIGN FEATURE. Citation tracing, SHAP over risk features, interpretable FIGARCH and GJR-GARCH parameters, and the orchestrator's weight vector as the decision-level record. Build the observability layer from the start, because the back-test will be short and underpowered and component-level metrics are what show the system works when the returns cannot.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.6" customHeight="1">
+    <row r="4" ht="134" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Evaluation Protocol</t>
@@ -9576,14 +9663,14 @@
           <t>The walk-forward and significance machinery comes from the diversified-portfolio framework, which runs 16 folds with HAC-adjusted and bootstrap tests and finds no significant mean-return outperformance anywhere. Against that, most of the agent literature reports single runs on one split. The reproducibility audit and reporting checklist from the Agentic Trading survey now supply an external standard to build the protocol chapter against.</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="41" t="inlineStr">
         <is>
           <t>Not a novelty claim. What does not exist is a CSE baseline set produced under it.</t>
         </is>
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t>The full CSE price and turnover history obtainable. The blocker is reframed rather than removed: a ten-year daily CSE INDEX series is demonstrably obtainable and has been published from the official database with a Bloomberg cross-check, which secures baselines, regime-split reporting and the persistence estimation. The per-counter track is roughly one year and is unprecedented in the published record, so building it is a contribution rather than a shortfall.</t>
+          <t>The full CSE price and turnover history obtainable. The blocker is reframed rather than removed: a ten-year daily CSE INDEX series is demonstrably obtainable and has been published from the official database with a Bloomberg cross-check, which secures baselines, regime-split reporting and the persistence estimation. The per-counter track is roughly one year, and I have not found a published per-counter CSE series of greater depth in the literature I have covered, so building it is a contribution rather than a shortfall.</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
@@ -9596,13 +9683,14 @@
           <t>With a small universe and short history, honest significance testing may return no significant outperformance, and that should be decided now as an acceptable outcome. A short-lookback cross-sectional design also needs a trading-day filter dropping counters with no genuine print before any median is computed, and the count that filter removes on an average day is itself a liquidity statistic worth reporting.</t>
         </is>
       </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="J4" s="42" t="inlineStr">
         <is>
           <t>EXPERIMENTAL METHODOLOGY. The equal-weight baseline still matters most, and Baseline 2 now has a reference implementation to build against rather than being an abstraction.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 21:55:57
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -17,6 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Research Gap Analysis'!$A$1:$N$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Conditioning Set'!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Reclassified Components'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dataset'!$A$1:$W$18</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -86,8 +87,23 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -194,6 +210,30 @@
         <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F5FA"/>
+        <bgColor rgb="FFF2F5FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -252,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -396,6 +436,75 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="25" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9701,2800 +9810,1775 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W24"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="4.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="8.5546875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.88671875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="10.109375" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="11.109375" bestFit="1" customWidth="1" min="14" max="14"/>
-    <col width="11.21875" bestFit="1" customWidth="1" min="15" max="15"/>
-    <col width="19.21875" bestFit="1" customWidth="1" min="16" max="16"/>
-    <col width="8.77734375" bestFit="1" customWidth="1" min="17" max="17"/>
-    <col width="11.88671875" bestFit="1" customWidth="1" min="19" max="19"/>
-    <col width="9.6640625" bestFit="1" customWidth="1" min="20" max="20"/>
-    <col width="8.5546875" bestFit="1" customWidth="1" min="21" max="21"/>
-    <col width="12.5546875" bestFit="1" customWidth="1" min="23" max="23"/>
+    <col width="7" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="18" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="40" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="44" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="40" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="34" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="44" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="54" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="36" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="50" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="50" bestFit="1" customWidth="1" min="20" max="20"/>
+    <col width="9" bestFit="1" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
+    <col width="50" bestFit="1" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1" ht="52.8" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="49" t="inlineStr">
         <is>
           <t>Source Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="49" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="49" t="inlineStr">
         <is>
           <t>Provider</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="49" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="49" t="inlineStr">
         <is>
           <t>Market / Coverage</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="49" t="inlineStr">
         <is>
           <t>Role &amp; Modality</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="49" t="inlineStr">
         <is>
           <t>Time Period</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="49" t="inlineStr">
         <is>
           <t>Granularity</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="49" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="49" t="inlineStr">
         <is>
           <t>Price / Volume Fields</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="49" t="inlineStr">
         <is>
           <t>Text &amp; Language</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="49" t="inlineStr">
         <is>
           <t>Labels / Annotations</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="49" t="inlineStr">
         <is>
           <t>Access Method</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="49" t="inlineStr">
         <is>
           <t>Licence / Legal Restrictions</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="49" t="inlineStr">
         <is>
           <t>Known Gaps &amp; Quality Issues</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="49" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="49" t="inlineStr">
         <is>
           <t>Which Agent It Feeds</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="49" t="inlineStr">
         <is>
           <t>Advantages</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="49" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="49" t="inlineStr">
         <is>
           <t>Suitability (1-5)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" s="49" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" s="49" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="409.6" customHeight="1">
-      <c r="A2" s="19" t="inlineStr">
+    <row r="2" ht="207" customHeight="1">
+      <c r="A2" s="50" t="inlineStr">
         <is>
           <t>D01</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="51" t="inlineStr">
         <is>
           <t>CSE undocumented JSON API</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="51" t="inlineStr">
         <is>
           <t>Price &amp; market data</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="51" t="inlineStr">
         <is>
           <t>Colombo Stock Exchange (unofficial, no published contract)</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="51" t="inlineStr">
         <is>
           <t>https://www.cse.lk/api/ (see github.com/GH0STH4CKER/Colombo-Stock-Exchange-CSE-API-Documentation)</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="51" t="inlineStr">
         <is>
           <t>CSE. All listed instruments, index level and per-ticker.</t>
         </is>
       </c>
-      <c r="G2" s="20" t="inlineStr">
+      <c r="G2" s="51" t="inlineStr">
         <is>
           <t>Primary price/volume feed. Structured JSON.</t>
         </is>
       </c>
-      <c r="H2" s="20" t="inlineStr">
+      <c r="H2" s="51" t="inlineStr">
         <is>
           <t>CONFIRMED by extraction, 4 October 2026: chartData serves daily history from 2012-01-02 to the previous trading day for every listed security. Historical depth is no longer unknown - see D22.</t>
         </is>
       </c>
-      <c r="I2" s="20" t="inlineStr">
+      <c r="I2" s="51" t="inlineStr">
         <is>
           <t>Daily snapshots plus an intraday 'today' price feed. Snapshot-oriented, not a bulk history endpoint.</t>
         </is>
       </c>
-      <c r="J2" s="20" t="inlineStr">
+      <c r="J2" s="51" t="inlineStr">
         <is>
           <t>~23 endpoints: companyInfoSummery, todaySharePrice, tradeSummary, chartData, aspiData, snpData, topGainers, topLooses, mostActiveTrades, detailedTrades, sector data, and 8 announcement endpoints (see D12).</t>
         </is>
       </c>
-      <c r="K2" s="20" t="inlineStr">
+      <c r="K2" s="51" t="inlineStr">
         <is>
           <t>Last-traded price, change, volume and turnover aggregates. No true OHLCV bars. No adjusted close, no corporate-action adjustment. No bid-ask or order book.</t>
         </is>
       </c>
-      <c r="L2" s="20" t="inlineStr">
+      <c r="L2" s="51" t="inlineStr">
         <is>
           <t>Announcement endpoints carry English text.</t>
         </is>
       </c>
-      <c r="M2" s="20" t="inlineStr">
+      <c r="M2" s="51" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="N2" s="20" t="inlineStr">
+      <c r="N2" s="51" t="inlineStr">
         <is>
           <t>Free, no auth. POST with form-encoded params; needs a Referer of https://www.cse.lk/ and a browser user agent. GET returns 405, which is how I confirmed the endpoints are live.</t>
         </is>
       </c>
-      <c r="O2" s="20" t="inlineStr">
-        <is>
-          <t>None published. Not an official product, so no terms of use covering it and no stability guarantee. cse.lk/robots.txt disallows only /cgi-bin/, so crawling isn't robots-prohibited - but robots.txt is not a licence. CSE's actual data-reuse terms are UNCONFIRMED and need resolving in writing.</t>
-        </is>
-      </c>
-      <c r="P2" s="20" t="inlineStr">
+      <c r="O2" s="51" t="inlineStr">
+        <is>
+          <t>None published. Not an official product, so no terms of use covering it and no stability guarantee. cse.lk/robots.txt disallows only /cgi-bin/, so crawling isn't robots-prohibited - but robots.txt is not a licence. CSE's actual data-reuse terms are UNCONFIRMED and need resolving in writing.  CLEAN-LICENCE ROUTE, folded in from D02 on 18 October 2026: the cse.lk PyPI wrapper (MIT, Production/Stable, wraps 13+ of these endpoints) is the only cleanly licensed way to reach this API. That does not cure the endpoint's own unconfirmed terms, but it does mean the client code carries no licence risk, which matters because D22 is extracted through this same API and its licence is on the critical path.</t>
+        </is>
+      </c>
+      <c r="P2" s="51" t="inlineStr">
         <is>
           <t>No OHLCV bars, so intraday high/low has to be reconstructed or done without. Schema can change without notice since it's reverse-engineered. No bulk historical dump - if I don't archive it daily I can't get the past back.</t>
         </is>
       </c>
-      <c r="Q2" s="20" t="inlineStr">
+      <c r="Q2" s="51" t="inlineStr">
         <is>
           <t>Verified by extraction, not by documentation. A full pull on 2026-10-04 returned 323 securities with 0 failures and 0 empty responses. The community API documentation remains the only written description of the endpoints.</t>
         </is>
       </c>
-      <c r="R2" s="20" t="inlineStr">
+      <c r="R2" s="51" t="inlineStr">
         <is>
           <t>A_T technical and A_L liquidity (price, volume, turnover), plus the friction-aware evaluation layer, which is gated on exactly the same data.</t>
         </is>
       </c>
-      <c r="S2" s="20" t="inlineStr">
+      <c r="S2" s="51" t="inlineStr">
         <is>
           <t>The only source with real per-ticker CSE coverage. Free, no auth, and the announcement endpoints are also how I discover the annual report PDFs.</t>
         </is>
       </c>
-      <c r="T2" s="20" t="inlineStr">
+      <c r="T2" s="51" t="inlineStr">
         <is>
           <t>Undocumented, unversioned, unlicensed and could break or be shut off at any point. Historical depth unknown.</t>
         </is>
       </c>
-      <c r="U2" s="21" t="n">
+      <c r="U2" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="V2" s="19" t="inlineStr">
+      <c r="V2" s="52" t="inlineStr">
         <is>
           <t>USE - primary price source</t>
         </is>
       </c>
-      <c r="W2" s="20" t="inlineStr">
+      <c r="W2" s="51" t="inlineStr">
         <is>
           <t>There is effectively no alternative. Yahoo and Investing.com are index-only, EODHD's CSE exchange code is contaminated, and TradingView has no free export. Build a local archive from day one and probe chartData depth in week one, because if the history is too short the whole RL design has to change.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="224.4" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>D02</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>cse.lk Python package</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+    <row r="3" ht="195" customHeight="1">
+      <c r="A3" s="53" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B3" s="54" t="inlineStr">
+        <is>
+          <t>CSE listed-company report PDFs</t>
+        </is>
+      </c>
+      <c r="C3" s="54" t="inlineStr">
+        <is>
+          <t>Filings / fundamentals</t>
+        </is>
+      </c>
+      <c r="D3" s="54" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange CDN</t>
+        </is>
+      </c>
+      <c r="E3" s="54" t="inlineStr">
+        <is>
+          <t>https://cdn.cse.lk/cmt/upload_report_file/&lt;id&gt;_&lt;epoch_ms&gt;.pdf (discovered via the D01 announcement endpoints)</t>
+        </is>
+      </c>
+      <c r="F3" s="54" t="inlineStr">
+        <is>
+          <t>All ~280-300 CSE-listed companies. Annual and quarterly reports.</t>
+        </is>
+      </c>
+      <c r="G3" s="54" t="inlineStr">
+        <is>
+          <t>RAG corpus. PDF - text, tables and figures.</t>
+        </is>
+      </c>
+      <c r="H3" s="54" t="inlineStr">
+        <is>
+          <t>Older filings thin, roughly pre-2015.</t>
+        </is>
+      </c>
+      <c r="I3" s="54" t="inlineStr">
+        <is>
+          <t>Quarterly and annual.</t>
+        </is>
+      </c>
+      <c r="J3" s="54" t="inlineStr">
+        <is>
+          <t>Hundreds of companies x multiple filings per year.</t>
+        </is>
+      </c>
+      <c r="K3" s="54" t="inlineStr">
+        <is>
+          <t>N/A - this is the fundamentals side.</t>
+        </is>
+      </c>
+      <c r="L3" s="54" t="inlineStr">
+        <is>
+          <t>English. Full audited statements: P&amp;L and OCI, financial position, changes in equity, cash flows, notes, auditor's report.</t>
+        </is>
+      </c>
+      <c r="M3" s="54" t="inlineStr">
+        <is>
+          <t>None - unlabelled documents.</t>
+        </is>
+      </c>
+      <c r="N3" s="54" t="inlineStr">
+        <is>
+          <t>Free direct HTTP GET, no auth. But filenames are opaque id/timestamp pairs, so links have to be harvested from the announcement endpoints rather than enumerated.</t>
+        </is>
+      </c>
+      <c r="O3" s="54" t="inlineStr">
+        <is>
+          <t>UNCONFIRMED. I could not retrieve a cse.lk terms-of-use page. Treat CSE data reuse rights as unresolved and email CSE before publishing anything derived.</t>
+        </is>
+      </c>
+      <c r="P3" s="54" t="inlineStr">
+        <is>
+          <t>No XBRL, so nothing is machine-structured. Report layout varies considerably company to company. Older filings more likely to be scanned rather than text-native, which is exactly the OCR failure mode P07 warns breaks element-based chunking.</t>
+        </is>
+      </c>
+      <c r="Q3" s="54" t="inlineStr">
+        <is>
+          <t>Verified - fetched the endpoint or page myself</t>
+        </is>
+      </c>
+      <c r="R3" s="54" t="inlineStr">
+        <is>
+          <t>A_F fundamental. After the September 2026 scope decision this is the framework's only text modality, so it carries the heterogeneity claim in the main gap.</t>
+        </is>
+      </c>
+      <c r="S3" s="54" t="inlineStr">
+        <is>
+          <t>The best-provisioned component of the whole project. Text-native full-statement PDFs for every listed company on an open CDN - I verified one end to end (Office Equipment PLC FY2025, full audited statements).</t>
+        </is>
+      </c>
+      <c r="T3" s="54" t="inlineStr">
+        <is>
+          <t>Discovery is awkward, structure is inconsistent, and the licensing question is unresolved.</t>
+        </is>
+      </c>
+      <c r="U3" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="V3" s="52" t="inlineStr">
+        <is>
+          <t>USE - primary RAG corpus</t>
+        </is>
+      </c>
+      <c r="W3" s="54" t="inlineStr">
+        <is>
+          <t>This is what A_F is built on, and after the scope cut it is the framework's only text channel rather than a demoted system feature. Text-native PDFs mean element-based chunking has something real to work with. The architectural novelty is closed by the 2025 CSE Neo4j Graph-RAG work (Shamila, Silva and Talagala, ERU 2025, DOI 10.31705/ERU.2025.35), now verified, so what remains for A_F is numeric statement extraction, point-in-time correctness and the orchestration that consumes the signal. Every document needs a publication-date field and a retrieval filter keyed to the simulation clock, because their graph is a static snapshot with no as-of field and that is a lookahead hazard in a backtest rather than an inconvenience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="50" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="B4" s="51" t="inlineStr">
+        <is>
+          <t>CSE exchange annual reports</t>
+        </is>
+      </c>
+      <c r="C4" s="51" t="inlineStr">
+        <is>
+          <t>Filings / fundamentals</t>
+        </is>
+      </c>
+      <c r="D4" s="51" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange</t>
+        </is>
+      </c>
+      <c r="E4" s="51" t="inlineStr">
+        <is>
+          <t>https://cdn.cse.lk/pdf/annual-reports/Annual-Report-YYYY.pdf</t>
+        </is>
+      </c>
+      <c r="F4" s="51" t="inlineStr">
+        <is>
+          <t>The exchange itself, not listed companies.</t>
+        </is>
+      </c>
+      <c r="G4" s="51" t="inlineStr">
+        <is>
+          <t>Market context. PDF.</t>
+        </is>
+      </c>
+      <c r="H4" s="51" t="inlineStr">
+        <is>
+          <t>2020-2024 confirmed loading.</t>
+        </is>
+      </c>
+      <c r="I4" s="51" t="inlineStr">
+        <is>
+          <t>Annual.</t>
+        </is>
+      </c>
+      <c r="J4" s="51" t="inlineStr">
+        <is>
+          <t>Five reports confirmed.</t>
+        </is>
+      </c>
+      <c r="K4" s="51" t="inlineStr">
+        <is>
+          <t>Market-level turnover and activity statistics.</t>
+        </is>
+      </c>
+      <c r="L4" s="51" t="inlineStr">
+        <is>
+          <t>English.</t>
+        </is>
+      </c>
+      <c r="M4" s="51" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="N4" s="51" t="inlineStr">
+        <is>
+          <t>Free direct download.</t>
+        </is>
+      </c>
+      <c r="O4" s="51" t="inlineStr">
+        <is>
+          <t>No explicit copyright notice in the documents I checked.</t>
+        </is>
+      </c>
+      <c r="P4" s="51" t="inlineStr">
+        <is>
+          <t>Exchange-level only - no company fundamentals.</t>
+        </is>
+      </c>
+      <c r="Q4" s="51" t="inlineStr">
+        <is>
+          <t>Verified - fetched the endpoint or page myself</t>
+        </is>
+      </c>
+      <c r="R4" s="51" t="inlineStr">
+        <is>
+          <t>None directly. Background for the Sub-gap 1 execution model, market structure and turnover context.</t>
+        </is>
+      </c>
+      <c r="S4" s="51" t="inlineStr">
+        <is>
+          <t>Useful for understanding CSE turnover patterns and market structure when I'm designing the simulated exchange.</t>
+        </is>
+      </c>
+      <c r="T4" s="51" t="inlineStr">
+        <is>
+          <t>Not a modelling input. Background reading.</t>
+        </is>
+      </c>
+      <c r="U4" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="V4" s="52" t="inlineStr">
+        <is>
+          <t>USE - background only</t>
+        </is>
+      </c>
+      <c r="W4" s="51" t="inlineStr">
+        <is>
+          <t>Worth reading for the microstructure and turnover context behind the execution model, but it doesn't feed any agent directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="53" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B5" s="54" t="inlineStr">
+        <is>
+          <t>CBSL Rates and Indicators</t>
+        </is>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="D5" s="54" t="inlineStr">
+        <is>
+          <t>Central Bank of Sri Lanka</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>https://www.cbsl.gov.lk/en/rates-and-indicators</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t>Sri Lanka.</t>
+        </is>
+      </c>
+      <c r="G5" s="54" t="inlineStr">
+        <is>
+          <t>Macro indicators. Web tables and PDFs.</t>
+        </is>
+      </c>
+      <c r="H5" s="54" t="inlineStr">
+        <is>
+          <t>Continuous archives with year/month filters.</t>
+        </is>
+      </c>
+      <c r="I5" s="54" t="inlineStr">
+        <is>
+          <t>Daily, weekly and monthly depending on series.</t>
+        </is>
+      </c>
+      <c r="J5" s="54" t="inlineStr">
+        <is>
+          <t>Multiple series.</t>
+        </is>
+      </c>
+      <c r="K5" s="54" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="L5" s="54" t="inlineStr">
+        <is>
+          <t>English, Sinhala and Tamil for the Monthly Bulletin.</t>
+        </is>
+      </c>
+      <c r="M5" s="54" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="N5" s="54" t="inlineStr">
+        <is>
+          <t>Free web. Navigate from the index page - constructed deep URLs (/interest-rates/t-bill-rates, /inflation, etc.) all 404.</t>
+        </is>
+      </c>
+      <c r="O5" s="54" t="inlineStr">
+        <is>
+          <t>cbsl.gov.lk/robots.txt sets Crawl-delay: 10 for all agents and explicitly disallows specific treasury-rate service endpoints - which directly touches what the risk agent would want. AhrefsBot fully blocked.</t>
+        </is>
+      </c>
+      <c r="P5" s="54" t="inlineStr">
+        <is>
+          <t>Download formats not stated on the index pages. The treasury-endpoint disallow is a real constraint, not a formality.</t>
+        </is>
+      </c>
+      <c r="Q5" s="54" t="inlineStr">
+        <is>
+          <t>Verified - fetched the endpoint or page myself</t>
+        </is>
+      </c>
+      <c r="R5" s="54" t="inlineStr">
+        <is>
+          <t>A_V, plus the risk-free rate for Sharpe and excess-return calculations in the evaluation layer.</t>
+        </is>
+      </c>
+      <c r="S5" s="54" t="inlineStr">
+        <is>
+          <t>Confirmed categories cover everything I need: CCPI and NCPI inflation, policy rates, exchange rates, SLIBOR, government securities (T-bill and T-bond yields), commercial bank lending and deposit rates, open market operations. P11 uses 91-day T-bill auction rates as the risk-free rate, and those live here.</t>
+        </is>
+      </c>
+      <c r="T5" s="54" t="inlineStr">
+        <is>
+          <t>Robots.txt disallows exactly the treasury-rate endpoints I'd most want to automate, and there's no API.</t>
+        </is>
+      </c>
+      <c r="U5" s="54" t="n">
+        <v>4</v>
+      </c>
+      <c r="V5" s="52" t="inlineStr">
+        <is>
+          <t>USE - respect the crawl-delay and the disallow list</t>
+        </is>
+      </c>
+      <c r="W5" s="54" t="inlineStr">
+        <is>
+          <t>Non-negotiable for the risk-free rate and regime context. But the disallowed treasury endpoints mean I need to pull those figures from the published tables rather than the service endpoints, and honour the 10-second crawl delay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="50" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>CSE announcements feed</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>Disclosures</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>Via the D01 POST API - 8 announcement categories</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="inlineStr">
+        <is>
+          <t>CSE. All listed companies.</t>
+        </is>
+      </c>
+      <c r="G6" s="51" t="inlineStr">
+        <is>
+          <t>Corporate disclosures. Structured JSON plus linked PDFs.</t>
+        </is>
+      </c>
+      <c r="H6" s="51" t="inlineStr">
+        <is>
+          <t>Not confirmed.</t>
+        </is>
+      </c>
+      <c r="I6" s="51" t="inlineStr">
+        <is>
+          <t>Event-driven.</t>
+        </is>
+      </c>
+      <c r="J6" s="51" t="inlineStr">
+        <is>
+          <t>8 announcement endpoints. The ones I could name from the community API documentation are financial, circular, compliance, listings, buy-in board and directives - the remaining two need confirming by enumerating the endpoints directly.</t>
+        </is>
+      </c>
+      <c r="K6" s="51" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="L6" s="51" t="inlineStr">
+        <is>
+          <t>English.</t>
+        </is>
+      </c>
+      <c r="M6" s="51" t="inlineStr">
+        <is>
+          <t>Unlabelled.</t>
+        </is>
+      </c>
+      <c r="N6" s="51" t="inlineStr">
+        <is>
+          <t>Same POST API as D01. No RSS found.</t>
+        </is>
+      </c>
+      <c r="O6" s="51" t="inlineStr">
+        <is>
+          <t>Same unconfirmed CSE terms as D01.</t>
+        </is>
+      </c>
+      <c r="P6" s="51" t="inlineStr">
+        <is>
+          <t>Historical depth unconfirmed, same as everything else on the CSE API.</t>
+        </is>
+      </c>
+      <c r="Q6" s="51" t="inlineStr">
+        <is>
+          <t>Verified - fetched the endpoint or page myself</t>
+        </is>
+      </c>
+      <c r="R6" s="51" t="inlineStr">
+        <is>
+          <t>A_F. This is how the report PDFs in D07 are discovered, which is the whole reason it survives the scope cut.</t>
+        </is>
+      </c>
+      <c r="S6" s="51" t="inlineStr">
+        <is>
+          <t>Primary-source corporate disclosure, which is higher-signal and less ambiguous than news coverage of the same events. Also the discovery mechanism for D07, the report PDFs.</t>
+        </is>
+      </c>
+      <c r="T6" s="51" t="inlineStr">
+        <is>
+          <t>Undocumented, and depth unknown.</t>
+        </is>
+      </c>
+      <c r="U6" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="V6" s="52" t="inlineStr">
+        <is>
+          <t>USE - primary disclosure feed</t>
+        </is>
+      </c>
+      <c r="W6" s="51" t="inlineStr">
+        <is>
+          <t>The only survivor of the news and social block, and it survives for a structural reason rather than a sentimental one: it is a primary disclosure feed, not commentary, and it is how the report PDFs in D07 are discovered. It also carries the timestamp that makes point-in-time retrieval possible - a document is only visible to A_F after the announcement datetime, which is what keeps the backtest free of lookahead. Treat it as metadata and routing for A_F, not as a text signal in its own right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="53" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t>CSE Price Index / ASPI ten-year daily series</t>
+        </is>
+      </c>
+      <c r="C7" s="56" t="inlineStr">
         <is>
           <t>Price &amp; market data</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>PyPI (community)</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>https://pypi.org/project/cse.lk/</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>CSE, wraps D01.</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Ingestion tooling.</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Same as D01.</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>Same as D01.</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Wraps 13+ CSE endpoints.</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Same as D01.</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>pip install. Python 3.8+.</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>MIT. One of the clean licences - see the Read Me for the full list.</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
-        <is>
-          <t>Inherits every limitation of D01, including no OHLCV and unknown history depth.</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>Ingestion layer for A_T and A_L.</t>
-        </is>
-      </c>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>Fastest route to a working prototype, and MIT-licensed so it's safe to build on. Marked Production/Stable.</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>Thin wrapper - it doesn't solve any of D01's underlying problems.</t>
-        </is>
-      </c>
-      <c r="U3" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="V3" s="7" t="inlineStr">
-        <is>
-          <t>USE - ingestion wrapper</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
-        <is>
-          <t>No reason to hand-roll the HTTP layer when a stable MIT-licensed wrapper exists. Just don't mistake it for a different data source.</t>
+      <c r="D7" s="56" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange official database</t>
+        </is>
+      </c>
+      <c r="E7" s="56" t="inlineStr">
+        <is>
+          <t>Via CSE directly; published route evidenced by the 2026 ARIMA study in the Literature Survey sheet</t>
+        </is>
+      </c>
+      <c r="F7" s="56" t="inlineStr">
+        <is>
+          <t>CSE, index level only.</t>
+        </is>
+      </c>
+      <c r="G7" s="56" t="inlineStr">
+        <is>
+          <t>Long index history. Time series.</t>
+        </is>
+      </c>
+      <c r="H7" s="56" t="inlineStr">
+        <is>
+          <t>OBTAINED 5 October 2026: 2012-01-02 to 2026-10-02.</t>
+        </is>
+      </c>
+      <c r="I7" s="56" t="inlineStr">
+        <is>
+          <t>Daily.</t>
+        </is>
+      </c>
+      <c r="J7" s="56" t="inlineStr">
+        <is>
+          <t>3,468 daily observations.</t>
+        </is>
+      </c>
+      <c r="K7" s="56" t="inlineStr">
+        <is>
+          <t>Traded Date and index Value (close) only. No index OHLC, no volume.</t>
+        </is>
+      </c>
+      <c r="L7" s="56" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="M7" s="56" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N7" s="56" t="inlineStr">
+        <is>
+          <t>Downloaded from the CSE site as 'Historical-Values-data-2026-10-05 (ASPI).csv'. S&amp;P SL20 obtained the same way on 2026-10-04. A separate 'Trading days.csv' gives the exchange calendar, which is what distinguishes a non-trading day from a zero-volume day everywhere else in this matrix.</t>
+        </is>
+      </c>
+      <c r="O7" s="56" t="inlineStr">
+        <is>
+          <t>Not stated in the source study. CSE data-reuse terms remain unconfirmed and should be resolved in the same written request as everything else.</t>
+        </is>
+      </c>
+      <c r="P7" s="56" t="inlineStr">
+        <is>
+          <t>Close only, so index-level Parkinson and Garman-Klass estimators cannot be computed from this file - V_t at index level is limited to close-to-close unless index OHLC is obtained separately. Rows are in descending date order with dates as '2 OCT 2026', so both need normalising on load.</t>
+        </is>
+      </c>
+      <c r="Q7" s="56" t="inlineStr">
+        <is>
+          <t>Obtained and held locally. Supersedes the second-hand 1 Jul 2014 - 30 Jun 2024 span previously recorded from a published study: the held series is longer at both ends.</t>
+        </is>
+      </c>
+      <c r="R7" s="56" t="inlineStr">
+        <is>
+          <t>A_V above all. Also the baselines and the regime-split reporting in the evaluation layer.</t>
+        </is>
+      </c>
+      <c r="S7" s="56" t="inlineStr">
+        <is>
+          <t>THE INDEX TRACK IS SECURE. Roughly 2,400 daily observations is in the same range as the 2,922 the CSE FIGARCH study used, so Sub-gap 2's persistence estimator can be fitted even if per-counter depth never improves. Three distinct regime episodes for labelling.</t>
+        </is>
+      </c>
+      <c r="T7" s="56" t="inlineStr">
+        <is>
+          <t>Index only. Per-regime it splits to roughly 1,500 / 500 / 600 observations, so the COVID window is thin for a fractional differencing estimate even though it is an order of magnitude past the four-month failure case in the literature.</t>
+        </is>
+      </c>
+      <c r="U7" s="56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V7" s="57" t="inlineStr">
+        <is>
+          <t>USE - obtained, and longer than the published span</t>
+        </is>
+      </c>
+      <c r="W7" s="56" t="inlineStr">
+        <is>
+          <t>This is the row that de-risks Sub-gap 2. The persistence work does not wait on the per-counter data request. Ask for it by name rather than asking for 'ten years of data', because an index series would satisfy that phrasing and leave A_T, A_L and the friction model no better off.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="396" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>D03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>stockanalysis.com CSE listing</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="50" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>Listing and delisting register with effective dates</t>
+        </is>
+      </c>
+      <c r="C8" s="58" t="inlineStr">
+        <is>
+          <t>Reference data</t>
+        </is>
+      </c>
+      <c r="D8" s="58" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange</t>
+        </is>
+      </c>
+      <c r="E8" s="58" t="inlineStr">
+        <is>
+          <t>Not located. Part of the CSE R&amp;D request.</t>
+        </is>
+      </c>
+      <c r="F8" s="58" t="inlineStr">
+        <is>
+          <t>CSE, all counters including those no longer listed.</t>
+        </is>
+      </c>
+      <c r="G8" s="58" t="inlineStr">
+        <is>
+          <t>Tradability mask. Reference table.</t>
+        </is>
+      </c>
+      <c r="H8" s="58" t="inlineStr">
+        <is>
+          <t>Snapshot as at 31 January 2024.</t>
+        </is>
+      </c>
+      <c r="I8" s="58" t="inlineStr">
+        <is>
+          <t>Event-level.</t>
+        </is>
+      </c>
+      <c r="J8" s="58" t="inlineStr">
+        <is>
+          <t>119 delisted companies.</t>
+        </is>
+      </c>
+      <c r="K8" s="58" t="inlineStr">
+        <is>
+          <t>None directly - this is the mask applied to the price data.</t>
+        </is>
+      </c>
+      <c r="L8" s="58" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="M8" s="58" t="inlineStr">
+        <is>
+          <t>Listing date, delisting date, and reason where available.</t>
+        </is>
+      </c>
+      <c r="N8" s="58" t="inlineStr">
+        <is>
+          <t>PARTIALLY OBTAINED. 'DE-LISTED-COMPANIES-31-01-2024.xlsx' is held, giving company code and company name for 119 delisted companies.</t>
+        </is>
+      </c>
+      <c r="O8" s="58" t="inlineStr">
+        <is>
+          <t>Unconfirmed.</t>
+        </is>
+      </c>
+      <c r="P8" s="58" t="inlineStr">
+        <is>
+          <t>Two gaps, and the first is the one that matters. (1) NO DELISTING DATES - the file is a list of names, so it supports a static exclusion but not a point-in-time tradability mask, and a static exclusion is the survivorship bias it was meant to fix. (2) The snapshot stops at 31 Jan 2024, so anything delisted since is missing. Separately, D22 already contains 61 securities whose history ends before the last trading day, which is an empirical lower bound on delistings and suspensions across the sample and can be cross-referenced against this list.</t>
+        </is>
+      </c>
+      <c r="Q8" s="58" t="inlineStr">
+        <is>
+          <t>Partially obtained - the list exists, the dates do not.</t>
+        </is>
+      </c>
+      <c r="R8" s="58" t="inlineStr">
+        <is>
+          <t>All four agents, via the universe definition, plus the evaluation layer.</t>
+        </is>
+      </c>
+      <c r="S8" s="58" t="inlineStr">
+        <is>
+          <t>A counter should leave the investable universe on the day it delisted, not retrospectively for the whole sample. This is the tradability-mask correction that the diversified-portfolio framework in the Literature Survey sheet builds explicitly from membership history, and whose absence is flagged there as a possible thirty-year survivorship filter in a comparable study.</t>
+        </is>
+      </c>
+      <c r="T8" s="58" t="inlineStr">
+        <is>
+          <t>May be unobtainable. The counters that delisted through the 2022 default and currency collapse are disproportionately the ones that failed, and they are also disproportionately thin - which is exactly the part of the book Sub-gap 1 is about, so excluding them removes the phenomenon under study.</t>
+        </is>
+      </c>
+      <c r="U8" s="58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V8" s="59" t="inlineStr">
+        <is>
+          <t>PARTIALLY OBTAINED - still ask the CSE for dated listing and delisting events  |  18 Oct 2026: Data Library item 06, New Listings and De-listings, is the official route to complete this and is included in the D24 purchase.</t>
+        </is>
+      </c>
+      <c r="W8" s="58" t="inlineStr">
+        <is>
+          <t>The names alone quantify how much of the universe is missing, which is already more than most projects on this market can state. What they do not support is a counter leaving the investable universe on the day it actually delisted. Ask the CSE specifically for EFFECTIVE DATES rather than for a delisting list, because the list is already held and asking for it again wastes the request. If dates cannot be obtained, use the D22 series-end dates as a proxy, state plainly that they are a proxy, and report the residual bias and its direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="53" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="B9" s="56" t="inlineStr">
+        <is>
+          <t>Counter liquidity screen and tier table</t>
+        </is>
+      </c>
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>Derived dataset</t>
+        </is>
+      </c>
+      <c r="D9" s="56" t="inlineStr">
+        <is>
+          <t>Own computation over D22</t>
+        </is>
+      </c>
+      <c r="E9" s="56" t="inlineStr">
+        <is>
+          <t>Derived from the D22 archive</t>
+        </is>
+      </c>
+      <c r="F9" s="56" t="inlineStr">
+        <is>
+          <t>CSE, all counters present in the archive.</t>
+        </is>
+      </c>
+      <c r="G9" s="56" t="inlineStr">
+        <is>
+          <t>Derived reference table sizing every downstream component.</t>
+        </is>
+      </c>
+      <c r="H9" s="56" t="inlineStr">
+        <is>
+          <t>The D22 span, 2012-01-02 to 2026-10-02. (Corrected 18 October 2026: this cell previously carried D13's 374-day span.)</t>
+        </is>
+      </c>
+      <c r="I9" s="56" t="inlineStr">
+        <is>
+          <t>Per counter.</t>
+        </is>
+      </c>
+      <c r="J9" s="56" t="inlineStr">
+        <is>
+          <t>323 securities x 829,070 observations available to screen, from D22.</t>
+        </is>
+      </c>
+      <c r="K9" s="56" t="inlineStr">
+        <is>
+          <t>Per counter from D22: share of trading days with non-zero volume, median and mean share_volume, median turnover, zero-return frequency reported separately from non-trading, Amihud mean of |return| over turnover, history length and missing-day count. Turnover and trade_volume are both present in D22, so Amihud is computable directly rather than proxied.</t>
+        </is>
+      </c>
+      <c r="L9" s="56" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="M9" s="56" t="inlineStr">
+        <is>
+          <t>Liquidity tier per counter.</t>
+        </is>
+      </c>
+      <c r="N9" s="56" t="inlineStr">
+        <is>
+          <t>One pass over data already held. No external dependency, no permission required.</t>
+        </is>
+      </c>
+      <c r="O9" s="56" t="inlineStr">
+        <is>
+          <t>n/a - derived.</t>
+        </is>
+      </c>
+      <c r="P9" s="56" t="inlineStr">
+        <is>
+          <t>A genuine flat print and a stale carry-forward both read as a zero return in a close-only series, so the screen must test volume rather than price change; the D15 exchange calendar is what separates a non-trading day from a zero-volume one. Liquidity regimes also shift across a 14.75-year span, so a screen fitted once is not valid throughout and must be re-run inside each training fold. Note that D22 carries a real example of the defect this guards against: ASPM.N0000 prints a close of 56.8 on days whose open, high and low are all 71.0, so close sits outside the high-low range.</t>
+        </is>
+      </c>
+      <c r="Q9" s="56" t="inlineStr">
+        <is>
+          <t>Not yet computed.</t>
+        </is>
+      </c>
+      <c r="R9" s="56" t="inlineStr">
+        <is>
+          <t>Sizes A_T, calibrates A_L, and sets the friction model's scale. Also the first empirical fit of the L_t conditioning variable.</t>
+        </is>
+      </c>
+      <c r="S9" s="56" t="inlineStr">
+        <is>
+          <t>The cheapest high-value computation available and it needs nothing that is not already held. It answers the question the cross-sectional reframe actually turns on, which is how many counters clear a liquidity screen rather than how many years of history exist. It is also a publishable CSE liquidity statistic in its own right.</t>
+        </is>
+      </c>
+      <c r="T9" s="56" t="inlineStr">
+        <is>
+          <t>Do not reduce it to a single threshold. Screening for liquid counters removes the thin-book conditions Sub-gap 1 is about, so report results BY TIER and let the cutoff become a result rather than a choice. That also aligns with the CSE finding that small caps are more exposed to illiquidity shocks than large, at -0.071 against -0.060.</t>
+        </is>
+      </c>
+      <c r="U9" s="56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V9" s="57" t="inlineStr">
+        <is>
+          <t>COMPUTE NEXT - no external dependency, and it now has 14.75 years to screen</t>
+        </is>
+      </c>
+      <c r="W9" s="56" t="inlineStr">
+        <is>
+          <t>At a 30-day lookback the D22 archive gives roughly 345 usable windows per counter, so with ~300 counters the sequence count is around 100,000, materially better than the earlier ~240-day working assumption. The tier table converts that headline into a per-tier figure, which is what actually sizes the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="50" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="B10" s="58" t="inlineStr">
+        <is>
+          <t>University of Moratuwa CSE Graph-RAG corpus and code</t>
+        </is>
+      </c>
+      <c r="C10" s="58" t="inlineStr">
+        <is>
+          <t>Filings / fundamentals</t>
+        </is>
+      </c>
+      <c r="D10" s="58" t="inlineStr">
+        <is>
+          <t>Shamila, Silva and Talagala, Dept of Computer Science and Engineering, University of Moratuwa</t>
+        </is>
+      </c>
+      <c r="E10" s="58" t="inlineStr">
+        <is>
+          <t>DOI 10.31705/ERU.2025.35, with a public GitHub repository linked from the paper</t>
+        </is>
+      </c>
+      <c r="F10" s="58" t="inlineStr">
+        <is>
+          <t>CSE annual reports. Company count and date range not reported.</t>
+        </is>
+      </c>
+      <c r="G10" s="58" t="inlineStr">
+        <is>
+          <t>Prior art for A_F, plus a data-access lead.</t>
+        </is>
+      </c>
+      <c r="H10" s="58" t="inlineStr">
+        <is>
+          <t>Not reported in the paper.</t>
+        </is>
+      </c>
+      <c r="I10" s="58" t="inlineStr">
+        <is>
+          <t>Document level.</t>
+        </is>
+      </c>
+      <c r="J10" s="58" t="inlineStr">
+        <is>
+          <t>Over 6,000 unique entities reported, against roughly 280 listed companies.</t>
+        </is>
+      </c>
+      <c r="K10" s="58" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="L10" s="58" t="inlineStr">
+        <is>
+          <t>English. CSE annual report PDFs.</t>
+        </is>
+      </c>
+      <c r="M10" s="58" t="inlineStr">
+        <is>
+          <t>A Neo4j knowledge graph of corporate structure, governance and ownership. Tabular financial data is explicitly out of scope in their work.</t>
+        </is>
+      </c>
+      <c r="N10" s="58" t="inlineStr">
+        <is>
+          <t>Public repository. The authors are at the same university and are reachable.</t>
+        </is>
+      </c>
+      <c r="O10" s="58" t="inlineStr">
+        <is>
+          <t>Not stated.</t>
+        </is>
+      </c>
+      <c r="P10" s="58" t="inlineStr">
+        <is>
+          <t>The paper gives NO information on how the CSE documents were obtained, how many companies, or what date range - which is the single most useful thing it could have reported for my purposes.</t>
+        </is>
+      </c>
+      <c r="Q10" s="58" t="inlineStr">
+        <is>
+          <t>Verified. Two-page extended abstract, ERU Symposium 2025.</t>
+        </is>
+      </c>
+      <c r="R10" s="58" t="inlineStr">
+        <is>
+          <t>A_F, as prior art and as adoptable tooling.</t>
+        </is>
+      </c>
+      <c r="S10" s="58" t="inlineStr">
+        <is>
+          <t>Closes the architectural novelty of structure-aware retrieval over CSE annual reports, which is settled and not recoverable. More useful to me now as a data-access lead: same department, same university, reachable, with working extraction code.</t>
+        </is>
+      </c>
+      <c r="T10" s="58" t="inlineStr">
+        <is>
+          <t>A two-page abstract, so the pipeline constants are adoptable as defaults but not as validated settings. Their graph is a static snapshot with no as-of field.</t>
+        </is>
+      </c>
+      <c r="U10" s="58" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V10" s="57" t="inlineStr">
+        <is>
+          <t>USE as prior art and as tooling; CONTACT the authors</t>
+        </is>
+      </c>
+      <c r="W10" s="58" t="inlineStr">
+        <is>
+          <t>The best warm route to the CSE data-access question. A local research group that already extracted CSE annual reports at scale knows how they got them, and that is worth an email before the formal R&amp;D request rather than after.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="53" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>FinQA</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="D11" s="56" t="inlineStr">
+        <is>
+          <t>Chen et al., EMNLP 2021</t>
+        </is>
+      </c>
+      <c r="E11" s="56" t="inlineStr">
+        <is>
+          <t>https://github.com/czyssrs/FinQA</t>
+        </is>
+      </c>
+      <c r="F11" s="56" t="inlineStr">
+        <is>
+          <t>US filings, English.</t>
+        </is>
+      </c>
+      <c r="G11" s="56" t="inlineStr">
+        <is>
+          <t>Development artefact for A_F. Tables plus text.</t>
+        </is>
+      </c>
+      <c r="H11" s="56" t="inlineStr">
+        <is>
+          <t>n/a.</t>
+        </is>
+      </c>
+      <c r="I11" s="56" t="inlineStr">
+        <is>
+          <t>Question level.</t>
+        </is>
+      </c>
+      <c r="J11" s="56" t="inlineStr">
+        <is>
+          <t>Built over FinTabNet.</t>
+        </is>
+      </c>
+      <c r="K11" s="56" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="L11" s="56" t="inlineStr">
+        <is>
+          <t>English.</t>
+        </is>
+      </c>
+      <c r="M11" s="56" t="inlineStr">
+        <is>
+          <t>Question, answer, and an executable reasoning program.</t>
+        </is>
+      </c>
+      <c r="N11" s="56" t="inlineStr">
+        <is>
+          <t>Public GitHub.</t>
+        </is>
+      </c>
+      <c r="O11" s="56" t="inlineStr">
+        <is>
+          <t>CDLA-Permissive via FinTabNet. The cleanest licence of the A_F development set.</t>
+        </is>
+      </c>
+      <c r="P11" s="56" t="inlineStr">
+        <is>
+          <t>US filings with page-local, pre-located context and no as-of notion, so it does not transfer to CSE documents as data.</t>
+        </is>
+      </c>
+      <c r="Q11" s="56" t="inlineStr">
+        <is>
+          <t>Verified.</t>
+        </is>
+      </c>
+      <c r="R11" s="56" t="inlineStr">
+        <is>
+          <t>A_F, development and the C_F,t confidence signal.</t>
+        </is>
+      </c>
+      <c r="S11" s="56" t="inlineStr">
+        <is>
+          <t>Pull the DSL and the program executor directly rather than reimplement. Supplies the retrieve-then-program architecture and, importantly, a structural confidence signal for A_F: whether the program parses under the grammar, whether every argument traces to a retrieved number, and program step count as a calibrated difficulty proxy at 67.61 / 59.08 / 22.78 per cent for one, two and three-plus steps.</t>
+        </is>
+      </c>
+      <c r="T11" s="56" t="inlineStr">
+        <is>
+          <t>Not usable as a CSE evaluation set. Its 61.24 / 91.16 difficulty prior is explicitly non-portable and should be cited as an order of magnitude, never as a target.</t>
+        </is>
+      </c>
+      <c r="U11" s="56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V11" s="57" t="inlineStr">
+        <is>
+          <t>USE - A_F development only</t>
+        </is>
+      </c>
+      <c r="W11" s="56" t="inlineStr">
+        <is>
+          <t>The planning band agreed across three independent papers is below 50% on computed quantities over CSE filings, nearer 40% than 60% on first build. A_F is expected to be unusable more often than not, and the orchestrator has to be designed for a channel that is frequently unusable rather than occasionally imperfect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="50" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t>ConvFinQA and TAT-QA</t>
+        </is>
+      </c>
+      <c r="C12" s="58" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="D12" s="58" t="inlineStr">
+        <is>
+          <t>Chen et al., EMNLP 2022; Zhu et al., ACL-IJCNLP 2021</t>
+        </is>
+      </c>
+      <c r="E12" s="58" t="inlineStr">
+        <is>
+          <t>https://github.com/czyssrs/ConvFinQA and https://nextplusplus.github.io/TAT-QA</t>
+        </is>
+      </c>
+      <c r="F12" s="58" t="inlineStr">
+        <is>
+          <t>US filings, English.</t>
+        </is>
+      </c>
+      <c r="G12" s="58" t="inlineStr">
+        <is>
+          <t>Development artefacts and taxonomy for A_F.</t>
+        </is>
+      </c>
+      <c r="H12" s="58" t="inlineStr">
+        <is>
+          <t>n/a.</t>
+        </is>
+      </c>
+      <c r="I12" s="58" t="inlineStr">
+        <is>
+          <t>Question level.</t>
+        </is>
+      </c>
+      <c r="J12" s="58" t="inlineStr">
+        <is>
+          <t>ConvFinQA: 3,037 / 421 / 434 conversations. TAT-QA: hybrid table-and-text questions.</t>
+        </is>
+      </c>
+      <c r="K12" s="58" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="L12" s="58" t="inlineStr">
+        <is>
+          <t>English.</t>
+        </is>
+      </c>
+      <c r="M12" s="58" t="inlineStr">
+        <is>
+          <t>ConvFinQA adds multi-turn context; TAT-QA adds a scale taxonomy of None / Thousand / Million / Billion / Percent and an answer-type by answer-source split.</t>
+        </is>
+      </c>
+      <c r="N12" s="58" t="inlineStr">
+        <is>
+          <t>Public.</t>
+        </is>
+      </c>
+      <c r="O12" s="58" t="inlineStr">
+        <is>
+          <t>ConvFinQA inherits FinTabNet. TAT-QA is public for NON-COMMERCIAL USE ONLY - the one explicit restriction in the A_F set.</t>
+        </is>
+      </c>
+      <c r="P12" s="58" t="inlineStr">
+        <is>
+          <t>Same non-transferability as D19.</t>
+        </is>
+      </c>
+      <c r="Q12" s="58" t="inlineStr">
+        <is>
+          <t>Verified.</t>
+        </is>
+      </c>
+      <c r="R12" s="58" t="inlineStr">
+        <is>
+          <t>A_F, probe-set design and taxonomy.</t>
+        </is>
+      </c>
+      <c r="S12" s="58" t="inlineStr">
+        <is>
+          <t>ConvFinQA pairs with FinQA as one probe corpus with and without conversational context, which is the cheapest available ablation on whether a reference-resolution layer does anything. TAT-QA's scale taxonomy and two-round validation pattern lift directly into the CSE probe-set design and are affordable at ten to twenty questions.</t>
+        </is>
+      </c>
+      <c r="T12" s="58" t="inlineStr">
+        <is>
+          <t>Neither is a CSE evaluation set. TAT-QA's operator accuracy runs from 100.0 down to 0.0 across classes, so a single posterior is not comparable across classes without per-operator reliability estimated on my own probe set.</t>
+        </is>
+      </c>
+      <c r="U12" s="58" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V12" s="57" t="inlineStr">
+        <is>
+          <t>USE - taxonomy and probe design</t>
+        </is>
+      </c>
+      <c r="W12" s="58" t="inlineStr">
+        <is>
+          <t>The convergent conclusion across the benchmark papers is the same: build a hand-checked probe set of ten to twenty questions over a handful of CSE annual reports, stratified by reasoning type and answer source, scored on the four-state taxonomy of correct, incorrect, failure-to-answer and no parseable answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>Level-III message data and multi-level depth for CSE</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
+        <is>
+          <t>Microstructure</t>
+        </is>
+      </c>
+      <c r="D13" s="56" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange</t>
+        </is>
+      </c>
+      <c r="E13" s="56" t="inlineStr">
+        <is>
+          <t>Not located. cse.lk/api/chartData almost certainly does not expose it.</t>
+        </is>
+      </c>
+      <c r="F13" s="56" t="inlineStr">
+        <is>
+          <t>CSE, per counter.</t>
+        </is>
+      </c>
+      <c r="G13" s="56" t="inlineStr">
+        <is>
+          <t>Order-book microstructure.</t>
+        </is>
+      </c>
+      <c r="H13" s="56" t="inlineStr">
+        <is>
+          <t>Unknown.</t>
+        </is>
+      </c>
+      <c r="I13" s="56" t="inlineStr">
+        <is>
+          <t>Tick or message level.</t>
+        </is>
+      </c>
+      <c r="J13" s="56" t="inlineStr">
+        <is>
+          <t>Unknown.</t>
+        </is>
+      </c>
+      <c r="K13" s="56" t="inlineStr">
+        <is>
+          <t>Order arrival, market order and cancellation intensities by queue size, or at minimum multi-level depth snapshots.</t>
+        </is>
+      </c>
+      <c r="L13" s="56" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="M13" s="56" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N13" s="56" t="inlineStr">
+        <is>
+          <t>Not available through any identified route. Whether the CSE exposes anything below top-of-book is unknown.</t>
+        </is>
+      </c>
+      <c r="O13" s="56" t="inlineStr">
+        <is>
+          <t>Unconfirmed.</t>
+        </is>
+      </c>
+      <c r="P13" s="56" t="inlineStr">
+        <is>
+          <t>Assessed as almost certainly out of reach. The queue-reactive execution simulator in the literature needs order-level message data; the deep LOB model needs ten levels per side tick-by-tick plus roughly 7,192 GPU hours in its own evidentiary standard.</t>
+        </is>
+      </c>
+      <c r="Q13" s="56" t="inlineStr">
+        <is>
+          <t>Not obtained; judged unlikely.</t>
+        </is>
+      </c>
+      <c r="R13" s="56" t="inlineStr">
+        <is>
+          <t>A_L and the friction-aware evaluation layer, which are gated on exactly the same data and should therefore be one workstream and one request.</t>
+        </is>
+      </c>
+      <c r="S13" s="56" t="inlineStr">
+        <is>
+          <t>There is a decisive and nearly free fallback that runs FIRST: the tick-size classification needs only the best bid, the best ask and the exchange's tick schedule. If liquid CSE counters come out small-tick, the microstructural route is ruled out at almost no cost and the friction work becomes daily-bar-based by necessity rather than by preference.</t>
+        </is>
+      </c>
+      <c r="T13" s="56" t="inlineStr">
+        <is>
+          <t>If none of it is observable, A_L falls back to turnover, traded value, zero-return frequency and Amihud-style measures from daily bars, and the friction model falls back to a parametric temporary and permanent impact model calibrated against observed turnover and daily price moves. Weaker, but honest.</t>
+        </is>
+      </c>
+      <c r="U13" s="56" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V13" s="59" t="inlineStr">
+        <is>
+          <t>EVALUATE via the top-of-book tick test first</t>
+        </is>
+      </c>
+      <c r="W13" s="56" t="inlineStr">
+        <is>
+          <t>Fold the level-III feature list and the queue-intensity calibration data into the SAME written request rather than two, because whatever cannot be observed also cannot be simulated, and the depth of the request determines how strong both A_L and the evaluation layer can be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="232" customHeight="1">
+      <c r="A14" s="61" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+      <c r="B14" s="62" t="inlineStr">
+        <is>
+          <t>CSE per-security daily OHLCV, turnover and trade count (own extraction)</t>
+        </is>
+      </c>
+      <c r="C14" s="62" t="inlineStr">
         <is>
           <t>Price &amp; market data</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Stock Analysis (commercial, freemium)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>https://stockanalysis.com/list/colombo-stock-exchange/</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>CSE. 296 actively traded stocks. (Coincidentally the same count as P11's 2010-2021 sample of 296 CSE-listed firms - almost certainly a coincidence, but worth confirming the live universe independently rather than assuming.)</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Ticker universe reference. Tabular.</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Current snapshot; deeper history behind the paid tier.</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Daily.</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>296 tickers.</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Symbol, name, market cap in LKR, price, % change, revenue. Has a download button.</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>English company names.</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>Free web with download; deeper data behind Stock Analysis Pro.</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Commercial site, standard ToU. Fine for bootstrapping a symbol list, not for redistribution.</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>Snapshot only on the free tier - no historical series.</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>Universe construction for all four agents.</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>The best free confirmation of the complete CSE ticker universe I found. 296 names with market caps is exactly what I need to define the investable set.</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>Not a historical data source. Free tier is a snapshot.</t>
-        </is>
-      </c>
-      <c r="U4" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="V4" s="7" t="inlineStr">
-        <is>
-          <t>USE - universe bootstrap only</t>
-        </is>
-      </c>
-      <c r="W4" s="3" t="inlineStr">
-        <is>
-          <t>Use it to build and sanity-check the ticker list, then pull actual prices from D01. Cross-checking the universe against a second source matters because D01 is reverse-engineered and I have no schema guarantee.</t>
+      <c r="D14" s="62" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange public JSON API (D01), extracted by me</t>
+        </is>
+      </c>
+      <c r="E14" s="62" t="inlineStr">
+        <is>
+          <t>https://github.com/Shaahid02/fyp-dataset  ·  commit d4017b0780a79d58c09f6291af259970476c50f7</t>
+        </is>
+      </c>
+      <c r="F14" s="62" t="inlineStr">
+        <is>
+          <t>CSE, 323 securities. 283 ordinary (.N), 21 non-voting (.X), 2 preference (.P), 17 rights (.R).</t>
+        </is>
+      </c>
+      <c r="G14" s="62" t="inlineStr">
+        <is>
+          <t>THE PRIMARY DATASET FOR THIS PROJECT. Per-security daily time series.</t>
+        </is>
+      </c>
+      <c r="H14" s="62" t="inlineStr">
+        <is>
+          <t>2012-01-02 to 2026-10-02. 14.75 years.</t>
+        </is>
+      </c>
+      <c r="I14" s="62" t="inlineStr">
+        <is>
+          <t>Daily, per security.</t>
+        </is>
+      </c>
+      <c r="J14" s="62" t="inlineStr">
+        <is>
+          <t>323 securities, 829,070 security-day observations. Per-security trading days: min 6, 10th percentile 1,081, median 2,935, 90th percentile 3,484, max 3,510. 304 securities have 250+ days, 295 have 1,000+, 248 have 2,000+, 155 have 3,000+.</t>
+        </is>
+      </c>
+      <c r="K14" s="62" t="inlineStr">
+        <is>
+          <t>date, open, high, low, close, turnover, share_volume, trade_volume. OPEN IS PRESENT, which the 20 September audit had flagged as not universally available in the official CSE files and which the OHLC bid-ask estimator in D23 depends on. TURNOVER AND TRADE COUNT ARE PRESENT - both were recorded as missing before this extraction and are not.</t>
+        </is>
+      </c>
+      <c r="L14" s="62" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="M14" s="62" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N14" s="62" t="inlineStr">
+        <is>
+          <t>Python client over the CSE chartData endpoint, requesting 2012-01-01 to the run date for every symbol in the listed-company set, one CSV per security plus a per-run log. Last full run 2026-10-04 19:43-19:53, log 'fetch_20261004_194323.log': 323 saved, 0 no-data, 0 skipped, 0 failed. Reproducible from the committed code; the run log records per-security row counts and date ranges and is the extraction evidence.</t>
+        </is>
+      </c>
+      <c r="O14" s="62" t="inlineStr">
+        <is>
+          <t>UNCONFIRMED AND ON THE CRITICAL PATH. Taken from an undocumented CSE endpoint with no published terms, so the same open question as D01 - and it now applies to the project's primary dataset rather than to a candidate source. Resolve reuse and publication rights in the CSE request. Do not redistribute the extracted data until that is answered; the repository is the extraction record, not a licence to publish.</t>
+        </is>
+      </c>
+      <c r="P14" s="62" t="inlineStr">
+        <is>
+          <t>Not yet profiled per counter - that is D17, and it is the next task. Four issues already visible. (1) Coverage is extremely uneven: the median security has 2,935 trading days and the 10th percentile has 1,081, so '14.75 years' is the envelope and not what most counters carry. (2) The 17 .R securities are rights issues, not counters - 6 to 11 days each - and belong out of the universe, leaving 306. (3) 61 securities (18.9%) end before 2026-10-02, which is delistings, suspensions and dormancy mixed together and not yet separated. (4) At least one security (ASPM.N0000) prints a close outside its own high-low range, so a high &gt;= close &gt;= low validation must run before anything is trusted. Corporate-action and adjustment treatment is UNKNOWN - the endpoint does not state whether prices are adjusted for splits, bonus issues or dividends, and on a market with frequent bonus issues that must be established before returns are computed.</t>
+        </is>
+      </c>
+      <c r="Q14" s="62" t="inlineStr">
+        <is>
+          <t>VERIFIED BY EXTRACTION. Figures in this row are parsed from the committed run log and the files themselves, not from a README or a claim.</t>
+        </is>
+      </c>
+      <c r="R14" s="62" t="inlineStr">
+        <is>
+          <t>A_T and A_L primarily, A_V for per-counter volatility and persistence, and the friction-aware evaluation layer. Effectively the whole quantitative side of the framework.</t>
+        </is>
+      </c>
+      <c r="S14" s="62" t="inlineStr">
+        <is>
+          <t>This is the row that closes the dataset blocker rated 1.5 on 20 September. It is materially better than the figure carried in the Progress Update: 323 securities rather than 270, 14.75 years rather than 10, and it carries turnover and trade count, which were both recorded as missing. Turnover makes Amihud directly computable rather than proxied, so L_t is measurable today. It contains 61 series that stop early, so dead counters are present rather than filtered out - the thin part of the book Sub-gap 1 is about. At a 30-day lookback across the 248 securities with 2,000+ days this is on the order of 480,000 training sequences.</t>
+        </is>
+      </c>
+      <c r="T14" s="62" t="inlineStr">
+        <is>
+          <t>Licence unconfirmed, which is the single largest risk in this matrix because it attaches to the primary dataset. ADJUSTMENT STATUS CONFIRMED 18 OCTOBER 2026: THE SERIES IS NOT ADJUSTED FOR CORPORATE ACTIONS. JKH closes at 212.50 on 2024-10-28 and 21.20 on 2024-11-06, a share split rendered as a -90% return; AAF shows +767% in 2019. Do not compute returns from this row directly, use D26. No bid, ask or depth - that gap is unchanged and is what D23 and the CSE request address. Coverage is uneven enough that any claim stated per-counter must be stated per-tier after D17.</t>
+        </is>
+      </c>
+      <c r="U14" s="62" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V14" s="63" t="inlineStr">
+        <is>
+          <t>USE - this is the project's primary dataset</t>
+        </is>
+      </c>
+      <c r="W14" s="62" t="inlineStr">
+        <is>
+          <t>Replaces the planning assumptions this matrix was built on. It also reassigns the CSE request: turnover and trade count are no longer needed, so the request narrows to BID/ASK AND DEPTH, DATED LISTING AND DELISTING EVENTS, and WRITTEN CONFIRMATION OF REUSE AND PUBLICATION RIGHTS - the last being the item that now carries the most risk. Freeze this extraction as a versioned snapshot and quote the commit in the proposal, so the experimental universe is reproducible even if the endpoint changes or disappears.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="277.2" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>D04</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>TradingView CSELK</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>TradingView</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>https://www.tradingview.com/symbols/CSELK-ASI/</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>CSE. Index (CSELK:ASI) and individual equities under the CSELK: prefix - confirmed Dialog Axiata, John Keells Holdings, Commercial Bank of Ceylon, Ceylon Tobacco.</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Cross-check / manual reference. Charts.</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>At least 10 years at index level (5Y +137.95%, 10Y +228.44% both shown).</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Daily and intraday on the platform.</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Full CSE universe appears to be covered.</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Full OHLCV on the platform.</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>Free web and charting. No bulk export on the free tier; paid API otherwise.</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>ToU forbids scraping. Realistic use is manual or paid-API only.</t>
-        </is>
-      </c>
-      <c r="P5" s="5" t="inlineStr">
-        <is>
-          <t>No programmatic access without paying, so it can't be part of an automated pipeline.</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R5" s="5" t="inlineStr">
-        <is>
-          <t>Manual cross-check for A_T. Confirmed ten years of depth at index level.</t>
-        </is>
-      </c>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>Best third-party per-stock CSE coverage I confirmed, and useful for eyeballing whether D01's numbers look right.</t>
-        </is>
-      </c>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>Can't be automated on the free tier. Not a pipeline source.</t>
-        </is>
-      </c>
-      <c r="U5" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>REFERENCE ONLY</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr">
-        <is>
-          <t>Valuable as a sanity check against D01 - if my archived prices disagree with TradingView's chart I've got a bug. Not usable as an actual feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="409.6" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Trading Economics - Sri Lanka stock market</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Trading Economics</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>https://tradingeconomics.com/sri-lanka/stock-market</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>CSE All Share index only.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Long index history. Time series.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>1993 to 2026 - the longest verified index history of any source here. Base 100 = 1985. (The page also showed an all-time-high figure that doesn't reconcile with TradingView's 5Y/10Y percentages in D04, so one of the two is a different series or a mis-read. Check before quoting any level figure from either.)</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Daily.</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>~33 years of daily index values.</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Index level. No per-ticker data.</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>Free web charts; historical download and API require a paid subscription.</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>Copyright Trading Economics, all rights reserved. Paid tiers for any programmatic use.</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t>Index only, and the useful access is paywalled.</t>
-        </is>
-      </c>
-      <c r="Q6" s="3" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R6" s="3" t="inlineStr">
-        <is>
-          <t>A_V volatility and risk - long index history for the persistence estimates and regime splitting.</t>
-        </is>
-      </c>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <t>1993-2026 daily index history would comfortably support the walk-forward scheme and regime decomposition, which is exactly what D01's unknown depth might not.</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>Paywalled for download, and no per-ticker data so it can't feed the trader agent.</t>
-        </is>
-      </c>
-      <c r="U6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="V6" s="6" t="inlineStr">
-        <is>
-          <t>EVALUATE - fallback for index history</t>
-        </is>
-      </c>
-      <c r="W6" s="3" t="inlineStr">
-        <is>
-          <t>Worth pricing up if D01's chartData turns out to be shallow. The volatility work (G2) only needs index series, so this could rescue that half of the project even if per-ticker history is short.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="237.6" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>D06</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Investing.com CSE All-Share</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Investing.com</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.investing.com/indices/cse-all-share-historical-data</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>CSE All-Share index. Individual Sri Lankan equities effectively absent - the equities page rendered exactly one name (Cargills Bank).</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Index history. Tabular.</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Date-range picker available; depth not confirmed.</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Daily.</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Index only.</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>Daily open, high, low, close, volume and % change in LKR.</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>Free web with a download option.</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>ToU prohibits automated scraping and redistribution; downloads are for personal use.</t>
-        </is>
-      </c>
-      <c r="P7" s="5" t="inlineStr">
-        <is>
-          <t>Index-only coverage is the killer. One Sri Lankan equity listed.</t>
-        </is>
-      </c>
-      <c r="Q7" s="5" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R7" s="5" t="inlineStr">
-        <is>
-          <t>A_V, as a cross-check on the index series.</t>
-        </is>
-      </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>Gives proper OHLCV at index level, which D01 does not.</t>
-        </is>
-      </c>
-      <c r="T7" s="5" t="inlineStr">
-        <is>
-          <t>No per-ticker coverage, and scraping is prohibited.</t>
-        </is>
-      </c>
-      <c r="U7" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="V7" s="6" t="inlineStr">
-        <is>
-          <t>REFERENCE ONLY</t>
-        </is>
-      </c>
-      <c r="W7" s="5" t="inlineStr">
-        <is>
-          <t>Useful to validate index OHLCV against, nothing more. The single-equity coverage rules it out as a real source.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="330" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>CSE listed-company report PDFs</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Filings / fundamentals</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange CDN</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>https://cdn.cse.lk/cmt/upload_report_file/&lt;id&gt;_&lt;epoch_ms&gt;.pdf (discovered via the D01 announcement endpoints)</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>All ~280-300 CSE-listed companies. Annual and quarterly reports.</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>RAG corpus. PDF - text, tables and figures.</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Older filings thin, roughly pre-2015.</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Quarterly and annual.</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>Hundreds of companies x multiple filings per year.</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>N/A - this is the fundamentals side.</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>English. Full audited statements: P&amp;L and OCI, financial position, changes in equity, cash flows, notes, auditor's report.</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>None - unlabelled documents.</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>Free direct HTTP GET, no auth. But filenames are opaque id/timestamp pairs, so links have to be harvested from the announcement endpoints rather than enumerated.</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>UNCONFIRMED. I could not retrieve a cse.lk terms-of-use page. Treat CSE data reuse rights as unresolved and email CSE before publishing anything derived.</t>
-        </is>
-      </c>
-      <c r="P8" s="5" t="inlineStr">
-        <is>
-          <t>No XBRL, so nothing is machine-structured. Report layout varies considerably company to company. Older filings more likely to be scanned rather than text-native, which is exactly the OCR failure mode P07 warns breaks element-based chunking.</t>
-        </is>
-      </c>
-      <c r="Q8" s="5" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R8" s="5" t="inlineStr">
-        <is>
-          <t>A_F fundamental. After the September 2026 scope decision this is the framework's only text modality, so it carries the heterogeneity claim in the main gap.</t>
-        </is>
-      </c>
-      <c r="S8" s="5" t="inlineStr">
-        <is>
-          <t>The best-provisioned component of the whole project. Text-native full-statement PDFs for every listed company on an open CDN - I verified one end to end (Office Equipment PLC FY2025, full audited statements).</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Discovery is awkward, structure is inconsistent, and the licensing question is unresolved.</t>
-        </is>
-      </c>
-      <c r="U8" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="V8" s="7" t="inlineStr">
-        <is>
-          <t>USE - primary RAG corpus</t>
-        </is>
-      </c>
-      <c r="W8" s="5" t="inlineStr">
-        <is>
-          <t>This is what A_F is built on, and after the scope cut it is the framework's only text channel rather than a demoted system feature. Text-native PDFs mean element-based chunking has something real to work with. The architectural novelty is closed by the 2025 CSE Neo4j Graph-RAG work (Shamila, Silva and Talagala, ERU 2025, DOI 10.31705/ERU.2025.35), now verified, so what remains for A_F is numeric statement extraction, point-in-time correctness and the orchestration that consumes the signal. Every document needs a publication-date field and a retrieval filter keyed to the simulation clock, because their graph is a static snapshot with no as-of field and that is a lookahead hazard in a backtest rather than an inconvenience.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="171.6" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>D08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>CSE exchange annual reports</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Filings / fundamentals</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>https://cdn.cse.lk/pdf/annual-reports/Annual-Report-YYYY.pdf</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>The exchange itself, not listed companies.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Market context. PDF.</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>2020-2024 confirmed loading.</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Annual.</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>Five reports confirmed.</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>Market-level turnover and activity statistics.</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>English.</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>Free direct download.</t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>No explicit copyright notice in the documents I checked.</t>
-        </is>
-      </c>
-      <c r="P9" s="3" t="inlineStr">
-        <is>
-          <t>Exchange-level only - no company fundamentals.</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>None directly. Background for the Sub-gap 1 execution model, market structure and turnover context.</t>
-        </is>
-      </c>
-      <c r="S9" s="3" t="inlineStr">
-        <is>
-          <t>Useful for understanding CSE turnover patterns and market structure when I'm designing the simulated exchange.</t>
-        </is>
-      </c>
-      <c r="T9" s="3" t="inlineStr">
-        <is>
-          <t>Not a modelling input. Background reading.</t>
-        </is>
-      </c>
-      <c r="U9" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="V9" s="7" t="inlineStr">
-        <is>
-          <t>USE - background only</t>
-        </is>
-      </c>
-      <c r="W9" s="3" t="inlineStr">
-        <is>
-          <t>Worth reading for the microstructure and turnover context behind the execution model, but it doesn't feed any agent directly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="250.8" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>CBSL Economic Data Library</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Central Bank of Sri Lanka</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cbsl.lk/eresearch/</t>
-        </is>
-      </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t>Sri Lanka. Organised by real, monetary, external, financial and fiscal sector.</t>
-        </is>
-      </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>Macro time series. Structured, format unconfirmed.</t>
-        </is>
-      </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Not stated on the landing page.</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>Varies by series.</t>
-        </is>
-      </c>
-      <c r="J10" s="20" t="inlineStr">
-        <is>
-          <t>Not stated.</t>
-        </is>
-      </c>
-      <c r="K10" s="20" t="inlineStr">
-        <is>
-          <t>Financial sector section includes share-market data.</t>
-        </is>
-      </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>English.</t>
-        </is>
-      </c>
-      <c r="M10" s="20" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N10" s="20" t="inlineStr">
-        <is>
-          <t>Web portal. Download formats, registration requirement and API existence are all NOT stated - this needs evaluating hands-on.</t>
-        </is>
-      </c>
-      <c r="O10" s="20" t="inlineStr">
-        <is>
-          <t>Not stated.</t>
-        </is>
-      </c>
-      <c r="P10" s="20" t="inlineStr">
-        <is>
-          <t>Note the domain: cbsl.lk, not cbsl.gov.lk - the .gov.lk/eresearch path 404s. Everything about access format is unconfirmed.</t>
-        </is>
-      </c>
-      <c r="Q10" s="20" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R10" s="20" t="inlineStr">
-        <is>
-          <t>A_V, and the macro context for regime labelling.</t>
-        </is>
-      </c>
-      <c r="S10" s="20" t="inlineStr">
-        <is>
-          <t>If it offers structured downloads it's a much better route than parsing the PDF-only publications (D10 and D11).</t>
-        </is>
-      </c>
-      <c r="T10" s="20" t="inlineStr">
-        <is>
-          <t>Completely unconfirmed on the things that matter - format, API, registration.</t>
-        </is>
-      </c>
-      <c r="U10" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="V10" s="19" t="inlineStr">
-        <is>
-          <t>EVALUATE FIRST - this decides the macro ingestion design</t>
-        </is>
-      </c>
-      <c r="W10" s="20" t="inlineStr">
-        <is>
-          <t>Worth an hour before committing to a PDF-extraction pipeline, because if this portal exports CSV the macro problem gets much easier. Evaluate it ahead of D10 and D11, which are PDF-first. The CSE macro papers confirm the acquisition method is manual in practice, mostly Excel downloads with inflation data transcribed out of PDFs, and name the Department of Census and Statistics as the NCPI source alongside CBSL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="369.6" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>CBSL Rates and Indicators</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Central Bank of Sri Lanka</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.cbsl.gov.lk/en/rates-and-indicators</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Sri Lanka.</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Macro indicators. Web tables and PDFs.</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Continuous archives with year/month filters.</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>Daily, weekly and monthly depending on series.</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Multiple series.</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>English, Sinhala and Tamil for the Monthly Bulletin.</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>Free web. Navigate from the index page - constructed deep URLs (/interest-rates/t-bill-rates, /inflation, etc.) all 404.</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>cbsl.gov.lk/robots.txt sets Crawl-delay: 10 for all agents and explicitly disallows specific treasury-rate service endpoints - which directly touches what the risk agent would want. AhrefsBot fully blocked.</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t>Download formats not stated on the index pages. The treasury-endpoint disallow is a real constraint, not a formality.</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R11" s="3" t="inlineStr">
-        <is>
-          <t>A_V, plus the risk-free rate for Sharpe and excess-return calculations in the evaluation layer.</t>
-        </is>
-      </c>
-      <c r="S11" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed categories cover everything I need: CCPI and NCPI inflation, policy rates, exchange rates, SLIBOR, government securities (T-bill and T-bond yields), commercial bank lending and deposit rates, open market operations. P11 uses 91-day T-bill auction rates as the risk-free rate, and those live here.</t>
-        </is>
-      </c>
-      <c r="T11" s="3" t="inlineStr">
-        <is>
-          <t>Robots.txt disallows exactly the treasury-rate endpoints I'd most want to automate, and there's no API.</t>
-        </is>
-      </c>
-      <c r="U11" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="V11" s="7" t="inlineStr">
-        <is>
-          <t>USE - respect the crawl-delay and the disallow list</t>
-        </is>
-      </c>
-      <c r="W11" s="3" t="inlineStr">
-        <is>
-          <t>Non-negotiable for the risk-free rate and regime context. But the disallowed treasury endpoints mean I need to pull those figures from the published tables rather than the service endpoints, and honour the 10-second crawl delay.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="290.4" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>CBSL Weekly Economic Indicators &amp; inflation releases</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Central Bank of Sri Lanka</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cbsl.gov.lk/en/statistics/economic-indicators/weekly-indicators</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>Sri Lanka - real, monetary, fiscal and external sectors.</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
-        <is>
-          <t>Macro time series trapped in PDFs.</t>
-        </is>
-      </c>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>Continuous archive with year/month filters; latest seen 11 Sep 2026. Inflation releases visible Feb 2025 - Jul 2026 with deeper archive behind pagination.</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="inlineStr">
-        <is>
-          <t>Weekly for indicators, monthly for inflation.</t>
-        </is>
-      </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>Long archive.</t>
-        </is>
-      </c>
-      <c r="K12" s="20" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="L12" s="20" t="inlineStr">
-        <is>
-          <t>English.</t>
-        </is>
-      </c>
-      <c r="M12" s="20" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="N12" s="20" t="inlineStr">
-        <is>
-          <t>Free download.</t>
-        </is>
-      </c>
-      <c r="O12" s="20" t="inlineStr">
-        <is>
-          <t>Same robots.txt constraints as D10.</t>
-        </is>
-      </c>
-      <c r="P12" s="20" t="inlineStr">
-        <is>
-          <t>PDF only - no Excel or CSV offered. This is a real ingestion cost, not a minor inconvenience.</t>
-        </is>
-      </c>
-      <c r="Q12" s="20" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R12" s="20" t="inlineStr">
-        <is>
-          <t>A_V.</t>
-        </is>
-      </c>
-      <c r="S12" s="20" t="inlineStr">
-        <is>
-          <t>Comprehensive and current, with a long archive.</t>
-        </is>
-      </c>
-      <c r="T12" s="20" t="inlineStr">
-        <is>
-          <t>PDF-first means the risk agent needs a table-extraction pipeline before it can use any of it. Ironically I'd be doing the same structural PDF parsing here that G4 does for company filings.</t>
-        </is>
-      </c>
-      <c r="U12" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="V12" s="19" t="inlineStr">
-        <is>
-          <t>USE - but evaluate D09 first</t>
-        </is>
-      </c>
-      <c r="W12" s="20" t="inlineStr">
-        <is>
-          <t>If D09 or Lanka Data can supply the same series as structured data, take that route. If not, at least the table-extraction work overlaps with the fundamental agent's pipeline so it's not entirely duplicated effort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="250.8" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>D12</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>CSE announcements feed</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Disclosures</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Via the D01 POST API - 8 announcement categories</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>CSE. All listed companies.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Corporate disclosures. Structured JSON plus linked PDFs.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Not confirmed.</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Event-driven.</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>8 announcement endpoints. The ones I could name from the community API documentation are financial, circular, compliance, listings, buy-in board and directives - the remaining two need confirming by enumerating the endpoints directly.</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>English.</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Unlabelled.</t>
-        </is>
-      </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>Same POST API as D01. No RSS found.</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>Same unconfirmed CSE terms as D01 and D11.</t>
-        </is>
-      </c>
-      <c r="P13" s="3" t="inlineStr">
-        <is>
-          <t>Historical depth unconfirmed, same as everything else on the CSE API.</t>
-        </is>
-      </c>
-      <c r="Q13" s="3" t="inlineStr">
-        <is>
-          <t>Verified - fetched the endpoint or page myself</t>
-        </is>
-      </c>
-      <c r="R13" s="3" t="inlineStr">
-        <is>
-          <t>A_F. This is how the report PDFs in D07 are discovered, which is the whole reason it survives the scope cut.</t>
-        </is>
-      </c>
-      <c r="S13" s="3" t="inlineStr">
-        <is>
-          <t>Primary-source corporate disclosure, which is higher-signal and less ambiguous than news coverage of the same events. Also the discovery mechanism for D11.</t>
-        </is>
-      </c>
-      <c r="T13" s="3" t="inlineStr">
-        <is>
-          <t>Undocumented, and depth unknown.</t>
-        </is>
-      </c>
-      <c r="U13" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="V13" s="7" t="inlineStr">
-        <is>
-          <t>USE - primary disclosure feed</t>
-        </is>
-      </c>
-      <c r="W13" s="3" t="inlineStr">
-        <is>
-          <t>The only survivor of the news and social block, and it survives for a structural reason rather than a sentimental one: it is a primary disclosure feed, not commentary, and it is how the report PDFs in D07 are discovered. It also carries the timestamp that makes point-in-time retrieval possible - a document is only visible to A_F after the announcement datetime, which is what keeps the backtest free of lookahead. Treat it as metadata and routing for A_F, not as a text signal in its own right.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="409.2" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Chindara/cse - CSE market-cap daily archive + scraper</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>GitHub (community, user Chindara)</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/Chindara/cse</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>CSE. Every company returned by the list_by_market_cap endpoint - 306 distinct symbols across the archive, around 301 per trading day.</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Ready-made historical archive plus a working daily-archiver pattern. CSV and JSON.</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>2025-04-10 to 2026-09-18. 374 trading days, 112,722 records. Verified by parsing the committed CSV, not by trusting the README.</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>One end-of-day snapshot per symbol per trading day. GitHub Actions cron at 10:00 UTC (15:30 SLT), Mon-Fri.</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>112,722 rows. ~20 MB CSV, ~60 MB JSON. 18-19 columns.</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>high, low, price (last traded), change, percentageChange, quantity, sharevolume, tradevolume, turnover, marketCap, marketCapPercentage, issuedQTY, lastTradedTime. No open, so no true OHLCV. No adjusted close, no corporate-action adjustment, no bid-ask.</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>N/A. Company name and symbol only, English.</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr">
+    <row r="15" ht="451" customHeight="1">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="B15" s="65" t="inlineStr">
+        <is>
+          <t>Effective bid-ask spread estimated from OHLC (derived) - LAST RESORT, MAY NEVER BE COMPUTED</t>
+        </is>
+      </c>
+      <c r="C15" s="65" t="inlineStr">
+        <is>
+          <t>Derived dataset</t>
+        </is>
+      </c>
+      <c r="D15" s="65" t="inlineStr">
+        <is>
+          <t>Own computation over D22, following Ardia, Guidotti &amp; Kroencke, Journal of Financial Economics 2024</t>
+        </is>
+      </c>
+      <c r="E15" s="65" t="inlineStr">
+        <is>
+          <t>Grid #61 in the Research Papers Grid; reference implementations are public</t>
+        </is>
+      </c>
+      <c r="F15" s="65" t="inlineStr">
+        <is>
+          <t>CSE, every security in D22 that survives the D17 screen.</t>
+        </is>
+      </c>
+      <c r="G15" s="65" t="inlineStr">
+        <is>
+          <t>Derived per-security daily spread estimate. The Level A proxy route for Sub-gap 1.</t>
+        </is>
+      </c>
+      <c r="H15" s="65" t="inlineStr">
+        <is>
+          <t>Same span as D22: 2012-01-02 to 2026-10-02.</t>
+        </is>
+      </c>
+      <c r="I15" s="65" t="inlineStr">
+        <is>
+          <t>Daily, per security.</t>
+        </is>
+      </c>
+      <c r="J15" s="65" t="inlineStr">
+        <is>
+          <t>Not yet computed. Upper bound is the D22 panel.</t>
+        </is>
+      </c>
+      <c r="K15" s="65" t="inlineStr">
+        <is>
+          <t>Estimated effective spread per security-day, from open, high, low and close.</t>
+        </is>
+      </c>
+      <c r="L15" s="65" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>Free. git clone or raw CSV/JSON from GitHub. Scraper is Python 3.10 + requests + pandas, POSTing to https://www.cse.lk/api/list_by_market_cap - i.e. it is D01 with 17 months of history already collected.</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t>No LICENCE file. Public but unlicensed, so default copyright applies and there is no grant to reuse either the code or the collected data. The data itself is D01's, so CSE's terms bind it as well. Two permissions to chase, not one.</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
-          <t>Column drift is the serious one: the CSE API added a logo field at position 3 on 2025-12-19 without the CSV header being rewritten, so 58,345 of the 112,722 rows carry 19 fields against an 18-field header. sync_json_from_csv.py patches this on read; anything that reads the raw CSV naively mis-maps every column after position 3. Stray header rows appear mid-file. Illiquid counters come through with empty price and volume fields. The writer is append-only with no de-duplication, so a re-run on the same date double-writes. The 15:30 SLT snapshot is not a confirmed official close.</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="inlineStr">
-        <is>
-          <t>Verified - cloned the repo and parsed the full CSV myself</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>A_T and A_L. The confirmed per-counter archive and currently the single most important row in this sheet.</t>
-        </is>
-      </c>
-      <c r="S14" s="3" t="inlineStr">
-        <is>
-          <t>Seventeen months of already-collected daily CSE cross-section, free, and it directly attacks the biggest unknown in this matrix - D01's retention depth - without waiting. Per-day market cap and issued quantity are not available from any other source I checked. The Actions workflow is a working template for my own archiver.</t>
-        </is>
-      </c>
-      <c r="T14" s="3" t="inlineStr">
-        <is>
-          <t>Unlicensed. No open price, so still not OHLCV. Starts 2025-04-10, which is short for anything volatility- or regime-related. Depends on one individual continuing to run a cron job. The column-drift bug has to be handled explicitly on ingest or every downstream number is wrong.</t>
-        </is>
-      </c>
-      <c r="U14" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="V14" s="7" t="inlineStr">
-        <is>
-          <t>USE - historical backfill, after normalising the column drift</t>
-        </is>
-      </c>
-      <c r="W14" s="3" t="inlineStr">
-        <is>
-          <t>The only meaningfully long, already-collected CSE daily cross-section I have found, and it costs nothing to take. Ingest once, normalise the 18/19-column split, treat it as read-only backfill sitting behind my own archive rather than as a live feed. Licence has to be settled with the author before any of it appears in the dissertation, and the CSE terms question (D01) applies on top.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="409.2" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>D14</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>cse-historical-data-scraper (TradingView route)</t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>GitHub (own repo, Shaahid02)</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>https://github.com/Shaahid02/cse-historical-data-scraper</t>
-        </is>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>CSE via TradingView's CSELK exchange. Driven by a bundled universe file of 285 companies (id, name, symbol, securityId).</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t>Historical OHLCV extraction. Per-symbol CSV.</t>
-        </is>
-      </c>
-      <c r="H15" s="20" t="inlineStr">
-        <is>
-          <t>scraper.py requests n_bars=365 daily bars per symbol; alt_scraper.py takes an explicit from/to and was run from 2021-01-01. True depth is whatever TradingView holds for CSELK - D04 confirmed 10 years at index level, so per-ticker depth still needs probing symbol by symbol.</t>
-        </is>
-      </c>
-      <c r="I15" s="20" t="inlineStr">
-        <is>
-          <t>Daily bars (Interval.in_daily). tvDatafeed exposes intraday intervals too, so minute and hourly are reachable if ever needed.</t>
-        </is>
-      </c>
-      <c r="J15" s="20" t="inlineStr">
-        <is>
-          <t>Code only - company_training_data/ is gitignored, so the repo ships no data. A full run is 285 symbols x 365 bars, roughly 104k bars.</t>
-        </is>
-      </c>
-      <c r="K15" s="20" t="inlineStr">
-        <is>
-          <t>True OHLCV - open, high, low, close, volume. This is the only source in the matrix that yields a real open price. No turnover, no market cap, no bid-ask. Whether the bars are corporate-action adjusted is TradingView's business and is undocumented.</t>
-        </is>
-      </c>
-      <c r="L15" s="20" t="inlineStr">
-        <is>
-          <t>N/A.</t>
-        </is>
-      </c>
-      <c r="M15" s="20" t="inlineStr">
+      <c r="M15" s="65" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t>Two routes. scraper.py uses tvDatafeed (unofficial client) with a TradingView username and password - placeholders in the repo since the 30 Jan 2026 commit. alt_scraper.py calls the UDF endpoint https://tvc4.tradingview.com/history directly with a browser User-Agent and no auth at all. Flat 2-second sleep between symbols.</t>
-        </is>
-      </c>
-      <c r="O15" s="20" t="inlineStr">
-        <is>
-          <t>No LICENCE file. The bigger problem is upstream: D04 already records that TradingView's ToU forbids scraping, and tvDatafeed is an unofficial client. The code is mine; the data is not, and no route here has permission behind it.</t>
-        </is>
-      </c>
-      <c r="P15" s="20" t="inlineStr">
-        <is>
-          <t>The ToU exposure is the real gap, not the code quality. Unofficial endpoints can change or be blocked without notice. n_bars=365 is hardcoded in scraper.py. No retry, no resume and no rate-limit backoff beyond the flat sleep - a failed symbol is printed and skipped. The bundled universe file is a static 285-company snapshot that will drift from D01/D03. Nothing verifies that CSELK bars agree with CSE's official close.</t>
-        </is>
-      </c>
-      <c r="Q15" s="20" t="inlineStr">
-        <is>
-          <t>Verified - cloned and read the source; the extraction has not been re-run end to end since 30 January 2026</t>
-        </is>
-      </c>
-      <c r="R15" s="20" t="inlineStr">
-        <is>
-          <t>A_T. The OHLCV feed D01 cannot provide.</t>
-        </is>
-      </c>
-      <c r="S15" s="20" t="inlineStr">
-        <is>
-          <t>The only route in the matrix to true per-ticker OHLCV with an open price and multi-year depth for CSE. It is my own code, so it does not depend on a third party maintaining anything, and alt_scraper.py needs no TradingView account at all.</t>
-        </is>
-      </c>
-      <c r="T15" s="20" t="inlineStr">
-        <is>
-          <t>Legally the weakest source in the matrix. It ties a core feed to an unofficial endpoint and a ToU I would be breaching, which is not defensible in a methodology chapter as it stands. Fragile by construction.</t>
-        </is>
-      </c>
-      <c r="U15" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="V15" s="19" t="inlineStr">
-        <is>
-          <t>SUPERSEDED by D22 - keep only as a ToU-free fallback</t>
-        </is>
-      </c>
-      <c r="W15" s="20" t="inlineStr">
-        <is>
-          <t>Superseded. The same OHLCV is now held from the CSE's own API (D22) with a longer span, more securities and turnover and trade-count fields this route never provided. That also removes the TradingView terms-of-use exposure from the critical path, which was this row's main risk. Keep the scraper as a fallback and as an independent cross-check on a sample of counters, and keep it out of the published pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="409.6" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>D15</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>CSE Price Index / ASPI ten-year daily series</t>
-        </is>
-      </c>
-      <c r="C16" s="22" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D16" s="22" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange official database</t>
-        </is>
-      </c>
-      <c r="E16" s="22" t="inlineStr">
-        <is>
-          <t>Via CSE directly; published route evidenced by the 2026 ARIMA study in the Literature Survey sheet</t>
-        </is>
-      </c>
-      <c r="F16" s="22" t="inlineStr">
-        <is>
-          <t>CSE, index level only.</t>
-        </is>
-      </c>
-      <c r="G16" s="22" t="inlineStr">
-        <is>
-          <t>Long index history. Time series.</t>
-        </is>
-      </c>
-      <c r="H16" s="22" t="inlineStr">
-        <is>
-          <t>OBTAINED 5 October 2026: 2012-01-02 to 2026-10-02.</t>
-        </is>
-      </c>
-      <c r="I16" s="22" t="inlineStr">
-        <is>
-          <t>Daily.</t>
-        </is>
-      </c>
-      <c r="J16" s="22" t="inlineStr">
-        <is>
-          <t>3,468 daily observations.</t>
-        </is>
-      </c>
-      <c r="K16" s="22" t="inlineStr">
-        <is>
-          <t>Traded Date and index Value (close) only. No index OHLC, no volume.</t>
-        </is>
-      </c>
-      <c r="L16" s="22" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="M16" s="22" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="N16" s="22" t="inlineStr">
-        <is>
-          <t>Downloaded from the CSE site as 'Historical-Values-data-2026-10-05 (ASPI).csv'. S&amp;P SL20 obtained the same way on 2026-10-04. A separate 'Trading days.csv' gives the exchange calendar, which is what distinguishes a non-trading day from a zero-volume day everywhere else in this matrix.</t>
-        </is>
-      </c>
-      <c r="O16" s="22" t="inlineStr">
-        <is>
-          <t>Not stated in the source study. CSE data-reuse terms remain unconfirmed and should be resolved in the same written request as everything else.</t>
-        </is>
-      </c>
-      <c r="P16" s="22" t="inlineStr">
-        <is>
-          <t>Close only, so index-level Parkinson and Garman-Klass estimators cannot be computed from this file - V_t at index level is limited to close-to-close unless index OHLC is obtained separately. Rows are in descending date order with dates as '2 OCT 2026', so both need normalising on load.</t>
-        </is>
-      </c>
-      <c r="Q16" s="22" t="inlineStr">
-        <is>
-          <t>Obtained and held locally. Supersedes the second-hand 1 Jul 2014 - 30 Jun 2024 span previously recorded from a published study: the held series is longer at both ends.</t>
-        </is>
-      </c>
-      <c r="R16" s="22" t="inlineStr">
-        <is>
-          <t>A_V above all. Also the baselines and the regime-split reporting in the evaluation layer.</t>
-        </is>
-      </c>
-      <c r="S16" s="22" t="inlineStr">
-        <is>
-          <t>THE INDEX TRACK IS SECURE. Roughly 2,400 daily observations is in the same range as the 2,922 the CSE FIGARCH study used, so Sub-gap 2's persistence estimator can be fitted even if per-counter depth never improves. Three distinct regime episodes for labelling.</t>
-        </is>
-      </c>
-      <c r="T16" s="22" t="inlineStr">
-        <is>
-          <t>Index only. Per-regime it splits to roughly 1,500 / 500 / 600 observations, so the COVID window is thin for a fractional differencing estimate even though it is an order of magnitude past the four-month failure case in the literature.</t>
-        </is>
-      </c>
-      <c r="U16" s="22" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="V16" s="22" t="inlineStr">
-        <is>
-          <t>USE - obtained, and longer than the published span</t>
-        </is>
-      </c>
-      <c r="W16" s="22" t="inlineStr">
-        <is>
-          <t>This is the row that de-risks Sub-gap 2. The persistence work does not wait on the per-counter data request. Ask for it by name rather than asking for 'ten years of data', because an index series would satisfy that phrasing and leave A_T, A_L and the friction model no better off.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="409.6" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>D16</t>
-        </is>
-      </c>
-      <c r="B17" s="22" t="inlineStr">
-        <is>
-          <t>Listing and delisting register with effective dates</t>
-        </is>
-      </c>
-      <c r="C17" s="22" t="inlineStr">
-        <is>
-          <t>Reference data</t>
-        </is>
-      </c>
-      <c r="D17" s="22" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange</t>
-        </is>
-      </c>
-      <c r="E17" s="22" t="inlineStr">
-        <is>
-          <t>Not located. Part of the CSE R&amp;D request.</t>
-        </is>
-      </c>
-      <c r="F17" s="22" t="inlineStr">
-        <is>
-          <t>CSE, all counters including those no longer listed.</t>
-        </is>
-      </c>
-      <c r="G17" s="22" t="inlineStr">
-        <is>
-          <t>Tradability mask. Reference table.</t>
-        </is>
-      </c>
-      <c r="H17" s="22" t="inlineStr">
-        <is>
-          <t>Snapshot as at 31 January 2024.</t>
-        </is>
-      </c>
-      <c r="I17" s="22" t="inlineStr">
-        <is>
-          <t>Event-level.</t>
-        </is>
-      </c>
-      <c r="J17" s="22" t="inlineStr">
-        <is>
-          <t>119 delisted companies.</t>
-        </is>
-      </c>
-      <c r="K17" s="22" t="inlineStr">
-        <is>
-          <t>None directly - this is the mask applied to the price data.</t>
-        </is>
-      </c>
-      <c r="L17" s="22" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="M17" s="22" t="inlineStr">
-        <is>
-          <t>Listing date, delisting date, and reason where available.</t>
-        </is>
-      </c>
-      <c r="N17" s="22" t="inlineStr">
-        <is>
-          <t>PARTIALLY OBTAINED. 'DE-LISTED-COMPANIES-31-01-2024.xlsx' is held, giving company code and company name for 119 delisted companies.</t>
-        </is>
-      </c>
-      <c r="O17" s="22" t="inlineStr">
-        <is>
-          <t>Unconfirmed.</t>
-        </is>
-      </c>
-      <c r="P17" s="22" t="inlineStr">
-        <is>
-          <t>Two gaps, and the first is the one that matters. (1) NO DELISTING DATES - the file is a list of names, so it supports a static exclusion but not a point-in-time tradability mask, and a static exclusion is the survivorship bias it was meant to fix. (2) The snapshot stops at 31 Jan 2024, so anything delisted since is missing. Separately, D22 already contains 61 securities whose history ends before the last trading day, which is an empirical lower bound on delistings and suspensions across the sample and can be cross-referenced against this list.</t>
-        </is>
-      </c>
-      <c r="Q17" s="22" t="inlineStr">
-        <is>
-          <t>Partially obtained - the list exists, the dates do not.</t>
-        </is>
-      </c>
-      <c r="R17" s="22" t="inlineStr">
-        <is>
-          <t>All four agents, via the universe definition, plus the evaluation layer.</t>
-        </is>
-      </c>
-      <c r="S17" s="22" t="inlineStr">
-        <is>
-          <t>A counter should leave the investable universe on the day it delisted, not retrospectively for the whole sample. This is the tradability-mask correction that the diversified-portfolio framework in the Literature Survey sheet builds explicitly from membership history, and whose absence is flagged there as a possible thirty-year survivorship filter in a comparable study.</t>
-        </is>
-      </c>
-      <c r="T17" s="22" t="inlineStr">
-        <is>
-          <t>May be unobtainable. The counters that delisted through the 2022 default and currency collapse are disproportionately the ones that failed, and they are also disproportionately thin - which is exactly the part of the book Sub-gap 1 is about, so excluding them removes the phenomenon under study.</t>
-        </is>
-      </c>
-      <c r="U17" s="22" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="V17" s="22" t="inlineStr">
-        <is>
-          <t>PARTIALLY OBTAINED - still ask the CSE for dated listing and delisting events</t>
-        </is>
-      </c>
-      <c r="W17" s="22" t="inlineStr">
-        <is>
-          <t>The names alone quantify how much of the universe is missing, which is already more than most projects on this market can state. What they do not support is a counter leaving the investable universe on the day it actually delisted. Ask the CSE specifically for EFFECTIVE DATES rather than for a delisting list, because the list is already held and asking for it again wastes the request. If dates cannot be obtained, use the D22 series-end dates as a proxy, state plainly that they are a proxy, and report the residual bias and its direction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="409.6" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>D17</t>
-        </is>
-      </c>
-      <c r="B18" s="22" t="inlineStr">
-        <is>
-          <t>Counter liquidity screen and tier table</t>
-        </is>
-      </c>
-      <c r="C18" s="22" t="inlineStr">
-        <is>
-          <t>Derived dataset</t>
-        </is>
-      </c>
-      <c r="D18" s="22" t="inlineStr">
-        <is>
-          <t>Own computation over D22</t>
-        </is>
-      </c>
-      <c r="E18" s="22" t="inlineStr">
-        <is>
-          <t>Derived from the D22 archive</t>
-        </is>
-      </c>
-      <c r="F18" s="22" t="inlineStr">
-        <is>
-          <t>CSE, all counters present in the archive.</t>
-        </is>
-      </c>
-      <c r="G18" s="22" t="inlineStr">
-        <is>
-          <t>Derived reference table sizing every downstream component.</t>
-        </is>
-      </c>
-      <c r="H18" s="22" t="inlineStr">
-        <is>
-          <t>The D22 span, 2025-04-10 to 2026-09-18.</t>
-        </is>
-      </c>
-      <c r="I18" s="22" t="inlineStr">
-        <is>
-          <t>Per counter.</t>
-        </is>
-      </c>
-      <c r="J18" s="22" t="inlineStr">
-        <is>
-          <t>323 securities x 829,070 observations available to screen, from D22.</t>
-        </is>
-      </c>
-      <c r="K18" s="22" t="inlineStr">
-        <is>
-          <t>Per counter from D22: share of trading days with non-zero volume, median and mean share_volume, median turnover, zero-return frequency reported separately from non-trading, Amihud mean of |return| over turnover, history length and missing-day count. Turnover and trade_volume are both present in D22, so Amihud is computable directly rather than proxied.</t>
-        </is>
-      </c>
-      <c r="L18" s="22" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="M18" s="22" t="inlineStr">
-        <is>
-          <t>Liquidity tier per counter.</t>
-        </is>
-      </c>
-      <c r="N18" s="22" t="inlineStr">
-        <is>
-          <t>One pass over data already held. No external dependency, no permission required.</t>
-        </is>
-      </c>
-      <c r="O18" s="22" t="inlineStr">
-        <is>
-          <t>n/a - derived.</t>
-        </is>
-      </c>
-      <c r="P18" s="22" t="inlineStr">
-        <is>
-          <t>A genuine flat print and a stale carry-forward both read as a zero return in a close-only series, so the screen must test volume rather than price change; the D15 exchange calendar is what separates a non-trading day from a zero-volume one. Liquidity regimes also shift across a 14.75-year span, so a screen fitted once is not valid throughout and must be re-run inside each training fold. Note that D22 carries a real example of the defect this guards against: ASPM.N0000 prints a close of 56.8 on days whose open, high and low are all 71.0, so close sits outside the high-low range.</t>
-        </is>
-      </c>
-      <c r="Q18" s="22" t="inlineStr">
-        <is>
-          <t>Not yet computed.</t>
-        </is>
-      </c>
-      <c r="R18" s="22" t="inlineStr">
-        <is>
-          <t>Sizes A_T, calibrates A_L, and sets the friction model's scale. Also the first empirical fit of the L_t conditioning variable.</t>
-        </is>
-      </c>
-      <c r="S18" s="22" t="inlineStr">
-        <is>
-          <t>The cheapest high-value computation available and it needs nothing that is not already held. It answers the question the cross-sectional reframe actually turns on, which is how many counters clear a liquidity screen rather than how many years of history exist. It is also a publishable CSE liquidity statistic in its own right.</t>
-        </is>
-      </c>
-      <c r="T18" s="22" t="inlineStr">
-        <is>
-          <t>Do not reduce it to a single threshold. Screening for liquid counters removes the thin-book conditions Sub-gap 1 is about, so report results BY TIER and let the cutoff become a result rather than a choice. That also aligns with the CSE finding that small caps are more exposed to illiquidity shocks than large, at -0.071 against -0.060.</t>
-        </is>
-      </c>
-      <c r="U18" s="22" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="V18" s="22" t="inlineStr">
-        <is>
-          <t>COMPUTE NEXT - no external dependency, and it now has 14.75 years to screen</t>
-        </is>
-      </c>
-      <c r="W18" s="22" t="inlineStr">
-        <is>
-          <t>At a 30-day lookback the D22 archive gives roughly 345 usable windows per counter, so with ~300 counters the sequence count is around 100,000, materially better than the earlier ~240-day working assumption. The tier table converts that headline into a per-tier figure, which is what actually sizes the model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="409.6" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>D18</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>University of Moratuwa CSE Graph-RAG corpus and code</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Filings / fundamentals</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>Shamila, Silva and Talagala, Dept of Computer Science and Engineering, University of Moratuwa</t>
-        </is>
-      </c>
-      <c r="E19" s="15" t="inlineStr">
-        <is>
-          <t>DOI 10.31705/ERU.2025.35, with a public GitHub repository linked from the paper</t>
-        </is>
-      </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>CSE annual reports. Company count and date range not reported.</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Prior art for A_F, plus a data-access lead.</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>Not reported in the paper.</t>
-        </is>
-      </c>
-      <c r="I19" s="15" t="inlineStr">
-        <is>
-          <t>Document level.</t>
-        </is>
-      </c>
-      <c r="J19" s="15" t="inlineStr">
-        <is>
-          <t>Over 6,000 unique entities reported, against roughly 280 listed companies.</t>
-        </is>
-      </c>
-      <c r="K19" s="15" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="L19" s="15" t="inlineStr">
-        <is>
-          <t>English. CSE annual report PDFs.</t>
-        </is>
-      </c>
-      <c r="M19" s="15" t="inlineStr">
-        <is>
-          <t>A Neo4j knowledge graph of corporate structure, governance and ownership. Tabular financial data is explicitly out of scope in their work.</t>
-        </is>
-      </c>
-      <c r="N19" s="15" t="inlineStr">
-        <is>
-          <t>Public repository. The authors are at the same university and are reachable.</t>
-        </is>
-      </c>
-      <c r="O19" s="15" t="inlineStr">
-        <is>
-          <t>Not stated.</t>
-        </is>
-      </c>
-      <c r="P19" s="15" t="inlineStr">
-        <is>
-          <t>The paper gives NO information on how the CSE documents were obtained, how many companies, or what date range - which is the single most useful thing it could have reported for my purposes.</t>
-        </is>
-      </c>
-      <c r="Q19" s="15" t="inlineStr">
-        <is>
-          <t>Verified. Two-page extended abstract, ERU Symposium 2025.</t>
-        </is>
-      </c>
-      <c r="R19" s="15" t="inlineStr">
-        <is>
-          <t>A_F, as prior art and as adoptable tooling.</t>
-        </is>
-      </c>
-      <c r="S19" s="15" t="inlineStr">
-        <is>
-          <t>Closes the architectural novelty of structure-aware retrieval over CSE annual reports, which is settled and not recoverable. More useful to me now as a data-access lead: same department, same university, reachable, with working extraction code.</t>
-        </is>
-      </c>
-      <c r="T19" s="15" t="inlineStr">
-        <is>
-          <t>A two-page abstract, so the pipeline constants are adoptable as defaults but not as validated settings. Their graph is a static snapshot with no as-of field.</t>
-        </is>
-      </c>
-      <c r="U19" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="V19" s="15" t="inlineStr">
-        <is>
-          <t>USE as prior art and as tooling; CONTACT the authors</t>
-        </is>
-      </c>
-      <c r="W19" s="15" t="inlineStr">
-        <is>
-          <t>The best warm route to the CSE data-access question. A local research group that already extracted CSE annual reports at scale knows how they got them, and that is worth an email before the formal R&amp;D request rather than after.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="409.6" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>D19</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>FinQA</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Benchmark</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>Chen et al., EMNLP 2021</t>
-        </is>
-      </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>https://github.com/czyssrs/FinQA</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>US filings, English.</t>
-        </is>
-      </c>
-      <c r="G20" s="15" t="inlineStr">
-        <is>
-          <t>Development artefact for A_F. Tables plus text.</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>n/a.</t>
-        </is>
-      </c>
-      <c r="I20" s="15" t="inlineStr">
-        <is>
-          <t>Question level.</t>
-        </is>
-      </c>
-      <c r="J20" s="15" t="inlineStr">
-        <is>
-          <t>Built over FinTabNet.</t>
-        </is>
-      </c>
-      <c r="K20" s="15" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="L20" s="15" t="inlineStr">
-        <is>
-          <t>English.</t>
-        </is>
-      </c>
-      <c r="M20" s="15" t="inlineStr">
-        <is>
-          <t>Question, answer, and an executable reasoning program.</t>
-        </is>
-      </c>
-      <c r="N20" s="15" t="inlineStr">
-        <is>
-          <t>Public GitHub.</t>
-        </is>
-      </c>
-      <c r="O20" s="15" t="inlineStr">
-        <is>
-          <t>CDLA-Permissive via FinTabNet. The cleanest licence of the A_F development set.</t>
-        </is>
-      </c>
-      <c r="P20" s="15" t="inlineStr">
-        <is>
-          <t>US filings with page-local, pre-located context and no as-of notion, so it does not transfer to CSE documents as data.</t>
-        </is>
-      </c>
-      <c r="Q20" s="15" t="inlineStr">
-        <is>
-          <t>Verified.</t>
-        </is>
-      </c>
-      <c r="R20" s="15" t="inlineStr">
-        <is>
-          <t>A_F, development and the C_F,t confidence signal.</t>
-        </is>
-      </c>
-      <c r="S20" s="15" t="inlineStr">
-        <is>
-          <t>Pull the DSL and the program executor directly rather than reimplement. Supplies the retrieve-then-program architecture and, importantly, a structural confidence signal for A_F: whether the program parses under the grammar, whether every argument traces to a retrieved number, and program step count as a calibrated difficulty proxy at 67.61 / 59.08 / 22.78 per cent for one, two and three-plus steps.</t>
-        </is>
-      </c>
-      <c r="T20" s="15" t="inlineStr">
-        <is>
-          <t>Not usable as a CSE evaluation set. Its 61.24 / 91.16 difficulty prior is explicitly non-portable and should be cited as an order of magnitude, never as a target.</t>
-        </is>
-      </c>
-      <c r="U20" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="V20" s="15" t="inlineStr">
-        <is>
-          <t>USE - A_F development only</t>
-        </is>
-      </c>
-      <c r="W20" s="15" t="inlineStr">
-        <is>
-          <t>The planning band agreed across three independent papers is below 50% on computed quantities over CSE filings, nearer 40% than 60% on first build. A_F is expected to be unusable more often than not, and the orchestrator has to be designed for a channel that is frequently unusable rather than occasionally imperfect.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="409.6" customHeight="1">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>D20</t>
-        </is>
-      </c>
-      <c r="B21" s="22" t="inlineStr">
-        <is>
-          <t>ConvFinQA and TAT-QA</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>Benchmark</t>
-        </is>
-      </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Chen et al., EMNLP 2022; Zhu et al., ACL-IJCNLP 2021</t>
-        </is>
-      </c>
-      <c r="E21" s="22" t="inlineStr">
-        <is>
-          <t>https://github.com/czyssrs/ConvFinQA and https://nextplusplus.github.io/TAT-QA</t>
-        </is>
-      </c>
-      <c r="F21" s="22" t="inlineStr">
-        <is>
-          <t>US filings, English.</t>
-        </is>
-      </c>
-      <c r="G21" s="22" t="inlineStr">
-        <is>
-          <t>Development artefacts and taxonomy for A_F.</t>
-        </is>
-      </c>
-      <c r="H21" s="22" t="inlineStr">
-        <is>
-          <t>n/a.</t>
-        </is>
-      </c>
-      <c r="I21" s="22" t="inlineStr">
-        <is>
-          <t>Question level.</t>
-        </is>
-      </c>
-      <c r="J21" s="22" t="inlineStr">
-        <is>
-          <t>ConvFinQA: 3,037 / 421 / 434 conversations. TAT-QA: hybrid table-and-text questions.</t>
-        </is>
-      </c>
-      <c r="K21" s="22" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="L21" s="22" t="inlineStr">
-        <is>
-          <t>English.</t>
-        </is>
-      </c>
-      <c r="M21" s="22" t="inlineStr">
-        <is>
-          <t>ConvFinQA adds multi-turn context; TAT-QA adds a scale taxonomy of None / Thousand / Million / Billion / Percent and an answer-type by answer-source split.</t>
-        </is>
-      </c>
-      <c r="N21" s="22" t="inlineStr">
-        <is>
-          <t>Public.</t>
-        </is>
-      </c>
-      <c r="O21" s="22" t="inlineStr">
-        <is>
-          <t>ConvFinQA inherits FinTabNet. TAT-QA is public for NON-COMMERCIAL USE ONLY - the one explicit restriction in the A_F set.</t>
-        </is>
-      </c>
-      <c r="P21" s="22" t="inlineStr">
-        <is>
-          <t>Same non-transferability as D19.</t>
-        </is>
-      </c>
-      <c r="Q21" s="22" t="inlineStr">
-        <is>
-          <t>Verified.</t>
-        </is>
-      </c>
-      <c r="R21" s="22" t="inlineStr">
-        <is>
-          <t>A_F, probe-set design and taxonomy.</t>
-        </is>
-      </c>
-      <c r="S21" s="22" t="inlineStr">
-        <is>
-          <t>ConvFinQA pairs with FinQA as one probe corpus with and without conversational context, which is the cheapest available ablation on whether a reference-resolution layer does anything. TAT-QA's scale taxonomy and two-round validation pattern lift directly into the CSE probe-set design and are affordable at ten to twenty questions.</t>
-        </is>
-      </c>
-      <c r="T21" s="22" t="inlineStr">
-        <is>
-          <t>Neither is a CSE evaluation set. TAT-QA's operator accuracy runs from 100.0 down to 0.0 across classes, so a single posterior is not comparable across classes without per-operator reliability estimated on my own probe set.</t>
-        </is>
-      </c>
-      <c r="U21" s="22" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="V21" s="22" t="inlineStr">
-        <is>
-          <t>USE - taxonomy and probe design</t>
-        </is>
-      </c>
-      <c r="W21" s="22" t="inlineStr">
-        <is>
-          <t>The convergent conclusion across the benchmark papers is the same: build a hand-checked probe set of ten to twenty questions over a handful of CSE annual reports, stratified by reasoning type and answer source, scored on the four-state taxonomy of correct, incorrect, failure-to-answer and no parseable answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="409.6" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>D21</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Level-III message data and multi-level depth for CSE</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Microstructure</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>Not located. cse.lk/api/chartData almost certainly does not expose it.</t>
-        </is>
-      </c>
-      <c r="F22" s="15" t="inlineStr">
-        <is>
-          <t>CSE, per counter.</t>
-        </is>
-      </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>Order-book microstructure.</t>
-        </is>
-      </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>Unknown.</t>
-        </is>
-      </c>
-      <c r="I22" s="15" t="inlineStr">
-        <is>
-          <t>Tick or message level.</t>
-        </is>
-      </c>
-      <c r="J22" s="15" t="inlineStr">
-        <is>
-          <t>Unknown.</t>
-        </is>
-      </c>
-      <c r="K22" s="15" t="inlineStr">
-        <is>
-          <t>Order arrival, market order and cancellation intensities by queue size, or at minimum multi-level depth snapshots.</t>
-        </is>
-      </c>
-      <c r="L22" s="15" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="M22" s="15" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="N22" s="15" t="inlineStr">
-        <is>
-          <t>Not available through any identified route. Whether the CSE exposes anything below top-of-book is unknown.</t>
-        </is>
-      </c>
-      <c r="O22" s="15" t="inlineStr">
-        <is>
-          <t>Unconfirmed.</t>
-        </is>
-      </c>
-      <c r="P22" s="15" t="inlineStr">
-        <is>
-          <t>Assessed as almost certainly out of reach. The queue-reactive execution simulator in the literature needs order-level message data; the deep LOB model needs ten levels per side tick-by-tick plus roughly 7,192 GPU hours in its own evidentiary standard.</t>
-        </is>
-      </c>
-      <c r="Q22" s="15" t="inlineStr">
-        <is>
-          <t>Not obtained; judged unlikely.</t>
-        </is>
-      </c>
-      <c r="R22" s="15" t="inlineStr">
-        <is>
-          <t>A_L and the friction-aware evaluation layer, which are gated on exactly the same data and should therefore be one workstream and one request.</t>
-        </is>
-      </c>
-      <c r="S22" s="15" t="inlineStr">
-        <is>
-          <t>There is a decisive and nearly free fallback that runs FIRST: the tick-size classification needs only the best bid, the best ask and the exchange's tick schedule. If liquid CSE counters come out small-tick, the microstructural route is ruled out at almost no cost and the friction work becomes daily-bar-based by necessity rather than by preference.</t>
-        </is>
-      </c>
-      <c r="T22" s="15" t="inlineStr">
-        <is>
-          <t>If none of it is observable, A_L falls back to turnover, traded value, zero-return frequency and Amihud-style measures from daily bars, and the friction model falls back to a parametric temporary and permanent impact model calibrated against observed turnover and daily price moves. Weaker, but honest.</t>
-        </is>
-      </c>
-      <c r="U22" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V22" s="15" t="inlineStr">
-        <is>
-          <t>EVALUATE via the top-of-book tick test first</t>
-        </is>
-      </c>
-      <c r="W22" s="15" t="inlineStr">
-        <is>
-          <t>Fold the level-III feature list and the queue-intensity calibration data into the SAME written request rather than two, because whatever cannot be observed also cannot be simulated, and the depth of the request determines how strong both A_L and the evaluation layer can be.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="409.6" customHeight="1">
-      <c r="A23" s="23" t="inlineStr">
-        <is>
-          <t>D22</t>
-        </is>
-      </c>
-      <c r="B23" s="24" t="inlineStr">
-        <is>
-          <t>CSE per-security daily OHLCV, turnover and trade count (own extraction)</t>
-        </is>
-      </c>
-      <c r="C23" s="24" t="inlineStr">
-        <is>
-          <t>Price &amp; market data</t>
-        </is>
-      </c>
-      <c r="D23" s="24" t="inlineStr">
-        <is>
-          <t>Colombo Stock Exchange public JSON API (D01), extracted by me</t>
-        </is>
-      </c>
-      <c r="E23" s="24" t="inlineStr">
-        <is>
-          <t>https://github.com/Shaahid02/fyp-dataset  ·  commit d4017b0780a79d58c09f6291af259970476c50f7</t>
-        </is>
-      </c>
-      <c r="F23" s="24" t="inlineStr">
-        <is>
-          <t>CSE, 323 securities. 283 ordinary (.N), 21 non-voting (.X), 2 preference (.P), 17 rights (.R).</t>
-        </is>
-      </c>
-      <c r="G23" s="24" t="inlineStr">
-        <is>
-          <t>THE PRIMARY DATASET FOR THIS PROJECT. Per-security daily time series.</t>
-        </is>
-      </c>
-      <c r="H23" s="24" t="inlineStr">
-        <is>
-          <t>2012-01-02 to 2026-10-02. 14.75 years.</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>Daily, per security.</t>
-        </is>
-      </c>
-      <c r="J23" s="24" t="inlineStr">
-        <is>
-          <t>323 securities, 829,070 security-day observations. Per-security trading days: min 6, 10th percentile 1,081, median 2,935, 90th percentile 3,484, max 3,510. 304 securities have 250+ days, 295 have 1,000+, 248 have 2,000+, 155 have 3,000+.</t>
-        </is>
-      </c>
-      <c r="K23" s="24" t="inlineStr">
-        <is>
-          <t>date, open, high, low, close, turnover, share_volume, trade_volume. OPEN IS PRESENT, which the 20 September audit had flagged as not universally available in the official CSE files and which the OHLC bid-ask estimator in D23 depends on. TURNOVER AND TRADE COUNT ARE PRESENT - both were recorded as missing before this extraction and are not.</t>
-        </is>
-      </c>
-      <c r="L23" s="24" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="M23" s="24" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="N23" s="24" t="inlineStr">
-        <is>
-          <t>Python client over the CSE chartData endpoint, requesting 2012-01-01 to the run date for every symbol in the listed-company set, one CSV per security plus a per-run log. Last full run 2026-10-04 19:43-19:53, log 'fetch_20261004_194323.log': 323 saved, 0 no-data, 0 skipped, 0 failed. Reproducible from the committed code; the run log records per-security row counts and date ranges and is the extraction evidence.</t>
-        </is>
-      </c>
-      <c r="O23" s="24" t="inlineStr">
-        <is>
-          <t>UNCONFIRMED AND ON THE CRITICAL PATH. Taken from an undocumented CSE endpoint with no published terms, so the same open question as D01 - and it now applies to the project's primary dataset rather than to a candidate source. Resolve reuse and publication rights in the CSE request. Do not redistribute the extracted data until that is answered; the repository is the extraction record, not a licence to publish.</t>
-        </is>
-      </c>
-      <c r="P23" s="24" t="inlineStr">
-        <is>
-          <t>Not yet profiled per counter - that is D17, and it is the next task. Four issues already visible. (1) Coverage is extremely uneven: the median security has 2,935 trading days and the 10th percentile has 1,081, so '14.75 years' is the envelope and not what most counters carry. (2) The 17 .R securities are rights issues, not counters - 6 to 11 days each - and belong out of the universe, leaving 306. (3) 61 securities (18.9%) end before 2026-10-02, which is delistings, suspensions and dormancy mixed together and not yet separated. (4) At least one security (ASPM.N0000) prints a close outside its own high-low range, so a high &gt;= close &gt;= low validation must run before anything is trusted. Corporate-action and adjustment treatment is UNKNOWN - the endpoint does not state whether prices are adjusted for splits, bonus issues or dividends, and on a market with frequent bonus issues that must be established before returns are computed.</t>
-        </is>
-      </c>
-      <c r="Q23" s="24" t="inlineStr">
-        <is>
-          <t>VERIFIED BY EXTRACTION. Figures in this row are parsed from the committed run log and the files themselves, not from a README or a claim.</t>
-        </is>
-      </c>
-      <c r="R23" s="24" t="inlineStr">
-        <is>
-          <t>A_T and A_L primarily, A_V for per-counter volatility and persistence, and the friction-aware evaluation layer. Effectively the whole quantitative side of the framework.</t>
-        </is>
-      </c>
-      <c r="S23" s="24" t="inlineStr">
-        <is>
-          <t>This is the row that closes the dataset blocker rated 1.5 on 20 September. It is materially better than the figure carried in the Progress Update: 323 securities rather than 270, 14.75 years rather than 10, and it carries turnover and trade count, which were both recorded as missing. Turnover makes Amihud directly computable rather than proxied, so L_t is measurable today. It contains 61 series that stop early, so dead counters are present rather than filtered out - the thin part of the book Sub-gap 1 is about. At a 30-day lookback across the 248 securities with 2,000+ days this is on the order of 480,000 training sequences.</t>
-        </is>
-      </c>
-      <c r="T23" s="24" t="inlineStr">
-        <is>
-          <t>Licence unconfirmed, which is the single largest risk in this matrix because it attaches to the primary dataset. Adjustment status unknown. No bid, ask or depth - that gap is unchanged and is what D23 and the CSE request address. Coverage is uneven enough that any claim stated per-counter must be stated per-tier after D17.</t>
-        </is>
-      </c>
-      <c r="U23" s="24" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="V23" s="24" t="inlineStr">
-        <is>
-          <t>USE - this is the project's primary dataset</t>
-        </is>
-      </c>
-      <c r="W23" s="24" t="inlineStr">
-        <is>
-          <t>Replaces the planning assumptions this matrix was built on. It also reassigns the CSE request: turnover and trade count are no longer needed, so the request narrows to BID/ASK AND DEPTH, DATED LISTING AND DELISTING EVENTS, and WRITTEN CONFIRMATION OF REUSE AND PUBLICATION RIGHTS - the last being the item that now carries the most risk. Freeze this extraction as a versioned snapshot and quote the commit in the proposal, so the experimental universe is reproducible even if the endpoint changes or disappears.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="409.6" customHeight="1">
-      <c r="A24" s="27" t="inlineStr">
-        <is>
-          <t>D23</t>
-        </is>
-      </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>Effective bid-ask spread estimated from OHLC (derived) - LAST RESORT, MAY NEVER BE COMPUTED</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t>Derived dataset</t>
-        </is>
-      </c>
-      <c r="D24" s="28" t="inlineStr">
-        <is>
-          <t>Own computation over D22, following Ardia, Guidotti &amp; Kroencke, Journal of Financial Economics 2024</t>
-        </is>
-      </c>
-      <c r="E24" s="28" t="inlineStr">
-        <is>
-          <t>Grid #61 in the Research Papers Grid; reference implementations are public</t>
-        </is>
-      </c>
-      <c r="F24" s="28" t="inlineStr">
-        <is>
-          <t>CSE, every security in D22 that survives the D17 screen.</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="inlineStr">
-        <is>
-          <t>Derived per-security daily spread estimate. The Level A proxy route for Sub-gap 1.</t>
-        </is>
-      </c>
-      <c r="H24" s="28" t="inlineStr">
-        <is>
-          <t>Same span as D22: 2012-01-02 to 2026-10-02.</t>
-        </is>
-      </c>
-      <c r="I24" s="28" t="inlineStr">
-        <is>
-          <t>Daily, per security.</t>
-        </is>
-      </c>
-      <c r="J24" s="28" t="inlineStr">
-        <is>
-          <t>Not yet computed. Upper bound is the D22 panel.</t>
-        </is>
-      </c>
-      <c r="K24" s="28" t="inlineStr">
-        <is>
-          <t>Estimated effective spread per security-day, from open, high, low and close.</t>
-        </is>
-      </c>
-      <c r="L24" s="28" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="M24" s="28" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="N24" s="28" t="inlineStr">
+      <c r="N15" s="65" t="inlineStr">
         <is>
           <t>One pass over data already held. No external dependency, no permission, no subscription.</t>
         </is>
       </c>
-      <c r="O24" s="28" t="inlineStr">
+      <c r="O15" s="65" t="inlineStr">
         <is>
           <t>n/a - derived. Inherits whatever terms attach to D22.</t>
         </is>
       </c>
-      <c r="P24" s="28" t="inlineStr">
+      <c r="P15" s="65" t="inlineStr">
         <is>
           <t>NOT YET COMPUTED. Three limits to state before relying on it. (1) It estimates the EFFECTIVE spread, not quoted spread and not depth, so it supports a cost model but not a queue-reactive one. (2) Accuracy is known to degrade in thin, frequently non-trading conditions - which is exactly the CSE case this is wanted for, so it must be reported by liquidity tier from D17 rather than pooled. (3) It is an estimate validated on other markets and not on the CSE; it needs checking against real quotes on whatever window can be obtained before any headline result rests on it.
 DECISION CHANGED 11 OCTOBER 2026 - the third limit below is now the governing one rather than one of three. The estimator is UNVALIDATED ON THIN AND FRONTIER MARKETS: the paper's empirical work is CRSP-TAQ US equities plus a Binance section carrying no quote benchmark at all, so no emerging or frontier market appears anywhere in it, and its own numbers put it at its weakest exactly where the CSE sits - 25.63% of daily-price estimates non-positive, 41% of large-cap stock-months negative before truncation, thinnest simulated panel roughly four expected trades per day with no-trade days forward-filled. A monthly window on D22 is about 21 observations, squarely inside that regime. The CSE has no quote data to check the output against, so an estimate produced here could not be falsified even in principle, which is a worse position than having no number because a number invites use.</t>
         </is>
       </c>
-      <c r="Q24" s="28" t="inlineStr">
+      <c r="Q15" s="65" t="inlineStr">
         <is>
           <t>Method verified - peer-reviewed in the Journal of Financial Economics. NOT VERIFIABLE ON THIS MARKET: there is no CSE quote data to validate the estimates against, and that is the reason for the demotion rather than any doubt about the method. The CSE estimates do not exist and may never be computed.</t>
         </is>
       </c>
-      <c r="R24" s="28" t="inlineStr">
+      <c r="R15" s="65" t="inlineStr">
         <is>
           <t>NONE AS OF 11 OCTOBER 2026. Previously A_L and the friction-aware evaluation layer; both now run on the proxies (Amihud, turnover, zero-return frequency, high-low range). If EDGE is ever computed it feeds a sensitivity check, not a component.</t>
         </is>
       </c>
-      <c r="S24" s="28" t="inlineStr">
+      <c r="S15" s="65" t="inlineStr">
         <is>
           <t>Converts the bid-ask gap from a blocker into a validation target. D22 carries open, high, low and close, which is exactly this estimator's input, so the Level A proxy route in the execution model can be built now rather than waiting on the CSE or on a MyCSE subscription. It also gives the CSE request a fallback: if bid/ask is refused, the sub-gap degrades to a proxy-based model with a published method behind it instead of collapsing.
 SUPERSEDED 11 OCTOBER 2026. The argument above still describes what EDGE would give; it is retained as the record of the case for computing it. What it does not weigh is whether the resulting number could be defended, which is the question the demotion turns on.</t>
         </is>
       </c>
-      <c r="T24" s="28" t="inlineStr">
+      <c r="T15" s="65" t="inlineStr">
         <is>
           <t>An estimate, not an observation. Does not provide depth, so the microstructure route (D21) stays closed without real order-book data. Its weakest regime is the thin-counter case the research is most interested in.
 11 OCTOBER 2026: and the weakest regime is not merely the thin-counter case the research is most interested in, it is also the case the paper never validates and this market cannot validate. Those two facts together are what moved the decision.</t>
         </is>
       </c>
-      <c r="U24" s="28" t="n">
+      <c r="U15" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="V24" s="28" t="inlineStr">
+      <c r="V15" s="66" t="inlineStr">
         <is>
           <t>LAST RESORT - DO NOT COMPUTE AS A COMPONENT. May never be computed at all.</t>
         </is>
       </c>
-      <c r="W24" s="28" t="inlineStr">
+      <c r="W15" s="65" t="inlineStr">
         <is>
           <t>DEMOTED 11 OCTOBER 2026, and the demotion does not change what the CSE request is for - it raises its priority. Bid/ask and depth were previously the validation set for an estimator already built; they are now the ONLY route to a measured spread, because the proxy route is not defensible on this market. Until they arrive the cost model runs on proxies and the write-up says so.
 IF EDGE IS COMPUTED AT ALL it is a sensitivity check reported alongside the proxies, never the spread term behind a headline result, and the fraction of non-positive estimates and the per-counter observation count are reported with it every time, because those two numbers are the only visible signal that the estimate came from the regime the paper never validates.
@@ -12503,7 +11587,359 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="207" customHeight="1">
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
+      <c r="B16" s="68" t="inlineStr">
+        <is>
+          <t>CSE Data Library (official statistics bundle, 40 files)</t>
+        </is>
+      </c>
+      <c r="C16" s="68" t="inlineStr">
+        <is>
+          <t>Price &amp; market data / reference</t>
+        </is>
+      </c>
+      <c r="D16" s="68" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange (official, paid)</t>
+        </is>
+      </c>
+      <c r="E16" s="68" t="inlineStr">
+        <is>
+          <t>Order form held in the dataset folder as CSE Data Library.pdf. Tel +94-11-2356525, info@cse.lk</t>
+        </is>
+      </c>
+      <c r="F16" s="68" t="inlineStr">
+        <is>
+          <t>CSE. All listed companies. Corporate actions, indices, sector and market statistics, and daily share price lists 1991 to 2025.</t>
+        </is>
+      </c>
+      <c r="G16" s="68" t="inlineStr">
+        <is>
+          <t>Official reference and corporate-action source. Files supplied by the exchange; format not stated on the order form.</t>
+        </is>
+      </c>
+      <c r="H16" s="68" t="inlineStr">
+        <is>
+          <t>Daily share price lists are split 1991-2000, 2001-2010, 2011-2020 and 2021-2025. The other series are not dated on the form.</t>
+        </is>
+      </c>
+      <c r="I16" s="68" t="inlineStr">
+        <is>
+          <t>Daily, monthly, quarterly and annual depending on the file.</t>
+        </is>
+      </c>
+      <c r="J16" s="68" t="inlineStr">
+        <is>
+          <t>40 numbered files. The ones this project needs: 01 Dividends, 02 Scrip Dividends, 03 Capitalisation of Reserves and Bonus Issues, 04 Rights Issues, 05 Sub Division and Share Splits, 06 New Listings and De-listings, 09 Total Returns Indices Daily, 11 and 12 Market Statistics Daily and Monthly, 16 List of Quoted Securities and Issued Quantity, 17 Public Holding Quarterly, 21 Market Capitalization, 29 Beta Values, 30 to 33 Daily Share Price Lists 1991 to 2025, and 39 GICS Daily. Not needed: 14 and 15 CDS Activities, 18 and 19 debt series, 20, 26, 27, 38 and 40 foreign flow and holding, 28 Closed End Funds, 37 Block Trades, 22 to 25 sector aggregates, and 34 to 36 periodic price summaries.</t>
+        </is>
+      </c>
+      <c r="K16" s="68" t="inlineStr">
+        <is>
+          <t>Daily share price lists plus monthly, quarterly and annual high, low and close summaries. NO BID, NO ASK, NO DEPTH AND NO ORDER BOOK anywhere in the forty items.</t>
+        </is>
+      </c>
+      <c r="L16" s="68" t="inlineStr">
+        <is>
+          <t>English.</t>
+        </is>
+      </c>
+      <c r="M16" s="68" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N16" s="68" t="inlineStr">
+        <is>
+          <t>Paid order form; cash, cheque or bank transfer. Rs 3,500 public for all files; Rs 1,500 for undergraduates of state universities for all files against a valid student ID; Rs 500 for the first selected file and Rs 250 per file thereafter.</t>
+        </is>
+      </c>
+      <c r="O16" s="68" t="inlineStr">
+        <is>
+          <t>Not stated on the order form. Reuse and publication rights must be settled in the same request, since D22's licence is also unconfirmed and this is the opportunity to resolve both at once.</t>
+        </is>
+      </c>
+      <c r="P16" s="68" t="inlineStr">
+        <is>
+          <t>The form does not state file formats, field layouts, or the periods covered by anything other than the daily share price lists. Confirm before depending on a specific field.</t>
+        </is>
+      </c>
+      <c r="Q16" s="68" t="inlineStr">
+        <is>
+          <t>Order form read in full, 18 October 2026. Contents not yet purchased or inspected.</t>
+        </is>
+      </c>
+      <c r="R16" s="68" t="inlineStr">
+        <is>
+          <t>All four indirectly, through D25 and D26. Directly: A_V and the evaluation layer via item 09, A_L via items 16, 17 and 21, and universe construction via items 06 and 39.</t>
+        </is>
+      </c>
+      <c r="S16" s="68" t="inlineStr">
+        <is>
+          <t>The student rate makes the arithmetic one-sided: five selected files already cost Rs 1,500, which is the price of all forty, and this project needs more than five. It is also the only official route to corporate actions, without which D22 cannot be corrected.</t>
+        </is>
+      </c>
+      <c r="T16" s="68" t="inlineStr">
+        <is>
+          <t>IT DOES NOT CLOSE SUB-GAP 1. There is no quote or depth data in any of the forty items, so the measurement half of the cost sub-gap is untouched and the separate CSE request for bid, ask and depth remains the only route to a measured spread.</t>
+        </is>
+      </c>
+      <c r="U16" s="68" t="n">
+        <v>5</v>
+      </c>
+      <c r="V16" s="69" t="inlineStr">
+        <is>
+          <t>BUY - the full set at the student rate</t>
+        </is>
+      </c>
+      <c r="W16" s="68" t="inlineStr">
+        <is>
+          <t>Required rather than optional, because D22 is unadjusted and items 01 to 05 are the only official source of the corporate actions needed to fix it. Everything else in the bundle is effectively free once the student rate is paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="B17" s="71" t="inlineStr">
+        <is>
+          <t>CSE corporate actions register (Data Library items 01 to 05)</t>
+        </is>
+      </c>
+      <c r="C17" s="71" t="inlineStr">
+        <is>
+          <t>Reference data</t>
+        </is>
+      </c>
+      <c r="D17" s="71" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange, supplied within D24</t>
+        </is>
+      </c>
+      <c r="E17" s="71" t="inlineStr">
+        <is>
+          <t>Supplied as part of D24.</t>
+        </is>
+      </c>
+      <c r="F17" s="71" t="inlineStr">
+        <is>
+          <t>CSE. All listed companies.</t>
+        </is>
+      </c>
+      <c r="G17" s="71" t="inlineStr">
+        <is>
+          <t>The adjustment factors. Tabular, event-level.</t>
+        </is>
+      </c>
+      <c r="H17" s="71" t="inlineStr">
+        <is>
+          <t>To be confirmed on delivery. Must reach back to 2012-01-02 at minimum to match D22.</t>
+        </is>
+      </c>
+      <c r="I17" s="71" t="inlineStr">
+        <is>
+          <t>Event-level.</t>
+        </is>
+      </c>
+      <c r="J17" s="71" t="inlineStr">
+        <is>
+          <t>Five files: dividends, scrip dividends, capitalisation of reserves and bonus issues, rights issues, and sub divisions and share splits.</t>
+        </is>
+      </c>
+      <c r="K17" s="71" t="inlineStr">
+        <is>
+          <t>Event dates, ratios and amounts rather than prices.</t>
+        </is>
+      </c>
+      <c r="L17" s="71" t="inlineStr">
+        <is>
+          <t>English.</t>
+        </is>
+      </c>
+      <c r="M17" s="71" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N17" s="71" t="inlineStr">
+        <is>
+          <t>Via D24.</t>
+        </is>
+      </c>
+      <c r="O17" s="71" t="inlineStr">
+        <is>
+          <t>As D24, unconfirmed.</t>
+        </is>
+      </c>
+      <c r="P17" s="71" t="inlineStr">
+        <is>
+          <t>Not yet obtained. Coverage before 2012 is unknown and may not matter. Ex-date against announcement date has to be checked, because adjusting on the wrong date introduces the same spurious return it is meant to remove.</t>
+        </is>
+      </c>
+      <c r="Q17" s="71" t="inlineStr">
+        <is>
+          <t>Not obtained. Identified from the D24 order form, 18 October 2026.</t>
+        </is>
+      </c>
+      <c r="R17" s="71" t="inlineStr">
+        <is>
+          <t>All four indirectly, by way of D26.</t>
+        </is>
+      </c>
+      <c r="S17" s="71" t="inlineStr">
+        <is>
+          <t>The only official source of the adjustment factors, and on current evidence the single highest-value purchase in this matrix.</t>
+        </is>
+      </c>
+      <c r="T17" s="71" t="inlineStr">
+        <is>
+          <t>Useless on its own. Its entire value is in producing D26.</t>
+        </is>
+      </c>
+      <c r="U17" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="V17" s="69" t="inlineStr">
+        <is>
+          <t>OBTAIN - highest priority in the data plan</t>
+        </is>
+      </c>
+      <c r="W17" s="71" t="inlineStr">
+        <is>
+          <t>Without it there is no correct return series, and therefore no trustworthy volatility estimate, Amihud measure, regime split or backtest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
+      <c r="B18" s="68" t="inlineStr">
+        <is>
+          <t>Adjusted per-security daily price and return series (derived)</t>
+        </is>
+      </c>
+      <c r="C18" s="68" t="inlineStr">
+        <is>
+          <t>Derived dataset</t>
+        </is>
+      </c>
+      <c r="D18" s="68" t="inlineStr">
+        <is>
+          <t>Own computation: D22 adjusted by D25</t>
+        </is>
+      </c>
+      <c r="E18" s="68" t="inlineStr">
+        <is>
+          <t>n/a - to be produced.</t>
+        </is>
+      </c>
+      <c r="F18" s="68" t="inlineStr">
+        <is>
+          <t>CSE, the D22 universe.</t>
+        </is>
+      </c>
+      <c r="G18" s="68" t="inlineStr">
+        <is>
+          <t>THE SERIES EVERY DOWNSTREAM COMPONENT SHOULD CONSUME. Per-security daily.</t>
+        </is>
+      </c>
+      <c r="H18" s="68" t="inlineStr">
+        <is>
+          <t>2012-01-02 to 2026-10-02, inherited from D22.</t>
+        </is>
+      </c>
+      <c r="I18" s="68" t="inlineStr">
+        <is>
+          <t>Daily.</t>
+        </is>
+      </c>
+      <c r="J18" s="68" t="inlineStr">
+        <is>
+          <t>As D22: 323 securities and roughly 829,070 security-day observations.</t>
+        </is>
+      </c>
+      <c r="K18" s="68" t="inlineStr">
+        <is>
+          <t>Adjusted open, high, low and close, with unadjusted turnover, share volume and trade count carried alongside, plus the adjustment factor and an event flag per security-day.</t>
+        </is>
+      </c>
+      <c r="L18" s="68" t="inlineStr">
+        <is>
+          <t>n/a.</t>
+        </is>
+      </c>
+      <c r="M18" s="68" t="inlineStr">
+        <is>
+          <t>An event flag marking every security-day that carries a corporate action, so the adjustment is auditable rather than silent.</t>
+        </is>
+      </c>
+      <c r="N18" s="68" t="inlineStr">
+        <is>
+          <t>Own pipeline.</t>
+        </is>
+      </c>
+      <c r="O18" s="68" t="inlineStr">
+        <is>
+          <t>Inherits the unconfirmed licences of D22 and D25.</t>
+        </is>
+      </c>
+      <c r="P18" s="68" t="inlineStr">
+        <is>
+          <t>Does not exist yet. Until it does, every return computed in this project is wrong on corporate-action days.</t>
+        </is>
+      </c>
+      <c r="Q18" s="68" t="inlineStr">
+        <is>
+          <t>CONFIRMED NECESSARY, 18 October 2026, by direct inspection of the staged files: D22 is unadjusted. JKH closes at 212.50 on 2024-10-28 and 21.20 on 2024-11-06, a share split rendered as a -90% return, and AAF shows a +767% move in 2019.</t>
+        </is>
+      </c>
+      <c r="R18" s="68" t="inlineStr">
+        <is>
+          <t>A_T, A_V and A_L directly, the evaluation layer, and the D17 liquidity screen.</t>
+        </is>
+      </c>
+      <c r="S18" s="68" t="inlineStr">
+        <is>
+          <t>Removes a defect that would otherwise contaminate every volatility estimate, every Amihud calculation and every backtest, and would manufacture false regime signals.</t>
+        </is>
+      </c>
+      <c r="T18" s="68" t="inlineStr">
+        <is>
+          <t>Quality is bounded by D25's completeness. Any corporate action missing from D25 survives as a spurious return, so the event flag and an outlier screen should be reported together.</t>
+        </is>
+      </c>
+      <c r="U18" s="68" t="n">
+        <v>5</v>
+      </c>
+      <c r="V18" s="69" t="inlineStr">
+        <is>
+          <t>BUILD - immediately after D25 arrives</t>
+        </is>
+      </c>
+      <c r="W18" s="68" t="inlineStr">
+        <is>
+          <t>This is the dataset the project actually runs on. D22 is the raw input to it rather than a substitute for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="451" customHeight="1"/>
+    <row r="20" ht="207" customHeight="1"/>
+    <row r="21" ht="150" customHeight="1"/>
+    <row r="22" ht="150" customHeight="1"/>
+    <row r="23" ht="409.6" customHeight="1"/>
+    <row r="24" ht="409.6" customHeight="1"/>
   </sheetData>
+  <autoFilter ref="A1:W18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-18 22:16:23
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Consolidated Research Matrix.xlsx
+++ b/FYP/Matrices/Consolidated Research Matrix.xlsx
@@ -9060,7 +9060,7 @@
       </c>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>Per-counter CSE daily price and turnover for L_t; ASPI and S&amp;P SL20 daily closes across the three regimes for P_t and V_t; A_F's retrieval output over CSE annual reports with a publication-date field on every document; and per-agent confidence, which is now specified rather than open (see the Conditioning Set sheet). The cross-sectional reframe changes what depth is needed: at a 30-day lookback with roughly 240 days and a couple of hundred tradable counters the sequence count reaches 40,000 to 50,000, so the sample is the cross-section rather than the history.</t>
+          <t>Per-counter CSE daily price and turnover for L_t; ASPI and S&amp;P SL20 daily closes across the three regimes for P_t and V_t; A_F's retrieval output over CSE annual reports with a publication-date field on every document; and per-agent confidence, which is now specified rather than open (see the Conditioning Set sheet). [CORRECTED 18 OCTOBER 2026] THE DATA-DEPTH POSITION HAS CHANGED AND THIS CELL PREVIOUSLY UNDERSTATED IT BY ROUGHLY A FACTOR OF NINE. The 374-day, February 2025 to February 2026 figure was the Chindara archive and is superseded. The project's own extraction holds 2012-01-02 to 2026-10-02, about 14.75 years, 323 securities and roughly 829,070 security-day observations, with turnover and trade count. At a 30-day lookback that is on the order of 820,000 sequences rather than 40,000 to 50,000. Coverage is uneven, so quote the envelope carefully: the median security carries about 2,935 trading days and the tenth percentile about 1,081. The cross-sectional reframe is therefore a convenience rather than a necessity, and all three regime episodes sit inside the sample. ONE NEW PRECONDITION: the series is not adjusted for corporate actions (a JKH split appears as a -90% return), so the adjusted series has to be built before any of this depth is usable.</t>
         </is>
       </c>
       <c r="J2" s="13" t="inlineStr">
@@ -9071,18 +9071,18 @@
       <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Three weighting schemes, then each state input ablated alone. The Graph-RAG paper supplies the discipline requirement that protects this: its fatal flaw is that the proposed system got both the graph and the agent scaffolding while the baseline got neither, so Baseline 2 has to be identical to the proposed system in every respect except the weighting function, and the ablations move one input at a time. Pre-registered diagnostics: weight-distribution ENTROPY over time, plus a cross-play check. A_F on/off inside the full framework is now required rather than optional, on the precedent that a text channel bolted onto a working structured pipeline cost 10.36 points with nothing able to notice. Report behavioural-fidelity metrics beside returns, equalise trade counts before comparing, report exposure time, holding period and turnover, and commit to dispersion and a paired significance test before seeing numbers.
-PRE-REGISTRATION, ADDED IN V6. Before the first run, record the margin over equal weights and the paired significance test that would count as the state-conditioned weighting having earned its place, together with the direction the forecast combination literature predicts. Both outcomes are reportable: the review states that comprehensive quantitative guidance on when estimated weights beat fixed ones does not yet exist in that literature, so a pre-registered answer on a thin frontier market is a contribution even if the answer is that equal weights win. Record also the absence of a pairwise interaction term as a deliberate choice rather than an oversight, since with four agents an interaction form is ten parameters against four on roughly 374 days, and the combination literature tried that first and moved away from it.</t>
+PRE-REGISTRATION, ADDED IN V6. Before the first run, record the margin over equal weights and the paired significance test that would count as the state-conditioned weighting having earned its place, together with the direction the forecast combination literature predicts. Both outcomes are reportable: the review states that comprehensive quantitative guidance on when estimated weights beat fixed ones does not yet exist in that literature, so a pre-registered answer on a thin frontier market is a contribution even if the answer is that equal weights win. Record also the absence of a pairwise interaction term as a deliberate choice rather than an oversight, since with four agents an interaction form is ten parameters against four. [CORRECTED 18 OCTOBER 2026] The denominator is roughly 3,400 trading days per counter, not the 374 previously recorded here, so ten parameters is no longer self-evidently too many and the omission has to rest on the instability of covariance estimates, which is what Bates and Granger and the authors after them actually argue, rather than on a parameter count.</t>
         </is>
       </c>
       <c r="L2" s="13" t="inlineStr">
         <is>
-          <t>Medium. The orchestrator is small and cheap relative to the agents beneath it, and the capacity constraint argues for keeping it small anyway. The binding constraints have changed since v4: agent confidence is no longer the open problem it was, and the cross-sectional reframe has softened the data-depth constraint, so the sharpest remaining constraint is whether a February 2025 to February 2026 series contains enough regime variation for a state-conditioned weighting to have anything to learn from.</t>
+          <t>Medium. The orchestrator is small and cheap relative to the agents beneath it, and the capacity constraint argues for keeping it small anyway. The binding constraints have changed since v4: agent confidence is no longer the open problem it was, and the cross-sectional reframe has softened the data-depth constraint, so the sharpest remaining constraint is no longer history length. [CORRECTED 18 OCTOBER 2026] The per-counter track is 2012-01-02 to 2026-10-02, not February 2025 to February 2026, and it contains the Easter attacks, COVID and the 2022 crisis, so regime variation is present rather than doubtful. The two binding constraints now are that the series is unadjusted for corporate actions and must be corrected first, and that per-counter coverage is uneven, so eligibility is a per-counter test rather than a blanket one.</t>
         </is>
       </c>
       <c r="M2" s="13" t="inlineStr">
         <is>
           <t>The entropy collapse risk stands and the pre-registered diagnostic stands with it. A second risk is now better defined: with A_F usable less than half the time, the orchestrator may learn to zero it permanently rather than conditionally, in which case the heterogeneity claim survives on paper while the system behaves as a three-agent one, and the weight trajectory around reporting dates is the natural test of whether the mechanism is conditional or merely selective. Third, the regularisation sign-flip observed on a larger dataset than the CSE offers means the orchestrator's own stability has to be swept and reported rather than tuned once. Fourth, the Agentic Trading cutoff means this gap statement has a shelf life and should be re-checked before submission.
-FIFTH, AND ADDED IN V6, THE FORECAST COMBINATION PUZZLE IS THE FIELD'S STANDING PRIOR AGAINST THIS DESIGN AND IT BELONGS IN THE WRITE-UP BEFORE THE RESULTS RATHER THAN AFTER THEM. Elliott bounds the available gain from optimal over equal weights as usually too small to pay for the estimation; Claeskens et al. show estimated weights can introduce bias into a combination of unbiased components and inflate variance past the fixed-weight case; and the probabilistic side reproduces the pattern independently. Everything that literature says about estimation error swamping the gains is worse in my setting, not better, because my components are themselves estimated on short, illiquid and intermittently traded series. The review's own two practical guidelines cut in opposite directions here: with limited historical data it recommends the simple average or weights that ignore covariances, which my roughly 374 trading days per counter argues for, while it also holds that structural change affects sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state. Which effect dominates on CSE data is the empirical question, and a failure to beat equal weights is the expected outcome under the field's prior rather than a surprise.</t>
+FIFTH, AND ADDED IN V6, THE FORECAST COMBINATION PUZZLE IS THE FIELD'S STANDING PRIOR AGAINST THIS DESIGN AND IT BELONGS IN THE WRITE-UP BEFORE THE RESULTS RATHER THAN AFTER THEM. Elliott bounds the available gain from optimal over equal weights as usually too small to pay for the estimation; Claeskens et al. show estimated weights can introduce bias into a combination of unbiased components and inflate variance past the fixed-weight case; and the probabilistic side reproduces the pattern independently. Everything that literature says about estimation error swamping the gains is worse in my setting, not better, because my components are themselves estimated on short, illiquid and intermittently traded series. The review's own two practical guidelines cut in opposite directions here: with limited historical data it recommends the simple average or weights that ignore covariances, which [CORRECTED 18 OCTOBER 2026] was written against a 374-day archive and is weaker than it reads, since the per-counter track is roughly 3,400 trading days; the guideline still bites because the components are themselves estimated on illiquid, intermittently traded series and calendar depth is not effective sample size, but equal weights is no longer favoured by data length alone. The review also holds that structural change affects sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state. Which effect dominates on CSE data is the empirical question, and a failure to beat equal weights is the expected outcome under the field's prior rather than a surprise.</t>
         </is>
       </c>
       <c r="N2" s="42" t="inlineStr">

</xml_diff>